<commit_message>
Cuadro de recursos centralizado y primer bloque de 7 partidas propias validadas
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/catalogo_partidas.xlsx
+++ b/basedatos_partidas/salida/catalogo_partidas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -489,12 +489,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ejemplo - Tabique de placa de yeso 15+70+15</t>
+          <t>Tabique autoportante de placa de yeso laminado 15+70+15.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Tabique autoportante de 100 mm de espesor total, formado por estructura de acero galvanizado de 70 mm y doble placa de yeso laminado de 15 mm a cada cara, con aislamiento de lana mineral. Incluye tratamiento de juntas, replanteo y limpieza.</t>
+          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a suelo y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos a contenedor. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -506,14 +506,242 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>38.5</v>
+        <v>67.11</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Albañilería</t>
+          <t>ALBAÑILERÍA</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DEMOLICIONES</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Demolición de pavimento cerámico existente y su capa de agarre.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de pavimento existente de baldosa cerámica o de gres y de su capa de agarre de mortero, ejecutada con martillo eléctrico manual, sin afectar a la capa de compresión del forjado ni a los elementos constructivos contiguos. Incluye protección previa de los paramentos y elementos que permanecen, control de polvo mediante aspiración, retirada manual de escombro en sacos hasta el punto de acopio y limpieza y barrido de la superficie resultante, dejándola preparada para recibir el nuevo soporte. No incluye el transporte a gestor autorizado, que se valora en su capítulo correspondiente. Medido en superficie realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>DEMOLICIONES</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>REVESTIMIENTOS</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Solado de gres porcelánico 60x60 cm, colocado en capa fina.</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y colocación de pavimento de baldosa de gres porcelánico esmaltado de 60x60 cm y 9 mm de espesor, gama media, sobre soporte previamente regularizado y limpio. Colocación en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido por la propiedad. Incluye replanteo previo para centrar despieces, cortes a inglete en encuentros, limpieza final de la superficie y retirada de restos. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>48.39</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>REVESTIMIENTOS</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>REVESTIMIENTOS</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Solado de gres porcelánico rectificado de gran formato 120x60 cm.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y colocación de pavimento de baldosa de gres porcelánico rectificado de gran formato, 120x60 cm y 10 mm de espesor, gama media. Colocación en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con sistema de ventosas, nivelación con cuñas para garantizar la planitud exigida por el formato y junta mínima de 2 mm rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>76.43000000000001</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>REVESTIMIENTOS</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>REVESTIMIENTOS</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Alicatado de gres porcelánico rectificado 30x90 cm en paramento interior.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y colocación de revestimiento de paramento interior con baldosa de gres porcelánico rectificado de 30x90 cm y 9 mm de espesor, gama media, en baños y cocinas. Colocación en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido, aplicado con llana dentada sobre soporte enfoscado y regularizado, con nivelación mediante crucetas y cuñas y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, ejecución de encuentros y limpieza final. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>60.68</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>REVESTIMIENTOS</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>REVESTIMIENTOS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Rodapié de gres porcelánico 8x60 cm a juego con el pavimento.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y colocación de rodapié de gres porcelánico de 8x60 cm, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los cercos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>11.18</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>REVESTIMIENTOS</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>REVESTIMIENTOS</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Regularización de soporte mediante mortero autonivelante de base cemento CT-C25-F6, de 5 mm de espesor medio, para dejar el soporte en condiciones de planitud aptas para la colocación de pavimento cerámico de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y tiempo de espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>14.21</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>REVESTIMIENTOS</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>incluida</t>
         </is>

</xml_diff>

<commit_message>
Reestructurar catalogo: costes Venezuela en USD, taxonomia jerarquica de 18 capitulos y separacion de productos de eleccion del cliente
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/catalogo_partidas.xlsx
+++ b/basedatos_partidas/salida/catalogo_partidas.xlsx
@@ -484,17 +484,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ALBAÑILERÍA</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tabique autoportante de placa de yeso laminado 15+70+15.</t>
+          <t>Demolición de pavimento cerámico existente y su capa de agarre.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a suelo y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos a contenedor. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Demolición de pavimento existente de baldosa cerámica o de porcelanato y de su capa de agarre de mortero, ejecutada con martillo eléctrico manual, sin afectar a la losa ni a los elementos constructivos contiguos. Incluye protección previa de los paramentos y elementos que permanecen, control de polvo mediante aspiración, retirada manual de escombro en sacos hasta el punto de acopio y limpieza y barrido de la superficie resultante, dejándola preparada para recibir el nuevo soporte. No incluye el transporte a vertedero, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -506,11 +506,11 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>67.11</v>
+        <v>4.62</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>ALBAÑILERÍA</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -522,17 +522,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DEMOLICIONES</t>
+          <t>Fachadas y particiones</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Demolición de pavimento cerámico existente y su capa de agarre.</t>
+          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Demolición de pavimento existente de baldosa cerámica o de gres y de su capa de agarre de mortero, ejecutada con martillo eléctrico manual, sin afectar a la capa de compresión del forjado ni a los elementos constructivos contiguos. Incluye protección previa de los paramentos y elementos que permanecen, control de polvo mediante aspiración, retirada manual de escombro en sacos hasta el punto de acopio y limpieza y barrido de la superficie resultante, dejándola preparada para recibir el nuevo soporte. No incluye el transporte a gestor autorizado, que se valora en su capítulo correspondiente. Medido en superficie realmente demolida.</t>
+          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -544,11 +544,11 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>14.7</v>
+        <v>52.4</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>DEMOLICIONES</t>
+          <t>Tabiquería de entramado autoportante</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -560,17 +560,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>REVESTIMIENTOS</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Solado de gres porcelánico 60x60 cm, colocado en capa fina.</t>
+          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Suministro y colocación de pavimento de baldosa de gres porcelánico esmaltado de 60x60 cm y 9 mm de espesor, gama media, sobre soporte previamente regularizado y limpio. Colocación en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido por la propiedad. Incluye replanteo previo para centrar despieces, cortes a inglete en encuentros, limpieza final de la superficie y retirada de restos. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -582,11 +582,11 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>48.39</v>
+        <v>10.87</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>REVESTIMIENTOS</t>
+          <t>Revestimientos de paramentos con piezas rígidas</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -598,17 +598,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>REVESTIMIENTOS</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Solado de gres porcelánico rectificado de gran formato 120x60 cm.</t>
+          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Suministro y colocación de pavimento de baldosa de gres porcelánico rectificado de gran formato, 120x60 cm y 10 mm de espesor, gama media. Colocación en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con sistema de ventosas, nivelación con cuñas para garantizar la planitud exigida por el formato y junta mínima de 2 mm rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -620,11 +620,11 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>76.43000000000001</v>
+        <v>8.02</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>REVESTIMIENTOS</t>
+          <t>Pavimentos</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -636,33 +636,33 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>REVESTIMIENTOS</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Alicatado de gres porcelánico rectificado 30x90 cm en paramento interior.</t>
+          <t>Colocación de rodapié cerámico o de porcelanato.</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Suministro y colocación de revestimiento de paramento interior con baldosa de gres porcelánico rectificado de 30x90 cm y 9 mm de espesor, gama media, en baños y cocinas. Colocación en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido, aplicado con llana dentada sobre soporte enfoscado y regularizado, con nivelación mediante crucetas y cuñas y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, ejecución de encuentros y limpieza final. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E6" t="n">
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>60.68</v>
+        <v>1.69</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>REVESTIMIENTOS</t>
+          <t>Pavimentos</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -674,33 +674,33 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>REVESTIMIENTOS</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Rodapié de gres porcelánico 8x60 cm a juego con el pavimento.</t>
+          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Suministro y colocación de rodapié de gres porcelánico de 8x60 cm, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los cercos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E7" t="n">
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>11.18</v>
+        <v>9.17</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>REVESTIMIENTOS</t>
+          <t>Pavimentos</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -712,17 +712,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>REVESTIMIENTOS</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Regularización de soporte mediante mortero autonivelante de base cemento CT-C25-F6, de 5 mm de espesor medio, para dejar el soporte en condiciones de planitud aptas para la colocación de pavimento cerámico de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y tiempo de espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -734,11 +734,11 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>14.21</v>
+        <v>12.51</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>REVESTIMIENTOS</t>
+          <t>Pavimentos</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">

</xml_diff>

<commit_message>
Herramienta de actualizacion de precios en bloque y 7 partidas nuevas de pinturas e instalaciones
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/catalogo_partidas.xlsx
+++ b/basedatos_partidas/salida/catalogo_partidas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -560,33 +560,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>10.87</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Revestimientos de paramentos con piezas rígidas</t>
+          <t>Eléctrica</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -598,33 +598,33 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E5" t="n">
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>8.02</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Eléctrica</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -636,17 +636,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -658,11 +658,11 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>1.69</v>
+        <v>7.45</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Fontanería</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -674,33 +674,33 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E7" t="n">
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>9.17</v>
+        <v>11.04</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Saneamiento y desagües</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -717,31 +717,297 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Revestimientos de paramentos con piezas rígidas</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Pinturas</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Pinturas</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Pinturas</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" t="n">
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
         <v>12.51</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Pavimentos</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>incluida</t>
         </is>

</xml_diff>

<commit_message>
13 partidas nuevas: cierra la cadena completa de reforma de bano (demoliciones, friso, cielo raso, puntos de instalacion, sanitarios y residuos)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/catalogo_partidas.xlsx
+++ b/basedatos_partidas/salida/catalogo_partidas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -489,28 +489,28 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Demolición de pavimento cerámico existente y su capa de agarre.</t>
+          <t>Desmontaje de aparato sanitario y su grifería.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Demolición de pavimento existente de baldosa cerámica o de porcelanato y de su capa de agarre de mortero, ejecutada con martillo eléctrico manual, sin afectar a la losa ni a los elementos constructivos contiguos. Incluye protección previa de los paramentos y elementos que permanecen, control de polvo mediante aspiración, retirada manual de escombro en sacos hasta el punto de acopio y limpieza y barrido de la superficie resultante, dejándola preparada para recibir el nuevo soporte. No incluye el transporte a vertedero, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de aparato sanitario existente, ya sea inodoro, lavamanos, bidé o fregadero, junto con su grifería y accesorios de conexión. Incluye cierre previo de la llave de paso y vaciado del aparato, desconexión de las tomas de agua y del desagüe, taponado provisional de las salidas para evitar olores y entrada de escombro, retirada del aparato hasta el punto de acopio y limpieza de la zona. Si el cliente desea conservar el aparato, se desmonta con cuidado y se acopia protegido. No incluye el transporte a vertedero. Medido por unidad desmontada.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E2" t="n">
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>4.62</v>
+        <v>4.55</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -522,17 +522,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fachadas y particiones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
+          <t>Demolición de tabique de bloque o ladrillo, incluidos sus revestimientos.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Demolición de tabique interior no estructural de bloque de concreto o ladrillo, con sus revestimientos por ambas caras, ejecutada con martillo eléctrico manual sin afectar a la estabilidad de los elementos constructivos contiguos. Incluye comprobación previa de que el tabique no es portante y de que no aloja instalaciones en servicio, protección del entorno, apeo puntual si fuera necesario, fragmentación del escombro en piezas manejables, retirada en sacos hasta el punto de acopio y limpieza de la zona. No incluye el transporte a vertedero. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -544,11 +544,11 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>52.4</v>
+        <v>5.42</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Tabiquería de entramado autoportante</t>
+          <t>Particiones</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -560,33 +560,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+          <t>Picado de revestimiento cerámico en paramento y su capa de agarre.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+          <t>Picado de revestimiento cerámico existente en paramento vertical, incluida su capa de agarre de mortero, ejecutado con martillo eléctrico manual hasta dejar el soporte a la vista, sin comprometer la estabilidad del muro ni dañar las instalaciones empotradas. Incluye protección previa de pisos, aparatos y carpintería, control de polvo mediante aspiración, retirada manual de escombro en sacos hasta el punto de acopio y limpieza de la superficie resultante, dejándola preparada para recibir el nuevo friso. No incluye el transporte a vertedero. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>8.369999999999999</v>
+        <v>5.95</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -598,33 +598,33 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+          <t>Demolición de pavimento cerámico existente y su capa de agarre.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+          <t>Demolición de pavimento existente de baldosa cerámica o de porcelanato y de su capa de agarre de mortero, ejecutada con martillo eléctrico manual, sin afectar a la losa ni a los elementos constructivos contiguos. Incluye protección previa de los paramentos y elementos que permanecen, control de polvo mediante aspiración, retirada manual de escombro en sacos hasta el punto de acopio y limpieza y barrido de la superficie resultante, dejándola preparada para recibir el nuevo soporte. No incluye el transporte a vertedero, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E5" t="n">
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>8.720000000000001</v>
+        <v>4.62</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -636,33 +636,33 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+          <t>Demolición de cielo raso y su estructura de soporte.</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+          <t>Demolición de cielo raso existente de yeso, machihembrado o placa, junto con su estructura de soporte y elementos de cuelgue, con medios manuales. Incluye desconexión previa de las luminarias y elementos alojados en el plano del cielo, protección del piso y del mobiliario, retirada de escombro en sacos hasta el punto de acopio y limpieza de la zona, dejando la losa a la vista. No incluye el transporte a vertedero. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E6" t="n">
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>7.45</v>
+        <v>2.37</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Fontanería</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -674,33 +674,33 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Fachadas y particiones</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E7" t="n">
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>11.04</v>
+        <v>52.4</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Saneamiento y desagües</t>
+          <t>Tabiquería de entramado autoportante</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -712,17 +712,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Fachadas y particiones</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+          <t>Tabique de bloque de concreto de 10 cm, recibido con mortero de pega.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Tabique interior no estructural de 10 cm de espesor, ejecutado con bloque hueco de concreto de 10x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Incluye replanteo y trazado sobre el piso, colocación de hiladas a nivel y plomo con la ayuda de reglas y cuerda, formación de huecos de paso, anclaje del tabique a los paramentos existentes, humedecido previo de las piezas y limpieza de restos. No incluye el friso ni los dinteles de los huecos, que se valoran aparte. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -734,11 +734,11 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>10.87</v>
+        <v>18.29</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Revestimientos de paramentos con piezas rígidas</t>
+          <t>Fábrica no estructural</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -750,33 +750,33 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Gestión de residuos</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+          <t>Retirada y transporte de escombro a vertedero autorizado.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Retirada de escombro procedente de demoliciones desde el punto de acopio de la obra y transporte en camión volqueta hasta vertedero o botadero autorizado, incluido el canon de vertido. Incluye la carga manual del escombro sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado con una distancia media considerada de 25 km, la descarga y la limpieza de la zona de carga. Medido por metro cúbico de escombro esponjado realmente retirado.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E9" t="n">
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>3.46</v>
+        <v>16.07</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Pinturas</t>
+          <t>Transporte de residuos</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -788,33 +788,33 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E10" t="n">
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>5.23</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Pinturas</t>
+          <t>Eléctrica</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -826,33 +826,33 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E11" t="n">
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>2.82</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Pinturas</t>
+          <t>Eléctrica</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -864,33 +864,33 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+          <t>Punto de agua fría y caliente para aparato sanitario.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>8.02</v>
+        <v>37.22</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Fontanería</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -902,33 +902,33 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E13" t="n">
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>1.69</v>
+        <v>13.52</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Fontanería</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -940,33 +940,33 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E14" t="n">
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>9.17</v>
+        <v>7.45</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Fontanería</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -978,36 +978,530 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Punto de desagüe para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>33.84</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Saneamiento y desagües</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Saneamiento y desagües</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Revestimientos y trasdosados</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Revestimientos de paramentos con piezas rígidas</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Pinturas</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Pinturas</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Pinturas</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Revestimientos continuos</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>m2</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" t="n">
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="n">
         <v>12.51</v>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>Pavimentos</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Falsos techos</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Señalización y equipamiento</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="n">
+        <v>23.45</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Señalización y equipamiento</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Instalación de lavamanos con su grifería y desagüe.</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="n">
+        <v>36.45</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
         <is>
           <t>incluida</t>
         </is>

</xml_diff>

<commit_message>
Completar grupo DRS de demoliciones de pisos con 16 partidas y anadir informe de cobertura
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/catalogo_partidas.xlsx
+++ b/basedatos_partidas/salida/catalogo_partidas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -603,12 +603,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Demolición de pavimento cerámico existente y su capa de agarre.</t>
+          <t>Demolición de piso cerámico y su capa de pega.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Demolición de pavimento existente de baldosa cerámica o de porcelanato y de su capa de agarre de mortero, ejecutada con martillo eléctrico manual, sin afectar a la losa ni a los elementos constructivos contiguos. Incluye protección previa de los paramentos y elementos que permanecen, control de polvo mediante aspiración, retirada manual de escombro en sacos hasta el punto de acopio y limpieza y barrido de la superficie resultante, dejándola preparada para recibir el nuevo soporte. No incluye el transporte a vertedero, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Demolición de piso existente de baldosa cerámica o de porcelanato, junto con su capa de pega de mortero, ejecutada con martillo eléctrico manual sin comprometer la losa ni los elementos constructivos vecinos. Incluye protección previa de paredes, puertas y ambientes contiguos, control de polvo mediante aspiración, retiro manual del escombro en sacos hasta el punto de acopio y barrido de la superficie resultante, dejándola lista para recibir el nuevo contrapiso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -620,7 +620,7 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>4.62</v>
+        <v>4.88</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -641,24 +641,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Demolición de cielo raso y su estructura de soporte.</t>
+          <t>Demolición de rodapié cerámico.</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Demolición de cielo raso existente de yeso, machihembrado o placa, junto con su estructura de soporte y elementos de cuelgue, con medios manuales. Incluye desconexión previa de las luminarias y elementos alojados en el plano del cielo, protección del piso y del mobiliario, retirada de escombro en sacos hasta el punto de acopio y limpieza de la zona, dejando la losa a la vista. No incluye el transporte a vertedero. Medido en superficie realmente demolida.</t>
+          <t>Demolición de rodapié existente de baldosa cerámica o de porcelanato y de su capa de pega, ejecutada con medios manuales y martillo eléctrico, cuidando de no dañar el friso de la pared por encima de la línea del rodapié. Incluye retiro manual del escombro en sacos hasta el punto de acopio, repicado de los restos de mortero adheridos y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E6" t="n">
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>2.37</v>
+        <v>1</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -674,17 +674,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fachadas y particiones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
+          <t>Demolición de piso de granito o terrazo en baldosa.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Demolición de piso existente de baldosa de granito o terrazo prefabricado, junto con su capa de asiento de mortero, ejecutada con martillo eléctrico manual. Por la dureza y el espesor de este tipo de baldosa el rendimiento es menor que en un piso cerámico y el escombro resulta más pesado, lo que se refleja en el rendimiento de la partida. Incluye protección previa de los ambientes contiguos, control de polvo, retiro manual del escombro en sacos y limpieza de la superficie. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -696,11 +696,11 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>52.4</v>
+        <v>5.9</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Tabiquería de entramado autoportante</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -712,33 +712,33 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Fachadas y particiones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tabique de bloque de concreto de 10 cm, recibido con mortero de pega.</t>
+          <t>Demolición de rodapié de granito o terrazo.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Tabique interior no estructural de 10 cm de espesor, ejecutado con bloque hueco de concreto de 10x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Incluye replanteo y trazado sobre el piso, colocación de hiladas a nivel y plomo con la ayuda de reglas y cuerda, formación de huecos de paso, anclaje del tabique a los paramentos existentes, humedecido previo de las piezas y limpieza de restos. No incluye el friso ni los dinteles de los huecos, que se valoran aparte. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Demolición de rodapié existente de granito o terrazo prefabricado y de su capa de asiento, ejecutada con martillo eléctrico manual, cuidando de no dañar el friso de la pared. Incluye repicado de los restos de mortero adheridos, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E8" t="n">
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>18.29</v>
+        <v>1.17</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Fábrica no estructural</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -750,33 +750,33 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Gestión de residuos</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Retirada y transporte de escombro a vertedero autorizado.</t>
+          <t>Demolición de piso de granito vaciado en sitio.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Retirada de escombro procedente de demoliciones desde el punto de acopio de la obra y transporte en camión volqueta hasta vertedero o botadero autorizado, incluido el canon de vertido. Incluye la carga manual del escombro sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado con una distancia media considerada de 25 km, la descarga y la limpieza de la zona de carga. Medido por metro cúbico de escombro esponjado realmente retirado.</t>
+          <t>Demolición de piso continuo de granito vaciado en sitio, incluida su base de mortero y las platinas divisorias de las juntas, ejecutada con martillo neumático por tratarse de una superficie monolítica de gran dureza. Incluye corte perimetral previo con amoladora de disco de diamante para delimitar la zona de intervención y evitar desprendimientos fuera de ella, protección de los ambientes contiguos, control de polvo, fragmentación del escombro en piezas manejables, retiro en sacos y limpieza. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E9" t="n">
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>16.07</v>
+        <v>13.04</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Transporte de residuos</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -788,33 +788,33 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+          <t>Demolición de piso de cemento pulido.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+          <t>Demolición de piso continuo de cemento pulido y de su base de mortero, ejecutada con martillo eléctrico manual, sin afectar a la losa estructural. Incluye corte perimetral con amoladora cuando la demolición sea parcial, protección de los ambientes contiguos, control de polvo mediante aspiración, fragmentación del escombro, retiro manual en sacos hasta el punto de acopio y limpieza de la superficie resultante. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E10" t="n">
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>8.369999999999999</v>
+        <v>6.92</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -826,33 +826,33 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+          <t>Demolición de rodapié de cemento.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+          <t>Demolición de rodapié corrido de mortero de cemento, ejecutada con medios manuales y cincel, cuidando de no dañar el friso de la pared por encima de la línea del rodapié. Incluye repicado de los restos adheridos al paramento, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E11" t="n">
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>8.720000000000001</v>
+        <v>0.91</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -864,33 +864,33 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+          <t>Demolición de piso de piedra natural.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+          <t>Demolición de piso existente de piedra natural, ya sea mármol, granito natural o laja, junto con su capa de asiento de mortero, ejecutada con martillo eléctrico manual. Si el cliente desea recuperar las piezas, se levantan una a una con cuidado, se limpian de mortero y se acopian protegidas, lo que reduce el rendimiento y debe advertirse en el presupuesto. Incluye protección de los ambientes contiguos, control de polvo, retiro manual del escombro en sacos y limpieza de la superficie. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>37.22</v>
+        <v>6.34</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Fontanería</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -902,33 +902,33 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+          <t>Demolición de rodapié de piedra natural.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+          <t>Demolición de rodapié existente de piedra natural y de su capa de asiento, ejecutada con martillo eléctrico manual, cuidando de no dañar el friso de la pared. Incluye repicado de los restos de mortero adheridos, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E13" t="n">
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>13.52</v>
+        <v>1.25</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Fontanería</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -940,33 +940,33 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+          <t>Levantado de piso de parquet o madera.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+          <t>Levantado de piso existente de parquet o de tablilla de madera, incluidos los rastreles o el adhesivo de fijación al contrapiso, ejecutado con medios manuales mediante palanca y espátula. Incluye el retiro previo de las molduras de remate, el rascado de los restos de adhesivo adheridos al contrapiso, la extracción de los clavos o tornillos que queden en la base, el retiro del material en sacos hasta el punto de acopio y la limpieza de la superficie resultante. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E14" t="n">
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>7.45</v>
+        <v>2.17</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Fontanería</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -978,33 +978,33 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Punto de desagüe para aparato sanitario.</t>
+          <t>Levantado de rodapié de madera.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+          <t>Levantado de rodapié existente de madera, ejecutado con medios manuales mediante palanca y espátula, cuidando de no dañar el friso de la pared. Incluye la extracción de los clavos, tornillos o tacos de fijación que queden en el paramento, el retiro del material en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente levantada.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E15" t="n">
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>33.84</v>
+        <v>0.43</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Saneamiento y desagües</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1016,33 +1016,33 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+          <t>Levantado de piso laminado.</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+          <t>Levantado de piso laminado flotante existente, incluidas la manta acústica y las molduras de remate perimetrales, ejecutado con medios manuales. Por tratarse de un sistema flotante de encastre el desmontaje es rápido y no genera escombro pesado. Incluye el desmontaje ordenado de las tablas, el retiro de la manta y del perfil perimetral, la limpieza y aspirado del contrapiso resultante y el retiro del material en sacos hasta el punto de acopio. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E16" t="n">
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>11.04</v>
+        <v>1.26</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Saneamiento y desagües</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1054,17 +1054,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+          <t>Levantado de piso vinílico, linóleo o alfombra.</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Levantado de revestimiento de piso flexible existente, ya sea vinílico en lámina o baldosa, linóleo o alfombra, incluido el adhesivo de fijación al contrapiso, ejecutado con medios manuales mediante espátula y rasqueta. Incluye la aplicación puntual de disolvente removedor en las zonas donde el adhesivo esté fuertemente adherido, el rascado hasta dejar el contrapiso limpio y sin restos que comprometan la adherencia del nuevo acabado, la ventilación del ambiente durante los trabajos, el retiro del material en sacos y la limpieza final. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1076,11 +1076,11 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>10.87</v>
+        <v>2.12</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Revestimientos de paramentos con piezas rígidas</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1092,17 +1092,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+          <t>Demolición de piso continuo de concreto.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Demolición de piso continuo de concreto de hasta 10 cm de espesor, ejecutada con martillo neumático, sin afectar a la losa estructural ni a las instalaciones que discurran por debajo. Incluye la comprobación previa de que no existen tuberías ni canalizaciones enterradas en la zona, el corte perimetral con amoladora de disco de diamante para delimitar la demolición, la protección de los ambientes contiguos, el control de polvo, la fragmentación del escombro en piezas manejables, el retiro en sacos hasta el punto de acopio y la limpieza. Si el piso está armado con malla electrosoldada se incluye su corte y retiro. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1114,11 +1114,11 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>3.46</v>
+        <v>15.33</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Pinturas</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1130,17 +1130,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+          <t>Demolición de contrapiso o base de mortero de nivelación.</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+          <t>Demolición de contrapiso o base de mortero de nivelación de hasta 5 cm de espesor, una vez retirado el piso de acabado, ejecutada con martillo eléctrico manual hasta dejar la losa estructural a la vista y limpia. Se emplea cuando la base existente está disgregada, hueca o fuera de nivel y no admite recibir el nuevo piso. Incluye la comprobación previa del estado de la base mediante golpeo, la protección de los ambientes contiguos, el control de polvo mediante aspiración, el retiro manual del escombro en sacos y el barrido final de la losa. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1152,11 +1152,11 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>5.23</v>
+        <v>7.18</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Pinturas</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1168,17 +1168,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+          <t>Desmontaje de piso técnico registrable.</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Desmontaje de piso técnico registrable existente, formado por paneles apoyados sobre pedestales regulables, ejecutado con medios manuales. Por tratarse de un sistema desmontable la operación es limpia y permite recuperar el material. Incluye la retirada ordenada de los paneles con ventosa, el desmontaje de los pedestales y travesaños, la clasificación de las piezas en aprovechables y desechables, el acopio protegido de las que el cliente desee conservar, el retiro del resto en sacos y la limpieza de la losa resultante. No incluye el bote del escombro. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1190,11 +1190,11 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>2.82</v>
+        <v>1.09</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Pinturas</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1206,17 +1206,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+          <t>Demolición de cielo raso y su estructura de soporte.</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Demolición de cielo raso existente de yeso, machihembrado o placa, junto con su estructura de soporte y elementos de cuelgue, con medios manuales. Incluye desconexión previa de las luminarias y elementos alojados en el plano del cielo, protección del piso y del mobiliario, retirada de escombro en sacos hasta el punto de acopio y limpieza de la zona, dejando la losa a la vista. No incluye el transporte a vertedero. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1228,11 +1228,11 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>10.75</v>
+        <v>2.37</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Revestimientos continuos</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1244,17 +1244,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Fachadas y particiones</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1266,11 +1266,11 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>8.02</v>
+        <v>52.4</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Tabiquería de entramado autoportante</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1282,33 +1282,33 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Fachadas y particiones</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+          <t>Tabique de bloque de concreto de 10 cm, recibido con mortero de pega.</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+          <t>Tabique interior no estructural de 10 cm de espesor, ejecutado con bloque hueco de concreto de 10x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Incluye replanteo y trazado sobre el piso, colocación de hiladas a nivel y plomo con la ayuda de reglas y cuerda, formación de huecos de paso, anclaje del tabique a los paramentos existentes, humedecido previo de las piezas y limpieza de restos. No incluye el friso ni los dinteles de los huecos, que se valoran aparte. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E23" t="n">
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>1.69</v>
+        <v>18.29</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Fábrica no estructural</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1320,33 +1320,33 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Gestión de residuos</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+          <t>Retirada y transporte de escombro a vertedero autorizado.</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Retirada de escombro procedente de demoliciones desde el punto de acopio de la obra y transporte en camión volqueta hasta vertedero o botadero autorizado, incluido el canon de vertido. Incluye la carga manual del escombro sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado con una distancia media considerada de 25 km, la descarga y la limpieza de la zona de carga. Medido por metro cúbico de escombro esponjado realmente retirado.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E24" t="n">
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>9.17</v>
+        <v>16.07</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Transporte de residuos</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1358,33 +1358,33 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E25" t="n">
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>12.51</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Eléctrica</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1396,33 +1396,33 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E26" t="n">
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>18.47</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Falsos techos</t>
+          <t>Eléctrica</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1434,17 +1434,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Señalización y equipamiento</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+          <t>Punto de agua fría y caliente para aparato sanitario.</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1456,11 +1456,11 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>23.45</v>
+        <v>37.22</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Fontanería</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1472,36 +1472,606 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="n">
+        <v>13.52</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Fontanería</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Fontanería</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Punto de desagüe para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" t="n">
+        <v>33.84</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Saneamiento y desagües</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Saneamiento y desagües</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Revestimientos de paramentos con piezas rígidas</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Pinturas</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Pinturas</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Pinturas</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Revestimientos continuos</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" t="n">
+        <v>12.51</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Falsos techos</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>Señalización y equipamiento</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="n">
+        <v>23.45</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Señalización y equipamiento</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
         <is>
           <t>Instalación de lavamanos con su grifería y desagüe.</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>ud</t>
         </is>
       </c>
-      <c r="E28" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" t="n">
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="n">
         <v>36.45</v>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>Aparatos sanitarios y grifería</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>incluida</t>
         </is>

</xml_diff>

<commit_message>
Cerrar el subcapitulo DR completo: 42 partidas en 8 grupos (pisos, enchapados, frisos, cielos rasos, trasdosados, decorativos, escaleras y fachada)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/catalogo_partidas.xlsx
+++ b/basedatos_partidas/salida/catalogo_partidas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -565,12 +565,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Picado de revestimiento cerámico en paramento y su capa de agarre.</t>
+          <t>Picado de enchapado cerámico en pared y su capa de pega.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Picado de revestimiento cerámico existente en paramento vertical, incluida su capa de agarre de mortero, ejecutado con martillo eléctrico manual hasta dejar el soporte a la vista, sin comprometer la estabilidad del muro ni dañar las instalaciones empotradas. Incluye protección previa de pisos, aparatos y carpintería, control de polvo mediante aspiración, retirada manual de escombro en sacos hasta el punto de acopio y limpieza de la superficie resultante, dejándola preparada para recibir el nuevo friso. No incluye el transporte a vertedero. Medido en superficie realmente picada.</t>
+          <t>Picado de enchapado cerámico o de porcelanato existente en pared, incluida su capa de pega de mortero, ejecutado con martillo eléctrico manual hasta dejar el friso o el bloque a la vista, sin comprometer la estabilidad del muro ni dañar las tuberías y canalizaciones empotradas. Incluye la localización previa de las instalaciones que discurren por el paramento, la protección de pisos, aparatos y puertas, el control de polvo mediante aspiración, el retiro manual del escombro en sacos hasta el punto de acopio y la limpieza de la superficie, dejándola lista para recibir el nuevo friso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -582,7 +582,7 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>5.95</v>
+        <v>6.25</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -603,12 +603,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Demolición de piso cerámico y su capa de pega.</t>
+          <t>Picado de enchapado de granito o terrazo en pared.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso existente de baldosa cerámica o de porcelanato, junto con su capa de pega de mortero, ejecutada con martillo eléctrico manual sin comprometer la losa ni los elementos constructivos vecinos. Incluye protección previa de paredes, puertas y ambientes contiguos, control de polvo mediante aspiración, retiro manual del escombro en sacos hasta el punto de acopio y barrido de la superficie resultante, dejándola lista para recibir el nuevo contrapiso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Picado de enchapado de granito o terrazo prefabricado existente en pared, incluida su capa de asiento de mortero, ejecutado con martillo eléctrico manual. Por el mayor espesor y peso de estas piezas frente al enchapado cerámico, el rendimiento es menor y el escombro más pesado. Incluye la protección de pisos y ambientes contiguos, el control de polvo, el retiro manual del escombro en sacos hasta el punto de acopio y el repicado de los restos de mortero adheridos al paramento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -620,7 +620,7 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>4.88</v>
+        <v>7.31</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -641,24 +641,24 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Demolición de rodapié cerámico.</t>
+          <t>Picado de enchapado de piedra natural en pared.</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Demolición de rodapié existente de baldosa cerámica o de porcelanato y de su capa de pega, ejecutada con medios manuales y martillo eléctrico, cuidando de no dañar el friso de la pared por encima de la línea del rodapié. Incluye retiro manual del escombro en sacos hasta el punto de acopio, repicado de los restos de mortero adheridos y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+          <t>Picado de enchapado de piedra natural existente en pared, ya sea mármol, laja o piedra de revestimiento, incluida su capa de asiento y los anclajes metálicos si los tuviera, ejecutado con martillo eléctrico manual. Si el cliente desea recuperar las piezas se desmontan una a una con cuidado, se limpian y se acopian protegidas, lo que reduce el rendimiento y debe advertirse en el presupuesto. Incluye la protección del entorno, el control de polvo, el retiro del escombro en sacos y el repicado de los restos adheridos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E6" t="n">
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>7.67</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -679,12 +679,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Demolición de piso de granito o terrazo en baldosa.</t>
+          <t>Desmontaje de enchapado de madera o machihembrado en pared.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso existente de baldosa de granito o terrazo prefabricado, junto con su capa de asiento de mortero, ejecutada con martillo eléctrico manual. Por la dureza y el espesor de este tipo de baldosa el rendimiento es menor que en un piso cerámico y el escombro resulta más pesado, lo que se refleja en el rendimiento de la partida. Incluye protección previa de los ambientes contiguos, control de polvo, retiro manual del escombro en sacos y limpieza de la superficie. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de revestimiento de madera existente en pared, ya sea machihembrado, tablilla o panel, junto con los rastreles de soporte fijados al paramento, ejecutado con medios manuales mediante palanca y barra. Incluye la extracción de los clavos, tornillos y tacos que queden en el muro, el retiro del material en sacos o atados hasta el punto de acopio, la clasificación de las piezas aprovechables si el cliente desea conservarlas y la limpieza del paramento resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -696,7 +696,7 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>5.9</v>
+        <v>2.21</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -717,24 +717,24 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Demolición de rodapié de granito o terrazo.</t>
+          <t>Desmontaje de revestimiento de láminas o paneles en pared.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Demolición de rodapié existente de granito o terrazo prefabricado y de su capa de asiento, ejecutada con martillo eléctrico manual, cuidando de no dañar el friso de la pared. Incluye repicado de los restos de mortero adheridos, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+          <t>Desmontaje de revestimiento de pared formado por láminas o paneles de PVC, aluminio, melamina o material similar, junto con su estructura o rastrelado de soporte, ejecutado con medios manuales. Incluye el retiro de los perfiles de remate y esquineros, la extracción de las fijaciones que queden en el paramento, el resane puntual de los huecos de anclaje, el retiro del material hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E8" t="n">
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>1.17</v>
+        <v>1.56</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -755,12 +755,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Demolición de piso de granito vaciado en sitio.</t>
+          <t>Retiro de papel tapiz en paramento.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso continuo de granito vaciado en sitio, incluida su base de mortero y las platinas divisorias de las juntas, ejecutada con martillo neumático por tratarse de una superficie monolítica de gran dureza. Incluye corte perimetral previo con amoladora de disco de diamante para delimitar la zona de intervención y evitar desprendimientos fuera de ella, protección de los ambientes contiguos, control de polvo, fragmentación del escombro en piezas manejables, retiro en sacos y limpieza. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Retiro de papel tapiz existente en paramento interior, junto con los restos de pegamento mural, ejecutado con medios manuales mediante humectación previa con solución reblandecedora y raspado con espátula ancha. Incluye la protección de pisos, rodapiés y mecanismos, la aplicación de la solución en varias pasadas hasta que el papel se desprenda sin arrancar el friso, el rascado de los residuos de pegamento, el lavado final del paramento y su secado, dejándolo listo para recibir el nuevo acabado. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -772,7 +772,7 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>13.04</v>
+        <v>2.2</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -793,24 +793,24 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Demolición de piso de cemento pulido.</t>
+          <t>Desmontaje de moldura decorativa de yeso o poliestireno.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso continuo de cemento pulido y de su base de mortero, ejecutada con martillo eléctrico manual, sin afectar a la losa estructural. Incluye corte perimetral con amoladora cuando la demolición sea parcial, protección de los ambientes contiguos, control de polvo mediante aspiración, fragmentación del escombro, retiro manual en sacos hasta el punto de acopio y limpieza de la superficie resultante. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de moldura decorativa corrida de yeso, poliestireno o poliuretano, situada en el encuentro de pared y cielo raso o como elemento decorativo en paramento, ejecutado con medios manuales mediante espátula y cincel. Incluye la protección del entorno, el corte previo de la línea de junta para evitar arrastrar el friso, el rascado de los restos de pasta o adhesivo, el resane puntual de los desconchados provocados, el retiro del material hasta el punto de acopio y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E10" t="n">
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>6.92</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -831,24 +831,24 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Demolición de rodapié de cemento.</t>
+          <t>Retiro de láminas decorativas, vinilos o espejos adheridos.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Demolición de rodapié corrido de mortero de cemento, ejecutada con medios manuales y cincel, cuidando de no dañar el friso de la pared por encima de la línea del rodapié. Incluye repicado de los restos adheridos al paramento, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+          <t>Retiro de revestimiento decorativo adherido al paramento, ya sea lámina vinílica, calcomanía mural o espejo pegado, junto con los restos de adhesivo. Incluye la protección del piso y del mobiliario, el calentamiento o humectación previa para reblandecer el adhesivo, el desprendimiento controlado del material con espátula, y en el caso de espejos el encintado previo de la superficie para evitar la proyección de fragmentos al fracturarse. Incluye el rascado de los restos de adhesivo, el retiro del material en sacos y la limpieza del paramento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E11" t="n">
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>0.91</v>
+        <v>1.6</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -869,12 +869,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Demolición de piso de piedra natural.</t>
+          <t>Demolición de revestimiento cerámico de escalera.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso existente de piedra natural, ya sea mármol, granito natural o laja, junto con su capa de asiento de mortero, ejecutada con martillo eléctrico manual. Si el cliente desea recuperar las piezas, se levantan una a una con cuidado, se limpian de mortero y se acopian protegidas, lo que reduce el rendimiento y debe advertirse en el presupuesto. Incluye protección de los ambientes contiguos, control de polvo, retiro manual del escombro en sacos y limpieza de la superficie. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Demolición del revestimiento cerámico de escalera, comprendiendo huellas, contrahuellas y su capa de pega, ejecutada con martillo eléctrico manual sin comprometer la losa de la escalera. El rendimiento es sensiblemente menor que en un piso corrido por la posición forzada de trabajo, la superficie fragmentada en peldaños y la dificultad de evacuar el escombro por la propia escalera. Incluye la protección del hueco y del pasamanos, el control de polvo, el retiro manual del escombro en sacos y la limpieza, dejando los peldaños listos para el nuevo revestimiento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida, desarrollando huella y contrahuella.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -886,7 +886,7 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>6.34</v>
+        <v>7.27</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -907,24 +907,24 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Demolición de rodapié de piedra natural.</t>
+          <t>Demolición de revestimiento de granito o piedra natural en escalera.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Demolición de rodapié existente de piedra natural y de su capa de asiento, ejecutada con martillo eléctrico manual, cuidando de no dañar el friso de la pared. Incluye repicado de los restos de mortero adheridos, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+          <t>Demolición del revestimiento de granito, terrazo o piedra natural de escalera, comprendiendo huellas, contrahuellas y su capa de asiento, ejecutada con martillo eléctrico manual. Al mayor espesor y peso de las piezas se suma la dificultad propia del trabajo en escalera, por lo que el rendimiento es el más bajo de los grupos de demolición de revestimientos. Incluye la protección del hueco y del pasamanos, el control de polvo, el retiro manual del escombro en sacos y el repicado de los restos de mortero adheridos a los peldaños. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida, desarrollando huella y contrahuella.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E13" t="n">
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>1.25</v>
+        <v>8.58</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -945,24 +945,24 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Levantado de piso de parquet o madera.</t>
+          <t>Demolición de zócalo escalonado de escalera.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Levantado de piso existente de parquet o de tablilla de madera, incluidos los rastreles o el adhesivo de fijación al contrapiso, ejecutado con medios manuales mediante palanca y espátula. Incluye el retiro previo de las molduras de remate, el rascado de los restos de adhesivo adheridos al contrapiso, la extracción de los clavos o tornillos que queden en la base, el retiro del material en sacos hasta el punto de acopio y la limpieza de la superficie resultante. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
+          <t>Demolición del zócalo o rodapié escalonado que acompaña a la escalera en su encuentro con el paramento, incluida su capa de pega, ejecutada con medios manuales y martillo eléctrico, cuidando de no dañar el friso por encima de la línea del zócalo. Incluye el repicado de los restos de mortero adheridos, el retiro del escombro en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud real de la línea inclinada del zócalo.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E14" t="n">
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>2.17</v>
+        <v>1.78</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -983,24 +983,24 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Levantado de rodapié de madera.</t>
+          <t>Picado de friso de mortero en paramento.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Levantado de rodapié existente de madera, ejecutado con medios manuales mediante palanca y espátula, cuidando de no dañar el friso de la pared. Incluye la extracción de los clavos, tornillos o tacos de fijación que queden en el paramento, el retiro del material en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente levantada.</t>
+          <t>Picado de friso de mortero de cemento existente en paramento interior o exterior, ejecutado con martillo eléctrico manual hasta dejar el bloque o el ladrillo a la vista, cuando el friso está disgregado, hueco o presenta fisuración generalizada. Incluye el sondeo previo por golpeo para delimitar las zonas sin adherencia, la protección de pisos y ambientes contiguos, el control de polvo mediante aspiración, el retiro manual del escombro en sacos hasta el punto de acopio y el barrido y limpieza del paramento, dejándolo listo para recibir el nuevo friso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E15" t="n">
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>0.43</v>
+        <v>5.86</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1021,12 +1021,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Levantado de piso laminado.</t>
+          <t>Picado de friso de yeso o pasta en paramento.</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Levantado de piso laminado flotante existente, incluidas la manta acústica y las molduras de remate perimetrales, ejecutado con medios manuales. Por tratarse de un sistema flotante de encastre el desmontaje es rápido y no genera escombro pesado. Incluye el desmontaje ordenado de las tablas, el retiro de la manta y del perfil perimetral, la limpieza y aspirado del contrapiso resultante y el retiro del material en sacos hasta el punto de acopio. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
+          <t>Picado de revestimiento de yeso o pasta existente en paramento interior, ejecutado con medios manuales mediante espátula ancha y cincel, con martillo eléctrico solo en las zonas de mayor espesor. Por tratarse de un material blando el rendimiento es sensiblemente mayor que en un friso de mortero, aunque genera abundante polvo fino. Incluye la protección del entorno, el control de polvo mediante aspiración continua, el retiro del escombro en sacos hasta el punto de acopio y la limpieza del paramento resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1038,7 +1038,7 @@
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>1.26</v>
+        <v>3.65</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1059,12 +1059,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Levantado de piso vinílico, linóleo o alfombra.</t>
+          <t>Picado de estuco o pasta decorativa en paramento.</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Levantado de revestimiento de piso flexible existente, ya sea vinílico en lámina o baldosa, linóleo o alfombra, incluido el adhesivo de fijación al contrapiso, ejecutado con medios manuales mediante espátula y rasqueta. Incluye la aplicación puntual de disolvente removedor en las zonas donde el adhesivo esté fuertemente adherido, el rascado hasta dejar el contrapiso limpio y sin restos que comprometan la adherencia del nuevo acabado, la ventilación del ambiente durante los trabajos, el retiro del material en sacos y la limpieza final. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
+          <t>Picado de revestimiento de estuco, pasta decorativa o revestimiento texturado existente en paramento, ejecutado con medios manuales y martillo eléctrico según el espesor y la dureza del material, hasta dejar el soporte limpio y apto para recibir el nuevo acabado. Incluye la cata previa para identificar el espesor y el tipo de soporte, la protección del entorno, el control de polvo, el retiro del escombro en sacos y la limpieza final. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1076,7 +1076,7 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>2.12</v>
+        <v>4.3</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1097,12 +1097,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Demolición de piso continuo de concreto.</t>
+          <t>Repicado de superficie de concreto para mejorar adherencia.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso continuo de concreto de hasta 10 cm de espesor, ejecutada con martillo neumático, sin afectar a la losa estructural ni a las instalaciones que discurran por debajo. Incluye la comprobación previa de que no existen tuberías ni canalizaciones enterradas en la zona, el corte perimetral con amoladora de disco de diamante para delimitar la demolición, la protección de los ambientes contiguos, el control de polvo, la fragmentación del escombro en piezas manejables, el retiro en sacos hasta el punto de acopio y la limpieza. Si el piso está armado con malla electrosoldada se incluye su corte y retiro. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Repicado superficial de paramento o losa de concreto, ejecutado con martillo eléctrico y puntero, para crear la rugosidad necesaria que garantice la adherencia del friso o del mortero de recrecido posterior. Incluye la limpieza previa de la superficie, el picado uniforme sin llegar a descubrir la armadura, la eliminación de lechadas superficiales y restos de desencofrante, el soplado y aspirado del polvo resultante y la retirada de los restos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente repicada.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1114,7 +1114,7 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>15.33</v>
+        <v>4.37</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1135,12 +1135,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Demolición de contrapiso o base de mortero de nivelación.</t>
+          <t>Eliminación de pintura en paramento mediante raspado y decapado.</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Demolición de contrapiso o base de mortero de nivelación de hasta 5 cm de espesor, una vez retirado el piso de acabado, ejecutada con martillo eléctrico manual hasta dejar la losa estructural a la vista y limpia. Se emplea cuando la base existente está disgregada, hueca o fuera de nivel y no admite recibir el nuevo piso. Incluye la comprobación previa del estado de la base mediante golpeo, la protección de los ambientes contiguos, el control de polvo mediante aspiración, el retiro manual del escombro en sacos y el barrido final de la losa. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Eliminación de las capas de pintura existentes en paramento interior o exterior, mediante raspado mecánico con espátula y lijado, con aplicación puntual de decapante químico en gel en las zonas de pintura muy adherida o de espesor elevado. Se emplea cuando la pintura existente está cuarteada, sopla o es incompatible con el nuevo acabado. Incluye la protección de pisos, carpintería y mobiliario, la ventilación del ambiente durante la aplicación del decapante, la neutralización y lavado de los restos químicos, el aspirado del polvo y la retirada de los residuos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1152,7 +1152,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>7.18</v>
+        <v>5.15</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1173,12 +1173,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Desmontaje de piso técnico registrable.</t>
+          <t>Picado de salpicado o graniplast en fachada.</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de piso técnico registrable existente, formado por paneles apoyados sobre pedestales regulables, ejecutado con medios manuales. Por tratarse de un sistema desmontable la operación es limpia y permite recuperar el material. Incluye la retirada ordenada de los paneles con ventosa, el desmontaje de los pedestales y travesaños, la clasificación de las piezas en aprovechables y desechables, el acopio protegido de las que el cliente desee conservar, el retiro del resto en sacos y la limpieza de la losa resultante. No incluye el bote del escombro. Medido en superficie realmente desmontada.</t>
+          <t>Picado de revestimiento de salpicado, graniplast o revestimiento pétreo proyectado en fachada, ejecutado con martillo eléctrico manual y espátula, hasta dejar el friso base sano o el bloque a la vista según el estado del soporte. Incluye el sondeo previo por golpeo para delimitar las zonas sin adherencia, el trabajo desde andamio con las protecciones colectivas correspondientes, la protección de carpinterías y de la zona de paso a pie de fachada, el control de la caída de escombro, su retiro en sacos hasta el punto de acopio y la limpieza del paramento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1190,7 +1190,7 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>1.09</v>
+        <v>7.11</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1211,12 +1211,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Demolición de cielo raso y su estructura de soporte.</t>
+          <t>Picado de mortero monocapa en fachada.</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Demolición de cielo raso existente de yeso, machihembrado o placa, junto con su estructura de soporte y elementos de cuelgue, con medios manuales. Incluye desconexión previa de las luminarias y elementos alojados en el plano del cielo, protección del piso y del mobiliario, retirada de escombro en sacos hasta el punto de acopio y limpieza de la zona, dejando la losa a la vista. No incluye el transporte a vertedero. Medido en superficie realmente demolida.</t>
+          <t>Picado de revestimiento de mortero monocapa en fachada, incluida su malla de refuerzo y los perfiles de arranque y goterón, ejecutado con martillo eléctrico manual hasta dejar el soporte limpio y apto para recibir el nuevo revestimiento. Incluye el sondeo previo del paramento, el trabajo desde andamio con las protecciones colectivas correspondientes, la protección de carpinterías y del paso a pie de fachada, el corte y retiro de la malla, el control de la caída de escombro, su retiro en sacos y la limpieza del soporte. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1228,7 +1228,7 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>2.37</v>
+        <v>8.02</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1244,17 +1244,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Fachadas y particiones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
+          <t>Demolición de trasdosado de yeso laminado y su estructura.</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Demolición de trasdosado autoportante de placa de yeso laminado adosado a muro, junto con la perfilería de acero galvanizado y el aislamiento alojado en la cámara, ejecutada con medios manuales. Incluye la localización y desconexión previa de los mecanismos e instalaciones que discurran por el trasdosado, la protección del piso y del mobiliario, el desmontaje ordenado de las placas, el retiro del aislamiento en sacos, el desmontaje de la perfilería y de las fijaciones al muro, y la limpieza de la zona dejando el paramento original a la vista. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1266,11 +1266,11 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>52.4</v>
+        <v>2.56</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Tabiquería de entramado autoportante</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1282,17 +1282,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Fachadas y particiones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Tabique de bloque de concreto de 10 cm, recibido con mortero de pega.</t>
+          <t>Demolición de trasdosado de bloque o ladrillo adosado a muro.</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Tabique interior no estructural de 10 cm de espesor, ejecutado con bloque hueco de concreto de 10x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Incluye replanteo y trazado sobre el piso, colocación de hiladas a nivel y plomo con la ayuda de reglas y cuerda, formación de huecos de paso, anclaje del tabique a los paramentos existentes, humedecido previo de las piezas y limpieza de restos. No incluye el friso ni los dinteles de los huecos, que se valoran aparte. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Demolición de tabique de bloque o ladrillo adosado a muro a modo de trasdosado, incluidos sus revestimientos y la cámara intermedia, ejecutada con martillo eléctrico manual sin dañar el muro original que permanece. Incluye la comprobación previa de que el trasdosado no cumple función estructural ni aloja instalaciones en servicio, la protección del entorno, el control de polvo, la fragmentación del escombro en piezas manejables, el retiro en sacos hasta el punto de acopio y el repicado de los restos de mortero adheridos al muro. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1304,11 +1304,11 @@
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>18.29</v>
+        <v>6.21</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Fábrica no estructural</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1320,33 +1320,33 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Gestión de residuos</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Retirada y transporte de escombro a vertedero autorizado.</t>
+          <t>Desmontaje de trasdosado directo de placa pegada al muro.</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Retirada de escombro procedente de demoliciones desde el punto de acopio de la obra y transporte en camión volqueta hasta vertedero o botadero autorizado, incluido el canon de vertido. Incluye la carga manual del escombro sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado con una distancia media considerada de 25 km, la descarga y la limpieza de la zona de carga. Medido por metro cúbico de escombro esponjado realmente retirado.</t>
+          <t>Desmontaje de trasdosado directo formado por placa de yeso laminado o panel aislante adherido al muro mediante pelladas de pasta, ejecutado con medios manuales mediante palanca y espátula. Incluye la protección del piso, el arranque de las placas, el rascado de los restos de pasta y adhesivo adheridos al muro hasta dejarlo apto para recibir el nuevo revestimiento, el retiro del material en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E24" t="n">
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>16.07</v>
+        <v>3.12</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Transporte de residuos</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1358,33 +1358,33 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+          <t>Demolición de piso cerámico y su capa de pega.</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+          <t>Demolición de piso existente de baldosa cerámica o de porcelanato, junto con su capa de pega de mortero, ejecutada con martillo eléctrico manual sin comprometer la losa ni los elementos constructivos vecinos. Incluye protección previa de paredes, puertas y ambientes contiguos, control de polvo mediante aspiración, retiro manual del escombro en sacos hasta el punto de acopio y barrido de la superficie resultante, dejándola lista para recibir el nuevo contrapiso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E25" t="n">
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>8.369999999999999</v>
+        <v>4.88</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1396,33 +1396,33 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+          <t>Demolición de rodapié cerámico.</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+          <t>Demolición de rodapié existente de baldosa cerámica o de porcelanato y de su capa de pega, ejecutada con medios manuales y martillo eléctrico, cuidando de no dañar el friso de la pared por encima de la línea del rodapié. Incluye retiro manual del escombro en sacos hasta el punto de acopio, repicado de los restos de mortero adheridos y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E26" t="n">
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>8.720000000000001</v>
+        <v>1</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1434,33 +1434,33 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+          <t>Demolición de piso de granito o terrazo en baldosa.</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+          <t>Demolición de piso existente de baldosa de granito o terrazo prefabricado, junto con su capa de asiento de mortero, ejecutada con martillo eléctrico manual. Por la dureza y el espesor de este tipo de baldosa el rendimiento es menor que en un piso cerámico y el escombro resulta más pesado, lo que se refleja en el rendimiento de la partida. Incluye protección previa de los ambientes contiguos, control de polvo, retiro manual del escombro en sacos y limpieza de la superficie. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E27" t="n">
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>37.22</v>
+        <v>5.9</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Fontanería</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1472,33 +1472,33 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+          <t>Demolición de rodapié de granito o terrazo.</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+          <t>Demolición de rodapié existente de granito o terrazo prefabricado y de su capa de asiento, ejecutada con martillo eléctrico manual, cuidando de no dañar el friso de la pared. Incluye repicado de los restos de mortero adheridos, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E28" t="n">
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>13.52</v>
+        <v>1.17</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Fontanería</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1510,33 +1510,33 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+          <t>Demolición de piso de granito vaciado en sitio.</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+          <t>Demolición de piso continuo de granito vaciado en sitio, incluida su base de mortero y las platinas divisorias de las juntas, ejecutada con martillo neumático por tratarse de una superficie monolítica de gran dureza. Incluye corte perimetral previo con amoladora de disco de diamante para delimitar la zona de intervención y evitar desprendimientos fuera de ella, protección de los ambientes contiguos, control de polvo, fragmentación del escombro en piezas manejables, retiro en sacos y limpieza. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E29" t="n">
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>7.45</v>
+        <v>13.04</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Fontanería</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1548,33 +1548,33 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Punto de desagüe para aparato sanitario.</t>
+          <t>Demolición de piso de cemento pulido.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+          <t>Demolición de piso continuo de cemento pulido y de su base de mortero, ejecutada con martillo eléctrico manual, sin afectar a la losa estructural. Incluye corte perimetral con amoladora cuando la demolición sea parcial, protección de los ambientes contiguos, control de polvo mediante aspiración, fragmentación del escombro, retiro manual en sacos hasta el punto de acopio y limpieza de la superficie resultante. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E30" t="n">
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>33.84</v>
+        <v>6.92</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Saneamiento y desagües</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1586,17 +1586,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+          <t>Demolición de rodapié de cemento.</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+          <t>Demolición de rodapié corrido de mortero de cemento, ejecutada con medios manuales y cincel, cuidando de no dañar el friso de la pared por encima de la línea del rodapié. Incluye repicado de los restos adheridos al paramento, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1608,11 +1608,11 @@
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>11.04</v>
+        <v>0.91</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Saneamiento y desagües</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1624,17 +1624,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+          <t>Demolición de piso de piedra natural.</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Demolición de piso existente de piedra natural, ya sea mármol, granito natural o laja, junto con su capa de asiento de mortero, ejecutada con martillo eléctrico manual. Si el cliente desea recuperar las piezas, se levantan una a una con cuidado, se limpian de mortero y se acopian protegidas, lo que reduce el rendimiento y debe advertirse en el presupuesto. Incluye protección de los ambientes contiguos, control de polvo, retiro manual del escombro en sacos y limpieza de la superficie. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1646,11 +1646,11 @@
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>10.87</v>
+        <v>6.34</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Revestimientos de paramentos con piezas rígidas</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1662,33 +1662,33 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+          <t>Demolición de rodapié de piedra natural.</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Demolición de rodapié existente de piedra natural y de su capa de asiento, ejecutada con martillo eléctrico manual, cuidando de no dañar el friso de la pared. Incluye repicado de los restos de mortero adheridos, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E33" t="n">
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>3.46</v>
+        <v>1.25</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Pinturas</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1700,17 +1700,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+          <t>Levantado de piso de parquet o madera.</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+          <t>Levantado de piso existente de parquet o de tablilla de madera, incluidos los rastreles o el adhesivo de fijación al contrapiso, ejecutado con medios manuales mediante palanca y espátula. Incluye el retiro previo de las molduras de remate, el rascado de los restos de adhesivo adheridos al contrapiso, la extracción de los clavos o tornillos que queden en la base, el retiro del material en sacos hasta el punto de acopio y la limpieza de la superficie resultante. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1722,11 +1722,11 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>5.23</v>
+        <v>2.17</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Pinturas</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1738,33 +1738,33 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+          <t>Levantado de rodapié de madera.</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Levantado de rodapié existente de madera, ejecutado con medios manuales mediante palanca y espátula, cuidando de no dañar el friso de la pared. Incluye la extracción de los clavos, tornillos o tacos de fijación que queden en el paramento, el retiro del material en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente levantada.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E35" t="n">
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>2.82</v>
+        <v>0.43</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Pinturas</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1776,17 +1776,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+          <t>Levantado de piso laminado.</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Levantado de piso laminado flotante existente, incluidas la manta acústica y las molduras de remate perimetrales, ejecutado con medios manuales. Por tratarse de un sistema flotante de encastre el desmontaje es rápido y no genera escombro pesado. Incluye el desmontaje ordenado de las tablas, el retiro de la manta y del perfil perimetral, la limpieza y aspirado del contrapiso resultante y el retiro del material en sacos hasta el punto de acopio. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1798,11 +1798,11 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>10.75</v>
+        <v>1.26</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Revestimientos continuos</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1814,17 +1814,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+          <t>Levantado de piso vinílico, linóleo o alfombra.</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+          <t>Levantado de revestimiento de piso flexible existente, ya sea vinílico en lámina o baldosa, linóleo o alfombra, incluido el adhesivo de fijación al contrapiso, ejecutado con medios manuales mediante espátula y rasqueta. Incluye la aplicación puntual de disolvente removedor en las zonas donde el adhesivo esté fuertemente adherido, el rascado hasta dejar el contrapiso limpio y sin restos que comprometan la adherencia del nuevo acabado, la ventilación del ambiente durante los trabajos, el retiro del material en sacos y la limpieza final. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1836,11 +1836,11 @@
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>8.02</v>
+        <v>2.12</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1852,33 +1852,33 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+          <t>Demolición de piso continuo de concreto.</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+          <t>Demolición de piso continuo de concreto de hasta 10 cm de espesor, ejecutada con martillo neumático, sin afectar a la losa estructural ni a las instalaciones que discurran por debajo. Incluye la comprobación previa de que no existen tuberías ni canalizaciones enterradas en la zona, el corte perimetral con amoladora de disco de diamante para delimitar la demolición, la protección de los ambientes contiguos, el control de polvo, la fragmentación del escombro en piezas manejables, el retiro en sacos hasta el punto de acopio y la limpieza. Si el piso está armado con malla electrosoldada se incluye su corte y retiro. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E38" t="n">
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>1.69</v>
+        <v>15.33</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -1890,17 +1890,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+          <t>Demolición de contrapiso o base de mortero de nivelación.</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Demolición de contrapiso o base de mortero de nivelación de hasta 5 cm de espesor, una vez retirado el piso de acabado, ejecutada con martillo eléctrico manual hasta dejar la losa estructural a la vista y limpia. Se emplea cuando la base existente está disgregada, hueca o fuera de nivel y no admite recibir el nuevo piso. Incluye la comprobación previa del estado de la base mediante golpeo, la protección de los ambientes contiguos, el control de polvo mediante aspiración, el retiro manual del escombro en sacos y el barrido final de la losa. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1912,11 +1912,11 @@
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>9.17</v>
+        <v>7.18</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1928,17 +1928,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+          <t>Desmontaje de piso técnico registrable.</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Desmontaje de piso técnico registrable existente, formado por paneles apoyados sobre pedestales regulables, ejecutado con medios manuales. Por tratarse de un sistema desmontable la operación es limpia y permite recuperar el material. Incluye la retirada ordenada de los paneles con ventosa, el desmontaje de los pedestales y travesaños, la clasificación de las piezas en aprovechables y desechables, el acopio protegido de las que el cliente desee conservar, el retiro del resto en sacos y la limpieza de la losa resultante. No incluye el bote del escombro. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1950,11 +1950,11 @@
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>12.51</v>
+        <v>1.09</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -1966,17 +1966,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+          <t>Demolición de cielo raso de yeso laminado y su estructura.</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+          <t>Demolición de cielo raso continuo de placa de yeso laminado, junto con la perfilería de acero galvanizado, las varillas de cuelgue y el ángulo perimetral, ejecutada con medios manuales. Incluye la desconexión y retiro previo de las luminarias, rejillas y difusores alojados en el plano del cielo, la protección del piso y del mobiliario, el descuelgue ordenado de las placas para evitar caídas incontroladas, el retiro del escombro en sacos y de la perfilería atada, y la limpieza de la zona dejando la losa a la vista. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1988,11 +1988,11 @@
         <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>18.47</v>
+        <v>2.69</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Falsos techos</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2004,33 +2004,33 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Señalización y equipamiento</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+          <t>Demolición de cielo raso de yeso vaciado o pasta.</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+          <t>Demolición de cielo raso de yeso vaciado, pasta o placa de yeso tradicional, junto con su estructura de soporte y elementos de cuelgue, ejecutada con medios manuales y martillo eléctrico donde el espesor lo requiera. Por tratarse de un material macizo genera más escombro y más polvo fino que un cielo de placa. Incluye la desconexión previa de las luminarias, la protección del piso y del mobiliario, el control de polvo mediante aspiración, el retiro del escombro en sacos y la limpieza de la losa resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E42" t="n">
         <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>23.45</v>
+        <v>4.91</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2042,36 +2042,948 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Desmontaje de cielo raso desmontable de fibra mineral.</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Desmontaje de cielo raso registrable existente, formado por paneles apoyados sobre perfilería vista en retícula, ejecutado con medios manuales. Por ser un sistema desmontable la operación es limpia, rápida y permite recuperar buena parte del material. Incluye la retirada ordenada de los paneles, el desmontaje de la perfilería y de los tensores de cuelgue, la clasificación de las piezas en aprovechables y desechables, el acopio protegido de las que el cliente desee conservar y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Desmontaje de cielo raso de machihembrado de madera.</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Desmontaje de cielo raso de machihembrado o tablilla de madera, junto con los rastreles y la estructura de soporte fijada a la losa, ejecutado con medios manuales mediante palanca y barra. Incluye la desconexión previa de las luminarias, la protección del piso y del mobiliario, la extracción de los clavos y tornillos que queden en la estructura, el retiro del material en atados hasta el punto de acopio, la clasificación de las piezas aprovechables y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Desmontaje de cielo raso de láminas de PVC o aluminio.</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Desmontaje de cielo raso formado por láminas de PVC, aluminio o material similar, junto con sus perfiles de soporte y remates perimetrales, ejecutado con medios manuales. Incluye la desconexión previa de las luminarias y rejillas, la protección del piso, el desencastre ordenado de las láminas para poder recuperarlas si el cliente lo desea, el desmontaje de la perfilería, el retiro del material hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Fachadas y particiones</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Tabiquería de entramado autoportante</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Fachadas y particiones</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Tabique de bloque de concreto de 10 cm, recibido con mortero de pega.</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>Tabique interior no estructural de 10 cm de espesor, ejecutado con bloque hueco de concreto de 10x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Incluye replanteo y trazado sobre el piso, colocación de hiladas a nivel y plomo con la ayuda de reglas y cuerda, formación de huecos de paso, anclaje del tabique a los paramentos existentes, humedecido previo de las piezas y limpieza de restos. No incluye el friso ni los dinteles de los huecos, que se valoran aparte. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" t="n">
+        <v>18.29</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Fábrica no estructural</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Gestión de residuos</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Retirada y transporte de escombro a vertedero autorizado.</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Retirada de escombro procedente de demoliciones desde el punto de acopio de la obra y transporte en camión volqueta hasta vertedero o botadero autorizado, incluido el canon de vertido. Incluye la carga manual del escombro sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado con una distancia media considerada de 25 km, la descarga y la limpieza de la zona de carga. Medido por metro cúbico de escombro esponjado realmente retirado.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" t="n">
+        <v>16.07</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Transporte de residuos</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" t="n">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Eléctrica</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" t="n">
+        <v>8.720000000000001</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Eléctrica</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" t="n">
+        <v>37.22</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Fontanería</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" t="n">
+        <v>13.52</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Fontanería</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Fontanería</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Punto de desagüe para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" t="n">
+        <v>33.84</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Saneamiento y desagües</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Saneamiento y desagües</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Revestimientos de paramentos con piezas rígidas</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Pinturas</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Pinturas</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Pinturas</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Revestimientos continuos</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F63" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" t="n">
+        <v>12.51</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Falsos techos</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
           <t>Señalización y equipamiento</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" t="n">
+        <v>23.45</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Señalización y equipamiento</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
         <is>
           <t>Instalación de lavamanos con su grifería y desagüe.</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
         <is>
           <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D67" t="inlineStr">
         <is>
           <t>ud</t>
         </is>
       </c>
-      <c r="E43" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" t="n">
+      <c r="E67" t="n">
+        <v>1</v>
+      </c>
+      <c r="F67" t="n">
         <v>36.45</v>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G67" t="inlineStr">
         <is>
           <t>Aparatos sanitarios y grifería</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H67" t="inlineStr">
         <is>
           <t>incluida</t>
         </is>

</xml_diff>

<commit_message>
Cerrar el capitulo D Demoliciones completo: 98 partidas en 13 subcapitulos y 42 grupos
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/catalogo_partidas.xlsx
+++ b/basedatos_partidas/salida/catalogo_partidas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -489,28 +489,28 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Desmontaje de aparato sanitario y su grifería.</t>
+          <t>Demolición de losa de fundación de concreto armado.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de aparato sanitario existente, ya sea inodoro, lavamanos, bidé o fregadero, junto con su grifería y accesorios de conexión. Incluye cierre previo de la llave de paso y vaciado del aparato, desconexión de las tomas de agua y del desagüe, taponado provisional de las salidas para evitar olores y entrada de escombro, retirada del aparato hasta el punto de acopio y limpieza de la zona. Si el cliente desea conservar el aparato, se desmonta con cuidado y se acopia protegido. No incluye el transporte a vertedero. Medido por unidad desmontada.</t>
+          <t>Demolición de losa de fundación de concreto armado, ejecutada con martillo hidráulico montado sobre retroexcavadora y corte de la malla de refuerzo. Incluye el corte perimetral previo para delimitar la zona de intervención, la comprobación de que no discurren instalaciones enterradas bajo la losa, la fragmentación del concreto en piezas cargables, el corte y separación del acero para su gestión diferenciada, el acopio del escombro y la limpieza del terreno resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en volumen realmente demolido.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E2" t="n">
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>4.55</v>
+        <v>119.83</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Cimentaciones</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -527,28 +527,28 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Demolición de tabique de bloque o ladrillo, incluidos sus revestimientos.</t>
+          <t>Demolición de viga de riostra o muro de contención de concreto.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Demolición de tabique interior no estructural de bloque de concreto o ladrillo, con sus revestimientos por ambas caras, ejecutada con martillo eléctrico manual sin afectar a la estabilidad de los elementos constructivos contiguos. Incluye comprobación previa de que el tabique no es portante y de que no aloja instalaciones en servicio, protección del entorno, apeo puntual si fuera necesario, fragmentación del escombro en piezas manejables, retirada en sacos hasta el punto de acopio y limpieza de la zona. No incluye el transporte a vertedero. Medido en superficie realmente demolida.</t>
+          <t>Demolición de viga de riostra, muro de contención o murete de concreto armado, ejecutada con martillo neumático y corte de armaduras. Incluye la comprobación previa de que el elemento no sostiene empujes de tierra activos o, en su caso, el sostenimiento provisional del terreno, la protección del entorno, el corte y retiro del acero de refuerzo, la fragmentación del concreto y su acopio, y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en volumen realmente demolido.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E3" t="n">
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>5.42</v>
+        <v>104.61</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Particiones</t>
+          <t>Cimentaciones</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -565,28 +565,28 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Picado de enchapado cerámico en pared y su capa de pega.</t>
+          <t>Demolición de zapata o pedestal de concreto armado.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Picado de enchapado cerámico o de porcelanato existente en pared, incluida su capa de pega de mortero, ejecutado con martillo eléctrico manual hasta dejar el friso o el bloque a la vista, sin comprometer la estabilidad del muro ni dañar las tuberías y canalizaciones empotradas. Incluye la localización previa de las instalaciones que discurren por el paramento, la protección de pisos, aparatos y puertas, el control de polvo mediante aspiración, el retiro manual del escombro en sacos hasta el punto de acopio y la limpieza de la superficie, dejándola lista para recibir el nuevo friso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Demolición de zapata aislada o pedestal de concreto armado, ejecutada con martillo neumático y corte de la armadura con oxicorte o amoladora. Requiere comprobación estructural previa de que el elemento ya no cumple función portante o de que la estructura está debidamente apeada. Incluye la excavación de descubrimiento del elemento si estuviera enterrado, la protección del entorno, el corte y retiro de las barras de acero, la fragmentación del concreto en piezas manejables y su acopio, y el relleno del hueco resultante si el proyecto lo requiere. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en volumen realmente demolido.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>6.25</v>
+        <v>113.98</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Cimentaciones</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -603,28 +603,28 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Picado de enchapado de granito o terrazo en pared.</t>
+          <t>Desmontaje de estructura metálica.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Picado de enchapado de granito o terrazo prefabricado existente en pared, incluida su capa de asiento de mortero, ejecutado con martillo eléctrico manual. Por el mayor espesor y peso de estas piezas frente al enchapado cerámico, el rendimiento es menor y el escombro más pesado. Incluye la protección de pisos y ambientes contiguos, el control de polvo, el retiro manual del escombro en sacos hasta el punto de acopio y el repicado de los restos de mortero adheridos al paramento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Desmontaje de estructura metálica de acero, formada por perfiles laminados o armados, ejecutado mediante oxicorte y desatornillado según el tipo de unión, con apeo previo de los elementos que permanecen. Incluye el estudio del orden de desmontaje para mantener la estabilidad del conjunto en todo momento, el eslingado y sostenimiento de las piezas antes de liberarlas, el corte en tramos transportables, el descenso a nivel de acopio y la clasificación del acero para su venta o gestión como chatarra, cuyo valor de recuperación puede descontarse al cliente. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en peso realmente desmontado.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E5" t="n">
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>7.31</v>
+        <v>0.52</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -641,28 +641,28 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Picado de enchapado de piedra natural en pared.</t>
+          <t>Demolición de columna de concreto armado.</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Picado de enchapado de piedra natural existente en pared, ya sea mármol, laja o piedra de revestimiento, incluida su capa de asiento y los anclajes metálicos si los tuviera, ejecutado con martillo eléctrico manual. Si el cliente desea recuperar las piezas se desmontan una a una con cuidado, se limpian y se acopian protegidas, lo que reduce el rendimiento y debe advertirse en el presupuesto. Incluye la protección del entorno, el control de polvo, el retiro del escombro en sacos y el repicado de los restos adheridos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Demolición de columna de concreto armado, ejecutada con martillo eléctrico o neumático según la sección, con corte previo de la armadura longitudinal. Exige apeo previo de la estructura que la columna soporta y validación del cálculo estructural, trabajos que se valoran aparte. Incluye la protección del entorno, la demolición descendente por tramos para mantener el control del elemento, el corte y retiro del acero, la fragmentación del concreto, el descenso del escombro y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en volumen realmente demolido.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E6" t="n">
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>7.67</v>
+        <v>119.95</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -679,28 +679,28 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Desmontaje de enchapado de madera o machihembrado en pared.</t>
+          <t>Demolición de viga de concreto armado.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de revestimiento de madera existente en pared, ya sea machihembrado, tablilla o panel, junto con los rastreles de soporte fijados al paramento, ejecutado con medios manuales mediante palanca y barra. Incluye la extracción de los clavos, tornillos y tacos que queden en el muro, el retiro del material en sacos o atados hasta el punto de acopio, la clasificación de las piezas aprovechables si el cliente desea conservarlas y la limpieza del paramento resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Demolición de viga de concreto armado, ejecutada con martillo eléctrico o neumático, con apeo previo de la losa o de los elementos que la viga sostiene. Incluye la validación estructural previa, el montaje del apeo provisional, la protección del entorno y del nivel inferior, la demolición por tramos controlados desde andamio, el corte y retiro de las barras de refuerzo, el descenso del escombro y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en volumen realmente demolido.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E7" t="n">
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>2.21</v>
+        <v>134.08</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -717,12 +717,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Desmontaje de revestimiento de láminas o paneles en pared.</t>
+          <t>Demolición de losa de entrepiso maciza o nervada.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de revestimiento de pared formado por láminas o paneles de PVC, aluminio, melamina o material similar, junto con su estructura o rastrelado de soporte, ejecutado con medios manuales. Incluye el retiro de los perfiles de remate y esquineros, la extracción de las fijaciones que queden en el paramento, el resane puntual de los huecos de anclaje, el retiro del material hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Demolición de losa de entrepiso de concreto armado, maciza o nervada, ejecutada con martillo neumático y corte de armaduras, con apeo previo de los tramos que permanecen. Incluye la validación estructural, el montaje del apeo, el acordonamiento y protección del nivel inferior para impedir el paso durante los trabajos, la demolición en franjas controladas desde los apoyos hacia el centro, el corte y separación del acero, el descenso del escombro y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -734,11 +734,11 @@
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>1.56</v>
+        <v>46.07</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -755,12 +755,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Retiro de papel tapiz en paramento.</t>
+          <t>Apertura de hueco en losa de concreto armado.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Retiro de papel tapiz existente en paramento interior, junto con los restos de pegamento mural, ejecutado con medios manuales mediante humectación previa con solución reblandecedora y raspado con espátula ancha. Incluye la protección de pisos, rodapiés y mecanismos, la aplicación de la solución en varias pasadas hasta que el papel se desprenda sin arrancar el friso, el rascado de los residuos de pegamento, el lavado final del paramento y su secado, dejándolo listo para recibir el nuevo acabado. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
+          <t>Apertura de hueco en losa de concreto armado para paso de escalera, ducto de instalaciones o claraboya, ejecutada mediante corte perimetral con disco de diamante y demolición interior con martillo eléctrico. Incluye la validación estructural previa y el refuerzo del borde si el cálculo lo exige, el apeo de la zona, el replanteo y corte perimetral que garantiza un borde limpio y sin fisuración hacia el resto de la losa, el corte de las armaduras, el descenso controlado del escombro y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de hueco realmente abierto.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -772,11 +772,11 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>2.2</v>
+        <v>36.26</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -793,28 +793,28 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Desmontaje de moldura decorativa de yeso o poliestireno.</t>
+          <t>Desmontaje de estructura de madera.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de moldura decorativa corrida de yeso, poliestireno o poliuretano, situada en el encuentro de pared y cielo raso o como elemento decorativo en paramento, ejecutado con medios manuales mediante espátula y cincel. Incluye la protección del entorno, el corte previo de la línea de junta para evitar arrastrar el friso, el rascado de los restos de pasta o adhesivo, el resane puntual de los desconchados provocados, el retiro del material hasta el punto de acopio y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
+          <t>Desmontaje de estructura de madera de entrepiso o de techo, formada por vigas, viguetas y entablado, ejecutado con medios manuales y sierra, con apeo previo. Incluye la inspección previa del estado de la madera para prever roturas por pudrición o ataque de xilófagos, el apeo provisional, el desmontaje ordenado desde el entablado hacia las vigas principales, la extracción de clavos y herrajes, la clasificación de las piezas aprovechables si el cliente desea conservarlas, el descenso del material y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E10" t="n">
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>0.9399999999999999</v>
+        <v>13.18</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -831,28 +831,28 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Retiro de láminas decorativas, vinilos o espejos adheridos.</t>
+          <t>Desmontaje de baranda o pasamanos de balcón.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Retiro de revestimiento decorativo adherido al paramento, ya sea lámina vinílica, calcomanía mural o espejo pegado, junto con los restos de adhesivo. Incluye la protección del piso y del mobiliario, el calentamiento o humectación previa para reblandecer el adhesivo, el desprendimiento controlado del material con espátula, y en el caso de espejos el encintado previo de la superficie para evitar la proyección de fragmentos al fracturarse. Incluye el rascado de los restos de adhesivo, el retiro del material en sacos y la limpieza del paramento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
+          <t>Desmontaje de baranda o antepecho metálico de balcón, terraza o escalera exterior, ejecutado mediante oxicorte o desatornillado según el anclaje, con sostenimiento previo del elemento. Incluye la instalación de una protección provisional del borde antes de retirar la baranda definitiva, requisito de seguridad ineludible cuando queda un vacío accesible, el corte de los anclajes al ras del soporte, el resane de los huecos de anclaje, el descenso del material y su acopio clasificado como chatarra. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E11" t="n">
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>1.6</v>
+        <v>5.79</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Fachadas</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -869,12 +869,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Demolición de revestimiento cerámico de escalera.</t>
+          <t>Desmontaje de reja de protección en fachada.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Demolición del revestimiento cerámico de escalera, comprendiendo huellas, contrahuellas y su capa de pega, ejecutada con martillo eléctrico manual sin comprometer la losa de la escalera. El rendimiento es sensiblemente menor que en un piso corrido por la posición forzada de trabajo, la superficie fragmentada en peldaños y la dificultad de evacuar el escombro por la propia escalera. Incluye la protección del hueco y del pasamanos, el control de polvo, el retiro manual del escombro en sacos y la limpieza, dejando los peldaños listos para el nuevo revestimiento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida, desarrollando huella y contrahuella.</t>
+          <t>Desmontaje de reja o protector metálico de ventana o puerta en fachada, ejecutado mediante oxicorte o amoladora sobre los anclajes empotrados en el paramento. Incluye el sostenimiento de la reja antes de liberar el último anclaje para evitar su caída, el corte de los elementos de fijación, el picado y resane de los huecos de anclaje que queden en el muro, el descenso del elemento y su acopio clasificado como chatarra. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -886,11 +886,11 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>7.27</v>
+        <v>5.62</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Fachadas</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -907,12 +907,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Demolición de revestimiento de granito o piedra natural en escalera.</t>
+          <t>Demolición de muro de fachada de bloque o ladrillo.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Demolición del revestimiento de granito, terrazo o piedra natural de escalera, comprendiendo huellas, contrahuellas y su capa de asiento, ejecutada con martillo eléctrico manual. Al mayor espesor y peso de las piezas se suma la dificultad propia del trabajo en escalera, por lo que el rendimiento es el más bajo de los grupos de demolición de revestimientos. Incluye la protección del hueco y del pasamanos, el control de polvo, el retiro manual del escombro en sacos y el repicado de los restos de mortero adheridos a los peldaños. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida, desarrollando huella y contrahuella.</t>
+          <t>Demolición de muro de cerramiento de fachada de bloque de concreto o ladrillo, incluidos sus revestimientos por ambas caras, ejecutada con martillo eléctrico manual desde andamio. Incluye la comprobación previa de que el muro no cumple función portante, el acordonamiento y señalización de la zona de caída a pie de fachada, la protección de las carpinterías que permanecen, la demolición descendente por hiladas para evitar vuelcos, el control de la caída de escombro, su retiro en sacos y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -924,11 +924,11 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>8.58</v>
+        <v>8.49</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Fachadas</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -945,28 +945,28 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Demolición de zócalo escalonado de escalera.</t>
+          <t>Desmontaje de cerramiento ligero de láminas metálicas.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Demolición del zócalo o rodapié escalonado que acompaña a la escalera en su encuentro con el paramento, incluida su capa de pega, ejecutada con medios manuales y martillo eléctrico, cuidando de no dañar el friso por encima de la línea del zócalo. Incluye el repicado de los restos de mortero adheridos, el retiro del escombro en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud real de la línea inclinada del zócalo.</t>
+          <t>Desmontaje de cerramiento de fachada formado por láminas metálicas, panel sándwich o material similar, junto con la perfilería de soporte, ejecutado con medios manuales y atornillador desde andamio. Incluye el acordonamiento de la zona a pie de fachada, el desmontaje ordenado de las láminas evitando que el viento las descontrole, el retiro de la perfilería y de las fijaciones, la clasificación del material recuperable, el descenso a nivel de acopio y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E14" t="n">
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>1.78</v>
+        <v>5.95</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Fachadas</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -983,28 +983,28 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Picado de friso de mortero en paramento.</t>
+          <t>Desmontaje de alféizar o repisa de ventana.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Picado de friso de mortero de cemento existente en paramento interior o exterior, ejecutado con martillo eléctrico manual hasta dejar el bloque o el ladrillo a la vista, cuando el friso está disgregado, hueco o presenta fisuración generalizada. Incluye el sondeo previo por golpeo para delimitar las zonas sin adherencia, la protección de pisos y ambientes contiguos, el control de polvo mediante aspiración, el retiro manual del escombro en sacos hasta el punto de acopio y el barrido y limpieza del paramento, dejándolo listo para recibir el nuevo friso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Desmontaje del alféizar o repisa de ventana, sea de granito, piedra, cerámica o concreto, incluida su capa de asiento, ejecutado con medios manuales y martillo eléctrico. Incluye el corte previo de la junta con el paramento para no arrastrar el friso al desprender la pieza, el picado del mortero de asiento, la limpieza del apoyo dejándolo plano y a nivel para recibir el nuevo alféizar, y el retiro del escombro en sacos. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido, lo que reduce el rendimiento y debe advertirse en el presupuesto. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E15" t="n">
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>5.86</v>
+        <v>2.93</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Remates</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1021,28 +1021,28 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Picado de friso de yeso o pasta en paramento.</t>
+          <t>Demolición de dintel prefabricado o cargadero.</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Picado de revestimiento de yeso o pasta existente en paramento interior, ejecutado con medios manuales mediante espátula ancha y cincel, con martillo eléctrico solo en las zonas de mayor espesor. Por tratarse de un material blando el rendimiento es sensiblemente mayor que en un friso de mortero, aunque genera abundante polvo fino. Incluye la protección del entorno, el control de polvo mediante aspiración continua, el retiro del escombro en sacos hasta el punto de acopio y la limpieza del paramento resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Demolición de dintel prefabricado o cargadero de concreto sobre hueco de puerta o ventana, ejecutada con martillo eléctrico previo apeo del muro superior. Incluye la validación previa de la carga que transmite el dintel y el montaje del apeo provisional mediante puntales, operación imprescindible antes de cualquier corte, la demolición por tramos, el corte de la armadura, el retiro del escombro y el repaso del apoyo para recibir el nuevo dintel. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E16" t="n">
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>3.65</v>
+        <v>12.52</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Remates</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1059,28 +1059,28 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Picado de estuco o pasta decorativa en paramento.</t>
+          <t>Desmontaje de pasamanos de escalera.</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Picado de revestimiento de estuco, pasta decorativa o revestimiento texturado existente en paramento, ejecutado con medios manuales y martillo eléctrico según el espesor y la dureza del material, hasta dejar el soporte limpio y apto para recibir el nuevo acabado. Incluye la cata previa para identificar el espesor y el tipo de soporte, la protección del entorno, el control de polvo, el retiro del escombro en sacos y la limpieza final. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Desmontaje de pasamanos de escalera, sea de madera, metálico o de obra, junto con sus soportes y anclajes al paramento o a la baranda. Ejecutado con medios manuales, atornillador y amoladora según el tipo de fijación. Incluye el sostenimiento del elemento durante el desmontaje, el corte o extracción de los anclajes, el resane de los huecos que queden en el paramento, la clasificación del material recuperable y el retiro hasta el punto de acopio. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido, lo que reduce el rendimiento y debe advertirse en el presupuesto. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E17" t="n">
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>4.3</v>
+        <v>2.26</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Remates</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1097,28 +1097,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Repicado de superficie de concreto para mejorar adherencia.</t>
+          <t>Desmontaje de equipo de aire acondicionado tipo split.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Repicado superficial de paramento o losa de concreto, ejecutado con martillo eléctrico y puntero, para crear la rugosidad necesaria que garantice la adherencia del friso o del mortero de recrecido posterior. Incluye la limpieza previa de la superficie, el picado uniforme sin llegar a descubrir la armadura, la eliminación de lechadas superficiales y restos de desencofrante, el soplado y aspirado del polvo resultante y la retirada de los restos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente repicada.</t>
+          <t>Desmontaje de equipo de aire acondicionado tipo split, comprendiendo la unidad evaporadora interior, la unidad condensadora exterior, la tubería frigorífica y el drenaje. Incluye la recuperación previa del gas refrigerante mediante equipo específico, operación obligatoria por normativa ambiental que no debe liberarse a la atmósfera, la desconexión eléctrica comprobada, el desmontaje de ambas unidades y de sus soportes, el retiro de la tubería y el drenaje, el resane de las perforaciones de paso y el descenso de los equipos. Si el cliente desea conservar el equipo, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por equipo desmontado.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E18" t="n">
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>4.37</v>
+        <v>16.84</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1135,28 +1135,28 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Eliminación de pintura en paramento mediante raspado y decapado.</t>
+          <t>Desmontaje de red eléctrica y sus mecanismos.</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Eliminación de las capas de pintura existentes en paramento interior o exterior, mediante raspado mecánico con espátula y lijado, con aplicación puntual de decapante químico en gel en las zonas de pintura muy adherida o de espesor elevado. Se emplea cuando la pintura existente está cuarteada, sopla o es incompatible con el nuevo acabado. Incluye la protección de pisos, carpintería y mobiliario, la ventilación del ambiente durante la aplicación del decapante, la neutralización y lavado de los restos químicos, el aspirado del polvo y la retirada de los residuos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
+          <t>Desmontaje de instalación eléctrica existente, comprendiendo la tubería conduit, el conductor, las cajas y los mecanismos, sea vista o empotrada. Incluye la desconexión previa en el tablero y la comprobación de ausencia de tensión con detector antes de manipular cualquier punto, requisito de seguridad ineludible, el picado de los tramos empotrados, la extracción del cableado y la tubería, el retiro de cajas y mecanismos, la clasificación del cobre para su recuperación y el resane de las rozas. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud de canalización realmente desmontada.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E19" t="n">
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>5.15</v>
+        <v>3.47</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1173,28 +1173,28 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Picado de salpicado o graniplast en fachada.</t>
+          <t>Desmontaje de tablero eléctrico.</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Picado de revestimiento de salpicado, graniplast o revestimiento pétreo proyectado en fachada, ejecutado con martillo eléctrico manual y espátula, hasta dejar el friso base sano o el bloque a la vista según el estado del soporte. Incluye el sondeo previo por golpeo para delimitar las zonas sin adherencia, el trabajo desde andamio con las protecciones colectivas correspondientes, la protección de carpinterías y de la zona de paso a pie de fachada, el control de la caída de escombro, su retiro en sacos hasta el punto de acopio y la limpieza del paramento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Desmontaje de tablero eléctrico de distribución, incluidos los interruptores termomagnéticos, el barraje y la caja. Incluye el corte previo del suministro desde el punto de acometida y su verificación con detector de tensión, el etiquetado de los circuitos existentes antes de desconectarlos para poder replantear la nueva instalación con la información del estado previo, la desconexión ordenada, el desmontaje de la caja empotrada, el resane del hueco y el retiro del material. Si el cliente desea conservar el equipo, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E20" t="n">
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>7.11</v>
+        <v>10.96</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1211,28 +1211,28 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Picado de mortero monocapa en fachada.</t>
+          <t>Desmontaje de red de tuberías de agua o desagüe.</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Picado de revestimiento de mortero monocapa en fachada, incluida su malla de refuerzo y los perfiles de arranque y goterón, ejecutado con martillo eléctrico manual hasta dejar el soporte limpio y apto para recibir el nuevo revestimiento. Incluye el sondeo previo del paramento, el trabajo desde andamio con las protecciones colectivas correspondientes, la protección de carpinterías y del paso a pie de fachada, el corte y retiro de la malla, el control de la caída de escombro, su retiro en sacos y la limpieza del soporte. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Desmontaje de red existente de tuberías de agua o de desagüe, vista o empotrada, incluidos sus accesorios y soportes. Incluye el cierre y comprobación previa de que la red está fuera de servicio y vaciada, el picado del paramento en los tramos empotrados, el corte y extracción de la tubería en tramos manejables, el taponado de las derivaciones que permanecen activas, el retiro del material clasificado según sea PVC, hierro galvanizado o cobre, y el resane de las rozas. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E21" t="n">
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>8.02</v>
+        <v>4.2</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1249,28 +1249,28 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Demolición de trasdosado de yeso laminado y su estructura.</t>
+          <t>Desmontaje de luminaria.</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Demolición de trasdosado autoportante de placa de yeso laminado adosado a muro, junto con la perfilería de acero galvanizado y el aislamiento alojado en la cámara, ejecutada con medios manuales. Incluye la localización y desconexión previa de los mecanismos e instalaciones que discurran por el trasdosado, la protección del piso y del mobiliario, el desmontaje ordenado de las placas, el retiro del aislamiento en sacos, el desmontaje de la perfilería y de las fijaciones al muro, y la limpieza de la zona dejando el paramento original a la vista. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de luminaria de techo o pared, sea empotrada, de sobreponer o colgante, incluidos sus soportes y accesorios. Incluye el corte previo del circuito y la comprobación de ausencia de tensión, la desconexión y aislamiento provisional de los conductores que permanecen, el desmontaje del cuerpo de la luminaria, el retiro de las lámparas con gestión diferenciada si son fluorescentes o de descarga por su contenido en mercurio, y el resane del punto si procede. Si el cliente desea conservar el equipo, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E22" t="n">
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>2.56</v>
+        <v>2.17</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1287,28 +1287,28 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Demolición de trasdosado de bloque o ladrillo adosado a muro.</t>
+          <t>Desmontaje de aparato sanitario y su grifería.</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Demolición de tabique de bloque o ladrillo adosado a muro a modo de trasdosado, incluidos sus revestimientos y la cámara intermedia, ejecutada con martillo eléctrico manual sin dañar el muro original que permanece. Incluye la comprobación previa de que el trasdosado no cumple función estructural ni aloja instalaciones en servicio, la protección del entorno, el control de polvo, la fragmentación del escombro en piezas manejables, el retiro en sacos hasta el punto de acopio y el repicado de los restos de mortero adheridos al muro. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de aparato sanitario existente, ya sea inodoro, lavamanos, bidé o fregadero, junto con su grifería y accesorios de conexión. Incluye cierre previo de la llave de paso y vaciado del aparato, desconexión de las tomas de agua y del desagüe, taponado provisional de las salidas para evitar olores y entrada de escombro, retirada del aparato hasta el punto de acopio y limpieza de la zona. Si el cliente desea conservar el aparato, se desmonta con cuidado y se acopia protegido. No incluye el transporte a vertedero. Medido por unidad desmontada.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E23" t="n">
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>6.21</v>
+        <v>4.55</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1325,28 +1325,28 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Desmontaje de trasdosado directo de placa pegada al muro.</t>
+          <t>Desmontaje de fregadero y su grifería.</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de trasdosado directo formado por placa de yeso laminado o panel aislante adherido al muro mediante pelladas de pasta, ejecutado con medios manuales mediante palanca y espátula. Incluye la protección del piso, el arranque de las placas, el rascado de los restos de pasta y adhesivo adheridos al muro hasta dejarlo apto para recibir el nuevo revestimiento, el retiro del material en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Desmontaje de fregadero de cocina con su grifería y accesorios de conexión. Incluye el cierre previo de las llaves de paso, la desconexión de las tomas de agua fría y caliente, el desmontaje del sifón y del desagüe con recogida del agua retenida, el corte del sellado perimetral con el mesón, la extracción de la pieza y el taponado provisional de las salidas para evitar olores y entrada de escombro. Si el cliente desea conservar el equipo, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E24" t="n">
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>3.12</v>
+        <v>4.12</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1363,28 +1363,28 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Demolición de piso cerámico y su capa de pega.</t>
+          <t>Desmontaje de calentador de agua.</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso existente de baldosa cerámica o de porcelanato, junto con su capa de pega de mortero, ejecutada con martillo eléctrico manual sin comprometer la losa ni los elementos constructivos vecinos. Incluye protección previa de paredes, puertas y ambientes contiguos, control de polvo mediante aspiración, retiro manual del escombro en sacos hasta el punto de acopio y barrido de la superficie resultante, dejándola lista para recibir el nuevo contrapiso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de calentador de agua eléctrico o a gas, incluidos sus soportes de anclaje y las conexiones de entrada y salida. Incluye el corte previo del suministro eléctrico o de gas y su comprobación con detector, el vaciado completo del tanque antes de liberarlo de sus soportes por el peso que retiene, la desconexión de las tuberías y su taponado, el desmontaje del anclaje al paramento, el resane de los huecos y el descenso del equipo hasta el punto de acopio. Si el cliente desea conservar el equipo, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E25" t="n">
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>4.88</v>
+        <v>9.43</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1401,28 +1401,28 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Demolición de rodapié cerámico.</t>
+          <t>Desmontaje de closet o mueble empotrado.</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Demolición de rodapié existente de baldosa cerámica o de porcelanato y de su capa de pega, ejecutada con medios manuales y martillo eléctrico, cuidando de no dañar el friso de la pared por encima de la línea del rodapié. Incluye retiro manual del escombro en sacos hasta el punto de acopio, repicado de los restos de mortero adheridos y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+          <t>Desmontaje de closet, alacena o mueble empotrado, incluidos las puertas, los entrepaños, la estructura interior y los rastreles de fijación al paramento, ejecutado con medios manuales y atornillador. Incluye el vaciado previo del contenido si el cliente no lo hubiera retirado, el desmontaje ordenado desde las puertas hacia la estructura, la extracción de tacos y tornillos del muro, el resane de los huecos de anclaje, la clasificación de las piezas aprovechables y el retiro del material. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de frente de mueble realmente desmontada.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E26" t="n">
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>4.62</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Carpintería, vidrios y protecciones solares</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Demolición de piso de granito o terrazo en baldosa.</t>
+          <t>Desmontaje de reja o protector metálico interior.</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso existente de baldosa de granito o terrazo prefabricado, junto con su capa de asiento de mortero, ejecutada con martillo eléctrico manual. Por la dureza y el espesor de este tipo de baldosa el rendimiento es menor que en un piso cerámico y el escombro resulta más pesado, lo que se refleja en el rendimiento de la partida. Incluye protección previa de los ambientes contiguos, control de polvo, retiro manual del escombro en sacos y limpieza de la superficie. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de reja, protector metálico o portón enrollable situado en el interior del inmueble, ejecutado mediante oxicorte o amoladora sobre sus anclajes. Incluye el sostenimiento del elemento antes de liberar el último punto de fijación, el corte de los anclajes al ras, el picado y resane de los huecos que queden en el paramento, el retiro del material hasta el punto de acopio y su clasificación como chatarra, cuyo valor de recuperación puede descontarse al cliente. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1456,11 +1456,11 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>5.9</v>
+        <v>4.71</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Carpintería, vidrios y protecciones solares</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1477,28 +1477,28 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Demolición de rodapié de granito o terrazo.</t>
+          <t>Retiro de vidrio de carpintería existente.</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Demolición de rodapié existente de granito o terrazo prefabricado y de su capa de asiento, ejecutada con martillo eléctrico manual, cuidando de no dañar el friso de la pared. Incluye repicado de los restos de mortero adheridos, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+          <t>Retiro de vidrio de carpintería que permanece en obra, ya sea por rotura, por sustitución del acristalamiento o para aligerar la ventana antes de su desmontaje. Ejecutado con medios manuales, retirando junquillos, masilla o silicona de sujeción. Incluye el encintado previo de la superficie del vidrio para que, si se fractura, los fragmentos queden contenidos en la lámina adhesiva, el uso de protección facial y guantes anticorte, la limpieza del galce, el retiro del vidrio en contenedor rígido específico y el barrido minucioso de esquirlas. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de vidrio realmente retirada.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E28" t="n">
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>1.17</v>
+        <v>3.38</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Carpintería, vidrios y protecciones solares</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1515,28 +1515,28 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Demolición de piso de granito vaciado en sitio.</t>
+          <t>Desmontaje de puerta interior con su marco.</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso continuo de granito vaciado en sitio, incluida su base de mortero y las platinas divisorias de las juntas, ejecutada con martillo neumático por tratarse de una superficie monolítica de gran dureza. Incluye corte perimetral previo con amoladora de disco de diamante para delimitar la zona de intervención y evitar desprendimientos fuera de ella, protección de los ambientes contiguos, control de polvo, fragmentación del escombro en piezas manejables, retiro en sacos y limpieza. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de puerta de paso interior, incluidas la hoja, el marco, las molduras de remate y la herrajería, ejecutado con medios manuales. Incluye el desmontaje previo de la hoja liberándola de sus bisagras, el desclavado o corte de los anclajes del marco al vano, el retiro de las molduras cuidando de no dañar el friso, el repicado de los restos de espuma o mortero de fijación y el retiro del material hasta el punto de acopio. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido, lo que reduce el rendimiento y debe advertirse en el presupuesto. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E29" t="n">
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>13.04</v>
+        <v>4.23</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Carpintería, vidrios y protecciones solares</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1553,28 +1553,28 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Demolición de piso de cemento pulido.</t>
+          <t>Desmontaje de puerta exterior o metálica con su marco.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso continuo de cemento pulido y de su base de mortero, ejecutada con martillo eléctrico manual, sin afectar a la losa estructural. Incluye corte perimetral con amoladora cuando la demolición sea parcial, protección de los ambientes contiguos, control de polvo mediante aspiración, fragmentación del escombro, retiro manual en sacos hasta el punto de acopio y limpieza de la superficie resultante. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de puerta exterior, de seguridad o metálica, incluidos la hoja, el marco y la herrajería, ejecutado mediante oxicorte o amoladora sobre los anclajes empotrados. Por su peso requiere dos operarios para el sostenimiento de la hoja durante la liberación del marco. Incluye el sostenimiento previo del conjunto, el corte de los anclajes, el picado y resane de los huecos que queden en el muro, el retiro del material hasta el punto de acopio y su clasificación como chatarra. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido, lo que reduce el rendimiento y debe advertirse en el presupuesto. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E30" t="n">
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>6.92</v>
+        <v>11.54</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Carpintería, vidrios y protecciones solares</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1591,28 +1591,28 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Demolición de rodapié de cemento.</t>
+          <t>Desmontaje de ventana con su marco.</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Demolición de rodapié corrido de mortero de cemento, ejecutada con medios manuales y cincel, cuidando de no dañar el friso de la pared por encima de la línea del rodapié. Incluye repicado de los restos adheridos al paramento, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+          <t>Desmontaje de ventana existente, incluidos el marco, las hojas, el vidrio y la herrajería, ejecutado con medios manuales y corte de anclajes. Incluye el retiro previo del vidrio para aligerar el conjunto y evitar roturas incontroladas durante la maniobra, el desmontaje de las hojas, el corte de los anclajes del marco al vano, el picado del mortero de recibido, el resane del hueco perimetral, el descenso del material y su clasificación para reciclaje o reutilización. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido, lo que reduce el rendimiento y debe advertirse en el presupuesto. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de hueco realmente desmontado.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E31" t="n">
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>0.91</v>
+        <v>7.02</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Carpintería, vidrios y protecciones solares</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1629,28 +1629,28 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Demolición de piso de piedra natural.</t>
+          <t>Demolición de brocal o cordón de acera.</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso existente de piedra natural, ya sea mármol, granito natural o laja, junto con su capa de asiento de mortero, ejecutada con martillo eléctrico manual. Si el cliente desea recuperar las piezas, se levantan una a una con cuidado, se limpian de mortero y se acopian protegidas, lo que reduce el rendimiento y debe advertirse en el presupuesto. Incluye protección de los ambientes contiguos, control de polvo, retiro manual del escombro en sacos y limpieza de la superficie. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Demolición de brocal, cordón o bordillo de acera, sea prefabricado o vaciado en sitio, junto con su dado de concreto de apoyo, ejecutada con martillo eléctrico manual. Incluye el acordonamiento y señalización del área de trabajo por su situación en zona de tránsito, el corte de las juntas entre piezas, la demolición del dado de apoyo, la extracción del escombro, el acopio de las piezas prefabricadas aprovechables si el cliente desea reutilizarlas y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E32" t="n">
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>6.34</v>
+        <v>7.1</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Firmes y pavimentos exteriores</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1667,28 +1667,28 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Demolición de rodapié de piedra natural.</t>
+          <t>Demolición de pavimento exterior de concreto.</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Demolición de rodapié existente de piedra natural y de su capa de asiento, ejecutada con martillo eléctrico manual, cuidando de no dañar el friso de la pared. Incluye repicado de los restos de mortero adheridos, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+          <t>Demolición de pavimento exterior de concreto, en acera, patio o vía de acceso, de hasta 15 cm de espesor, ejecutada con martillo hidráulico montado sobre retroexcavadora. Incluye la comprobación previa de que no discurren instalaciones enterradas bajo el pavimento, el corte perimetral con disco de diamante para delimitar la zona de intervención, el acordonamiento del área de trabajo, la fragmentación del concreto en piezas cargables, el corte y separación de la malla de refuerzo si la tuviera, el acopio del escombro y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E33" t="n">
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>1.25</v>
+        <v>12.66</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Firmes y pavimentos exteriores</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1705,12 +1705,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Levantado de piso de parquet o madera.</t>
+          <t>Demolición de pavimento asfáltico.</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Levantado de piso existente de parquet o de tablilla de madera, incluidos los rastreles o el adhesivo de fijación al contrapiso, ejecutado con medios manuales mediante palanca y espátula. Incluye el retiro previo de las molduras de remate, el rascado de los restos de adhesivo adheridos al contrapiso, la extracción de los clavos o tornillos que queden en la base, el retiro del material en sacos hasta el punto de acopio y la limpieza de la superficie resultante. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
+          <t>Demolición de pavimento asfáltico de hasta 10 cm de espesor, ejecutada con martillo hidráulico montado sobre retroexcavadora, con corte perimetral previo para obtener un borde recto que facilite la reposición. Incluye la comprobación de instalaciones enterradas, el acordonamiento y señalización del área, el corte perimetral con disco, el arranque y fragmentación del asfalto, el acopio diferenciado del material fresado por admitir reciclaje específico, y la limpieza y barrido de la base resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1722,11 +1722,11 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>2.17</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Firmes y pavimentos exteriores</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1743,28 +1743,28 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Levantado de rodapié de madera.</t>
+          <t>Levantado de pavimento de adoquín.</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Levantado de rodapié existente de madera, ejecutado con medios manuales mediante palanca y espátula, cuidando de no dañar el friso de la pared. Incluye la extracción de los clavos, tornillos o tacos de fijación que queden en el paramento, el retiro del material en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente levantada.</t>
+          <t>Levantado de pavimento exterior de adoquín de concreto o piedra, junto con su cama de arena, ejecutado con medios manuales mediante palanca y pico. Por tratarse de piezas independientes el levantado permite recuperar un porcentaje elevado del material para su reutilización. Incluye el levantado ordenado desde un borde libre, la limpieza de las piezas retirando la arena y el mortero adherido, su clasificación en aprovechables y desechables, el paletizado o acopio de las recuperables, el retiro de la cama de arena y el barrido de la base. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente levantada.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E35" t="n">
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>0.43</v>
+        <v>3.35</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Firmes y pavimentos exteriores</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1781,12 +1781,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Levantado de piso laminado.</t>
+          <t>Retiro de aislamiento térmico o acústico.</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Levantado de piso laminado flotante existente, incluidas la manta acústica y las molduras de remate perimetrales, ejecutado con medios manuales. Por tratarse de un sistema flotante de encastre el desmontaje es rápido y no genera escombro pesado. Incluye el desmontaje ordenado de las tablas, el retiro de la manta y del perfil perimetral, la limpieza y aspirado del contrapiso resultante y el retiro del material en sacos hasta el punto de acopio. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
+          <t>Retiro de aislamiento térmico o acústico existente, sea de lana mineral, poliestireno o poliuretano, alojado en cámara de tabique, cielo raso o cubierta. Incluye el uso de mascarilla y guantes por la irritación que producen las fibras minerales, el desmontaje del material en piezas completas cuando el estado lo permita, el ensacado inmediato para evitar la dispersión de fibras por el ambiente, el aspirado de los restos y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente retirada.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1798,11 +1798,11 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>1.26</v>
+        <v>1.99</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Aislamientos e impermeabilizaciones</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1819,12 +1819,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Levantado de piso vinílico, linóleo o alfombra.</t>
+          <t>Retiro de manto asfáltico en cubierta.</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Levantado de revestimiento de piso flexible existente, ya sea vinílico en lámina o baldosa, linóleo o alfombra, incluido el adhesivo de fijación al contrapiso, ejecutado con medios manuales mediante espátula y rasqueta. Incluye la aplicación puntual de disolvente removedor en las zonas donde el adhesivo esté fuertemente adherido, el rascado hasta dejar el contrapiso limpio y sin restos que comprometan la adherencia del nuevo acabado, la ventilación del ambiente durante los trabajos, el retiro del material en sacos y la limpieza final. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
+          <t>Retiro de impermeabilización existente de manto asfáltico en cubierta, incluidos los solapes, los refuerzos de encuentro y la imprimación adherida al soporte, ejecutado con medios manuales mediante espátula y palanca, con aplicación puntual de calor para reblandecer las zonas fuertemente adheridas. Incluye la protección de los desagües para impedir que se obstruyan con restos, el corte del manto en franjas manejables, el rascado del soporte hasta dejarlo limpio y apto para recibir la nueva impermeabilización, el retiro del material en rollos atados y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente retirada.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1836,11 +1836,11 @@
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>2.12</v>
+        <v>3.44</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Aislamientos e impermeabilizaciones</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1857,12 +1857,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Demolición de piso continuo de concreto.</t>
+          <t>Retiro de impermeabilización líquida o acrílica.</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso continuo de concreto de hasta 10 cm de espesor, ejecutada con martillo neumático, sin afectar a la losa estructural ni a las instalaciones que discurran por debajo. Incluye la comprobación previa de que no existen tuberías ni canalizaciones enterradas en la zona, el corte perimetral con amoladora de disco de diamante para delimitar la demolición, la protección de los ambientes contiguos, el control de polvo, la fragmentación del escombro en piezas manejables, el retiro en sacos hasta el punto de acopio y la limpieza. Si el piso está armado con malla electrosoldada se incluye su corte y retiro. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Retiro de recubrimiento impermeabilizante líquido, acrílico o cementoso existente en cubierta o terraza, ejecutado con medios manuales mediante rasqueta y lijado mecánico, hasta dejar el soporte limpio y con la rugosidad adecuada para recibir el nuevo sistema. Incluye la protección de los desagües, el rascado de las zonas con burbujas o desprendimientos, el lijado de la superficie remanente, el aspirado del polvo generado y el retiro de los residuos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1874,11 +1874,11 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>15.33</v>
+        <v>3.34</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Aislamientos e impermeabilizaciones</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -1895,12 +1895,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Demolición de contrapiso o base de mortero de nivelación.</t>
+          <t>Demolición de tabique de bloque o ladrillo, incluidos sus revestimientos.</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Demolición de contrapiso o base de mortero de nivelación de hasta 5 cm de espesor, una vez retirado el piso de acabado, ejecutada con martillo eléctrico manual hasta dejar la losa estructural a la vista y limpia. Se emplea cuando la base existente está disgregada, hueca o fuera de nivel y no admite recibir el nuevo piso. Incluye la comprobación previa del estado de la base mediante golpeo, la protección de los ambientes contiguos, el control de polvo mediante aspiración, el retiro manual del escombro en sacos y el barrido final de la losa. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Demolición de tabique interior no estructural de bloque de concreto o ladrillo, con sus revestimientos por ambas caras, ejecutada con martillo eléctrico manual sin afectar a la estabilidad de los elementos constructivos contiguos. Incluye comprobación previa de que el tabique no es portante y de que no aloja instalaciones en servicio, protección del entorno, apeo puntual si fuera necesario, fragmentación del escombro en piezas manejables, retirada en sacos hasta el punto de acopio y limpieza de la zona. No incluye el transporte a vertedero. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1912,11 +1912,11 @@
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>7.18</v>
+        <v>5.42</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Particiones</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1933,12 +1933,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Desmontaje de piso técnico registrable.</t>
+          <t>Demolición de tabique de yeso laminado y su estructura.</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de piso técnico registrable existente, formado por paneles apoyados sobre pedestales regulables, ejecutado con medios manuales. Por tratarse de un sistema desmontable la operación es limpia y permite recuperar el material. Incluye la retirada ordenada de los paneles con ventosa, el desmontaje de los pedestales y travesaños, la clasificación de las piezas en aprovechables y desechables, el acopio protegido de las que el cliente desee conservar, el retiro del resto en sacos y la limpieza de la losa resultante. No incluye el bote del escombro. Medido en superficie realmente desmontada.</t>
+          <t>Demolición de tabique interior de placa de yeso laminado, junto con la perfilería de acero galvanizado y el aislamiento de la cámara, ejecutada con medios manuales. Incluye la localización y desconexión previa de las instalaciones que discurran por el interior del tabique, operación crítica en este sistema porque las tuberías y el cableado quedan ocultos y sin señalizar, la protección del piso, el desmontaje ordenado de las placas, el retiro del aislamiento, el desmontaje de la perfilería y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1950,11 +1950,11 @@
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>1.09</v>
+        <v>2.89</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Particiones</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -1971,12 +1971,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Demolición de cielo raso de yeso laminado y su estructura.</t>
+          <t>Demolición de muro de concreto no estructural.</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Demolición de cielo raso continuo de placa de yeso laminado, junto con la perfilería de acero galvanizado, las varillas de cuelgue y el ángulo perimetral, ejecutada con medios manuales. Incluye la desconexión y retiro previo de las luminarias, rejillas y difusores alojados en el plano del cielo, la protección del piso y del mobiliario, el descuelgue ordenado de las placas para evitar caídas incontroladas, el retiro del escombro en sacos y de la perfilería atada, y la limpieza de la zona dejando la losa a la vista. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Demolición de muro interior de concreto no estructural, incluidos sus revestimientos, ejecutada con martillo neumático y corte de la malla de refuerzo si la tuviera. Incluye la comprobación estructural previa que acredite que el muro no es portante ni de arriostramiento, requisito imprescindible antes de intervenir, el corte perimetral con disco de diamante, la protección del entorno, el control de polvo, la fragmentación del escombro y su retiro en sacos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1988,11 +1988,11 @@
         <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>2.69</v>
+        <v>17.5</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Particiones</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2009,12 +2009,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Demolición de cielo raso de yeso vaciado o pasta.</t>
+          <t>Apertura de vano en pared de bloque o ladrillo.</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Demolición de cielo raso de yeso vaciado, pasta o placa de yeso tradicional, junto con su estructura de soporte y elementos de cuelgue, ejecutada con medios manuales y martillo eléctrico donde el espesor lo requiera. Por tratarse de un material macizo genera más escombro y más polvo fino que un cielo de placa. Incluye la desconexión previa de las luminarias, la protección del piso y del mobiliario, el control de polvo mediante aspiración, el retiro del escombro en sacos y la limpieza de la losa resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Apertura de vano para puerta, ventana o paso en pared existente de bloque o ladrillo, ejecutada con corte perimetral mediante disco de diamante y demolición interior con martillo eléctrico. Incluye el replanteo del vano, el apeo provisional del dintel mediante puntales antes de iniciar la demolición, el corte perimetral que garantiza jambas rectas y sin desgarros hacia el resto del muro, la demolición controlada desde la parte superior, el retiro del escombro y el repaso de las jambas dejándolas aplomadas. No incluye el dintel definitivo ni el resane de las jambas, que se valoran aparte. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de vano realmente abierto.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2026,11 +2026,11 @@
         <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>4.91</v>
+        <v>17.78</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Particiones</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2047,12 +2047,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Desmontaje de cielo raso desmontable de fibra mineral.</t>
+          <t>Demolición de tabique de bloque de vidrio.</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de cielo raso registrable existente, formado por paneles apoyados sobre perfilería vista en retícula, ejecutado con medios manuales. Por ser un sistema desmontable la operación es limpia, rápida y permite recuperar buena parte del material. Incluye la retirada ordenada de los paneles, el desmontaje de la perfilería y de los tensores de cuelgue, la clasificación de las piezas en aprovechables y desechables, el acopio protegido de las que el cliente desee conservar y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Demolición de tabique o paño de bloque de vidrio, incluidas las juntas de mortero y la armadura de refuerzo entre hiladas, ejecutada con medios manuales y martillo eléctrico. Requiere precauciones específicas frente a la proyección de fragmentos cortantes: se encinta previamente la superficie de los bloques para que rompan de forma contenida y se emplea protección facial y guantes anticorte. Incluye la protección del entorno, la demolición descendente por hiladas, el retiro cuidadoso del material en sacos reforzados y la limpieza minuciosa de esquirlas. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2064,11 +2064,11 @@
         <v>1</v>
       </c>
       <c r="F43" t="n">
-        <v>1.65</v>
+        <v>6.79</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Particiones</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2085,28 +2085,28 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Desmontaje de cielo raso de machihembrado de madera.</t>
+          <t>Desmontaje de canal de aguas lluvias.</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de cielo raso de machihembrado o tablilla de madera, junto con los rastreles y la estructura de soporte fijada a la losa, ejecutado con medios manuales mediante palanca y barra. Incluye la desconexión previa de las luminarias, la protección del piso y del mobiliario, la extracción de los clavos y tornillos que queden en la estructura, el retiro del material en atados hasta el punto de acopio, la clasificación de las piezas aprovechables y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Desmontaje de canal o canalón de recogida de aguas lluvias, incluidos los soportes, las uniones y las piezas especiales, ejecutado con medios manuales desde andamio. Incluye el acordonamiento de la zona inferior, el desmontaje por tramos con sostenimiento previo, la extracción de los ganchos y anclajes al alero, el resane de los puntos de fijación, el descenso del material y su clasificación para reciclaje. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E44" t="n">
         <v>1</v>
       </c>
       <c r="F44" t="n">
-        <v>2.82</v>
+        <v>2.7</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Cubiertas</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2123,28 +2123,28 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Desmontaje de cielo raso de láminas de PVC o aluminio.</t>
+          <t>Desmontaje de bajante de aguas lluvias.</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de cielo raso formado por láminas de PVC, aluminio o material similar, junto con sus perfiles de soporte y remates perimetrales, ejecutado con medios manuales. Incluye la desconexión previa de las luminarias y rejillas, la protección del piso, el desencastre ordenado de las láminas para poder recuperarlas si el cliente lo desea, el desmontaje de la perfilería, el retiro del material hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Desmontaje de bajante de aguas lluvias, vista o empotrada, incluidos las abrazaderas, los codos y las piezas de conexión, ejecutado con medios manuales desde andamio. Incluye el acordonamiento de la zona inferior, el corte de la bajante en tramos manejables, la extracción de las abrazaderas ancladas a la fachada, el resane de los huecos de anclaje, el taponado provisional de la conexión a la red que permanece y el retiro del material. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E45" t="n">
         <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>1.76</v>
+        <v>2.72</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Cubiertas</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2156,17 +2156,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Fachadas y particiones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
+          <t>Desmontaje de cubierta de teja.</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Desmontaje de cubierta de teja criolla, teja plana o similar, incluidos el mortero de fijación y los caballetes de cumbrera, ejecutado con medios manuales desde andamio y con línea de vida. Incluye la comprobación previa del estado de la estructura de soporte antes de que el personal transite sobre ella, el desmontaje ordenado desde la cumbrera hacia el alero, el descenso de las tejas por medios mecánicos evitando el lanzamiento, la clasificación de las piezas aprovechables y el acopio del material. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2178,11 +2178,11 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>52.4</v>
+        <v>9.44</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Tabiquería de entramado autoportante</t>
+          <t>Cubiertas</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2194,17 +2194,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Fachadas y particiones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Tabique de bloque de concreto de 10 cm, recibido con mortero de pega.</t>
+          <t>Desmontaje de cubierta de lámina metálica o acerolit.</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Tabique interior no estructural de 10 cm de espesor, ejecutado con bloque hueco de concreto de 10x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Incluye replanteo y trazado sobre el piso, colocación de hiladas a nivel y plomo con la ayuda de reglas y cuerda, formación de huecos de paso, anclaje del tabique a los paramentos existentes, humedecido previo de las piezas y limpieza de restos. No incluye el friso ni los dinteles de los huecos, que se valoran aparte. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Desmontaje de cubierta de lámina metálica, acerolit, zinc o fibrocemento, incluidos los ganchos, tornillos y elementos de fijación a la estructura, ejecutado con medios manuales desde andamio y con línea de vida. Si la lámina es de fibrocemento antiguo debe verificarse la posible presencia de amianto, en cuyo caso el desmontaje queda fuera de esta partida y exige empresa autorizada. Incluye el desmontaje ordenado con sujeción de las láminas frente al viento, el descenso controlado, la clasificación del material y el acopio. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2216,11 +2216,11 @@
         <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>18.29</v>
+        <v>6.81</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Fábrica no estructural</t>
+          <t>Cubiertas</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2232,33 +2232,33 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Gestión de residuos</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Retirada y transporte de escombro a vertedero autorizado.</t>
+          <t>Desmontaje de estructura de techo.</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Retirada de escombro procedente de demoliciones desde el punto de acopio de la obra y transporte en camión volqueta hasta vertedero o botadero autorizado, incluido el canon de vertido. Incluye la carga manual del escombro sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado con una distancia media considerada de 25 km, la descarga y la limpieza de la zona de carga. Medido por metro cúbico de escombro esponjado realmente retirado.</t>
+          <t>Desmontaje de la estructura de soporte de cubierta, formada por correas, cerchas o perfiles de madera o metal, una vez retirado el material de cubrición. Ejecutado con sierra, oxicorte o desatornillado según el material, con apeo previo y eslingado de los elementos antes de liberarlos. Incluye el estudio del orden de desmontaje para conservar la estabilidad del conjunto, el sostenimiento de cada pieza antes del corte, el descenso mecánico, la clasificación del material recuperable y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de cubierta cuya estructura se desmonta.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E48" t="n">
         <v>1</v>
       </c>
       <c r="F48" t="n">
-        <v>16.07</v>
+        <v>14.46</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Transporte de residuos</t>
+          <t>Cubiertas</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2270,33 +2270,33 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+          <t>Demolición de pendientado y protección de cubierta plana.</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+          <t>Demolición de la capa de pendientado y de la protección de cubierta plana, comprendiendo el relleno aligerado de formación de pendiente, la capa de mortero de protección y el acabado superficial, hasta descubrir la losa. Ejecutada con martillo eléctrico manual. Incluye la protección y taponado provisional de los desagües, la comprobación de no perforar la losa, el control del acopio de escombro sobre la cubierta para no sobrecargarla, su descenso por medios mecánicos y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E49" t="n">
         <v>1</v>
       </c>
       <c r="F49" t="n">
-        <v>8.369999999999999</v>
+        <v>11.27</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Cubiertas</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2308,33 +2308,33 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+          <t>Picado de enchapado cerámico en pared y su capa de pega.</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+          <t>Picado de enchapado cerámico o de porcelanato existente en pared, incluida su capa de pega de mortero, ejecutado con martillo eléctrico manual hasta dejar el friso o el bloque a la vista, sin comprometer la estabilidad del muro ni dañar las tuberías y canalizaciones empotradas. Incluye la localización previa de las instalaciones que discurren por el paramento, la protección de pisos, aparatos y puertas, el control de polvo mediante aspiración, el retiro manual del escombro en sacos hasta el punto de acopio y la limpieza de la superficie, dejándola lista para recibir el nuevo friso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E50" t="n">
         <v>1</v>
       </c>
       <c r="F50" t="n">
-        <v>8.720000000000001</v>
+        <v>6.25</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2346,33 +2346,33 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+          <t>Picado de enchapado de granito o terrazo en pared.</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+          <t>Picado de enchapado de granito o terrazo prefabricado existente en pared, incluida su capa de asiento de mortero, ejecutado con martillo eléctrico manual. Por el mayor espesor y peso de estas piezas frente al enchapado cerámico, el rendimiento es menor y el escombro más pesado. Incluye la protección de pisos y ambientes contiguos, el control de polvo, el retiro manual del escombro en sacos hasta el punto de acopio y el repicado de los restos de mortero adheridos al paramento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E51" t="n">
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>37.22</v>
+        <v>7.31</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Fontanería</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2384,33 +2384,33 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+          <t>Picado de enchapado de piedra natural en pared.</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+          <t>Picado de enchapado de piedra natural existente en pared, ya sea mármol, laja o piedra de revestimiento, incluida su capa de asiento y los anclajes metálicos si los tuviera, ejecutado con martillo eléctrico manual. Si el cliente desea recuperar las piezas se desmontan una a una con cuidado, se limpian y se acopian protegidas, lo que reduce el rendimiento y debe advertirse en el presupuesto. Incluye la protección del entorno, el control de polvo, el retiro del escombro en sacos y el repicado de los restos adheridos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E52" t="n">
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>13.52</v>
+        <v>7.67</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Fontanería</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2422,33 +2422,33 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+          <t>Desmontaje de enchapado de madera o machihembrado en pared.</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+          <t>Desmontaje de revestimiento de madera existente en pared, ya sea machihembrado, tablilla o panel, junto con los rastreles de soporte fijados al paramento, ejecutado con medios manuales mediante palanca y barra. Incluye la extracción de los clavos, tornillos y tacos que queden en el muro, el retiro del material en sacos o atados hasta el punto de acopio, la clasificación de las piezas aprovechables si el cliente desea conservarlas y la limpieza del paramento resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E53" t="n">
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>7.45</v>
+        <v>2.21</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Fontanería</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2460,33 +2460,33 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Punto de desagüe para aparato sanitario.</t>
+          <t>Desmontaje de revestimiento de láminas o paneles en pared.</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+          <t>Desmontaje de revestimiento de pared formado por láminas o paneles de PVC, aluminio, melamina o material similar, junto con su estructura o rastrelado de soporte, ejecutado con medios manuales. Incluye el retiro de los perfiles de remate y esquineros, la extracción de las fijaciones que queden en el paramento, el resane puntual de los huecos de anclaje, el retiro del material hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E54" t="n">
         <v>1</v>
       </c>
       <c r="F54" t="n">
-        <v>33.84</v>
+        <v>1.56</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Saneamiento y desagües</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2498,33 +2498,33 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+          <t>Retiro de papel tapiz en paramento.</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+          <t>Retiro de papel tapiz existente en paramento interior, junto con los restos de pegamento mural, ejecutado con medios manuales mediante humectación previa con solución reblandecedora y raspado con espátula ancha. Incluye la protección de pisos, rodapiés y mecanismos, la aplicación de la solución en varias pasadas hasta que el papel se desprenda sin arrancar el friso, el rascado de los residuos de pegamento, el lavado final del paramento y su secado, dejándolo listo para recibir el nuevo acabado. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E55" t="n">
         <v>1</v>
       </c>
       <c r="F55" t="n">
-        <v>11.04</v>
+        <v>2.2</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Saneamiento y desagües</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2536,33 +2536,33 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+          <t>Desmontaje de moldura decorativa de yeso o poliestireno.</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Desmontaje de moldura decorativa corrida de yeso, poliestireno o poliuretano, situada en el encuentro de pared y cielo raso o como elemento decorativo en paramento, ejecutado con medios manuales mediante espátula y cincel. Incluye la protección del entorno, el corte previo de la línea de junta para evitar arrastrar el friso, el rascado de los restos de pasta o adhesivo, el resane puntual de los desconchados provocados, el retiro del material hasta el punto de acopio y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E56" t="n">
         <v>1</v>
       </c>
       <c r="F56" t="n">
-        <v>10.87</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Revestimientos de paramentos con piezas rígidas</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2574,17 +2574,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+          <t>Retiro de láminas decorativas, vinilos o espejos adheridos.</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Retiro de revestimiento decorativo adherido al paramento, ya sea lámina vinílica, calcomanía mural o espejo pegado, junto con los restos de adhesivo. Incluye la protección del piso y del mobiliario, el calentamiento o humectación previa para reblandecer el adhesivo, el desprendimiento controlado del material con espátula, y en el caso de espejos el encintado previo de la superficie para evitar la proyección de fragmentos al fracturarse. Incluye el rascado de los restos de adhesivo, el retiro del material en sacos y la limpieza del paramento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2596,11 +2596,11 @@
         <v>1</v>
       </c>
       <c r="F57" t="n">
-        <v>3.46</v>
+        <v>1.6</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Pinturas</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2612,17 +2612,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+          <t>Demolición de revestimiento cerámico de escalera.</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+          <t>Demolición del revestimiento cerámico de escalera, comprendiendo huellas, contrahuellas y su capa de pega, ejecutada con martillo eléctrico manual sin comprometer la losa de la escalera. El rendimiento es sensiblemente menor que en un piso corrido por la posición forzada de trabajo, la superficie fragmentada en peldaños y la dificultad de evacuar el escombro por la propia escalera. Incluye la protección del hueco y del pasamanos, el control de polvo, el retiro manual del escombro en sacos y la limpieza, dejando los peldaños listos para el nuevo revestimiento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida, desarrollando huella y contrahuella.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2634,11 +2634,11 @@
         <v>1</v>
       </c>
       <c r="F58" t="n">
-        <v>5.23</v>
+        <v>7.27</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Pinturas</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2650,17 +2650,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+          <t>Demolición de revestimiento de granito o piedra natural en escalera.</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Demolición del revestimiento de granito, terrazo o piedra natural de escalera, comprendiendo huellas, contrahuellas y su capa de asiento, ejecutada con martillo eléctrico manual. Al mayor espesor y peso de las piezas se suma la dificultad propia del trabajo en escalera, por lo que el rendimiento es el más bajo de los grupos de demolición de revestimientos. Incluye la protección del hueco y del pasamanos, el control de polvo, el retiro manual del escombro en sacos y el repicado de los restos de mortero adheridos a los peldaños. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida, desarrollando huella y contrahuella.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2672,11 +2672,11 @@
         <v>1</v>
       </c>
       <c r="F59" t="n">
-        <v>2.82</v>
+        <v>8.58</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Pinturas</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2688,33 +2688,33 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+          <t>Demolición de zócalo escalonado de escalera.</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Demolición del zócalo o rodapié escalonado que acompaña a la escalera en su encuentro con el paramento, incluida su capa de pega, ejecutada con medios manuales y martillo eléctrico, cuidando de no dañar el friso por encima de la línea del zócalo. Incluye el repicado de los restos de mortero adheridos, el retiro del escombro en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud real de la línea inclinada del zócalo.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E60" t="n">
         <v>1</v>
       </c>
       <c r="F60" t="n">
-        <v>10.75</v>
+        <v>1.78</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Revestimientos continuos</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -2726,17 +2726,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+          <t>Picado de friso de mortero en paramento.</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+          <t>Picado de friso de mortero de cemento existente en paramento interior o exterior, ejecutado con martillo eléctrico manual hasta dejar el bloque o el ladrillo a la vista, cuando el friso está disgregado, hueco o presenta fisuración generalizada. Incluye el sondeo previo por golpeo para delimitar las zonas sin adherencia, la protección de pisos y ambientes contiguos, el control de polvo mediante aspiración, el retiro manual del escombro en sacos hasta el punto de acopio y el barrido y limpieza del paramento, dejándolo listo para recibir el nuevo friso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2748,11 +2748,11 @@
         <v>1</v>
       </c>
       <c r="F61" t="n">
-        <v>8.02</v>
+        <v>5.86</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -2764,33 +2764,33 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+          <t>Picado de friso de yeso o pasta en paramento.</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+          <t>Picado de revestimiento de yeso o pasta existente en paramento interior, ejecutado con medios manuales mediante espátula ancha y cincel, con martillo eléctrico solo en las zonas de mayor espesor. Por tratarse de un material blando el rendimiento es sensiblemente mayor que en un friso de mortero, aunque genera abundante polvo fino. Incluye la protección del entorno, el control de polvo mediante aspiración continua, el retiro del escombro en sacos hasta el punto de acopio y la limpieza del paramento resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E62" t="n">
         <v>1</v>
       </c>
       <c r="F62" t="n">
-        <v>1.69</v>
+        <v>3.65</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -2802,17 +2802,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+          <t>Picado de estuco o pasta decorativa en paramento.</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Picado de revestimiento de estuco, pasta decorativa o revestimiento texturado existente en paramento, ejecutado con medios manuales y martillo eléctrico según el espesor y la dureza del material, hasta dejar el soporte limpio y apto para recibir el nuevo acabado. Incluye la cata previa para identificar el espesor y el tipo de soporte, la protección del entorno, el control de polvo, el retiro del escombro en sacos y la limpieza final. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2824,11 +2824,11 @@
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>9.17</v>
+        <v>4.3</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -2840,17 +2840,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+          <t>Repicado de superficie de concreto para mejorar adherencia.</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Repicado superficial de paramento o losa de concreto, ejecutado con martillo eléctrico y puntero, para crear la rugosidad necesaria que garantice la adherencia del friso o del mortero de recrecido posterior. Incluye la limpieza previa de la superficie, el picado uniforme sin llegar a descubrir la armadura, la eliminación de lechadas superficiales y restos de desencofrante, el soplado y aspirado del polvo resultante y la retirada de los restos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente repicada.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2862,11 +2862,11 @@
         <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>12.51</v>
+        <v>4.37</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -2878,17 +2878,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+          <t>Eliminación de pintura en paramento mediante raspado y decapado.</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+          <t>Eliminación de las capas de pintura existentes en paramento interior o exterior, mediante raspado mecánico con espátula y lijado, con aplicación puntual de decapante químico en gel en las zonas de pintura muy adherida o de espesor elevado. Se emplea cuando la pintura existente está cuarteada, sopla o es incompatible con el nuevo acabado. Incluye la protección de pisos, carpintería y mobiliario, la ventilación del ambiente durante la aplicación del decapante, la neutralización y lavado de los restos químicos, el aspirado del polvo y la retirada de los residuos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2900,11 +2900,11 @@
         <v>1</v>
       </c>
       <c r="F65" t="n">
-        <v>18.47</v>
+        <v>5.15</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Falsos techos</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -2916,33 +2916,33 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Señalización y equipamiento</t>
+          <t>Demoliciones</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+          <t>Picado de salpicado o graniplast en fachada.</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+          <t>Picado de revestimiento de salpicado, graniplast o revestimiento pétreo proyectado en fachada, ejecutado con martillo eléctrico manual y espátula, hasta dejar el friso base sano o el bloque a la vista según el estado del soporte. Incluye el sondeo previo por golpeo para delimitar las zonas sin adherencia, el trabajo desde andamio con las protecciones colectivas correspondientes, la protección de carpinterías y de la zona de paso a pie de fachada, el control de la caída de escombro, su retiro en sacos hasta el punto de acopio y la limpieza del paramento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E66" t="n">
         <v>1</v>
       </c>
       <c r="F66" t="n">
-        <v>23.45</v>
+        <v>7.11</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Revestimientos y trasdosados</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -2954,36 +2954,2088 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Picado de mortero monocapa en fachada.</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Picado de revestimiento de mortero monocapa en fachada, incluida su malla de refuerzo y los perfiles de arranque y goterón, ejecutado con martillo eléctrico manual hasta dejar el soporte limpio y apto para recibir el nuevo revestimiento. Incluye el sondeo previo del paramento, el trabajo desde andamio con las protecciones colectivas correspondientes, la protección de carpinterías y del paso a pie de fachada, el corte y retiro de la malla, el control de la caída de escombro, su retiro en sacos y la limpieza del soporte. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>1</v>
+      </c>
+      <c r="F67" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Demolición de trasdosado de yeso laminado y su estructura.</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de trasdosado autoportante de placa de yeso laminado adosado a muro, junto con la perfilería de acero galvanizado y el aislamiento alojado en la cámara, ejecutada con medios manuales. Incluye la localización y desconexión previa de los mecanismos e instalaciones que discurran por el trasdosado, la protección del piso y del mobiliario, el desmontaje ordenado de las placas, el retiro del aislamiento en sacos, el desmontaje de la perfilería y de las fijaciones al muro, y la limpieza de la zona dejando el paramento original a la vista. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Demolición de trasdosado de bloque o ladrillo adosado a muro.</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de tabique de bloque o ladrillo adosado a muro a modo de trasdosado, incluidos sus revestimientos y la cámara intermedia, ejecutada con martillo eléctrico manual sin dañar el muro original que permanece. Incluye la comprobación previa de que el trasdosado no cumple función estructural ni aloja instalaciones en servicio, la protección del entorno, el control de polvo, la fragmentación del escombro en piezas manejables, el retiro en sacos hasta el punto de acopio y el repicado de los restos de mortero adheridos al muro. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Desmontaje de trasdosado directo de placa pegada al muro.</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Desmontaje de trasdosado directo formado por placa de yeso laminado o panel aislante adherido al muro mediante pelladas de pasta, ejecutado con medios manuales mediante palanca y espátula. Incluye la protección del piso, el arranque de las placas, el rascado de los restos de pasta y adhesivo adheridos al muro hasta dejarlo apto para recibir el nuevo revestimiento, el retiro del material en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Demolición de piso cerámico y su capa de pega.</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de piso existente de baldosa cerámica o de porcelanato, junto con su capa de pega de mortero, ejecutada con martillo eléctrico manual sin comprometer la losa ni los elementos constructivos vecinos. Incluye protección previa de paredes, puertas y ambientes contiguos, control de polvo mediante aspiración, retiro manual del escombro en sacos hasta el punto de acopio y barrido de la superficie resultante, dejándola lista para recibir el nuevo contrapiso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>1</v>
+      </c>
+      <c r="F71" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Demolición de rodapié cerámico.</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de rodapié existente de baldosa cerámica o de porcelanato y de su capa de pega, ejecutada con medios manuales y martillo eléctrico, cuidando de no dañar el friso de la pared por encima de la línea del rodapié. Incluye retiro manual del escombro en sacos hasta el punto de acopio, repicado de los restos de mortero adheridos y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Demolición de piso de granito o terrazo en baldosa.</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de piso existente de baldosa de granito o terrazo prefabricado, junto con su capa de asiento de mortero, ejecutada con martillo eléctrico manual. Por la dureza y el espesor de este tipo de baldosa el rendimiento es menor que en un piso cerámico y el escombro resulta más pesado, lo que se refleja en el rendimiento de la partida. Incluye protección previa de los ambientes contiguos, control de polvo, retiro manual del escombro en sacos y limpieza de la superficie. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>1</v>
+      </c>
+      <c r="F73" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Demolición de rodapié de granito o terrazo.</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de rodapié existente de granito o terrazo prefabricado y de su capa de asiento, ejecutada con martillo eléctrico manual, cuidando de no dañar el friso de la pared. Incluye repicado de los restos de mortero adheridos, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>1</v>
+      </c>
+      <c r="F74" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Demolición de piso de granito vaciado en sitio.</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de piso continuo de granito vaciado en sitio, incluida su base de mortero y las platinas divisorias de las juntas, ejecutada con martillo neumático por tratarse de una superficie monolítica de gran dureza. Incluye corte perimetral previo con amoladora de disco de diamante para delimitar la zona de intervención y evitar desprendimientos fuera de ella, protección de los ambientes contiguos, control de polvo, fragmentación del escombro en piezas manejables, retiro en sacos y limpieza. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>1</v>
+      </c>
+      <c r="F75" t="n">
+        <v>13.04</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Demolición de piso de cemento pulido.</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de piso continuo de cemento pulido y de su base de mortero, ejecutada con martillo eléctrico manual, sin afectar a la losa estructural. Incluye corte perimetral con amoladora cuando la demolición sea parcial, protección de los ambientes contiguos, control de polvo mediante aspiración, fragmentación del escombro, retiro manual en sacos hasta el punto de acopio y limpieza de la superficie resultante. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>1</v>
+      </c>
+      <c r="F76" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Demolición de rodapié de cemento.</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de rodapié corrido de mortero de cemento, ejecutada con medios manuales y cincel, cuidando de no dañar el friso de la pared por encima de la línea del rodapié. Incluye repicado de los restos adheridos al paramento, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>1</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Demolición de piso de piedra natural.</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de piso existente de piedra natural, ya sea mármol, granito natural o laja, junto con su capa de asiento de mortero, ejecutada con martillo eléctrico manual. Si el cliente desea recuperar las piezas, se levantan una a una con cuidado, se limpian de mortero y se acopian protegidas, lo que reduce el rendimiento y debe advertirse en el presupuesto. Incluye protección de los ambientes contiguos, control de polvo, retiro manual del escombro en sacos y limpieza de la superficie. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>1</v>
+      </c>
+      <c r="F78" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Demolición de rodapié de piedra natural.</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de rodapié existente de piedra natural y de su capa de asiento, ejecutada con martillo eléctrico manual, cuidando de no dañar el friso de la pared. Incluye repicado de los restos de mortero adheridos, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>1</v>
+      </c>
+      <c r="F79" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Levantado de piso de parquet o madera.</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Levantado de piso existente de parquet o de tablilla de madera, incluidos los rastreles o el adhesivo de fijación al contrapiso, ejecutado con medios manuales mediante palanca y espátula. Incluye el retiro previo de las molduras de remate, el rascado de los restos de adhesivo adheridos al contrapiso, la extracción de los clavos o tornillos que queden en la base, el retiro del material en sacos hasta el punto de acopio y la limpieza de la superficie resultante. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>1</v>
+      </c>
+      <c r="F80" t="n">
+        <v>2.17</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Levantado de rodapié de madera.</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Levantado de rodapié existente de madera, ejecutado con medios manuales mediante palanca y espátula, cuidando de no dañar el friso de la pared. Incluye la extracción de los clavos, tornillos o tacos de fijación que queden en el paramento, el retiro del material en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente levantada.</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>1</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Levantado de piso laminado.</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Levantado de piso laminado flotante existente, incluidas la manta acústica y las molduras de remate perimetrales, ejecutado con medios manuales. Por tratarse de un sistema flotante de encastre el desmontaje es rápido y no genera escombro pesado. Incluye el desmontaje ordenado de las tablas, el retiro de la manta y del perfil perimetral, la limpieza y aspirado del contrapiso resultante y el retiro del material en sacos hasta el punto de acopio. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Levantado de piso vinílico, linóleo o alfombra.</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Levantado de revestimiento de piso flexible existente, ya sea vinílico en lámina o baldosa, linóleo o alfombra, incluido el adhesivo de fijación al contrapiso, ejecutado con medios manuales mediante espátula y rasqueta. Incluye la aplicación puntual de disolvente removedor en las zonas donde el adhesivo esté fuertemente adherido, el rascado hasta dejar el contrapiso limpio y sin restos que comprometan la adherencia del nuevo acabado, la ventilación del ambiente durante los trabajos, el retiro del material en sacos y la limpieza final. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>1</v>
+      </c>
+      <c r="F83" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Demolición de piso continuo de concreto.</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de piso continuo de concreto de hasta 10 cm de espesor, ejecutada con martillo neumático, sin afectar a la losa estructural ni a las instalaciones que discurran por debajo. Incluye la comprobación previa de que no existen tuberías ni canalizaciones enterradas en la zona, el corte perimetral con amoladora de disco de diamante para delimitar la demolición, la protección de los ambientes contiguos, el control de polvo, la fragmentación del escombro en piezas manejables, el retiro en sacos hasta el punto de acopio y la limpieza. Si el piso está armado con malla electrosoldada se incluye su corte y retiro. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>1</v>
+      </c>
+      <c r="F84" t="n">
+        <v>15.33</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Demolición de contrapiso o base de mortero de nivelación.</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de contrapiso o base de mortero de nivelación de hasta 5 cm de espesor, una vez retirado el piso de acabado, ejecutada con martillo eléctrico manual hasta dejar la losa estructural a la vista y limpia. Se emplea cuando la base existente está disgregada, hueca o fuera de nivel y no admite recibir el nuevo piso. Incluye la comprobación previa del estado de la base mediante golpeo, la protección de los ambientes contiguos, el control de polvo mediante aspiración, el retiro manual del escombro en sacos y el barrido final de la losa. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>1</v>
+      </c>
+      <c r="F85" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Desmontaje de piso técnico registrable.</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Desmontaje de piso técnico registrable existente, formado por paneles apoyados sobre pedestales regulables, ejecutado con medios manuales. Por tratarse de un sistema desmontable la operación es limpia y permite recuperar el material. Incluye la retirada ordenada de los paneles con ventosa, el desmontaje de los pedestales y travesaños, la clasificación de las piezas en aprovechables y desechables, el acopio protegido de las que el cliente desee conservar, el retiro del resto en sacos y la limpieza de la losa resultante. No incluye el bote del escombro. Medido en superficie realmente desmontada.</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>1</v>
+      </c>
+      <c r="F86" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Demolición de cielo raso de yeso laminado y su estructura.</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de cielo raso continuo de placa de yeso laminado, junto con la perfilería de acero galvanizado, las varillas de cuelgue y el ángulo perimetral, ejecutada con medios manuales. Incluye la desconexión y retiro previo de las luminarias, rejillas y difusores alojados en el plano del cielo, la protección del piso y del mobiliario, el descuelgue ordenado de las placas para evitar caídas incontroladas, el retiro del escombro en sacos y de la perfilería atada, y la limpieza de la zona dejando la losa a la vista. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>1</v>
+      </c>
+      <c r="F87" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Demolición de cielo raso de yeso vaciado o pasta.</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de cielo raso de yeso vaciado, pasta o placa de yeso tradicional, junto con su estructura de soporte y elementos de cuelgue, ejecutada con medios manuales y martillo eléctrico donde el espesor lo requiera. Por tratarse de un material macizo genera más escombro y más polvo fino que un cielo de placa. Incluye la desconexión previa de las luminarias, la protección del piso y del mobiliario, el control de polvo mediante aspiración, el retiro del escombro en sacos y la limpieza de la losa resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>1</v>
+      </c>
+      <c r="F88" t="n">
+        <v>4.91</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Desmontaje de cielo raso desmontable de fibra mineral.</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Desmontaje de cielo raso registrable existente, formado por paneles apoyados sobre perfilería vista en retícula, ejecutado con medios manuales. Por ser un sistema desmontable la operación es limpia, rápida y permite recuperar buena parte del material. Incluye la retirada ordenada de los paneles, el desmontaje de la perfilería y de los tensores de cuelgue, la clasificación de las piezas en aprovechables y desechables, el acopio protegido de las que el cliente desee conservar y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>1</v>
+      </c>
+      <c r="F89" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Desmontaje de cielo raso de machihembrado de madera.</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Desmontaje de cielo raso de machihembrado o tablilla de madera, junto con los rastreles y la estructura de soporte fijada a la losa, ejecutado con medios manuales mediante palanca y barra. Incluye la desconexión previa de las luminarias, la protección del piso y del mobiliario, la extracción de los clavos y tornillos que queden en la estructura, el retiro del material en atados hasta el punto de acopio, la clasificación de las piezas aprovechables y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>1</v>
+      </c>
+      <c r="F90" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Desmontaje de cielo raso de láminas de PVC o aluminio.</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Desmontaje de cielo raso formado por láminas de PVC, aluminio o material similar, junto con sus perfiles de soporte y remates perimetrales, ejecutado con medios manuales. Incluye la desconexión previa de las luminarias y rejillas, la protección del piso, el desencastre ordenado de las láminas para poder recuperarlas si el cliente lo desea, el desmontaje de la perfilería, el retiro del material hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>1</v>
+      </c>
+      <c r="F91" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Desmontaje de mueble de baño y sus accesorios.</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Desmontaje de mueble de baño con su lavamanos integrado, espejo y accesorios como toalleros, jaboneras y portarrollos. Ejecutado con medios manuales y atornillador. Incluye el cierre previo de las llaves de paso, la desconexión de las tomas de agua y del desagüe con recogida del agua retenida en el sifón, el corte del sellado perimetral, el desmontaje del mueble y del espejo con sostenimiento previo, la extracción de los anclajes, el resane de los huecos y el retiro del material. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por conjunto realmente desmontado.</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>1</v>
+      </c>
+      <c r="F92" t="n">
+        <v>6.86</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Equipamiento</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Desmontaje de mueble de cocina alto o bajo.</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Desmontaje de mueble de cocina alto o bajo, incluidas las puertas, los entrepaños, los cajones y los herrajes de fijación al paramento. Ejecutado con medios manuales y atornillador. Incluye el vaciado previo del contenido si el cliente no lo hubiera retirado, la desconexión de las instalaciones que atraviesen el mueble, el desmontaje ordenado desde las puertas hacia el cuerpo, la extracción de tacos y tornillos del muro, el resane de los huecos de anclaje y la clasificación de las piezas aprovechables. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud de frente de mueble realmente desmontada.</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>1</v>
+      </c>
+      <c r="F93" t="n">
+        <v>5.11</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Equipamiento</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Desmontaje de mesón de cocina y su salpicadero.</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Desmontaje de mesón o tope de cocina, sea de granito, cuarzo, concreto o laminado, junto con su salpicadero y la estructura de apoyo. Ejecutado con medios manuales, amoladora y martillo eléctrico según el material. Incluye el desmontaje previo del fregadero y de la placa de cocción si permanecieran, el corte del sellado perimetral, el sostenimiento del tablero por dos operarios dado su peso, el corte en tramos manejables cuando no pueda extraerse entero, el picado de los apoyos de obra, el resane del paramento y el retiro del material. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud de mesón realmente desmontada.</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>1</v>
+      </c>
+      <c r="F94" t="n">
+        <v>8.76</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Equipamiento</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Desmontaje de mobiliario fijo diverso.</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Desmontaje de mobiliario fijo no clasificado en las partidas anteriores, tal como repisas de obra, bancos, barras, mostradores o estanterías ancladas al paramento. Ejecutado con medios manuales, atornillador, amoladora y martillo eléctrico según el material y el tipo de anclaje. Incluye el vaciado previo, el sostenimiento del elemento antes de liberar el último anclaje, la extracción de las fijaciones, el picado de los apoyos de obra si los tuviera, el resane de los huecos y el retiro del material clasificado. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de frente realmente desmontada.</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>1</v>
+      </c>
+      <c r="F95" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Equipamiento</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Demolición de muro de cerca perimetral.</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de muro de cerca perimetral de bloque, ladrillo o concreto, incluidos sus revestimientos y las columnas de arriostramiento, ejecutada con martillo eléctrico o neumático según el espesor. Incluye el acordonamiento y señalización de la zona a ambos lados del muro, la comprobación de que no existen instalaciones adosadas ni servidumbres del vecino, la demolición descendente por hiladas para evitar vuelcos incontrolados, el corte de las armaduras de las columnas, el acopio del escombro y la limpieza del terreno. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>1</v>
+      </c>
+      <c r="F96" t="n">
+        <v>11.27</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Urbanización interior de la parcela</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Desmontaje de cerca de malla ciclónica.</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Desmontaje de cerca de malla ciclónica o alfajol, incluidos los tubos o postes de soporte, los tensores, el alambre de púas de coronación y las bases de concreto de los postes. Ejecutado con medios manuales, amoladora y martillo eléctrico. Incluye el destensado previo de la malla, el corte y enrollado en tramos manejables, la extracción de los postes con demolición de sus dados de concreto, el relleno de los huecos resultantes, la clasificación del material recuperable y el retiro. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>1</v>
+      </c>
+      <c r="F97" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Urbanización interior de la parcela</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Demolición de tanquilla o registro enterrado.</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de tanquilla, registro o caja de paso enterrada de concreto o mampostería, incluidas su tapa, sus paredes y su solera, ejecutada con martillo eléctrico previa excavación de descubrimiento. Incluye la comprobación previa de que la tanquilla está fuera de servicio, el vaciado y limpieza de su interior, el taponado de las tuberías que acometen y permanecen activas, la demolición de las paredes y la solera, la extracción del escombro y el relleno y compactación del hueco resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad demolida.</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>1</v>
+      </c>
+      <c r="F98" t="n">
+        <v>33.71</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Urbanización interior de la parcela</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Demoliciones</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Tala y destronque de árbol.</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Tala y destronque de árbol de porte medio situado en el interior de la parcela, incluidos el desrame previo, el troceado del fuste, la extracción del tocón y del sistema radicular superficial y el relleno del hueco resultante. Ejecutado con motosierra y retroexcavadora. Incluye la comprobación previa de que la especie no está protegida y de que se cuenta con la autorización municipal cuando sea exigible, el acordonamiento de la zona de caída, el desrame descendente, el troceado en piezas transportables, la extracción del tocón y el relleno y compactación del hueco. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad talada.</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>1</v>
+      </c>
+      <c r="F99" t="n">
+        <v>89.09999999999999</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Urbanización interior de la parcela</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Fachadas y particiones</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>1</v>
+      </c>
+      <c r="F100" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Tabiquería de entramado autoportante</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Fachadas y particiones</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Tabique de bloque de concreto de 10 cm, recibido con mortero de pega.</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Tabique interior no estructural de 10 cm de espesor, ejecutado con bloque hueco de concreto de 10x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Incluye replanteo y trazado sobre el piso, colocación de hiladas a nivel y plomo con la ayuda de reglas y cuerda, formación de huecos de paso, anclaje del tabique a los paramentos existentes, humedecido previo de las piezas y limpieza de restos. No incluye el friso ni los dinteles de los huecos, que se valoran aparte. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>1</v>
+      </c>
+      <c r="F101" t="n">
+        <v>18.29</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Fábrica no estructural</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Gestión de residuos</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Retirada y transporte de escombro a vertedero autorizado.</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Retirada de escombro procedente de demoliciones desde el punto de acopio de la obra y transporte en camión volqueta hasta vertedero o botadero autorizado, incluido el canon de vertido. Incluye la carga manual del escombro sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado con una distancia media considerada de 25 km, la descarga y la limpieza de la zona de carga. Medido por metro cúbico de escombro esponjado realmente retirado.</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>1</v>
+      </c>
+      <c r="F102" t="n">
+        <v>16.07</v>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Transporte de residuos</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>1</v>
+      </c>
+      <c r="F103" t="n">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Eléctrica</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>1</v>
+      </c>
+      <c r="F104" t="n">
+        <v>8.720000000000001</v>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Eléctrica</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>1</v>
+      </c>
+      <c r="F105" t="n">
+        <v>37.22</v>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Fontanería</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F106" t="n">
+        <v>13.52</v>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Fontanería</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>1</v>
+      </c>
+      <c r="F107" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Fontanería</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Punto de desagüe para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>1</v>
+      </c>
+      <c r="F108" t="n">
+        <v>33.84</v>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Saneamiento y desagües</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Instalaciones</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>1</v>
+      </c>
+      <c r="F109" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Saneamiento y desagües</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>1</v>
+      </c>
+      <c r="F110" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Revestimientos de paramentos con piezas rígidas</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>1</v>
+      </c>
+      <c r="F111" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Pinturas</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>1</v>
+      </c>
+      <c r="F112" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Pinturas</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>1</v>
+      </c>
+      <c r="F113" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Pinturas</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>1</v>
+      </c>
+      <c r="F114" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Revestimientos continuos</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>1</v>
+      </c>
+      <c r="F115" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>1</v>
+      </c>
+      <c r="F116" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>1</v>
+      </c>
+      <c r="F117" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>1</v>
+      </c>
+      <c r="F118" t="n">
+        <v>12.51</v>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Pavimentos</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Revestimientos y trasdosados</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>1</v>
+      </c>
+      <c r="F119" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Falsos techos</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
           <t>Señalización y equipamiento</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>1</v>
+      </c>
+      <c r="F120" t="n">
+        <v>23.45</v>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Señalización y equipamiento</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
         <is>
           <t>Instalación de lavamanos con su grifería y desagüe.</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
+      <c r="C121" s="2" t="inlineStr">
         <is>
           <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D121" t="inlineStr">
         <is>
           <t>ud</t>
         </is>
       </c>
-      <c r="E67" t="n">
-        <v>1</v>
-      </c>
-      <c r="F67" t="n">
+      <c r="E121" t="n">
+        <v>1</v>
+      </c>
+      <c r="F121" t="n">
         <v>36.45</v>
       </c>
-      <c r="G67" t="inlineStr">
+      <c r="G121" t="inlineStr">
         <is>
           <t>Aparatos sanitarios y grifería</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr">
+      <c r="H121" t="inlineStr">
         <is>
           <t>incluida</t>
         </is>

</xml_diff>

<commit_message>
Migrar a codificacion propia CotizaT y estructura venezolana de 20 capitulos; separar ambitos reforma y obra nueva
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/catalogo_partidas.xlsx
+++ b/basedatos_partidas/salida/catalogo_partidas.xlsx
@@ -484,33 +484,33 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Demolición de losa de fundación de concreto armado.</t>
+          <t>Demolición de piso cerámico y su capa de pega.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Demolición de losa de fundación de concreto armado, ejecutada con martillo hidráulico montado sobre retroexcavadora y corte de la malla de refuerzo. Incluye el corte perimetral previo para delimitar la zona de intervención, la comprobación de que no discurren instalaciones enterradas bajo la losa, la fragmentación del concreto en piezas cargables, el corte y separación del acero para su gestión diferenciada, el acopio del escombro y la limpieza del terreno resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en volumen realmente demolido.</t>
+          <t>Demolición de piso existente de baldosa cerámica o de porcelanato, junto con su capa de pega de mortero, ejecutada con martillo eléctrico manual sin comprometer la losa ni los elementos constructivos vecinos. Incluye protección previa de paredes, puertas y ambientes contiguos, control de polvo mediante aspiración, retiro manual del escombro en sacos hasta el punto de acopio y barrido de la superficie resultante, dejándola lista para recibir el nuevo contrapiso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E2" t="n">
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>119.83</v>
+        <v>4.88</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Cimentaciones</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -522,33 +522,33 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Demolición de viga de riostra o muro de contención de concreto.</t>
+          <t>Demolición de rodapié cerámico.</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Demolición de viga de riostra, muro de contención o murete de concreto armado, ejecutada con martillo neumático y corte de armaduras. Incluye la comprobación previa de que el elemento no sostiene empujes de tierra activos o, en su caso, el sostenimiento provisional del terreno, la protección del entorno, el corte y retiro del acero de refuerzo, la fragmentación del concreto y su acopio, y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en volumen realmente demolido.</t>
+          <t>Demolición de rodapié existente de baldosa cerámica o de porcelanato y de su capa de pega, ejecutada con medios manuales y martillo eléctrico, cuidando de no dañar el friso de la pared por encima de la línea del rodapié. Incluye retiro manual del escombro en sacos hasta el punto de acopio, repicado de los restos de mortero adheridos y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E3" t="n">
         <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>104.61</v>
+        <v>1</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Cimentaciones</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -560,33 +560,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Demolición de zapata o pedestal de concreto armado.</t>
+          <t>Demolición de piso de granito o terrazo en baldosa.</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Demolición de zapata aislada o pedestal de concreto armado, ejecutada con martillo neumático y corte de la armadura con oxicorte o amoladora. Requiere comprobación estructural previa de que el elemento ya no cumple función portante o de que la estructura está debidamente apeada. Incluye la excavación de descubrimiento del elemento si estuviera enterrado, la protección del entorno, el corte y retiro de las barras de acero, la fragmentación del concreto en piezas manejables y su acopio, y el relleno del hueco resultante si el proyecto lo requiere. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en volumen realmente demolido.</t>
+          <t>Demolición de piso existente de baldosa de granito o terrazo prefabricado, junto con su capa de asiento de mortero, ejecutada con martillo eléctrico manual. Por la dureza y el espesor de este tipo de baldosa el rendimiento es menor que en un piso cerámico y el escombro resulta más pesado, lo que se refleja en el rendimiento de la partida. Incluye protección previa de los ambientes contiguos, control de polvo, retiro manual del escombro en sacos y limpieza de la superficie. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>113.98</v>
+        <v>5.9</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Cimentaciones</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -598,33 +598,33 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Desmontaje de estructura metálica.</t>
+          <t>Demolición de rodapié de granito o terrazo.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de estructura metálica de acero, formada por perfiles laminados o armados, ejecutado mediante oxicorte y desatornillado según el tipo de unión, con apeo previo de los elementos que permanecen. Incluye el estudio del orden de desmontaje para mantener la estabilidad del conjunto en todo momento, el eslingado y sostenimiento de las piezas antes de liberarlas, el corte en tramos transportables, el descenso a nivel de acopio y la clasificación del acero para su venta o gestión como chatarra, cuyo valor de recuperación puede descontarse al cliente. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en peso realmente desmontado.</t>
+          <t>Demolición de rodapié existente de granito o terrazo prefabricado y de su capa de asiento, ejecutada con martillo eléctrico manual, cuidando de no dañar el friso de la pared. Incluye repicado de los restos de mortero adheridos, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E5" t="n">
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0.52</v>
+        <v>1.17</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Estructuras</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -636,33 +636,33 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Demolición de columna de concreto armado.</t>
+          <t>Demolición de piso de granito vaciado en sitio.</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Demolición de columna de concreto armado, ejecutada con martillo eléctrico o neumático según la sección, con corte previo de la armadura longitudinal. Exige apeo previo de la estructura que la columna soporta y validación del cálculo estructural, trabajos que se valoran aparte. Incluye la protección del entorno, la demolición descendente por tramos para mantener el control del elemento, el corte y retiro del acero, la fragmentación del concreto, el descenso del escombro y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en volumen realmente demolido.</t>
+          <t>Demolición de piso continuo de granito vaciado en sitio, incluida su base de mortero y las platinas divisorias de las juntas, ejecutada con martillo neumático por tratarse de una superficie monolítica de gran dureza. Incluye corte perimetral previo con amoladora de disco de diamante para delimitar la zona de intervención y evitar desprendimientos fuera de ella, protección de los ambientes contiguos, control de polvo, fragmentación del escombro en piezas manejables, retiro en sacos y limpieza. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E6" t="n">
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>119.95</v>
+        <v>13.04</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Estructuras</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -674,33 +674,33 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Demolición de viga de concreto armado.</t>
+          <t>Demolición de piso de cemento pulido.</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Demolición de viga de concreto armado, ejecutada con martillo eléctrico o neumático, con apeo previo de la losa o de los elementos que la viga sostiene. Incluye la validación estructural previa, el montaje del apeo provisional, la protección del entorno y del nivel inferior, la demolición por tramos controlados desde andamio, el corte y retiro de las barras de refuerzo, el descenso del escombro y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en volumen realmente demolido.</t>
+          <t>Demolición de piso continuo de cemento pulido y de su base de mortero, ejecutada con martillo eléctrico manual, sin afectar a la losa estructural. Incluye corte perimetral con amoladora cuando la demolición sea parcial, protección de los ambientes contiguos, control de polvo mediante aspiración, fragmentación del escombro, retiro manual en sacos hasta el punto de acopio y limpieza de la superficie resultante. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E7" t="n">
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>134.08</v>
+        <v>6.92</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Estructuras</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -712,33 +712,33 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Demolición de losa de entrepiso maciza o nervada.</t>
+          <t>Demolición de rodapié de cemento.</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Demolición de losa de entrepiso de concreto armado, maciza o nervada, ejecutada con martillo neumático y corte de armaduras, con apeo previo de los tramos que permanecen. Incluye la validación estructural, el montaje del apeo, el acordonamiento y protección del nivel inferior para impedir el paso durante los trabajos, la demolición en franjas controladas desde los apoyos hacia el centro, el corte y separación del acero, el descenso del escombro y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Demolición de rodapié corrido de mortero de cemento, ejecutada con medios manuales y cincel, cuidando de no dañar el friso de la pared por encima de la línea del rodapié. Incluye repicado de los restos adheridos al paramento, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E8" t="n">
         <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>46.07</v>
+        <v>0.91</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Estructuras</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -750,17 +750,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Apertura de hueco en losa de concreto armado.</t>
+          <t>Demolición de piso de piedra natural.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Apertura de hueco en losa de concreto armado para paso de escalera, ducto de instalaciones o claraboya, ejecutada mediante corte perimetral con disco de diamante y demolición interior con martillo eléctrico. Incluye la validación estructural previa y el refuerzo del borde si el cálculo lo exige, el apeo de la zona, el replanteo y corte perimetral que garantiza un borde limpio y sin fisuración hacia el resto de la losa, el corte de las armaduras, el descenso controlado del escombro y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de hueco realmente abierto.</t>
+          <t>Demolición de piso existente de piedra natural, ya sea mármol, granito natural o laja, junto con su capa de asiento de mortero, ejecutada con martillo eléctrico manual. Si el cliente desea recuperar las piezas, se levantan una a una con cuidado, se limpian de mortero y se acopian protegidas, lo que reduce el rendimiento y debe advertirse en el presupuesto. Incluye protección de los ambientes contiguos, control de polvo, retiro manual del escombro en sacos y limpieza de la superficie. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -772,11 +772,11 @@
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>36.26</v>
+        <v>6.34</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Estructuras</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -788,33 +788,33 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Desmontaje de estructura de madera.</t>
+          <t>Demolición de rodapié de piedra natural.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de estructura de madera de entrepiso o de techo, formada por vigas, viguetas y entablado, ejecutado con medios manuales y sierra, con apeo previo. Incluye la inspección previa del estado de la madera para prever roturas por pudrición o ataque de xilófagos, el apeo provisional, el desmontaje ordenado desde el entablado hacia las vigas principales, la extracción de clavos y herrajes, la clasificación de las piezas aprovechables si el cliente desea conservarlas, el descenso del material y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Demolición de rodapié existente de piedra natural y de su capa de asiento, ejecutada con martillo eléctrico manual, cuidando de no dañar el friso de la pared. Incluye repicado de los restos de mortero adheridos, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E10" t="n">
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>13.18</v>
+        <v>1.25</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Estructuras</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -826,33 +826,33 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Desmontaje de baranda o pasamanos de balcón.</t>
+          <t>Levantado de piso de parquet o madera.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de baranda o antepecho metálico de balcón, terraza o escalera exterior, ejecutado mediante oxicorte o desatornillado según el anclaje, con sostenimiento previo del elemento. Incluye la instalación de una protección provisional del borde antes de retirar la baranda definitiva, requisito de seguridad ineludible cuando queda un vacío accesible, el corte de los anclajes al ras del soporte, el resane de los huecos de anclaje, el descenso del material y su acopio clasificado como chatarra. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
+          <t>Levantado de piso existente de parquet o de tablilla de madera, incluidos los rastreles o el adhesivo de fijación al contrapiso, ejecutado con medios manuales mediante palanca y espátula. Incluye el retiro previo de las molduras de remate, el rascado de los restos de adhesivo adheridos al contrapiso, la extracción de los clavos o tornillos que queden en la base, el retiro del material en sacos hasta el punto de acopio y la limpieza de la superficie resultante. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E11" t="n">
         <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>5.79</v>
+        <v>2.17</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Fachadas</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -864,33 +864,33 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Desmontaje de reja de protección en fachada.</t>
+          <t>Levantado de rodapié de madera.</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de reja o protector metálico de ventana o puerta en fachada, ejecutado mediante oxicorte o amoladora sobre los anclajes empotrados en el paramento. Incluye el sostenimiento de la reja antes de liberar el último anclaje para evitar su caída, el corte de los elementos de fijación, el picado y resane de los huecos de anclaje que queden en el muro, el descenso del elemento y su acopio clasificado como chatarra. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Levantado de rodapié existente de madera, ejecutado con medios manuales mediante palanca y espátula, cuidando de no dañar el friso de la pared. Incluye la extracción de los clavos, tornillos o tacos de fijación que queden en el paramento, el retiro del material en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente levantada.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E12" t="n">
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>5.62</v>
+        <v>0.43</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Fachadas</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -902,17 +902,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Demolición de muro de fachada de bloque o ladrillo.</t>
+          <t>Levantado de piso laminado.</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Demolición de muro de cerramiento de fachada de bloque de concreto o ladrillo, incluidos sus revestimientos por ambas caras, ejecutada con martillo eléctrico manual desde andamio. Incluye la comprobación previa de que el muro no cumple función portante, el acordonamiento y señalización de la zona de caída a pie de fachada, la protección de las carpinterías que permanecen, la demolición descendente por hiladas para evitar vuelcos, el control de la caída de escombro, su retiro en sacos y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Levantado de piso laminado flotante existente, incluidas la manta acústica y las molduras de remate perimetrales, ejecutado con medios manuales. Por tratarse de un sistema flotante de encastre el desmontaje es rápido y no genera escombro pesado. Incluye el desmontaje ordenado de las tablas, el retiro de la manta y del perfil perimetral, la limpieza y aspirado del contrapiso resultante y el retiro del material en sacos hasta el punto de acopio. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -924,11 +924,11 @@
         <v>1</v>
       </c>
       <c r="F13" t="n">
-        <v>8.49</v>
+        <v>1.26</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Fachadas</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -940,17 +940,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Desmontaje de cerramiento ligero de láminas metálicas.</t>
+          <t>Levantado de piso vinílico, linóleo o alfombra.</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de cerramiento de fachada formado por láminas metálicas, panel sándwich o material similar, junto con la perfilería de soporte, ejecutado con medios manuales y atornillador desde andamio. Incluye el acordonamiento de la zona a pie de fachada, el desmontaje ordenado de las láminas evitando que el viento las descontrole, el retiro de la perfilería y de las fijaciones, la clasificación del material recuperable, el descenso a nivel de acopio y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Levantado de revestimiento de piso flexible existente, ya sea vinílico en lámina o baldosa, linóleo o alfombra, incluido el adhesivo de fijación al contrapiso, ejecutado con medios manuales mediante espátula y rasqueta. Incluye la aplicación puntual de disolvente removedor en las zonas donde el adhesivo esté fuertemente adherido, el rascado hasta dejar el contrapiso limpio y sin restos que comprometan la adherencia del nuevo acabado, la ventilación del ambiente durante los trabajos, el retiro del material en sacos y la limpieza final. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -962,11 +962,11 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>5.95</v>
+        <v>2.12</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Fachadas</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -978,33 +978,33 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Desmontaje de alféizar o repisa de ventana.</t>
+          <t>Demolición de piso continuo de concreto.</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje del alféizar o repisa de ventana, sea de granito, piedra, cerámica o concreto, incluida su capa de asiento, ejecutado con medios manuales y martillo eléctrico. Incluye el corte previo de la junta con el paramento para no arrastrar el friso al desprender la pieza, el picado del mortero de asiento, la limpieza del apoyo dejándolo plano y a nivel para recibir el nuevo alféizar, y el retiro del escombro en sacos. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido, lo que reduce el rendimiento y debe advertirse en el presupuesto. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
+          <t>Demolición de piso continuo de concreto de hasta 10 cm de espesor, ejecutada con martillo neumático, sin afectar a la losa estructural ni a las instalaciones que discurran por debajo. Incluye la comprobación previa de que no existen tuberías ni canalizaciones enterradas en la zona, el corte perimetral con amoladora de disco de diamante para delimitar la demolición, la protección de los ambientes contiguos, el control de polvo, la fragmentación del escombro en piezas manejables, el retiro en sacos hasta el punto de acopio y la limpieza. Si el piso está armado con malla electrosoldada se incluye su corte y retiro. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E15" t="n">
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>2.93</v>
+        <v>15.33</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Remates</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1016,33 +1016,33 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Demolición de dintel prefabricado o cargadero.</t>
+          <t>Demolición de contrapiso o base de mortero de nivelación.</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Demolición de dintel prefabricado o cargadero de concreto sobre hueco de puerta o ventana, ejecutada con martillo eléctrico previo apeo del muro superior. Incluye la validación previa de la carga que transmite el dintel y el montaje del apeo provisional mediante puntales, operación imprescindible antes de cualquier corte, la demolición por tramos, el corte de la armadura, el retiro del escombro y el repaso del apoyo para recibir el nuevo dintel. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente demolida.</t>
+          <t>Demolición de contrapiso o base de mortero de nivelación de hasta 5 cm de espesor, una vez retirado el piso de acabado, ejecutada con martillo eléctrico manual hasta dejar la losa estructural a la vista y limpia. Se emplea cuando la base existente está disgregada, hueca o fuera de nivel y no admite recibir el nuevo piso. Incluye la comprobación previa del estado de la base mediante golpeo, la protección de los ambientes contiguos, el control de polvo mediante aspiración, el retiro manual del escombro en sacos y el barrido final de la losa. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E16" t="n">
         <v>1</v>
       </c>
       <c r="F16" t="n">
-        <v>12.52</v>
+        <v>7.18</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Remates</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1054,33 +1054,33 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Desmontaje de pasamanos de escalera.</t>
+          <t>Desmontaje de piso técnico registrable.</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de pasamanos de escalera, sea de madera, metálico o de obra, junto con sus soportes y anclajes al paramento o a la baranda. Ejecutado con medios manuales, atornillador y amoladora según el tipo de fijación. Incluye el sostenimiento del elemento durante el desmontaje, el corte o extracción de los anclajes, el resane de los huecos que queden en el paramento, la clasificación del material recuperable y el retiro hasta el punto de acopio. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido, lo que reduce el rendimiento y debe advertirse en el presupuesto. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
+          <t>Desmontaje de piso técnico registrable existente, formado por paneles apoyados sobre pedestales regulables, ejecutado con medios manuales. Por tratarse de un sistema desmontable la operación es limpia y permite recuperar el material. Incluye la retirada ordenada de los paneles con ventosa, el desmontaje de los pedestales y travesaños, la clasificación de las piezas en aprovechables y desechables, el acopio protegido de las que el cliente desee conservar, el retiro del resto en sacos y la limpieza de la losa resultante. No incluye el bote del escombro. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E17" t="n">
         <v>1</v>
       </c>
       <c r="F17" t="n">
-        <v>2.26</v>
+        <v>1.09</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Remates</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1092,33 +1092,33 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Desmontaje de equipo de aire acondicionado tipo split.</t>
+          <t>Picado de enchapado cerámico en pared y su capa de pega.</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de equipo de aire acondicionado tipo split, comprendiendo la unidad evaporadora interior, la unidad condensadora exterior, la tubería frigorífica y el drenaje. Incluye la recuperación previa del gas refrigerante mediante equipo específico, operación obligatoria por normativa ambiental que no debe liberarse a la atmósfera, la desconexión eléctrica comprobada, el desmontaje de ambas unidades y de sus soportes, el retiro de la tubería y el drenaje, el resane de las perforaciones de paso y el descenso de los equipos. Si el cliente desea conservar el equipo, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por equipo desmontado.</t>
+          <t>Picado de enchapado cerámico o de porcelanato existente en pared, incluida su capa de pega de mortero, ejecutado con martillo eléctrico manual hasta dejar el friso o el bloque a la vista, sin comprometer la estabilidad del muro ni dañar las tuberías y canalizaciones empotradas. Incluye la localización previa de las instalaciones que discurren por el paramento, la protección de pisos, aparatos y puertas, el control de polvo mediante aspiración, el retiro manual del escombro en sacos hasta el punto de acopio y la limpieza de la superficie, dejándola lista para recibir el nuevo friso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E18" t="n">
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>16.84</v>
+        <v>6.25</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Revestimientos y frisos de pared</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1130,33 +1130,33 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Desmontaje de red eléctrica y sus mecanismos.</t>
+          <t>Picado de enchapado de granito o terrazo en pared.</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de instalación eléctrica existente, comprendiendo la tubería conduit, el conductor, las cajas y los mecanismos, sea vista o empotrada. Incluye la desconexión previa en el tablero y la comprobación de ausencia de tensión con detector antes de manipular cualquier punto, requisito de seguridad ineludible, el picado de los tramos empotrados, la extracción del cableado y la tubería, el retiro de cajas y mecanismos, la clasificación del cobre para su recuperación y el resane de las rozas. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud de canalización realmente desmontada.</t>
+          <t>Picado de enchapado de granito o terrazo prefabricado existente en pared, incluida su capa de asiento de mortero, ejecutado con martillo eléctrico manual. Por el mayor espesor y peso de estas piezas frente al enchapado cerámico, el rendimiento es menor y el escombro más pesado. Incluye la protección de pisos y ambientes contiguos, el control de polvo, el retiro manual del escombro en sacos hasta el punto de acopio y el repicado de los restos de mortero adheridos al paramento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E19" t="n">
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>3.47</v>
+        <v>7.31</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Revestimientos y frisos de pared</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1168,33 +1168,33 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Desmontaje de tablero eléctrico.</t>
+          <t>Picado de enchapado de piedra natural en pared.</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de tablero eléctrico de distribución, incluidos los interruptores termomagnéticos, el barraje y la caja. Incluye el corte previo del suministro desde el punto de acometida y su verificación con detector de tensión, el etiquetado de los circuitos existentes antes de desconectarlos para poder replantear la nueva instalación con la información del estado previo, la desconexión ordenada, el desmontaje de la caja empotrada, el resane del hueco y el retiro del material. Si el cliente desea conservar el equipo, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
+          <t>Picado de enchapado de piedra natural existente en pared, ya sea mármol, laja o piedra de revestimiento, incluida su capa de asiento y los anclajes metálicos si los tuviera, ejecutado con martillo eléctrico manual. Si el cliente desea recuperar las piezas se desmontan una a una con cuidado, se limpian y se acopian protegidas, lo que reduce el rendimiento y debe advertirse en el presupuesto. Incluye la protección del entorno, el control de polvo, el retiro del escombro en sacos y el repicado de los restos adheridos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E20" t="n">
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>10.96</v>
+        <v>7.67</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Revestimientos y frisos de pared</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1206,33 +1206,33 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Desmontaje de red de tuberías de agua o desagüe.</t>
+          <t>Desmontaje de enchapado de madera o machihembrado en pared.</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de red existente de tuberías de agua o de desagüe, vista o empotrada, incluidos sus accesorios y soportes. Incluye el cierre y comprobación previa de que la red está fuera de servicio y vaciada, el picado del paramento en los tramos empotrados, el corte y extracción de la tubería en tramos manejables, el taponado de las derivaciones que permanecen activas, el retiro del material clasificado según sea PVC, hierro galvanizado o cobre, y el resane de las rozas. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
+          <t>Desmontaje de revestimiento de madera existente en pared, ya sea machihembrado, tablilla o panel, junto con los rastreles de soporte fijados al paramento, ejecutado con medios manuales mediante palanca y barra. Incluye la extracción de los clavos, tornillos y tacos que queden en el muro, el retiro del material en sacos o atados hasta el punto de acopio, la clasificación de las piezas aprovechables si el cliente desea conservarlas y la limpieza del paramento resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E21" t="n">
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>4.2</v>
+        <v>2.21</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Revestimientos y frisos de pared</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1244,33 +1244,33 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Desmontaje de luminaria.</t>
+          <t>Desmontaje de revestimiento de láminas o paneles en pared.</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de luminaria de techo o pared, sea empotrada, de sobreponer o colgante, incluidos sus soportes y accesorios. Incluye el corte previo del circuito y la comprobación de ausencia de tensión, la desconexión y aislamiento provisional de los conductores que permanecen, el desmontaje del cuerpo de la luminaria, el retiro de las lámparas con gestión diferenciada si son fluorescentes o de descarga por su contenido en mercurio, y el resane del punto si procede. Si el cliente desea conservar el equipo, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
+          <t>Desmontaje de revestimiento de pared formado por láminas o paneles de PVC, aluminio, melamina o material similar, junto con su estructura o rastrelado de soporte, ejecutado con medios manuales. Incluye el retiro de los perfiles de remate y esquineros, la extracción de las fijaciones que queden en el paramento, el resane puntual de los huecos de anclaje, el retiro del material hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E22" t="n">
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>2.17</v>
+        <v>1.56</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Revestimientos y frisos de pared</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1282,33 +1282,33 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Desmontaje de aparato sanitario y su grifería.</t>
+          <t>Picado de friso de mortero en paramento.</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de aparato sanitario existente, ya sea inodoro, lavamanos, bidé o fregadero, junto con su grifería y accesorios de conexión. Incluye cierre previo de la llave de paso y vaciado del aparato, desconexión de las tomas de agua y del desagüe, taponado provisional de las salidas para evitar olores y entrada de escombro, retirada del aparato hasta el punto de acopio y limpieza de la zona. Si el cliente desea conservar el aparato, se desmonta con cuidado y se acopia protegido. No incluye el transporte a vertedero. Medido por unidad desmontada.</t>
+          <t>Picado de friso de mortero de cemento existente en paramento interior o exterior, ejecutado con martillo eléctrico manual hasta dejar el bloque o el ladrillo a la vista, cuando el friso está disgregado, hueco o presenta fisuración generalizada. Incluye el sondeo previo por golpeo para delimitar las zonas sin adherencia, la protección de pisos y ambientes contiguos, el control de polvo mediante aspiración, el retiro manual del escombro en sacos hasta el punto de acopio y el barrido y limpieza del paramento, dejándolo listo para recibir el nuevo friso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E23" t="n">
         <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>4.55</v>
+        <v>5.86</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Revestimientos y frisos de pared</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1320,33 +1320,33 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Desmontaje de fregadero y su grifería.</t>
+          <t>Picado de friso de yeso o pasta en paramento.</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de fregadero de cocina con su grifería y accesorios de conexión. Incluye el cierre previo de las llaves de paso, la desconexión de las tomas de agua fría y caliente, el desmontaje del sifón y del desagüe con recogida del agua retenida, el corte del sellado perimetral con el mesón, la extracción de la pieza y el taponado provisional de las salidas para evitar olores y entrada de escombro. Si el cliente desea conservar el equipo, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
+          <t>Picado de revestimiento de yeso o pasta existente en paramento interior, ejecutado con medios manuales mediante espátula ancha y cincel, con martillo eléctrico solo en las zonas de mayor espesor. Por tratarse de un material blando el rendimiento es sensiblemente mayor que en un friso de mortero, aunque genera abundante polvo fino. Incluye la protección del entorno, el control de polvo mediante aspiración continua, el retiro del escombro en sacos hasta el punto de acopio y la limpieza del paramento resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E24" t="n">
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>4.12</v>
+        <v>3.65</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Revestimientos y frisos de pared</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1358,33 +1358,33 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Desmontaje de calentador de agua.</t>
+          <t>Picado de estuco o pasta decorativa en paramento.</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de calentador de agua eléctrico o a gas, incluidos sus soportes de anclaje y las conexiones de entrada y salida. Incluye el corte previo del suministro eléctrico o de gas y su comprobación con detector, el vaciado completo del tanque antes de liberarlo de sus soportes por el peso que retiene, la desconexión de las tuberías y su taponado, el desmontaje del anclaje al paramento, el resane de los huecos y el descenso del equipo hasta el punto de acopio. Si el cliente desea conservar el equipo, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
+          <t>Picado de revestimiento de estuco, pasta decorativa o revestimiento texturado existente en paramento, ejecutado con medios manuales y martillo eléctrico según el espesor y la dureza del material, hasta dejar el soporte limpio y apto para recibir el nuevo acabado. Incluye la cata previa para identificar el espesor y el tipo de soporte, la protección del entorno, el control de polvo, el retiro del escombro en sacos y la limpieza final. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E25" t="n">
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>9.43</v>
+        <v>4.3</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Revestimientos y frisos de pared</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1396,17 +1396,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Desmontaje de closet o mueble empotrado.</t>
+          <t>Repicado de superficie de concreto para mejorar adherencia.</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de closet, alacena o mueble empotrado, incluidos las puertas, los entrepaños, la estructura interior y los rastreles de fijación al paramento, ejecutado con medios manuales y atornillador. Incluye el vaciado previo del contenido si el cliente no lo hubiera retirado, el desmontaje ordenado desde las puertas hacia la estructura, la extracción de tacos y tornillos del muro, el resane de los huecos de anclaje, la clasificación de las piezas aprovechables y el retiro del material. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de frente de mueble realmente desmontada.</t>
+          <t>Repicado superficial de paramento o losa de concreto, ejecutado con martillo eléctrico y puntero, para crear la rugosidad necesaria que garantice la adherencia del friso o del mortero de recrecido posterior. Incluye la limpieza previa de la superficie, el picado uniforme sin llegar a descubrir la armadura, la eliminación de lechadas superficiales y restos de desencofrante, el soplado y aspirado del polvo resultante y la retirada de los restos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente repicada.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1418,11 +1418,11 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>4.62</v>
+        <v>4.37</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Carpintería, vidrios y protecciones solares</t>
+          <t>Revestimientos y frisos de pared</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1434,17 +1434,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Desmontaje de reja o protector metálico interior.</t>
+          <t>Eliminación de pintura en paramento mediante raspado y decapado.</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de reja, protector metálico o portón enrollable situado en el interior del inmueble, ejecutado mediante oxicorte o amoladora sobre sus anclajes. Incluye el sostenimiento del elemento antes de liberar el último punto de fijación, el corte de los anclajes al ras, el picado y resane de los huecos que queden en el paramento, el retiro del material hasta el punto de acopio y su clasificación como chatarra, cuyo valor de recuperación puede descontarse al cliente. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Eliminación de las capas de pintura existentes en paramento interior o exterior, mediante raspado mecánico con espátula y lijado, con aplicación puntual de decapante químico en gel en las zonas de pintura muy adherida o de espesor elevado. Se emplea cuando la pintura existente está cuarteada, sopla o es incompatible con el nuevo acabado. Incluye la protección de pisos, carpintería y mobiliario, la ventilación del ambiente durante la aplicación del decapante, la neutralización y lavado de los restos químicos, el aspirado del polvo y la retirada de los residuos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1456,11 +1456,11 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>4.71</v>
+        <v>5.15</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Carpintería, vidrios y protecciones solares</t>
+          <t>Revestimientos y frisos de pared</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1472,17 +1472,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Retiro de vidrio de carpintería existente.</t>
+          <t>Demolición de cielo raso de yeso laminado y su estructura.</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Retiro de vidrio de carpintería que permanece en obra, ya sea por rotura, por sustitución del acristalamiento o para aligerar la ventana antes de su desmontaje. Ejecutado con medios manuales, retirando junquillos, masilla o silicona de sujeción. Incluye el encintado previo de la superficie del vidrio para que, si se fractura, los fragmentos queden contenidos en la lámina adhesiva, el uso de protección facial y guantes anticorte, la limpieza del galce, el retiro del vidrio en contenedor rígido específico y el barrido minucioso de esquirlas. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de vidrio realmente retirada.</t>
+          <t>Demolición de cielo raso continuo de placa de yeso laminado, junto con la perfilería de acero galvanizado, las varillas de cuelgue y el ángulo perimetral, ejecutada con medios manuales. Incluye la desconexión y retiro previo de las luminarias, rejillas y difusores alojados en el plano del cielo, la protección del piso y del mobiliario, el descuelgue ordenado de las placas para evitar caídas incontroladas, el retiro del escombro en sacos y de la perfilería atada, y la limpieza de la zona dejando la losa a la vista. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1494,11 +1494,11 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>3.38</v>
+        <v>2.69</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Carpintería, vidrios y protecciones solares</t>
+          <t>Cielos rasos</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1510,33 +1510,33 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Desmontaje de puerta interior con su marco.</t>
+          <t>Demolición de cielo raso de yeso vaciado o pasta.</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de puerta de paso interior, incluidas la hoja, el marco, las molduras de remate y la herrajería, ejecutado con medios manuales. Incluye el desmontaje previo de la hoja liberándola de sus bisagras, el desclavado o corte de los anclajes del marco al vano, el retiro de las molduras cuidando de no dañar el friso, el repicado de los restos de espuma o mortero de fijación y el retiro del material hasta el punto de acopio. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido, lo que reduce el rendimiento y debe advertirse en el presupuesto. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
+          <t>Demolición de cielo raso de yeso vaciado, pasta o placa de yeso tradicional, junto con su estructura de soporte y elementos de cuelgue, ejecutada con medios manuales y martillo eléctrico donde el espesor lo requiera. Por tratarse de un material macizo genera más escombro y más polvo fino que un cielo de placa. Incluye la desconexión previa de las luminarias, la protección del piso y del mobiliario, el control de polvo mediante aspiración, el retiro del escombro en sacos y la limpieza de la losa resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E29" t="n">
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>4.23</v>
+        <v>4.91</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Carpintería, vidrios y protecciones solares</t>
+          <t>Cielos rasos</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1548,33 +1548,33 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Desmontaje de puerta exterior o metálica con su marco.</t>
+          <t>Desmontaje de cielo raso desmontable de fibra mineral.</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de puerta exterior, de seguridad o metálica, incluidos la hoja, el marco y la herrajería, ejecutado mediante oxicorte o amoladora sobre los anclajes empotrados. Por su peso requiere dos operarios para el sostenimiento de la hoja durante la liberación del marco. Incluye el sostenimiento previo del conjunto, el corte de los anclajes, el picado y resane de los huecos que queden en el muro, el retiro del material hasta el punto de acopio y su clasificación como chatarra. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido, lo que reduce el rendimiento y debe advertirse en el presupuesto. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
+          <t>Desmontaje de cielo raso registrable existente, formado por paneles apoyados sobre perfilería vista en retícula, ejecutado con medios manuales. Por ser un sistema desmontable la operación es limpia, rápida y permite recuperar buena parte del material. Incluye la retirada ordenada de los paneles, el desmontaje de la perfilería y de los tensores de cuelgue, la clasificación de las piezas en aprovechables y desechables, el acopio protegido de las que el cliente desee conservar y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E30" t="n">
         <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>11.54</v>
+        <v>1.65</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Carpintería, vidrios y protecciones solares</t>
+          <t>Cielos rasos</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1586,17 +1586,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Desmontaje de ventana con su marco.</t>
+          <t>Desmontaje de cielo raso de machihembrado de madera.</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de ventana existente, incluidos el marco, las hojas, el vidrio y la herrajería, ejecutado con medios manuales y corte de anclajes. Incluye el retiro previo del vidrio para aligerar el conjunto y evitar roturas incontroladas durante la maniobra, el desmontaje de las hojas, el corte de los anclajes del marco al vano, el picado del mortero de recibido, el resane del hueco perimetral, el descenso del material y su clasificación para reciclaje o reutilización. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido, lo que reduce el rendimiento y debe advertirse en el presupuesto. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de hueco realmente desmontado.</t>
+          <t>Desmontaje de cielo raso de machihembrado o tablilla de madera, junto con los rastreles y la estructura de soporte fijada a la losa, ejecutado con medios manuales mediante palanca y barra. Incluye la desconexión previa de las luminarias, la protección del piso y del mobiliario, la extracción de los clavos y tornillos que queden en la estructura, el retiro del material en atados hasta el punto de acopio, la clasificación de las piezas aprovechables y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1608,11 +1608,11 @@
         <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>7.02</v>
+        <v>2.82</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Carpintería, vidrios y protecciones solares</t>
+          <t>Cielos rasos</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1624,33 +1624,33 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Demolición de brocal o cordón de acera.</t>
+          <t>Desmontaje de cielo raso de láminas de PVC o aluminio.</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Demolición de brocal, cordón o bordillo de acera, sea prefabricado o vaciado en sitio, junto con su dado de concreto de apoyo, ejecutada con martillo eléctrico manual. Incluye el acordonamiento y señalización del área de trabajo por su situación en zona de tránsito, el corte de las juntas entre piezas, la demolición del dado de apoyo, la extracción del escombro, el acopio de las piezas prefabricadas aprovechables si el cliente desea reutilizarlas y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente demolida.</t>
+          <t>Desmontaje de cielo raso formado por láminas de PVC, aluminio o material similar, junto con sus perfiles de soporte y remates perimetrales, ejecutado con medios manuales. Incluye la desconexión previa de las luminarias y rejillas, la protección del piso, el desencastre ordenado de las láminas para poder recuperarlas si el cliente lo desea, el desmontaje de la perfilería, el retiro del material hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E32" t="n">
         <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>7.1</v>
+        <v>1.76</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Firmes y pavimentos exteriores</t>
+          <t>Cielos rasos</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1662,17 +1662,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Demolición de pavimento exterior de concreto.</t>
+          <t>Demolición de trasdosado de yeso laminado y su estructura.</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Demolición de pavimento exterior de concreto, en acera, patio o vía de acceso, de hasta 15 cm de espesor, ejecutada con martillo hidráulico montado sobre retroexcavadora. Incluye la comprobación previa de que no discurren instalaciones enterradas bajo el pavimento, el corte perimetral con disco de diamante para delimitar la zona de intervención, el acordonamiento del área de trabajo, la fragmentación del concreto en piezas cargables, el corte y separación de la malla de refuerzo si la tuviera, el acopio del escombro y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Demolición de trasdosado autoportante de placa de yeso laminado adosado a muro, junto con la perfilería de acero galvanizado y el aislamiento alojado en la cámara, ejecutada con medios manuales. Incluye la localización y desconexión previa de los mecanismos e instalaciones que discurran por el trasdosado, la protección del piso y del mobiliario, el desmontaje ordenado de las placas, el retiro del aislamiento en sacos, el desmontaje de la perfilería y de las fijaciones al muro, y la limpieza de la zona dejando el paramento original a la vista. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1684,11 +1684,11 @@
         <v>1</v>
       </c>
       <c r="F33" t="n">
-        <v>12.66</v>
+        <v>2.56</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Firmes y pavimentos exteriores</t>
+          <t>Trasdosados y forros</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1700,17 +1700,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Demolición de pavimento asfáltico.</t>
+          <t>Demolición de trasdosado de bloque o ladrillo adosado a muro.</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Demolición de pavimento asfáltico de hasta 10 cm de espesor, ejecutada con martillo hidráulico montado sobre retroexcavadora, con corte perimetral previo para obtener un borde recto que facilite la reposición. Incluye la comprobación de instalaciones enterradas, el acordonamiento y señalización del área, el corte perimetral con disco, el arranque y fragmentación del asfalto, el acopio diferenciado del material fresado por admitir reciclaje específico, y la limpieza y barrido de la base resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Demolición de tabique de bloque o ladrillo adosado a muro a modo de trasdosado, incluidos sus revestimientos y la cámara intermedia, ejecutada con martillo eléctrico manual sin dañar el muro original que permanece. Incluye la comprobación previa de que el trasdosado no cumple función estructural ni aloja instalaciones en servicio, la protección del entorno, el control de polvo, la fragmentación del escombro en piezas manejables, el retiro en sacos hasta el punto de acopio y el repicado de los restos de mortero adheridos al muro. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1722,11 +1722,11 @@
         <v>1</v>
       </c>
       <c r="F34" t="n">
-        <v>8.800000000000001</v>
+        <v>6.21</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Firmes y pavimentos exteriores</t>
+          <t>Trasdosados y forros</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1738,17 +1738,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Levantado de pavimento de adoquín.</t>
+          <t>Desmontaje de trasdosado directo de placa pegada al muro.</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Levantado de pavimento exterior de adoquín de concreto o piedra, junto con su cama de arena, ejecutado con medios manuales mediante palanca y pico. Por tratarse de piezas independientes el levantado permite recuperar un porcentaje elevado del material para su reutilización. Incluye el levantado ordenado desde un borde libre, la limpieza de las piezas retirando la arena y el mortero adherido, su clasificación en aprovechables y desechables, el paletizado o acopio de las recuperables, el retiro de la cama de arena y el barrido de la base. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente levantada.</t>
+          <t>Desmontaje de trasdosado directo formado por placa de yeso laminado o panel aislante adherido al muro mediante pelladas de pasta, ejecutado con medios manuales mediante palanca y espátula. Incluye la protección del piso, el arranque de las placas, el rascado de los restos de pasta y adhesivo adheridos al muro hasta dejarlo apto para recibir el nuevo revestimiento, el retiro del material en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1760,11 +1760,11 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>3.35</v>
+        <v>3.12</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Firmes y pavimentos exteriores</t>
+          <t>Trasdosados y forros</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1776,17 +1776,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Retiro de aislamiento térmico o acústico.</t>
+          <t>Retiro de papel tapiz en paramento.</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Retiro de aislamiento térmico o acústico existente, sea de lana mineral, poliestireno o poliuretano, alojado en cámara de tabique, cielo raso o cubierta. Incluye el uso de mascarilla y guantes por la irritación que producen las fibras minerales, el desmontaje del material en piezas completas cuando el estado lo permita, el ensacado inmediato para evitar la dispersión de fibras por el ambiente, el aspirado de los restos y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente retirada.</t>
+          <t>Retiro de papel tapiz existente en paramento interior, junto con los restos de pegamento mural, ejecutado con medios manuales mediante humectación previa con solución reblandecedora y raspado con espátula ancha. Incluye la protección de pisos, rodapiés y mecanismos, la aplicación de la solución en varias pasadas hasta que el papel se desprenda sin arrancar el friso, el rascado de los residuos de pegamento, el lavado final del paramento y su secado, dejándolo listo para recibir el nuevo acabado. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1798,11 +1798,11 @@
         <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>1.99</v>
+        <v>2.2</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Aislamientos e impermeabilizaciones</t>
+          <t>Revestimientos decorativos</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1814,33 +1814,33 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Retiro de manto asfáltico en cubierta.</t>
+          <t>Desmontaje de moldura decorativa de yeso o poliestireno.</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Retiro de impermeabilización existente de manto asfáltico en cubierta, incluidos los solapes, los refuerzos de encuentro y la imprimación adherida al soporte, ejecutado con medios manuales mediante espátula y palanca, con aplicación puntual de calor para reblandecer las zonas fuertemente adheridas. Incluye la protección de los desagües para impedir que se obstruyan con restos, el corte del manto en franjas manejables, el rascado del soporte hasta dejarlo limpio y apto para recibir la nueva impermeabilización, el retiro del material en rollos atados y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente retirada.</t>
+          <t>Desmontaje de moldura decorativa corrida de yeso, poliestireno o poliuretano, situada en el encuentro de pared y cielo raso o como elemento decorativo en paramento, ejecutado con medios manuales mediante espátula y cincel. Incluye la protección del entorno, el corte previo de la línea de junta para evitar arrastrar el friso, el rascado de los restos de pasta o adhesivo, el resane puntual de los desconchados provocados, el retiro del material hasta el punto de acopio y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E37" t="n">
         <v>1</v>
       </c>
       <c r="F37" t="n">
-        <v>3.44</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Aislamientos e impermeabilizaciones</t>
+          <t>Revestimientos decorativos</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1852,17 +1852,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Retiro de impermeabilización líquida o acrílica.</t>
+          <t>Retiro de láminas decorativas, vinilos o espejos adheridos.</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Retiro de recubrimiento impermeabilizante líquido, acrílico o cementoso existente en cubierta o terraza, ejecutado con medios manuales mediante rasqueta y lijado mecánico, hasta dejar el soporte limpio y con la rugosidad adecuada para recibir el nuevo sistema. Incluye la protección de los desagües, el rascado de las zonas con burbujas o desprendimientos, el lijado de la superficie remanente, el aspirado del polvo generado y el retiro de los residuos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
+          <t>Retiro de revestimiento decorativo adherido al paramento, ya sea lámina vinílica, calcomanía mural o espejo pegado, junto con los restos de adhesivo. Incluye la protección del piso y del mobiliario, el calentamiento o humectación previa para reblandecer el adhesivo, el desprendimiento controlado del material con espátula, y en el caso de espejos el encintado previo de la superficie para evitar la proyección de fragmentos al fracturarse. Incluye el rascado de los restos de adhesivo, el retiro del material en sacos y la limpieza del paramento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1874,11 +1874,11 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>3.34</v>
+        <v>1.6</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Aislamientos e impermeabilizaciones</t>
+          <t>Revestimientos decorativos</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -1890,17 +1890,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Demolición de tabique de bloque o ladrillo, incluidos sus revestimientos.</t>
+          <t>Demolición de revestimiento cerámico de escalera.</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Demolición de tabique interior no estructural de bloque de concreto o ladrillo, con sus revestimientos por ambas caras, ejecutada con martillo eléctrico manual sin afectar a la estabilidad de los elementos constructivos contiguos. Incluye comprobación previa de que el tabique no es portante y de que no aloja instalaciones en servicio, protección del entorno, apeo puntual si fuera necesario, fragmentación del escombro en piezas manejables, retirada en sacos hasta el punto de acopio y limpieza de la zona. No incluye el transporte a vertedero. Medido en superficie realmente demolida.</t>
+          <t>Demolición del revestimiento cerámico de escalera, comprendiendo huellas, contrahuellas y su capa de pega, ejecutada con martillo eléctrico manual sin comprometer la losa de la escalera. El rendimiento es sensiblemente menor que en un piso corrido por la posición forzada de trabajo, la superficie fragmentada en peldaños y la dificultad de evacuar el escombro por la propia escalera. Incluye la protección del hueco y del pasamanos, el control de polvo, el retiro manual del escombro en sacos y la limpieza, dejando los peldaños listos para el nuevo revestimiento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida, desarrollando huella y contrahuella.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1912,11 +1912,11 @@
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>5.42</v>
+        <v>7.27</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Particiones</t>
+          <t>Escaleras</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -1928,17 +1928,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Demolición de tabique de yeso laminado y su estructura.</t>
+          <t>Demolición de revestimiento de granito o piedra natural en escalera.</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Demolición de tabique interior de placa de yeso laminado, junto con la perfilería de acero galvanizado y el aislamiento de la cámara, ejecutada con medios manuales. Incluye la localización y desconexión previa de las instalaciones que discurran por el interior del tabique, operación crítica en este sistema porque las tuberías y el cableado quedan ocultos y sin señalizar, la protección del piso, el desmontaje ordenado de las placas, el retiro del aislamiento, el desmontaje de la perfilería y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Demolición del revestimiento de granito, terrazo o piedra natural de escalera, comprendiendo huellas, contrahuellas y su capa de asiento, ejecutada con martillo eléctrico manual. Al mayor espesor y peso de las piezas se suma la dificultad propia del trabajo en escalera, por lo que el rendimiento es el más bajo de los grupos de demolición de revestimientos. Incluye la protección del hueco y del pasamanos, el control de polvo, el retiro manual del escombro en sacos y el repicado de los restos de mortero adheridos a los peldaños. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida, desarrollando huella y contrahuella.</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1950,11 +1950,11 @@
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>2.89</v>
+        <v>8.58</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Particiones</t>
+          <t>Escaleras</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -1966,33 +1966,33 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Demolición de muro de concreto no estructural.</t>
+          <t>Demolición de zócalo escalonado de escalera.</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Demolición de muro interior de concreto no estructural, incluidos sus revestimientos, ejecutada con martillo neumático y corte de la malla de refuerzo si la tuviera. Incluye la comprobación estructural previa que acredite que el muro no es portante ni de arriostramiento, requisito imprescindible antes de intervenir, el corte perimetral con disco de diamante, la protección del entorno, el control de polvo, la fragmentación del escombro y su retiro en sacos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Demolición del zócalo o rodapié escalonado que acompaña a la escalera en su encuentro con el paramento, incluida su capa de pega, ejecutada con medios manuales y martillo eléctrico, cuidando de no dañar el friso por encima de la línea del zócalo. Incluye el repicado de los restos de mortero adheridos, el retiro del escombro en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud real de la línea inclinada del zócalo.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E41" t="n">
         <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>17.5</v>
+        <v>1.78</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Particiones</t>
+          <t>Escaleras</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2004,33 +2004,33 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Apertura de vano en pared de bloque o ladrillo.</t>
+          <t>Desmontaje de baranda o pasamanos de balcón.</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Apertura de vano para puerta, ventana o paso en pared existente de bloque o ladrillo, ejecutada con corte perimetral mediante disco de diamante y demolición interior con martillo eléctrico. Incluye el replanteo del vano, el apeo provisional del dintel mediante puntales antes de iniciar la demolición, el corte perimetral que garantiza jambas rectas y sin desgarros hacia el resto del muro, la demolición controlada desde la parte superior, el retiro del escombro y el repaso de las jambas dejándolas aplomadas. No incluye el dintel definitivo ni el resane de las jambas, que se valoran aparte. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de vano realmente abierto.</t>
+          <t>Desmontaje de baranda o antepecho metálico de balcón, terraza o escalera exterior, ejecutado mediante oxicorte o desatornillado según el anclaje, con sostenimiento previo del elemento. Incluye la instalación de una protección provisional del borde antes de retirar la baranda definitiva, requisito de seguridad ineludible cuando queda un vacío accesible, el corte de los anclajes al ras del soporte, el resane de los huecos de anclaje, el descenso del material y su acopio clasificado como chatarra. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E42" t="n">
         <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>17.78</v>
+        <v>5.79</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Particiones</t>
+          <t>Fachadas y revestimientos exteriores</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -2042,17 +2042,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Demolición de tabique de bloque de vidrio.</t>
+          <t>Desmontaje de reja de protección en fachada.</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Demolición de tabique o paño de bloque de vidrio, incluidas las juntas de mortero y la armadura de refuerzo entre hiladas, ejecutada con medios manuales y martillo eléctrico. Requiere precauciones específicas frente a la proyección de fragmentos cortantes: se encinta previamente la superficie de los bloques para que rompan de forma contenida y se emplea protección facial y guantes anticorte. Incluye la protección del entorno, la demolición descendente por hiladas, el retiro cuidadoso del material en sacos reforzados y la limpieza minuciosa de esquirlas. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de reja o protector metálico de ventana o puerta en fachada, ejecutado mediante oxicorte o amoladora sobre los anclajes empotrados en el paramento. Incluye el sostenimiento de la reja antes de liberar el último anclaje para evitar su caída, el corte de los elementos de fijación, el picado y resane de los huecos de anclaje que queden en el muro, el descenso del elemento y su acopio clasificado como chatarra. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2064,11 +2064,11 @@
         <v>1</v>
       </c>
       <c r="F43" t="n">
-        <v>6.79</v>
+        <v>5.62</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Particiones</t>
+          <t>Fachadas y revestimientos exteriores</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2080,33 +2080,33 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Desmontaje de canal de aguas lluvias.</t>
+          <t>Demolición de muro de fachada de bloque o ladrillo.</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de canal o canalón de recogida de aguas lluvias, incluidos los soportes, las uniones y las piezas especiales, ejecutado con medios manuales desde andamio. Incluye el acordonamiento de la zona inferior, el desmontaje por tramos con sostenimiento previo, la extracción de los ganchos y anclajes al alero, el resane de los puntos de fijación, el descenso del material y su clasificación para reciclaje. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
+          <t>Demolición de muro de cerramiento de fachada de bloque de concreto o ladrillo, incluidos sus revestimientos por ambas caras, ejecutada con martillo eléctrico manual desde andamio. Incluye la comprobación previa de que el muro no cumple función portante, el acordonamiento y señalización de la zona de caída a pie de fachada, la protección de las carpinterías que permanecen, la demolición descendente por hiladas para evitar vuelcos, el control de la caída de escombro, su retiro en sacos y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E44" t="n">
         <v>1</v>
       </c>
       <c r="F44" t="n">
-        <v>2.7</v>
+        <v>8.49</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Cubiertas</t>
+          <t>Fachadas y revestimientos exteriores</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2118,33 +2118,33 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Desmontaje de bajante de aguas lluvias.</t>
+          <t>Desmontaje de cerramiento ligero de láminas metálicas.</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de bajante de aguas lluvias, vista o empotrada, incluidos las abrazaderas, los codos y las piezas de conexión, ejecutado con medios manuales desde andamio. Incluye el acordonamiento de la zona inferior, el corte de la bajante en tramos manejables, la extracción de las abrazaderas ancladas a la fachada, el resane de los huecos de anclaje, el taponado provisional de la conexión a la red que permanece y el retiro del material. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
+          <t>Desmontaje de cerramiento de fachada formado por láminas metálicas, panel sándwich o material similar, junto con la perfilería de soporte, ejecutado con medios manuales y atornillador desde andamio. Incluye el acordonamiento de la zona a pie de fachada, el desmontaje ordenado de las láminas evitando que el viento las descontrole, el retiro de la perfilería y de las fijaciones, la clasificación del material recuperable, el descenso a nivel de acopio y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E45" t="n">
         <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>2.72</v>
+        <v>5.95</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Cubiertas</t>
+          <t>Fachadas y revestimientos exteriores</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2156,17 +2156,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Desmontaje de cubierta de teja.</t>
+          <t>Picado de salpicado o graniplast en fachada.</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de cubierta de teja criolla, teja plana o similar, incluidos el mortero de fijación y los caballetes de cumbrera, ejecutado con medios manuales desde andamio y con línea de vida. Incluye la comprobación previa del estado de la estructura de soporte antes de que el personal transite sobre ella, el desmontaje ordenado desde la cumbrera hacia el alero, el descenso de las tejas por medios mecánicos evitando el lanzamiento, la clasificación de las piezas aprovechables y el acopio del material. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Picado de revestimiento de salpicado, graniplast o revestimiento pétreo proyectado en fachada, ejecutado con martillo eléctrico manual y espátula, hasta dejar el friso base sano o el bloque a la vista según el estado del soporte. Incluye el sondeo previo por golpeo para delimitar las zonas sin adherencia, el trabajo desde andamio con las protecciones colectivas correspondientes, la protección de carpinterías y de la zona de paso a pie de fachada, el control de la caída de escombro, su retiro en sacos hasta el punto de acopio y la limpieza del paramento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2178,11 +2178,11 @@
         <v>1</v>
       </c>
       <c r="F46" t="n">
-        <v>9.44</v>
+        <v>7.11</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Cubiertas</t>
+          <t>Fachadas y revestimientos exteriores</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2194,17 +2194,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Desmontaje de cubierta de lámina metálica o acerolit.</t>
+          <t>Picado de mortero monocapa en fachada.</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de cubierta de lámina metálica, acerolit, zinc o fibrocemento, incluidos los ganchos, tornillos y elementos de fijación a la estructura, ejecutado con medios manuales desde andamio y con línea de vida. Si la lámina es de fibrocemento antiguo debe verificarse la posible presencia de amianto, en cuyo caso el desmontaje queda fuera de esta partida y exige empresa autorizada. Incluye el desmontaje ordenado con sujeción de las láminas frente al viento, el descenso controlado, la clasificación del material y el acopio. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Picado de revestimiento de mortero monocapa en fachada, incluida su malla de refuerzo y los perfiles de arranque y goterón, ejecutado con martillo eléctrico manual hasta dejar el soporte limpio y apto para recibir el nuevo revestimiento. Incluye el sondeo previo del paramento, el trabajo desde andamio con las protecciones colectivas correspondientes, la protección de carpinterías y del paso a pie de fachada, el corte y retiro de la malla, el control de la caída de escombro, su retiro en sacos y la limpieza del soporte. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2216,11 +2216,11 @@
         <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>6.81</v>
+        <v>8.02</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Cubiertas</t>
+          <t>Fachadas y revestimientos exteriores</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2232,17 +2232,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Desmontaje de estructura de techo.</t>
+          <t>Demolición de tabique de bloque o ladrillo, incluidos sus revestimientos.</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de la estructura de soporte de cubierta, formada por correas, cerchas o perfiles de madera o metal, una vez retirado el material de cubrición. Ejecutado con sierra, oxicorte o desatornillado según el material, con apeo previo y eslingado de los elementos antes de liberarlos. Incluye el estudio del orden de desmontaje para conservar la estabilidad del conjunto, el sostenimiento de cada pieza antes del corte, el descenso mecánico, la clasificación del material recuperable y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de cubierta cuya estructura se desmonta.</t>
+          <t>Demolición de tabique interior no estructural de bloque de concreto o ladrillo, con sus revestimientos por ambas caras, ejecutada con martillo eléctrico manual sin afectar a la estabilidad de los elementos constructivos contiguos. Incluye comprobación previa de que el tabique no es portante y de que no aloja instalaciones en servicio, protección del entorno, apeo puntual si fuera necesario, fragmentación del escombro en piezas manejables, retirada en sacos hasta el punto de acopio y limpieza de la zona. No incluye el transporte a vertedero. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2254,11 +2254,11 @@
         <v>1</v>
       </c>
       <c r="F48" t="n">
-        <v>14.46</v>
+        <v>5.42</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Cubiertas</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2270,17 +2270,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Demolición de pendientado y protección de cubierta plana.</t>
+          <t>Demolición de tabique de yeso laminado y su estructura.</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Demolición de la capa de pendientado y de la protección de cubierta plana, comprendiendo el relleno aligerado de formación de pendiente, la capa de mortero de protección y el acabado superficial, hasta descubrir la losa. Ejecutada con martillo eléctrico manual. Incluye la protección y taponado provisional de los desagües, la comprobación de no perforar la losa, el control del acopio de escombro sobre la cubierta para no sobrecargarla, su descenso por medios mecánicos y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Demolición de tabique interior de placa de yeso laminado, junto con la perfilería de acero galvanizado y el aislamiento de la cámara, ejecutada con medios manuales. Incluye la localización y desconexión previa de las instalaciones que discurran por el interior del tabique, operación crítica en este sistema porque las tuberías y el cableado quedan ocultos y sin señalizar, la protección del piso, el desmontaje ordenado de las placas, el retiro del aislamiento, el desmontaje de la perfilería y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2292,11 +2292,11 @@
         <v>1</v>
       </c>
       <c r="F49" t="n">
-        <v>11.27</v>
+        <v>2.89</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Cubiertas</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -2308,17 +2308,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Picado de enchapado cerámico en pared y su capa de pega.</t>
+          <t>Demolición de muro de concreto no estructural.</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Picado de enchapado cerámico o de porcelanato existente en pared, incluida su capa de pega de mortero, ejecutado con martillo eléctrico manual hasta dejar el friso o el bloque a la vista, sin comprometer la estabilidad del muro ni dañar las tuberías y canalizaciones empotradas. Incluye la localización previa de las instalaciones que discurren por el paramento, la protección de pisos, aparatos y puertas, el control de polvo mediante aspiración, el retiro manual del escombro en sacos hasta el punto de acopio y la limpieza de la superficie, dejándola lista para recibir el nuevo friso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Demolición de muro interior de concreto no estructural, incluidos sus revestimientos, ejecutada con martillo neumático y corte de la malla de refuerzo si la tuviera. Incluye la comprobación estructural previa que acredite que el muro no es portante ni de arriostramiento, requisito imprescindible antes de intervenir, el corte perimetral con disco de diamante, la protección del entorno, el control de polvo, la fragmentación del escombro y su retiro en sacos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2330,11 +2330,11 @@
         <v>1</v>
       </c>
       <c r="F50" t="n">
-        <v>6.25</v>
+        <v>17.5</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2346,17 +2346,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Picado de enchapado de granito o terrazo en pared.</t>
+          <t>Apertura de vano en pared de bloque o ladrillo.</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Picado de enchapado de granito o terrazo prefabricado existente en pared, incluida su capa de asiento de mortero, ejecutado con martillo eléctrico manual. Por el mayor espesor y peso de estas piezas frente al enchapado cerámico, el rendimiento es menor y el escombro más pesado. Incluye la protección de pisos y ambientes contiguos, el control de polvo, el retiro manual del escombro en sacos hasta el punto de acopio y el repicado de los restos de mortero adheridos al paramento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Apertura de vano para puerta, ventana o paso en pared existente de bloque o ladrillo, ejecutada con corte perimetral mediante disco de diamante y demolición interior con martillo eléctrico. Incluye el replanteo del vano, el apeo provisional del dintel mediante puntales antes de iniciar la demolición, el corte perimetral que garantiza jambas rectas y sin desgarros hacia el resto del muro, la demolición controlada desde la parte superior, el retiro del escombro y el repaso de las jambas dejándolas aplomadas. No incluye el dintel definitivo ni el resane de las jambas, que se valoran aparte. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de vano realmente abierto.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2368,11 +2368,11 @@
         <v>1</v>
       </c>
       <c r="F51" t="n">
-        <v>7.31</v>
+        <v>17.78</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -2384,17 +2384,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Picado de enchapado de piedra natural en pared.</t>
+          <t>Demolición de tabique de bloque de vidrio.</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Picado de enchapado de piedra natural existente en pared, ya sea mármol, laja o piedra de revestimiento, incluida su capa de asiento y los anclajes metálicos si los tuviera, ejecutado con martillo eléctrico manual. Si el cliente desea recuperar las piezas se desmontan una a una con cuidado, se limpian y se acopian protegidas, lo que reduce el rendimiento y debe advertirse en el presupuesto. Incluye la protección del entorno, el control de polvo, el retiro del escombro en sacos y el repicado de los restos adheridos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Demolición de tabique o paño de bloque de vidrio, incluidas las juntas de mortero y la armadura de refuerzo entre hiladas, ejecutada con medios manuales y martillo eléctrico. Requiere precauciones específicas frente a la proyección de fragmentos cortantes: se encinta previamente la superficie de los bloques para que rompan de forma contenida y se emplea protección facial y guantes anticorte. Incluye la protección del entorno, la demolición descendente por hiladas, el retiro cuidadoso del material en sacos reforzados y la limpieza minuciosa de esquirlas. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2406,11 +2406,11 @@
         <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>7.67</v>
+        <v>6.79</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2422,17 +2422,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Desmontaje de enchapado de madera o machihembrado en pared.</t>
+          <t>Desmontaje de closet o mueble empotrado.</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de revestimiento de madera existente en pared, ya sea machihembrado, tablilla o panel, junto con los rastreles de soporte fijados al paramento, ejecutado con medios manuales mediante palanca y barra. Incluye la extracción de los clavos, tornillos y tacos que queden en el muro, el retiro del material en sacos o atados hasta el punto de acopio, la clasificación de las piezas aprovechables si el cliente desea conservarlas y la limpieza del paramento resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Desmontaje de closet, alacena o mueble empotrado, incluidos las puertas, los entrepaños, la estructura interior y los rastreles de fijación al paramento, ejecutado con medios manuales y atornillador. Incluye el vaciado previo del contenido si el cliente no lo hubiera retirado, el desmontaje ordenado desde las puertas hacia la estructura, la extracción de tacos y tornillos del muro, el resane de los huecos de anclaje, la clasificación de las piezas aprovechables y el retiro del material. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de frente de mueble realmente desmontada.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2444,11 +2444,11 @@
         <v>1</v>
       </c>
       <c r="F53" t="n">
-        <v>2.21</v>
+        <v>4.62</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Carpintería, herrería y vidrios</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2460,17 +2460,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Desmontaje de revestimiento de láminas o paneles en pared.</t>
+          <t>Desmontaje de reja o protector metálico interior.</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de revestimiento de pared formado por láminas o paneles de PVC, aluminio, melamina o material similar, junto con su estructura o rastrelado de soporte, ejecutado con medios manuales. Incluye el retiro de los perfiles de remate y esquineros, la extracción de las fijaciones que queden en el paramento, el resane puntual de los huecos de anclaje, el retiro del material hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Desmontaje de reja, protector metálico o portón enrollable situado en el interior del inmueble, ejecutado mediante oxicorte o amoladora sobre sus anclajes. Incluye el sostenimiento del elemento antes de liberar el último punto de fijación, el corte de los anclajes al ras, el picado y resane de los huecos que queden en el paramento, el retiro del material hasta el punto de acopio y su clasificación como chatarra, cuyo valor de recuperación puede descontarse al cliente. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2482,11 +2482,11 @@
         <v>1</v>
       </c>
       <c r="F54" t="n">
-        <v>1.56</v>
+        <v>4.71</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Carpintería, herrería y vidrios</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2498,17 +2498,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Retiro de papel tapiz en paramento.</t>
+          <t>Retiro de vidrio de carpintería existente.</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Retiro de papel tapiz existente en paramento interior, junto con los restos de pegamento mural, ejecutado con medios manuales mediante humectación previa con solución reblandecedora y raspado con espátula ancha. Incluye la protección de pisos, rodapiés y mecanismos, la aplicación de la solución en varias pasadas hasta que el papel se desprenda sin arrancar el friso, el rascado de los residuos de pegamento, el lavado final del paramento y su secado, dejándolo listo para recibir el nuevo acabado. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
+          <t>Retiro de vidrio de carpintería que permanece en obra, ya sea por rotura, por sustitución del acristalamiento o para aligerar la ventana antes de su desmontaje. Ejecutado con medios manuales, retirando junquillos, masilla o silicona de sujeción. Incluye el encintado previo de la superficie del vidrio para que, si se fractura, los fragmentos queden contenidos en la lámina adhesiva, el uso de protección facial y guantes anticorte, la limpieza del galce, el retiro del vidrio en contenedor rígido específico y el barrido minucioso de esquirlas. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de vidrio realmente retirada.</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2520,11 +2520,11 @@
         <v>1</v>
       </c>
       <c r="F55" t="n">
-        <v>2.2</v>
+        <v>3.38</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Carpintería, herrería y vidrios</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2536,33 +2536,33 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Desmontaje de moldura decorativa de yeso o poliestireno.</t>
+          <t>Desmontaje de puerta interior con su marco.</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de moldura decorativa corrida de yeso, poliestireno o poliuretano, situada en el encuentro de pared y cielo raso o como elemento decorativo en paramento, ejecutado con medios manuales mediante espátula y cincel. Incluye la protección del entorno, el corte previo de la línea de junta para evitar arrastrar el friso, el rascado de los restos de pasta o adhesivo, el resane puntual de los desconchados provocados, el retiro del material hasta el punto de acopio y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
+          <t>Desmontaje de puerta de paso interior, incluidas la hoja, el marco, las molduras de remate y la herrajería, ejecutado con medios manuales. Incluye el desmontaje previo de la hoja liberándola de sus bisagras, el desclavado o corte de los anclajes del marco al vano, el retiro de las molduras cuidando de no dañar el friso, el repicado de los restos de espuma o mortero de fijación y el retiro del material hasta el punto de acopio. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido, lo que reduce el rendimiento y debe advertirse en el presupuesto. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E56" t="n">
         <v>1</v>
       </c>
       <c r="F56" t="n">
-        <v>0.9399999999999999</v>
+        <v>4.23</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Carpintería, herrería y vidrios</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -2574,33 +2574,33 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Retiro de láminas decorativas, vinilos o espejos adheridos.</t>
+          <t>Desmontaje de puerta exterior o metálica con su marco.</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Retiro de revestimiento decorativo adherido al paramento, ya sea lámina vinílica, calcomanía mural o espejo pegado, junto con los restos de adhesivo. Incluye la protección del piso y del mobiliario, el calentamiento o humectación previa para reblandecer el adhesivo, el desprendimiento controlado del material con espátula, y en el caso de espejos el encintado previo de la superficie para evitar la proyección de fragmentos al fracturarse. Incluye el rascado de los restos de adhesivo, el retiro del material en sacos y la limpieza del paramento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
+          <t>Desmontaje de puerta exterior, de seguridad o metálica, incluidos la hoja, el marco y la herrajería, ejecutado mediante oxicorte o amoladora sobre los anclajes empotrados. Por su peso requiere dos operarios para el sostenimiento de la hoja durante la liberación del marco. Incluye el sostenimiento previo del conjunto, el corte de los anclajes, el picado y resane de los huecos que queden en el muro, el retiro del material hasta el punto de acopio y su clasificación como chatarra. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido, lo que reduce el rendimiento y debe advertirse en el presupuesto. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E57" t="n">
         <v>1</v>
       </c>
       <c r="F57" t="n">
-        <v>1.6</v>
+        <v>11.54</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Carpintería, herrería y vidrios</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2612,17 +2612,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Demolición de revestimiento cerámico de escalera.</t>
+          <t>Desmontaje de ventana con su marco.</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Demolición del revestimiento cerámico de escalera, comprendiendo huellas, contrahuellas y su capa de pega, ejecutada con martillo eléctrico manual sin comprometer la losa de la escalera. El rendimiento es sensiblemente menor que en un piso corrido por la posición forzada de trabajo, la superficie fragmentada en peldaños y la dificultad de evacuar el escombro por la propia escalera. Incluye la protección del hueco y del pasamanos, el control de polvo, el retiro manual del escombro en sacos y la limpieza, dejando los peldaños listos para el nuevo revestimiento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida, desarrollando huella y contrahuella.</t>
+          <t>Desmontaje de ventana existente, incluidos el marco, las hojas, el vidrio y la herrajería, ejecutado con medios manuales y corte de anclajes. Incluye el retiro previo del vidrio para aligerar el conjunto y evitar roturas incontroladas durante la maniobra, el desmontaje de las hojas, el corte de los anclajes del marco al vano, el picado del mortero de recibido, el resane del hueco perimetral, el descenso del material y su clasificación para reciclaje o reutilización. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido, lo que reduce el rendimiento y debe advertirse en el presupuesto. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de hueco realmente desmontado.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2634,11 +2634,11 @@
         <v>1</v>
       </c>
       <c r="F58" t="n">
-        <v>7.27</v>
+        <v>7.02</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Carpintería, herrería y vidrios</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -2650,33 +2650,33 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Demolición de revestimiento de granito o piedra natural en escalera.</t>
+          <t>Desmontaje de alféizar o repisa de ventana.</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Demolición del revestimiento de granito, terrazo o piedra natural de escalera, comprendiendo huellas, contrahuellas y su capa de asiento, ejecutada con martillo eléctrico manual. Al mayor espesor y peso de las piezas se suma la dificultad propia del trabajo en escalera, por lo que el rendimiento es el más bajo de los grupos de demolición de revestimientos. Incluye la protección del hueco y del pasamanos, el control de polvo, el retiro manual del escombro en sacos y el repicado de los restos de mortero adheridos a los peldaños. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida, desarrollando huella y contrahuella.</t>
+          <t>Desmontaje del alféizar o repisa de ventana, sea de granito, piedra, cerámica o concreto, incluida su capa de asiento, ejecutado con medios manuales y martillo eléctrico. Incluye el corte previo de la junta con el paramento para no arrastrar el friso al desprender la pieza, el picado del mortero de asiento, la limpieza del apoyo dejándolo plano y a nivel para recibir el nuevo alféizar, y el retiro del escombro en sacos. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido, lo que reduce el rendimiento y debe advertirse en el presupuesto. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E59" t="n">
         <v>1</v>
       </c>
       <c r="F59" t="n">
-        <v>8.58</v>
+        <v>2.93</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Remates y elementos accesorios</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -2688,17 +2688,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Demolición de zócalo escalonado de escalera.</t>
+          <t>Demolición de dintel prefabricado o cargadero.</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Demolición del zócalo o rodapié escalonado que acompaña a la escalera en su encuentro con el paramento, incluida su capa de pega, ejecutada con medios manuales y martillo eléctrico, cuidando de no dañar el friso por encima de la línea del zócalo. Incluye el repicado de los restos de mortero adheridos, el retiro del escombro en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud real de la línea inclinada del zócalo.</t>
+          <t>Demolición de dintel prefabricado o cargadero de concreto sobre hueco de puerta o ventana, ejecutada con martillo eléctrico previo apeo del muro superior. Incluye la validación previa de la carga que transmite el dintel y el montaje del apeo provisional mediante puntales, operación imprescindible antes de cualquier corte, la demolición por tramos, el corte de la armadura, el retiro del escombro y el repaso del apoyo para recibir el nuevo dintel. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2710,11 +2710,11 @@
         <v>1</v>
       </c>
       <c r="F60" t="n">
-        <v>1.78</v>
+        <v>12.52</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Remates y elementos accesorios</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -2726,33 +2726,33 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Picado de friso de mortero en paramento.</t>
+          <t>Desmontaje de pasamanos de escalera.</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Picado de friso de mortero de cemento existente en paramento interior o exterior, ejecutado con martillo eléctrico manual hasta dejar el bloque o el ladrillo a la vista, cuando el friso está disgregado, hueco o presenta fisuración generalizada. Incluye el sondeo previo por golpeo para delimitar las zonas sin adherencia, la protección de pisos y ambientes contiguos, el control de polvo mediante aspiración, el retiro manual del escombro en sacos hasta el punto de acopio y el barrido y limpieza del paramento, dejándolo listo para recibir el nuevo friso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Desmontaje de pasamanos de escalera, sea de madera, metálico o de obra, junto con sus soportes y anclajes al paramento o a la baranda. Ejecutado con medios manuales, atornillador y amoladora según el tipo de fijación. Incluye el sostenimiento del elemento durante el desmontaje, el corte o extracción de los anclajes, el resane de los huecos que queden en el paramento, la clasificación del material recuperable y el retiro hasta el punto de acopio. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido, lo que reduce el rendimiento y debe advertirse en el presupuesto. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E61" t="n">
         <v>1</v>
       </c>
       <c r="F61" t="n">
-        <v>5.86</v>
+        <v>2.26</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Remates y elementos accesorios</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -2764,33 +2764,33 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Picado de friso de yeso o pasta en paramento.</t>
+          <t>Desmontaje de equipo de aire acondicionado tipo split.</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Picado de revestimiento de yeso o pasta existente en paramento interior, ejecutado con medios manuales mediante espátula ancha y cincel, con martillo eléctrico solo en las zonas de mayor espesor. Por tratarse de un material blando el rendimiento es sensiblemente mayor que en un friso de mortero, aunque genera abundante polvo fino. Incluye la protección del entorno, el control de polvo mediante aspiración continua, el retiro del escombro en sacos hasta el punto de acopio y la limpieza del paramento resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Desmontaje de equipo de aire acondicionado tipo split, comprendiendo la unidad evaporadora interior, la unidad condensadora exterior, la tubería frigorífica y el drenaje. Incluye la recuperación previa del gas refrigerante mediante equipo específico, operación obligatoria por normativa ambiental que no debe liberarse a la atmósfera, la desconexión eléctrica comprobada, el desmontaje de ambas unidades y de sus soportes, el retiro de la tubería y el drenaje, el resane de las perforaciones de paso y el descenso de los equipos. Si el cliente desea conservar el equipo, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por equipo desmontado.</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E62" t="n">
         <v>1</v>
       </c>
       <c r="F62" t="n">
-        <v>3.65</v>
+        <v>16.84</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
@@ -2802,33 +2802,33 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Picado de estuco o pasta decorativa en paramento.</t>
+          <t>Desmontaje de red eléctrica y sus mecanismos.</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Picado de revestimiento de estuco, pasta decorativa o revestimiento texturado existente en paramento, ejecutado con medios manuales y martillo eléctrico según el espesor y la dureza del material, hasta dejar el soporte limpio y apto para recibir el nuevo acabado. Incluye la cata previa para identificar el espesor y el tipo de soporte, la protección del entorno, el control de polvo, el retiro del escombro en sacos y la limpieza final. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Desmontaje de instalación eléctrica existente, comprendiendo la tubería conduit, el conductor, las cajas y los mecanismos, sea vista o empotrada. Incluye la desconexión previa en el tablero y la comprobación de ausencia de tensión con detector antes de manipular cualquier punto, requisito de seguridad ineludible, el picado de los tramos empotrados, la extracción del cableado y la tubería, el retiro de cajas y mecanismos, la clasificación del cobre para su recuperación y el resane de las rozas. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud de canalización realmente desmontada.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E63" t="n">
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>4.3</v>
+        <v>3.47</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
@@ -2840,33 +2840,33 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Repicado de superficie de concreto para mejorar adherencia.</t>
+          <t>Desmontaje de tablero eléctrico.</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Repicado superficial de paramento o losa de concreto, ejecutado con martillo eléctrico y puntero, para crear la rugosidad necesaria que garantice la adherencia del friso o del mortero de recrecido posterior. Incluye la limpieza previa de la superficie, el picado uniforme sin llegar a descubrir la armadura, la eliminación de lechadas superficiales y restos de desencofrante, el soplado y aspirado del polvo resultante y la retirada de los restos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente repicada.</t>
+          <t>Desmontaje de tablero eléctrico de distribución, incluidos los interruptores termomagnéticos, el barraje y la caja. Incluye el corte previo del suministro desde el punto de acometida y su verificación con detector de tensión, el etiquetado de los circuitos existentes antes de desconectarlos para poder replantear la nueva instalación con la información del estado previo, la desconexión ordenada, el desmontaje de la caja empotrada, el resane del hueco y el retiro del material. Si el cliente desea conservar el equipo, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E64" t="n">
         <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>4.37</v>
+        <v>10.96</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -2878,33 +2878,33 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Eliminación de pintura en paramento mediante raspado y decapado.</t>
+          <t>Desmontaje de red de tuberías de agua o desagüe.</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Eliminación de las capas de pintura existentes en paramento interior o exterior, mediante raspado mecánico con espátula y lijado, con aplicación puntual de decapante químico en gel en las zonas de pintura muy adherida o de espesor elevado. Se emplea cuando la pintura existente está cuarteada, sopla o es incompatible con el nuevo acabado. Incluye la protección de pisos, carpintería y mobiliario, la ventilación del ambiente durante la aplicación del decapante, la neutralización y lavado de los restos químicos, el aspirado del polvo y la retirada de los residuos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
+          <t>Desmontaje de red existente de tuberías de agua o de desagüe, vista o empotrada, incluidos sus accesorios y soportes. Incluye el cierre y comprobación previa de que la red está fuera de servicio y vaciada, el picado del paramento en los tramos empotrados, el corte y extracción de la tubería en tramos manejables, el taponado de las derivaciones que permanecen activas, el retiro del material clasificado según sea PVC, hierro galvanizado o cobre, y el resane de las rozas. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E65" t="n">
         <v>1</v>
       </c>
       <c r="F65" t="n">
-        <v>5.15</v>
+        <v>4.2</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -2916,33 +2916,33 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Picado de salpicado o graniplast en fachada.</t>
+          <t>Desmontaje de luminaria.</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Picado de revestimiento de salpicado, graniplast o revestimiento pétreo proyectado en fachada, ejecutado con martillo eléctrico manual y espátula, hasta dejar el friso base sano o el bloque a la vista según el estado del soporte. Incluye el sondeo previo por golpeo para delimitar las zonas sin adherencia, el trabajo desde andamio con las protecciones colectivas correspondientes, la protección de carpinterías y de la zona de paso a pie de fachada, el control de la caída de escombro, su retiro en sacos hasta el punto de acopio y la limpieza del paramento. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Desmontaje de luminaria de techo o pared, sea empotrada, de sobreponer o colgante, incluidos sus soportes y accesorios. Incluye el corte previo del circuito y la comprobación de ausencia de tensión, la desconexión y aislamiento provisional de los conductores que permanecen, el desmontaje del cuerpo de la luminaria, el retiro de las lámparas con gestión diferenciada si son fluorescentes o de descarga por su contenido en mercurio, y el resane del punto si procede. Si el cliente desea conservar el equipo, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E66" t="n">
         <v>1</v>
       </c>
       <c r="F66" t="n">
-        <v>7.11</v>
+        <v>2.17</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -2954,33 +2954,33 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Picado de mortero monocapa en fachada.</t>
+          <t>Desmontaje de aparato sanitario y su grifería.</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Picado de revestimiento de mortero monocapa en fachada, incluida su malla de refuerzo y los perfiles de arranque y goterón, ejecutado con martillo eléctrico manual hasta dejar el soporte limpio y apto para recibir el nuevo revestimiento. Incluye el sondeo previo del paramento, el trabajo desde andamio con las protecciones colectivas correspondientes, la protección de carpinterías y del paso a pie de fachada, el corte y retiro de la malla, el control de la caída de escombro, su retiro en sacos y la limpieza del soporte. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente picada.</t>
+          <t>Desmontaje de aparato sanitario existente, ya sea inodoro, lavamanos, bidé o fregadero, junto con su grifería y accesorios de conexión. Incluye cierre previo de la llave de paso y vaciado del aparato, desconexión de las tomas de agua y del desagüe, taponado provisional de las salidas para evitar olores y entrada de escombro, retirada del aparato hasta el punto de acopio y limpieza de la zona. Si el cliente desea conservar el aparato, se desmonta con cuidado y se acopia protegido. No incluye el transporte a vertedero. Medido por unidad desmontada.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E67" t="n">
         <v>1</v>
       </c>
       <c r="F67" t="n">
-        <v>8.02</v>
+        <v>4.55</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
@@ -2992,33 +2992,33 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Demolición de trasdosado de yeso laminado y su estructura.</t>
+          <t>Desmontaje de fregadero y su grifería.</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Demolición de trasdosado autoportante de placa de yeso laminado adosado a muro, junto con la perfilería de acero galvanizado y el aislamiento alojado en la cámara, ejecutada con medios manuales. Incluye la localización y desconexión previa de los mecanismos e instalaciones que discurran por el trasdosado, la protección del piso y del mobiliario, el desmontaje ordenado de las placas, el retiro del aislamiento en sacos, el desmontaje de la perfilería y de las fijaciones al muro, y la limpieza de la zona dejando el paramento original a la vista. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de fregadero de cocina con su grifería y accesorios de conexión. Incluye el cierre previo de las llaves de paso, la desconexión de las tomas de agua fría y caliente, el desmontaje del sifón y del desagüe con recogida del agua retenida, el corte del sellado perimetral con el mesón, la extracción de la pieza y el taponado provisional de las salidas para evitar olores y entrada de escombro. Si el cliente desea conservar el equipo, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E68" t="n">
         <v>1</v>
       </c>
       <c r="F68" t="n">
-        <v>2.56</v>
+        <v>4.12</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3030,33 +3030,33 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Demolición de trasdosado de bloque o ladrillo adosado a muro.</t>
+          <t>Desmontaje de calentador de agua.</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Demolición de tabique de bloque o ladrillo adosado a muro a modo de trasdosado, incluidos sus revestimientos y la cámara intermedia, ejecutada con martillo eléctrico manual sin dañar el muro original que permanece. Incluye la comprobación previa de que el trasdosado no cumple función estructural ni aloja instalaciones en servicio, la protección del entorno, el control de polvo, la fragmentación del escombro en piezas manejables, el retiro en sacos hasta el punto de acopio y el repicado de los restos de mortero adheridos al muro. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de calentador de agua eléctrico o a gas, incluidos sus soportes de anclaje y las conexiones de entrada y salida. Incluye el corte previo del suministro eléctrico o de gas y su comprobación con detector, el vaciado completo del tanque antes de liberarlo de sus soportes por el peso que retiene, la desconexión de las tuberías y su taponado, el desmontaje del anclaje al paramento, el resane de los huecos y el descenso del equipo hasta el punto de acopio. Si el cliente desea conservar el equipo, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por unidad desmontada.</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E69" t="n">
         <v>1</v>
       </c>
       <c r="F69" t="n">
-        <v>6.21</v>
+        <v>9.43</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3068,17 +3068,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Desmontaje de trasdosado directo de placa pegada al muro.</t>
+          <t>Retiro de aislamiento térmico o acústico.</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de trasdosado directo formado por placa de yeso laminado o panel aislante adherido al muro mediante pelladas de pasta, ejecutado con medios manuales mediante palanca y espátula. Incluye la protección del piso, el arranque de las placas, el rascado de los restos de pasta y adhesivo adheridos al muro hasta dejarlo apto para recibir el nuevo revestimiento, el retiro del material en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Retiro de aislamiento térmico o acústico existente, sea de lana mineral, poliestireno o poliuretano, alojado en cámara de tabique, cielo raso o cubierta. Incluye el uso de mascarilla y guantes por la irritación que producen las fibras minerales, el desmontaje del material en piezas completas cuando el estado lo permita, el ensacado inmediato para evitar la dispersión de fibras por el ambiente, el aspirado de los restos y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente retirada.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3090,11 +3090,11 @@
         <v>1</v>
       </c>
       <c r="F70" t="n">
-        <v>3.12</v>
+        <v>1.99</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Impermeabilizaciones y aislamientos</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3106,17 +3106,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Demolición de piso cerámico y su capa de pega.</t>
+          <t>Retiro de manto asfáltico en cubierta.</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso existente de baldosa cerámica o de porcelanato, junto con su capa de pega de mortero, ejecutada con martillo eléctrico manual sin comprometer la losa ni los elementos constructivos vecinos. Incluye protección previa de paredes, puertas y ambientes contiguos, control de polvo mediante aspiración, retiro manual del escombro en sacos hasta el punto de acopio y barrido de la superficie resultante, dejándola lista para recibir el nuevo contrapiso. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Retiro de impermeabilización existente de manto asfáltico en cubierta, incluidos los solapes, los refuerzos de encuentro y la imprimación adherida al soporte, ejecutado con medios manuales mediante espátula y palanca, con aplicación puntual de calor para reblandecer las zonas fuertemente adheridas. Incluye la protección de los desagües para impedir que se obstruyan con restos, el corte del manto en franjas manejables, el rascado del soporte hasta dejarlo limpio y apto para recibir la nueva impermeabilización, el retiro del material en rollos atados y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente retirada.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3128,11 +3128,11 @@
         <v>1</v>
       </c>
       <c r="F71" t="n">
-        <v>4.88</v>
+        <v>3.44</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Impermeabilizaciones y aislamientos</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -3144,33 +3144,33 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Demolición de rodapié cerámico.</t>
+          <t>Retiro de impermeabilización líquida o acrílica.</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Demolición de rodapié existente de baldosa cerámica o de porcelanato y de su capa de pega, ejecutada con medios manuales y martillo eléctrico, cuidando de no dañar el friso de la pared por encima de la línea del rodapié. Incluye retiro manual del escombro en sacos hasta el punto de acopio, repicado de los restos de mortero adheridos y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+          <t>Retiro de recubrimiento impermeabilizante líquido, acrílico o cementoso existente en cubierta o terraza, ejecutado con medios manuales mediante rasqueta y lijado mecánico, hasta dejar el soporte limpio y con la rugosidad adecuada para recibir el nuevo sistema. Incluye la protección de los desagües, el rascado de las zonas con burbujas o desprendimientos, el lijado de la superficie remanente, el aspirado del polvo generado y el retiro de los residuos. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente tratada.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E72" t="n">
         <v>1</v>
       </c>
       <c r="F72" t="n">
-        <v>1</v>
+        <v>3.34</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Impermeabilizaciones y aislamientos</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -3182,33 +3182,33 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Demolición de piso de granito o terrazo en baldosa.</t>
+          <t>Desmontaje de canal de aguas lluvias.</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso existente de baldosa de granito o terrazo prefabricado, junto con su capa de asiento de mortero, ejecutada con martillo eléctrico manual. Por la dureza y el espesor de este tipo de baldosa el rendimiento es menor que en un piso cerámico y el escombro resulta más pesado, lo que se refleja en el rendimiento de la partida. Incluye protección previa de los ambientes contiguos, control de polvo, retiro manual del escombro en sacos y limpieza de la superficie. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de canal o canalón de recogida de aguas lluvias, incluidos los soportes, las uniones y las piezas especiales, ejecutado con medios manuales desde andamio. Incluye el acordonamiento de la zona inferior, el desmontaje por tramos con sostenimiento previo, la extracción de los ganchos y anclajes al alero, el resane de los puntos de fijación, el descenso del material y su clasificación para reciclaje. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E73" t="n">
         <v>1</v>
       </c>
       <c r="F73" t="n">
-        <v>5.9</v>
+        <v>2.7</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Techos y cubiertas</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -3220,17 +3220,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Demolición de rodapié de granito o terrazo.</t>
+          <t>Desmontaje de bajante de aguas lluvias.</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Demolición de rodapié existente de granito o terrazo prefabricado y de su capa de asiento, ejecutada con martillo eléctrico manual, cuidando de no dañar el friso de la pared. Incluye repicado de los restos de mortero adheridos, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+          <t>Desmontaje de bajante de aguas lluvias, vista o empotrada, incluidos las abrazaderas, los codos y las piezas de conexión, ejecutado con medios manuales desde andamio. Incluye el acordonamiento de la zona inferior, el corte de la bajante en tramos manejables, la extracción de las abrazaderas ancladas a la fachada, el resane de los huecos de anclaje, el taponado provisional de la conexión a la red que permanece y el retiro del material. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente desmontada.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3242,11 +3242,11 @@
         <v>1</v>
       </c>
       <c r="F74" t="n">
-        <v>1.17</v>
+        <v>2.72</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Techos y cubiertas</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3258,17 +3258,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Demolición de piso de granito vaciado en sitio.</t>
+          <t>Desmontaje de cubierta de teja.</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso continuo de granito vaciado en sitio, incluida su base de mortero y las platinas divisorias de las juntas, ejecutada con martillo neumático por tratarse de una superficie monolítica de gran dureza. Incluye corte perimetral previo con amoladora de disco de diamante para delimitar la zona de intervención y evitar desprendimientos fuera de ella, protección de los ambientes contiguos, control de polvo, fragmentación del escombro en piezas manejables, retiro en sacos y limpieza. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de cubierta de teja criolla, teja plana o similar, incluidos el mortero de fijación y los caballetes de cumbrera, ejecutado con medios manuales desde andamio y con línea de vida. Incluye la comprobación previa del estado de la estructura de soporte antes de que el personal transite sobre ella, el desmontaje ordenado desde la cumbrera hacia el alero, el descenso de las tejas por medios mecánicos evitando el lanzamiento, la clasificación de las piezas aprovechables y el acopio del material. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3280,11 +3280,11 @@
         <v>1</v>
       </c>
       <c r="F75" t="n">
-        <v>13.04</v>
+        <v>9.44</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Techos y cubiertas</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -3296,17 +3296,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Demolición de piso de cemento pulido.</t>
+          <t>Desmontaje de cubierta de lámina metálica o acerolit.</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso continuo de cemento pulido y de su base de mortero, ejecutada con martillo eléctrico manual, sin afectar a la losa estructural. Incluye corte perimetral con amoladora cuando la demolición sea parcial, protección de los ambientes contiguos, control de polvo mediante aspiración, fragmentación del escombro, retiro manual en sacos hasta el punto de acopio y limpieza de la superficie resultante. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de cubierta de lámina metálica, acerolit, zinc o fibrocemento, incluidos los ganchos, tornillos y elementos de fijación a la estructura, ejecutado con medios manuales desde andamio y con línea de vida. Si la lámina es de fibrocemento antiguo debe verificarse la posible presencia de amianto, en cuyo caso el desmontaje queda fuera de esta partida y exige empresa autorizada. Incluye el desmontaje ordenado con sujeción de las láminas frente al viento, el descenso controlado, la clasificación del material y el acopio. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3318,11 +3318,11 @@
         <v>1</v>
       </c>
       <c r="F76" t="n">
-        <v>6.92</v>
+        <v>6.81</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Techos y cubiertas</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -3334,33 +3334,33 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Demolición de rodapié de cemento.</t>
+          <t>Desmontaje de estructura de techo.</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Demolición de rodapié corrido de mortero de cemento, ejecutada con medios manuales y cincel, cuidando de no dañar el friso de la pared por encima de la línea del rodapié. Incluye repicado de los restos adheridos al paramento, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+          <t>Desmontaje de la estructura de soporte de cubierta, formada por correas, cerchas o perfiles de madera o metal, una vez retirado el material de cubrición. Ejecutado con sierra, oxicorte o desatornillado según el material, con apeo previo y eslingado de los elementos antes de liberarlos. Incluye el estudio del orden de desmontaje para conservar la estabilidad del conjunto, el sostenimiento de cada pieza antes del corte, el descenso mecánico, la clasificación del material recuperable y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de cubierta cuya estructura se desmonta.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E77" t="n">
         <v>1</v>
       </c>
       <c r="F77" t="n">
-        <v>0.91</v>
+        <v>14.46</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Techos y cubiertas</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -3372,17 +3372,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Demolición de piso de piedra natural.</t>
+          <t>Demolición de pendientado y protección de cubierta plana.</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso existente de piedra natural, ya sea mármol, granito natural o laja, junto con su capa de asiento de mortero, ejecutada con martillo eléctrico manual. Si el cliente desea recuperar las piezas, se levantan una a una con cuidado, se limpian de mortero y se acopian protegidas, lo que reduce el rendimiento y debe advertirse en el presupuesto. Incluye protección de los ambientes contiguos, control de polvo, retiro manual del escombro en sacos y limpieza de la superficie. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Demolición de la capa de pendientado y de la protección de cubierta plana, comprendiendo el relleno aligerado de formación de pendiente, la capa de mortero de protección y el acabado superficial, hasta descubrir la losa. Ejecutada con martillo eléctrico manual. Incluye la protección y taponado provisional de los desagües, la comprobación de no perforar la losa, el control del acopio de escombro sobre la cubierta para no sobrecargarla, su descenso por medios mecánicos y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -3394,11 +3394,11 @@
         <v>1</v>
       </c>
       <c r="F78" t="n">
-        <v>6.34</v>
+        <v>11.27</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Techos y cubiertas</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -3410,33 +3410,33 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Demolición de rodapié de piedra natural.</t>
+          <t>Desmontaje de mueble de baño y sus accesorios.</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Demolición de rodapié existente de piedra natural y de su capa de asiento, ejecutada con martillo eléctrico manual, cuidando de no dañar el friso de la pared. Incluye repicado de los restos de mortero adheridos, retiro manual del escombro en sacos hasta el punto de acopio y limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente demolida.</t>
+          <t>Desmontaje de mueble de baño con su lavamanos integrado, espejo y accesorios como toalleros, jaboneras y portarrollos. Ejecutado con medios manuales y atornillador. Incluye el cierre previo de las llaves de paso, la desconexión de las tomas de agua y del desagüe con recogida del agua retenida en el sifón, el corte del sellado perimetral, el desmontaje del mueble y del espejo con sostenimiento previo, la extracción de los anclajes, el resane de los huecos y el retiro del material. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por conjunto realmente desmontado.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E79" t="n">
         <v>1</v>
       </c>
       <c r="F79" t="n">
-        <v>1.25</v>
+        <v>6.86</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Equipamiento y mobiliario fijo</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -3448,33 +3448,33 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Levantado de piso de parquet o madera.</t>
+          <t>Desmontaje de mueble de cocina alto o bajo.</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Levantado de piso existente de parquet o de tablilla de madera, incluidos los rastreles o el adhesivo de fijación al contrapiso, ejecutado con medios manuales mediante palanca y espátula. Incluye el retiro previo de las molduras de remate, el rascado de los restos de adhesivo adheridos al contrapiso, la extracción de los clavos o tornillos que queden en la base, el retiro del material en sacos hasta el punto de acopio y la limpieza de la superficie resultante. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
+          <t>Desmontaje de mueble de cocina alto o bajo, incluidas las puertas, los entrepaños, los cajones y los herrajes de fijación al paramento. Ejecutado con medios manuales y atornillador. Incluye el vaciado previo del contenido si el cliente no lo hubiera retirado, la desconexión de las instalaciones que atraviesen el mueble, el desmontaje ordenado desde las puertas hacia el cuerpo, la extracción de tacos y tornillos del muro, el resane de los huecos de anclaje y la clasificación de las piezas aprovechables. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud de frente de mueble realmente desmontada.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E80" t="n">
         <v>1</v>
       </c>
       <c r="F80" t="n">
-        <v>2.17</v>
+        <v>5.11</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Equipamiento y mobiliario fijo</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -3486,17 +3486,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Levantado de rodapié de madera.</t>
+          <t>Desmontaje de mesón de cocina y su salpicadero.</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Levantado de rodapié existente de madera, ejecutado con medios manuales mediante palanca y espátula, cuidando de no dañar el friso de la pared. Incluye la extracción de los clavos, tornillos o tacos de fijación que queden en el paramento, el retiro del material en sacos hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro. Medido en longitud realmente levantada.</t>
+          <t>Desmontaje de mesón o tope de cocina, sea de granito, cuarzo, concreto o laminado, junto con su salpicadero y la estructura de apoyo. Ejecutado con medios manuales, amoladora y martillo eléctrico según el material. Incluye el desmontaje previo del fregadero y de la placa de cocción si permanecieran, el corte del sellado perimetral, el sostenimiento del tablero por dos operarios dado su peso, el corte en tramos manejables cuando no pueda extraerse entero, el picado de los apoyos de obra, el resane del paramento y el retiro del material. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud de mesón realmente desmontada.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -3508,11 +3508,11 @@
         <v>1</v>
       </c>
       <c r="F81" t="n">
-        <v>0.43</v>
+        <v>8.76</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Equipamiento y mobiliario fijo</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -3524,17 +3524,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Levantado de piso laminado.</t>
+          <t>Desmontaje de mobiliario fijo diverso.</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Levantado de piso laminado flotante existente, incluidas la manta acústica y las molduras de remate perimetrales, ejecutado con medios manuales. Por tratarse de un sistema flotante de encastre el desmontaje es rápido y no genera escombro pesado. Incluye el desmontaje ordenado de las tablas, el retiro de la manta y del perfil perimetral, la limpieza y aspirado del contrapiso resultante y el retiro del material en sacos hasta el punto de acopio. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
+          <t>Desmontaje de mobiliario fijo no clasificado en las partidas anteriores, tal como repisas de obra, bancos, barras, mostradores o estanterías ancladas al paramento. Ejecutado con medios manuales, atornillador, amoladora y martillo eléctrico según el material y el tipo de anclaje. Incluye el vaciado previo, el sostenimiento del elemento antes de liberar el último anclaje, la extracción de las fijaciones, el picado de los apoyos de obra si los tuviera, el resane de los huecos y el retiro del material clasificado. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de frente realmente desmontada.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3546,11 +3546,11 @@
         <v>1</v>
       </c>
       <c r="F82" t="n">
-        <v>1.26</v>
+        <v>6.41</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Equipamiento y mobiliario fijo</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -3562,33 +3562,33 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Levantado de piso vinílico, linóleo o alfombra.</t>
+          <t>Desmontaje de estructura metálica.</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Levantado de revestimiento de piso flexible existente, ya sea vinílico en lámina o baldosa, linóleo o alfombra, incluido el adhesivo de fijación al contrapiso, ejecutado con medios manuales mediante espátula y rasqueta. Incluye la aplicación puntual de disolvente removedor en las zonas donde el adhesivo esté fuertemente adherido, el rascado hasta dejar el contrapiso limpio y sin restos que comprometan la adherencia del nuevo acabado, la ventilación del ambiente durante los trabajos, el retiro del material en sacos y la limpieza final. No incluye el bote del escombro. Medido en superficie realmente levantada.</t>
+          <t>Desmontaje de estructura metálica de acero, formada por perfiles laminados o armados, ejecutado mediante oxicorte y desatornillado según el tipo de unión, con apeo previo de los elementos que permanecen. Incluye el estudio del orden de desmontaje para mantener la estabilidad del conjunto en todo momento, el eslingado y sostenimiento de las piezas antes de liberarlas, el corte en tramos transportables, el descenso a nivel de acopio y la clasificación del acero para su venta o gestión como chatarra, cuyo valor de recuperación puede descontarse al cliente. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en peso realmente desmontado.</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E83" t="n">
         <v>1</v>
       </c>
       <c r="F83" t="n">
-        <v>2.12</v>
+        <v>0.52</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -3600,33 +3600,33 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Demolición de piso continuo de concreto.</t>
+          <t>Demolición de columna de concreto armado.</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Demolición de piso continuo de concreto de hasta 10 cm de espesor, ejecutada con martillo neumático, sin afectar a la losa estructural ni a las instalaciones que discurran por debajo. Incluye la comprobación previa de que no existen tuberías ni canalizaciones enterradas en la zona, el corte perimetral con amoladora de disco de diamante para delimitar la demolición, la protección de los ambientes contiguos, el control de polvo, la fragmentación del escombro en piezas manejables, el retiro en sacos hasta el punto de acopio y la limpieza. Si el piso está armado con malla electrosoldada se incluye su corte y retiro. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Demolición de columna de concreto armado, ejecutada con martillo eléctrico o neumático según la sección, con corte previo de la armadura longitudinal. Exige apeo previo de la estructura que la columna soporta y validación del cálculo estructural, trabajos que se valoran aparte. Incluye la protección del entorno, la demolición descendente por tramos para mantener el control del elemento, el corte y retiro del acero, la fragmentación del concreto, el descenso del escombro y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en volumen realmente demolido.</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E84" t="n">
         <v>1</v>
       </c>
       <c r="F84" t="n">
-        <v>15.33</v>
+        <v>119.95</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -3638,33 +3638,33 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Demolición de contrapiso o base de mortero de nivelación.</t>
+          <t>Demolición de viga de concreto armado.</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Demolición de contrapiso o base de mortero de nivelación de hasta 5 cm de espesor, una vez retirado el piso de acabado, ejecutada con martillo eléctrico manual hasta dejar la losa estructural a la vista y limpia. Se emplea cuando la base existente está disgregada, hueca o fuera de nivel y no admite recibir el nuevo piso. Incluye la comprobación previa del estado de la base mediante golpeo, la protección de los ambientes contiguos, el control de polvo mediante aspiración, el retiro manual del escombro en sacos y el barrido final de la losa. No incluye el bote del escombro. Medido en superficie realmente demolida.</t>
+          <t>Demolición de viga de concreto armado, ejecutada con martillo eléctrico o neumático, con apeo previo de la losa o de los elementos que la viga sostiene. Incluye la validación estructural previa, el montaje del apeo provisional, la protección del entorno y del nivel inferior, la demolición por tramos controlados desde andamio, el corte y retiro de las barras de refuerzo, el descenso del escombro y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en volumen realmente demolido.</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E85" t="n">
         <v>1</v>
       </c>
       <c r="F85" t="n">
-        <v>7.18</v>
+        <v>134.08</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
@@ -3676,17 +3676,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Desmontaje de piso técnico registrable.</t>
+          <t>Demolición de losa de entrepiso maciza o nervada.</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de piso técnico registrable existente, formado por paneles apoyados sobre pedestales regulables, ejecutado con medios manuales. Por tratarse de un sistema desmontable la operación es limpia y permite recuperar el material. Incluye la retirada ordenada de los paneles con ventosa, el desmontaje de los pedestales y travesaños, la clasificación de las piezas en aprovechables y desechables, el acopio protegido de las que el cliente desee conservar, el retiro del resto en sacos y la limpieza de la losa resultante. No incluye el bote del escombro. Medido en superficie realmente desmontada.</t>
+          <t>Demolición de losa de entrepiso de concreto armado, maciza o nervada, ejecutada con martillo neumático y corte de armaduras, con apeo previo de los tramos que permanecen. Incluye la validación estructural, el montaje del apeo, el acordonamiento y protección del nivel inferior para impedir el paso durante los trabajos, la demolición en franjas controladas desde los apoyos hacia el centro, el corte y separación del acero, el descenso del escombro y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -3698,11 +3698,11 @@
         <v>1</v>
       </c>
       <c r="F86" t="n">
-        <v>1.09</v>
+        <v>46.07</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -3714,17 +3714,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Demolición de cielo raso de yeso laminado y su estructura.</t>
+          <t>Apertura de hueco en losa de concreto armado.</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Demolición de cielo raso continuo de placa de yeso laminado, junto con la perfilería de acero galvanizado, las varillas de cuelgue y el ángulo perimetral, ejecutada con medios manuales. Incluye la desconexión y retiro previo de las luminarias, rejillas y difusores alojados en el plano del cielo, la protección del piso y del mobiliario, el descuelgue ordenado de las placas para evitar caídas incontroladas, el retiro del escombro en sacos y de la perfilería atada, y la limpieza de la zona dejando la losa a la vista. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Apertura de hueco en losa de concreto armado para paso de escalera, ducto de instalaciones o claraboya, ejecutada mediante corte perimetral con disco de diamante y demolición interior con martillo eléctrico. Incluye la validación estructural previa y el refuerzo del borde si el cálculo lo exige, el apeo de la zona, el replanteo y corte perimetral que garantiza un borde limpio y sin fisuración hacia el resto de la losa, el corte de las armaduras, el descenso controlado del escombro y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de hueco realmente abierto.</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3736,11 +3736,11 @@
         <v>1</v>
       </c>
       <c r="F87" t="n">
-        <v>2.69</v>
+        <v>36.26</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -3752,17 +3752,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Demolición de cielo raso de yeso vaciado o pasta.</t>
+          <t>Desmontaje de estructura de madera.</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Demolición de cielo raso de yeso vaciado, pasta o placa de yeso tradicional, junto con su estructura de soporte y elementos de cuelgue, ejecutada con medios manuales y martillo eléctrico donde el espesor lo requiera. Por tratarse de un material macizo genera más escombro y más polvo fino que un cielo de placa. Incluye la desconexión previa de las luminarias, la protección del piso y del mobiliario, el control de polvo mediante aspiración, el retiro del escombro en sacos y la limpieza de la losa resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
+          <t>Desmontaje de estructura de madera de entrepiso o de techo, formada por vigas, viguetas y entablado, ejecutado con medios manuales y sierra, con apeo previo. Incluye la inspección previa del estado de la madera para prever roturas por pudrición o ataque de xilófagos, el apeo provisional, el desmontaje ordenado desde el entablado hacia las vigas principales, la extracción de clavos y herrajes, la clasificación de las piezas aprovechables si el cliente desea conservarlas, el descenso del material y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -3774,11 +3774,11 @@
         <v>1</v>
       </c>
       <c r="F88" t="n">
-        <v>4.91</v>
+        <v>13.18</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -3790,33 +3790,33 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Desmontaje de cielo raso desmontable de fibra mineral.</t>
+          <t>Demolición de losa de fundación de concreto armado.</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de cielo raso registrable existente, formado por paneles apoyados sobre perfilería vista en retícula, ejecutado con medios manuales. Por ser un sistema desmontable la operación es limpia, rápida y permite recuperar buena parte del material. Incluye la retirada ordenada de los paneles, el desmontaje de la perfilería y de los tensores de cuelgue, la clasificación de las piezas en aprovechables y desechables, el acopio protegido de las que el cliente desee conservar y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Demolición de losa de fundación de concreto armado, ejecutada con martillo hidráulico montado sobre retroexcavadora y corte de la malla de refuerzo. Incluye el corte perimetral previo para delimitar la zona de intervención, la comprobación de que no discurren instalaciones enterradas bajo la losa, la fragmentación del concreto en piezas cargables, el corte y separación del acero para su gestión diferenciada, el acopio del escombro y la limpieza del terreno resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en volumen realmente demolido.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E89" t="n">
         <v>1</v>
       </c>
       <c r="F89" t="n">
-        <v>1.65</v>
+        <v>119.83</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -3828,33 +3828,33 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Desmontaje de cielo raso de machihembrado de madera.</t>
+          <t>Demolición de viga de riostra o muro de contención de concreto.</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de cielo raso de machihembrado o tablilla de madera, junto con los rastreles y la estructura de soporte fijada a la losa, ejecutado con medios manuales mediante palanca y barra. Incluye la desconexión previa de las luminarias, la protección del piso y del mobiliario, la extracción de los clavos y tornillos que queden en la estructura, el retiro del material en atados hasta el punto de acopio, la clasificación de las piezas aprovechables y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Demolición de viga de riostra, muro de contención o murete de concreto armado, ejecutada con martillo neumático y corte de armaduras. Incluye la comprobación previa de que el elemento no sostiene empujes de tierra activos o, en su caso, el sostenimiento provisional del terreno, la protección del entorno, el corte y retiro del acero de refuerzo, la fragmentación del concreto y su acopio, y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en volumen realmente demolido.</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E90" t="n">
         <v>1</v>
       </c>
       <c r="F90" t="n">
-        <v>2.82</v>
+        <v>104.61</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -3866,33 +3866,33 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Desmontaje de cielo raso de láminas de PVC o aluminio.</t>
+          <t>Demolición de zapata o pedestal de concreto armado.</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de cielo raso formado por láminas de PVC, aluminio o material similar, junto con sus perfiles de soporte y remates perimetrales, ejecutado con medios manuales. Incluye la desconexión previa de las luminarias y rejillas, la protección del piso, el desencastre ordenado de las láminas para poder recuperarlas si el cliente lo desea, el desmontaje de la perfilería, el retiro del material hasta el punto de acopio y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente desmontada.</t>
+          <t>Demolición de zapata aislada o pedestal de concreto armado, ejecutada con martillo neumático y corte de la armadura con oxicorte o amoladora. Requiere comprobación estructural previa de que el elemento ya no cumple función portante o de que la estructura está debidamente apeada. Incluye la excavación de descubrimiento del elemento si estuviera enterrado, la protección del entorno, el corte y retiro de las barras de acero, la fragmentación del concreto en piezas manejables y su acopio, y el relleno del hueco resultante si el proyecto lo requiere. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en volumen realmente demolido.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E91" t="n">
         <v>1</v>
       </c>
       <c r="F91" t="n">
-        <v>1.76</v>
+        <v>113.98</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -3904,33 +3904,33 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Desmontaje de mueble de baño y sus accesorios.</t>
+          <t>Demolición de brocal o cordón de acera.</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de mueble de baño con su lavamanos integrado, espejo y accesorios como toalleros, jaboneras y portarrollos. Ejecutado con medios manuales y atornillador. Incluye el cierre previo de las llaves de paso, la desconexión de las tomas de agua y del desagüe con recogida del agua retenida en el sifón, el corte del sellado perimetral, el desmontaje del mueble y del espejo con sostenimiento previo, la extracción de los anclajes, el resane de los huecos y el retiro del material. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido por conjunto realmente desmontado.</t>
+          <t>Demolición de brocal, cordón o bordillo de acera, sea prefabricado o vaciado en sitio, junto con su dado de concreto de apoyo, ejecutada con martillo eléctrico manual. Incluye el acordonamiento y señalización del área de trabajo por su situación en zona de tránsito, el corte de las juntas entre piezas, la demolición del dado de apoyo, la extracción del escombro, el acopio de las piezas prefabricadas aprovechables si el cliente desea reutilizarlas y la limpieza de la zona. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud realmente demolida.</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E92" t="n">
         <v>1</v>
       </c>
       <c r="F92" t="n">
-        <v>6.86</v>
+        <v>7.1</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Equipamiento</t>
+          <t>Obras exteriores y urbanismo</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
@@ -3942,33 +3942,33 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Desmontaje de mueble de cocina alto o bajo.</t>
+          <t>Demolición de pavimento exterior de concreto.</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de mueble de cocina alto o bajo, incluidas las puertas, los entrepaños, los cajones y los herrajes de fijación al paramento. Ejecutado con medios manuales y atornillador. Incluye el vaciado previo del contenido si el cliente no lo hubiera retirado, la desconexión de las instalaciones que atraviesen el mueble, el desmontaje ordenado desde las puertas hacia el cuerpo, la extracción de tacos y tornillos del muro, el resane de los huecos de anclaje y la clasificación de las piezas aprovechables. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud de frente de mueble realmente desmontada.</t>
+          <t>Demolición de pavimento exterior de concreto, en acera, patio o vía de acceso, de hasta 15 cm de espesor, ejecutada con martillo hidráulico montado sobre retroexcavadora. Incluye la comprobación previa de que no discurren instalaciones enterradas bajo el pavimento, el corte perimetral con disco de diamante para delimitar la zona de intervención, el acordonamiento del área de trabajo, la fragmentación del concreto en piezas cargables, el corte y separación de la malla de refuerzo si la tuviera, el acopio del escombro y la limpieza. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E93" t="n">
         <v>1</v>
       </c>
       <c r="F93" t="n">
-        <v>5.11</v>
+        <v>12.66</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Equipamiento</t>
+          <t>Obras exteriores y urbanismo</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -3980,33 +3980,33 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Desmontaje de mesón de cocina y su salpicadero.</t>
+          <t>Demolición de pavimento asfáltico.</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de mesón o tope de cocina, sea de granito, cuarzo, concreto o laminado, junto con su salpicadero y la estructura de apoyo. Ejecutado con medios manuales, amoladora y martillo eléctrico según el material. Incluye el desmontaje previo del fregadero y de la placa de cocción si permanecieran, el corte del sellado perimetral, el sostenimiento del tablero por dos operarios dado su peso, el corte en tramos manejables cuando no pueda extraerse entero, el picado de los apoyos de obra, el resane del paramento y el retiro del material. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en longitud de mesón realmente desmontada.</t>
+          <t>Demolición de pavimento asfáltico de hasta 10 cm de espesor, ejecutada con martillo hidráulico montado sobre retroexcavadora, con corte perimetral previo para obtener un borde recto que facilite la reposición. Incluye la comprobación de instalaciones enterradas, el acordonamiento y señalización del área, el corte perimetral con disco, el arranque y fragmentación del asfalto, el acopio diferenciado del material fresado por admitir reciclaje específico, y la limpieza y barrido de la base resultante. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente demolida.</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E94" t="n">
         <v>1</v>
       </c>
       <c r="F94" t="n">
-        <v>8.76</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Equipamiento</t>
+          <t>Obras exteriores y urbanismo</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -4018,17 +4018,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Desmontaje de mobiliario fijo diverso.</t>
+          <t>Levantado de pavimento de adoquín.</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Desmontaje de mobiliario fijo no clasificado en las partidas anteriores, tal como repisas de obra, bancos, barras, mostradores o estanterías ancladas al paramento. Ejecutado con medios manuales, atornillador, amoladora y martillo eléctrico según el material y el tipo de anclaje. Incluye el vaciado previo, el sostenimiento del elemento antes de liberar el último anclaje, la extracción de las fijaciones, el picado de los apoyos de obra si los tuviera, el resane de los huecos y el retiro del material clasificado. Si el cliente desea conservar el elemento, se desmonta con cuidado y se acopia protegido. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie de frente realmente desmontada.</t>
+          <t>Levantado de pavimento exterior de adoquín de concreto o piedra, junto con su cama de arena, ejecutado con medios manuales mediante palanca y pico. Por tratarse de piezas independientes el levantado permite recuperar un porcentaje elevado del material para su reutilización. Incluye el levantado ordenado desde un borde libre, la limpieza de las piezas retirando la arena y el mortero adherido, su clasificación en aprovechables y desechables, el paletizado o acopio de las recuperables, el retiro de la cama de arena y el barrido de la base. No incluye el bote del escombro, que se valora en el capítulo de gestión de residuos. Medido en superficie realmente levantada.</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -4040,11 +4040,11 @@
         <v>1</v>
       </c>
       <c r="F95" t="n">
-        <v>6.41</v>
+        <v>3.35</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Equipamiento</t>
+          <t>Obras exteriores y urbanismo</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -4056,7 +4056,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Urbanización interior de la parcela</t>
+          <t>Obras exteriores y urbanismo</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -4094,7 +4094,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Urbanización interior de la parcela</t>
+          <t>Obras exteriores y urbanismo</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -4132,7 +4132,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Urbanización interior de la parcela</t>
+          <t>Obras exteriores y urbanismo</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -4170,7 +4170,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Demoliciones</t>
+          <t>Demoliciones y desmontajes</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4196,7 +4196,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Urbanización interior de la parcela</t>
+          <t>Obras exteriores y urbanismo</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
@@ -4208,17 +4208,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Fachadas y particiones</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
+          <t>Tabique de bloque de concreto de 10 cm, recibido con mortero de pega.</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Tabique interior no estructural de 10 cm de espesor, ejecutado con bloque hueco de concreto de 10x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Incluye replanteo y trazado sobre el piso, colocación de hiladas a nivel y plomo con la ayuda de reglas y cuerda, formación de huecos de paso, anclaje del tabique a los paramentos existentes, humedecido previo de las piezas y limpieza de restos. No incluye el friso ni los dinteles de los huecos, que se valoran aparte. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -4230,11 +4230,11 @@
         <v>1</v>
       </c>
       <c r="F100" t="n">
-        <v>52.4</v>
+        <v>18.29</v>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Tabiquería de entramado autoportante</t>
+          <t>Bloque de concreto</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
@@ -4246,17 +4246,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Fachadas y particiones</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Tabique de bloque de concreto de 10 cm, recibido con mortero de pega.</t>
+          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Tabique interior no estructural de 10 cm de espesor, ejecutado con bloque hueco de concreto de 10x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Incluye replanteo y trazado sobre el piso, colocación de hiladas a nivel y plomo con la ayuda de reglas y cuerda, formación de huecos de paso, anclaje del tabique a los paramentos existentes, humedecido previo de las piezas y limpieza de restos. No incluye el friso ni los dinteles de los huecos, que se valoran aparte. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -4268,11 +4268,11 @@
         <v>1</v>
       </c>
       <c r="F101" t="n">
-        <v>18.29</v>
+        <v>52.4</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Fábrica no estructural</t>
+          <t>Tabiquería de yeso laminado</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -4284,33 +4284,33 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Gestión de residuos</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Retirada y transporte de escombro a vertedero autorizado.</t>
+          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Retirada de escombro procedente de demoliciones desde el punto de acopio de la obra y transporte en camión volqueta hasta vertedero o botadero autorizado, incluido el canon de vertido. Incluye la carga manual del escombro sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado con una distancia media considerada de 25 km, la descarga y la limpieza de la zona de carga. Medido por metro cúbico de escombro esponjado realmente retirado.</t>
+          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E102" t="n">
         <v>1</v>
       </c>
       <c r="F102" t="n">
-        <v>16.07</v>
+        <v>10.75</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Transporte de residuos</t>
+          <t>Frisos y enlucidos de mortero</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -4322,33 +4322,33 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E103" t="n">
         <v>1</v>
       </c>
       <c r="F103" t="n">
-        <v>8.369999999999999</v>
+        <v>10.87</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Enchapado cerámico y porcelanato</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -4360,33 +4360,33 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E104" t="n">
         <v>1</v>
       </c>
       <c r="F104" t="n">
-        <v>8.720000000000001</v>
+        <v>8.02</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Eléctrica</t>
+          <t>Bases, contrapisos y nivelación</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
@@ -4398,33 +4398,33 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E105" t="n">
         <v>1</v>
       </c>
       <c r="F105" t="n">
-        <v>37.22</v>
+        <v>9.17</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Fontanería</t>
+          <t>Pisos cerámicos y porcelanato</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -4436,33 +4436,33 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E106" t="n">
         <v>1</v>
       </c>
       <c r="F106" t="n">
-        <v>13.52</v>
+        <v>12.51</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Fontanería</t>
+          <t>Pisos cerámicos y porcelanato</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
@@ -4474,17 +4474,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+          <t>Colocación de rodapié cerámico o de porcelanato.</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -4496,11 +4496,11 @@
         <v>1</v>
       </c>
       <c r="F107" t="n">
-        <v>7.45</v>
+        <v>1.69</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Fontanería</t>
+          <t>Rodapiés y remates de piso</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
@@ -4512,33 +4512,33 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Cielos rasos</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Punto de desagüe para aparato sanitario.</t>
+          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E108" t="n">
         <v>1</v>
       </c>
       <c r="F108" t="n">
-        <v>33.84</v>
+        <v>18.47</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Saneamiento y desagües</t>
+          <t>Yeso laminado continuo</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
@@ -4550,17 +4550,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Instalaciones</t>
+          <t>Instalaciones sanitarias</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -4572,11 +4572,11 @@
         <v>1</v>
       </c>
       <c r="F109" t="n">
-        <v>11.04</v>
+        <v>7.45</v>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Saneamiento y desagües</t>
+          <t>Tuberías y montantes de agua</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
@@ -4588,33 +4588,33 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones sanitarias</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+          <t>Punto de agua fría y caliente para aparato sanitario.</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E110" t="n">
         <v>1</v>
       </c>
       <c r="F110" t="n">
-        <v>10.87</v>
+        <v>37.22</v>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>Revestimientos de paramentos con piezas rígidas</t>
+          <t>Puntos de agua</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -4626,33 +4626,33 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones sanitarias</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E111" t="n">
         <v>1</v>
       </c>
       <c r="F111" t="n">
-        <v>3.46</v>
+        <v>13.52</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Pinturas</t>
+          <t>Llaves y valvulería</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -4664,33 +4664,33 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones sanitarias</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E112" t="n">
         <v>1</v>
       </c>
       <c r="F112" t="n">
-        <v>5.23</v>
+        <v>23.45</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Pinturas</t>
+          <t>Aparatos sanitarios y grifería</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
@@ -4702,33 +4702,33 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones sanitarias</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+          <t>Instalación de lavamanos con su grifería y desagüe.</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E113" t="n">
         <v>1</v>
       </c>
       <c r="F113" t="n">
-        <v>2.82</v>
+        <v>36.45</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Pinturas</t>
+          <t>Aparatos sanitarios y grifería</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -4740,33 +4740,33 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones sanitarias</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E114" t="n">
         <v>1</v>
       </c>
       <c r="F114" t="n">
-        <v>10.75</v>
+        <v>11.04</v>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Revestimientos continuos</t>
+          <t>Tuberías y bajantes de desagüe</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -4778,33 +4778,33 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones sanitarias</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+          <t>Punto de desagüe para aparato sanitario.</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E115" t="n">
         <v>1</v>
       </c>
       <c r="F115" t="n">
-        <v>8.02</v>
+        <v>33.84</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Puntos de desagüe</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -4816,17 +4816,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones eléctricas</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -4838,11 +4838,11 @@
         <v>1</v>
       </c>
       <c r="F116" t="n">
-        <v>1.69</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Canalizaciones y cableado</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -4854,33 +4854,33 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Instalaciones eléctricas</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>ud</t>
         </is>
       </c>
       <c r="E117" t="n">
         <v>1</v>
       </c>
       <c r="F117" t="n">
-        <v>9.17</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Puntos, mecanismos y tomas</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -4892,17 +4892,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Pintura y acabados</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -4914,11 +4914,11 @@
         <v>1</v>
       </c>
       <c r="F118" t="n">
-        <v>12.51</v>
+        <v>2.82</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>Pavimentos</t>
+          <t>Preparación de soportes</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -4930,17 +4930,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Revestimientos y trasdosados</t>
+          <t>Pintura y acabados</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -4952,11 +4952,11 @@
         <v>1</v>
       </c>
       <c r="F119" t="n">
-        <v>18.47</v>
+        <v>3.46</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Falsos techos</t>
+          <t>Pintura interior</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -4968,33 +4968,33 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Señalización y equipamiento</t>
+          <t>Pintura y acabados</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E120" t="n">
         <v>1</v>
       </c>
       <c r="F120" t="n">
-        <v>23.45</v>
+        <v>5.23</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Esmaltes sobre madera y metal</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -5006,33 +5006,33 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Señalización y equipamiento</t>
+          <t>Gestión de residuos y limpieza</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Instalación de lavamanos con su grifería y desagüe.</t>
+          <t>Retirada y transporte de escombro a vertedero autorizado.</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
+          <t>Retirada de escombro procedente de demoliciones desde el punto de acopio de la obra y transporte en camión volqueta hasta vertedero o botadero autorizado, incluido el canon de vertido. Incluye la carga manual del escombro sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado con una distancia media considerada de 25 km, la descarga y la limpieza de la zona de carga. Medido por metro cúbico de escombro esponjado realmente retirado.</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E121" t="n">
         <v>1</v>
       </c>
       <c r="F121" t="n">
-        <v>36.45</v>
+        <v>16.07</v>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Retiro y transporte de escombro</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">

</xml_diff>

<commit_message>
Cerrar el capitulo 03 Movimiento de tierras con 22 partidas en 4 subcapitulos
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/catalogo_partidas.xlsx
+++ b/basedatos_partidas/salida/catalogo_partidas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H145"/>
+  <dimension ref="A1:H167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5120,17 +5120,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Paredes y tabiquería</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Tabique de bloque de concreto de 10 cm, recibido con mortero de pega.</t>
+          <t>Limpieza y desbroce manual del terreno.</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>Tabique interior no estructural de 10 cm de espesor, ejecutado con bloque hueco de concreto de 10x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Incluye replanteo y trazado sobre el piso, colocación de hiladas a nivel y plomo con la ayuda de reglas y cuerda, formación de huecos de paso, anclaje del tabique a los paramentos existentes, humedecido previo de las piezas y limpieza de restos. No incluye el friso ni los dinteles de los huecos, que se valoran aparte. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Limpieza y desbroce manual del terreno, con retiro de maleza, hierba, arbustos y basura acumulada, hasta dejar la superficie despejada para el replanteo. Se emplea en parcelas pequeñas o de acceso restringido donde no entra maquinaria. Incluye el corte de la vegetación con desbrozadora, el arranque manual de raíces superficiales, el recogido y ensacado de los residuos, su traslado al punto de acopio y el barrido final de la superficie. No incluye el transporte del material sobrante a botadero, que se valora en el subcapítulo de transporte de tierras. Medido en superficie realmente desbrozada.</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -5142,11 +5142,11 @@
         <v>1</v>
       </c>
       <c r="F124" t="n">
-        <v>18.29</v>
+        <v>1.08</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Bloque de concreto</t>
+          <t>Limpieza y desbroce</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -5158,17 +5158,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Paredes y tabiquería</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
+          <t>Limpieza y desbroce mecanizado del terreno.</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Limpieza y desbroce mecanizado del terreno mediante retroexcavadora o minicargadora, con retiro de maleza, arbustos, raíces y escombro superficial, hasta dejar la superficie despejada y groseramente nivelada. Rinde frente al desbroce manual a partir de superficies medianas y con acceso para maquinaria. Incluye el acordonamiento de la zona de trabajo, el barrido mecánico de la superficie, el amontonamiento del material retirado en el punto de acopio y el repaso manual de los bordes y esquinas donde no alcanza la máquina. No incluye el transporte del material sobrante a botadero, que se valora en el subcapítulo de transporte de tierras. Medido en superficie realmente desbrozada.</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -5180,11 +5180,11 @@
         <v>1</v>
       </c>
       <c r="F125" t="n">
-        <v>52.4</v>
+        <v>0.91</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Tabiquería de yeso laminado</t>
+          <t>Limpieza y desbroce</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -5196,17 +5196,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Frisos y revestimientos de pared</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+          <t>Descapote y retiro de capa vegetal.</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Descapote del terreno mediante retiro de la capa vegetal superficial, de unos 20 cm de espesor medio, hasta alcanzar el terreno firme apto para recibir fundaciones o rellenos. La capa vegetal es compresible y no admite carga, de modo que su retiro es condición previa a cualquier cimentación. Incluye el replanteo del área, la excavación de la capa con medios mecánicos o manuales según el acceso, su amontonamiento separado del resto del material por si el cliente desea reutilizarla en jardinería, y el perfilado de la superficie resultante. No incluye el transporte del material sobrante a botadero, que se valora en el subcapítulo de transporte de tierras. Medido en superficie realmente descapotada.</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -5218,11 +5218,11 @@
         <v>1</v>
       </c>
       <c r="F126" t="n">
-        <v>10.75</v>
+        <v>1.65</v>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Frisos y enlucidos de mortero</t>
+          <t>Limpieza y desbroce</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -5234,17 +5234,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Frisos y revestimientos de pared</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+          <t>Retiro de raíces y obstáculos menores enterrados.</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Retiro de raíces, restos de fundaciones antiguas, tuberías fuera de servicio y demás obstáculos menores que aparecen enterrados al despejar el terreno. Incluye la localización y descubrimiento del obstáculo, su extracción con medios manuales o con retroexcavadora según el tamaño, el corte con motosierra o amoladora cuando sea necesario fragmentarlo, el relleno y compactación del hueco resultante con material del sitio y la separación del material extraído según sea escombro, chatarra o vegetal. No incluye el transporte del material sobrante a botadero, que se valora en el subcapítulo de transporte de tierras. Medido en superficie de terreno realmente sondeada y liberada de obstáculos.</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -5256,11 +5256,11 @@
         <v>1</v>
       </c>
       <c r="F127" t="n">
-        <v>10.87</v>
+        <v>2.87</v>
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Enchapado cerámico y porcelanato</t>
+          <t>Limpieza y desbroce</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -5272,33 +5272,33 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+          <t>Excavación manual en zanja para fundaciones.</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+          <t>Excavación manual en zanja o pozo para fundaciones, en terreno de consistencia media, hasta la cota y con las dimensiones de proyecto. Es la solución habitual en obra de reforma y en ampliaciones donde no hay acceso para maquinaria o el volumen no la justifica. Incluye el replanteo de la zanja, la excavación con pico y pala por capas, el acopio del material a distancia suficiente del borde para no sobrecargarlo, el perfilado de paredes y fondo, y la extracción del material hasta el punto de carga. No incluye el transporte del material sobrante a botadero, que se valora en el subcapítulo de transporte de tierras. Medido en volumen teórico de excavación según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E128" t="n">
         <v>1</v>
       </c>
       <c r="F128" t="n">
-        <v>8.02</v>
+        <v>12.77</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Bases, contrapisos y nivelación</t>
+          <t>Excavaciones</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -5310,33 +5310,33 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+          <t>Excavación mecanizada en zanja para fundaciones.</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Excavación mecanizada en zanja o pozo para fundaciones mediante retroexcavadora, en terreno de consistencia media, hasta la cota y con las dimensiones de proyecto. Incluye el replanteo, la excavación con la máquina, el acopio del material a distancia suficiente del borde, el refine manual de paredes y fondo que la máquina no puede dar, y la vigilancia durante la excavación para detener los trabajos si aparecen instalaciones enterradas no previstas. No incluye el transporte del material sobrante a botadero, que se valora en el subcapítulo de transporte de tierras. Medido en volumen teórico de excavación según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E129" t="n">
         <v>1</v>
       </c>
       <c r="F129" t="n">
-        <v>9.17</v>
+        <v>7.38</v>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Pisos cerámicos y porcelanato</t>
+          <t>Excavaciones</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -5348,33 +5348,33 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+          <t>Excavación manual en zanja para instalaciones enterradas.</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Excavación manual en zanja de sección reducida para el tendido de tuberías de agua, desagüe o canalizaciones eléctricas enterradas, con la pendiente que exija la instalación. Se ejecuta a mano precisamente porque en zonas construidas el riesgo de romper una instalación existente hace desaconsejable la máquina. Incluye el replanteo del trazado, la excavación por capas con vigilancia continua, el acopio del material junto a la zanja, el perfilado del fondo con la pendiente requerida y el mantenimiento de la zanja señalizada mientras permanezca abierta. No incluye el transporte del material sobrante a botadero, que se valora en el subcapítulo de transporte de tierras. Medido en volumen teórico de excavación según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E130" t="n">
         <v>1</v>
       </c>
       <c r="F130" t="n">
-        <v>12.51</v>
+        <v>12.32</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Pisos cerámicos y porcelanato</t>
+          <t>Excavaciones</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -5386,33 +5386,33 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+          <t>Excavación mecanizada a cielo abierto.</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+          <t>Excavación mecanizada a cielo abierto para vaciado general, rebaje de cota o formación de plataforma, mediante retroexcavadora o minicargadora, en terreno de consistencia media. Incluye el replanteo y marcado de la cota final, la excavación por tongadas, el acopio del material en obra o su carga directa sobre camión, el refine manual de los bordes y taludes, y el control topográfico de la cota alcanzada. No incluye el transporte del material sobrante a botadero, que se valora en el subcapítulo de transporte de tierras. Medido en volumen teórico de excavación según las cotas de proyecto.</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E131" t="n">
         <v>1</v>
       </c>
       <c r="F131" t="n">
-        <v>1.69</v>
+        <v>5.19</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Rodapiés y remates de piso</t>
+          <t>Excavaciones</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -5424,33 +5424,33 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Cielos rasos</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+          <t>Excavación en material duro o roca.</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+          <t>Excavación en terreno de alta compacidad, material cementado o roca, mediante martillo hidráulico montado sobre retroexcavadora, con apoyo de martillo neumático manual en los rincones. Se aplica cuando el rendimiento de la excavación convencional cae por debajo de lo aceptable, circunstancia que debe dejarse acreditada en obra para justificar el cambio de partida. Incluye el fracturado del material, su extracción y acopio, el refine de paredes y fondo, y el control de las vibraciones cuando existan edificaciones colindantes. No incluye el transporte del material sobrante a botadero, que se valora en el subcapítulo de transporte de tierras. Medido en volumen teórico de excavación según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E132" t="n">
         <v>1</v>
       </c>
       <c r="F132" t="n">
-        <v>18.47</v>
+        <v>30.21</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Yeso laminado continuo</t>
+          <t>Excavaciones</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -5462,33 +5462,33 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+          <t>Excavación para tanque séptico, sumidero o tanque enterrado.</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+          <t>Excavación para el alojamiento de tanque séptico, sumidero, tanque de agua enterrado o similar, con las dimensiones de proyecto más el sobreancho de trabajo necesario para el montaje y el posterior relleno perimetral. Incluye el replanteo, la excavación con medios mecánicos y refine manual, el perfilado del fondo a la cota exacta de apoyo, la comprobación de la estabilidad de las paredes y su entibado si la profundidad lo exige, y la señalización y cubrición del hueco mientras permanezca abierto. No incluye el transporte del material sobrante a botadero, que se valora en el subcapítulo de transporte de tierras. Medido en volumen teórico de excavación según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E133" t="n">
         <v>1</v>
       </c>
       <c r="F133" t="n">
-        <v>7.45</v>
+        <v>11.95</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Tuberías y montantes de agua</t>
+          <t>Excavaciones</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -5500,33 +5500,33 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+          <t>Entibado de zanja con madera.</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+          <t>Entibado de las paredes de zanja mediante tablones y puntales de madera, para sostener el terreno y permitir el trabajo seguro en el interior. Es obligatorio a partir de la profundidad en que el terreno deja de ser autoestable, y su ausencia es la causa principal de los accidentes graves en zanja. Incluye el montaje del entibado conforme avanza la excavación y nunca después, la colocación de tablones y puntales con el apriete necesario, la revisión diaria del conjunto y tras cada lluvia, y el desmontaje escalonado a medida que se ejecuta el relleno. Medido en superficie de pared de zanja realmente entibada.</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E134" t="n">
         <v>1</v>
       </c>
       <c r="F134" t="n">
-        <v>37.22</v>
+        <v>8.83</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>Puntos de agua</t>
+          <t>Excavaciones</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -5538,33 +5538,33 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+          <t>Perfilado y compactación del fondo de excavación.</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+          <t>Perfilado, refine y compactación del fondo de la excavación hasta dejarlo a la cota exacta, plano y con la densidad requerida para recibir la fundación o la base del pavimento. Incluye la retirada del material suelto y descomprimido del fondo, el refine manual hasta la cota de proyecto, la humectación del terreno hasta la humedad óptima y la compactación con plancha vibratoria o compactador de impacto según el ancho disponible. Medido en superficie de fondo realmente perfilada.</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E135" t="n">
         <v>1</v>
       </c>
       <c r="F135" t="n">
-        <v>13.52</v>
+        <v>1.1</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>Llaves y valvulería</t>
+          <t>Excavaciones</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -5576,33 +5576,33 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+          <t>Achicamiento de agua en excavación.</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+          <t>Agotamiento del agua acumulada en la excavación mediante bomba sumergible con manguera de descarga a punto autorizado, para permitir el trabajo en seco. Se aplica cuando aparece nivel freático, filtraciones o agua de lluvia acumulada. Incluye el emplazamiento de la bomba en el punto bajo, el tendido de la manguera de descarga a un punto donde el vertido no erosione ni inunde otras zonas, la vigilancia del funcionamiento, la limpieza periódica del filtro de aspiración y el retiro del equipo. Medido por hora de funcionamiento efectivo del equipo.</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="E136" t="n">
         <v>1</v>
       </c>
       <c r="F136" t="n">
-        <v>23.45</v>
+        <v>4.3</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Excavaciones</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -5614,33 +5614,33 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Instalación de lavamanos con su grifería y desagüe.</t>
+          <t>Relleno y compactación con material del sitio.</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
+          <t>Relleno de zanjas, trasdós de muros o rebajes con el propio material procedente de la excavación, siempre que sea apto por no contener materia orgánica ni elementos compresibles, extendido y compactado en capas de 20 cm de espesor máximo. Incluye la selección y cribado grosero del material acopiado, su extendido por tongadas, la humectación hasta la humedad óptima, la compactación de cada capa con compactador de impacto o plancha vibratoria según el espacio, y la comprobación del nivel final. Medido en volumen de relleno compactado según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E137" t="n">
         <v>1</v>
       </c>
       <c r="F137" t="n">
-        <v>36.45</v>
+        <v>5.37</v>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Rellenos y compactación</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -5652,33 +5652,33 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+          <t>Relleno y compactación con material granular de préstamo.</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+          <t>Relleno con material granular seleccionado de préstamo, tipo granzón natural, extendido y compactado en capas de 20 cm de espesor máximo, empleado cuando el material del sitio no reúne las condiciones exigidas. Incluye el suministro y puesta en obra del material, su extendido por tongadas, la humectación hasta la humedad óptima, la compactación de cada capa hasta alcanzar la densidad especificada y el control del nivel final. Medido en volumen de relleno compactado según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E138" t="n">
         <v>1</v>
       </c>
       <c r="F138" t="n">
-        <v>11.04</v>
+        <v>34.71</v>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Tuberías y bajantes de desagüe</t>
+          <t>Rellenos y compactación</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -5690,33 +5690,33 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Punto de desagüe para aparato sanitario.</t>
+          <t>Relleno de zanja de instalaciones con arena.</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+          <t>Relleno de zanja de instalaciones con arena lavada, formando la cama de asiento bajo la tubería y el recubrimiento envolvente hasta 20 cm por encima de su generatriz superior, para protegerla de cargas puntuales y del contacto con material grueso. Incluye el suministro y puesta en obra de la arena, la formación de la cama con la pendiente de la instalación, el relleno lateral y superior por capas con compactación manual cuidadosa para no desplazar ni dañar la tubería, y la colocación de la cinta de señalización sobre el recubrimiento. Medido en volumen de arena realmente colocada.</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E139" t="n">
         <v>1</v>
       </c>
       <c r="F139" t="n">
-        <v>33.84</v>
+        <v>39.23</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>Puntos de desagüe</t>
+          <t>Rellenos y compactación</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -5728,33 +5728,33 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Instalaciones eléctricas</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+          <t>Base de piedra picada compactada.</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+          <t>Base de piedra picada extendida y compactada bajo pisos, aceras o pavimentos exteriores, con función de capa drenante y de reparto de cargas, y de rotura del ascenso capilar de humedad hacia el piso. Incluye el suministro y puesta en obra de la piedra, su extendido por tongadas de 15 cm, el acuñado con material fino cuando se requiera cerrar la superficie, la compactación con plancha vibratoria y la comprobación del nivel y la planitud finales. Medido en volumen de base compactada según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E140" t="n">
         <v>1</v>
       </c>
       <c r="F140" t="n">
-        <v>8.369999999999999</v>
+        <v>45.36</v>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>Canalizaciones y cableado</t>
+          <t>Rellenos y compactación</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -5766,33 +5766,33 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Instalaciones eléctricas</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+          <t>Nivelación y compactación de terreno.</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+          <t>Nivelación y compactación de la superficie del terreno tras el desbroce o el relleno, hasta dejarla a la cota y con la pendiente de proyecto y con la densidad necesaria para recibir la capa siguiente. Incluye el repaso de la superficie con retirada de los puntos altos y aporte en los bajos, la humectación hasta la humedad óptima, la compactación con plancha vibratoria en pasadas cruzadas y la comprobación de cotas y pendientes con nivel láser. Medido en superficie realmente nivelada y compactada.</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E141" t="n">
         <v>1</v>
       </c>
       <c r="F141" t="n">
-        <v>8.720000000000001</v>
+        <v>1.22</v>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Puntos, mecanismos y tomas</t>
+          <t>Rellenos y compactación</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
@@ -5804,33 +5804,33 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+          <t>Carga manual y transporte de tierra sobrante a botadero.</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Carga manual del material sobrante de excavación sobre camión volqueta y transporte a botadero autorizado, incluido el canon de vertido, con una distancia media considerada de 25 km. Se emplea cuando el acopio es inaccesible para la maquinaria de carga. Incluye la carga a pala sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado, la descarga y la limpieza de la zona de carga. Medido en volumen de material esponjado realmente retirado.</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E142" t="n">
         <v>1</v>
       </c>
       <c r="F142" t="n">
-        <v>2.82</v>
+        <v>14.17</v>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Preparación de soportes</t>
+          <t>Transporte de tierras</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -5842,33 +5842,33 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+          <t>Carga mecanizada y transporte de tierra sobrante a botadero.</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Carga mecanizada del material sobrante de excavación con retroexcavadora sobre camión volqueta y transporte a botadero autorizado, incluido el canon de vertido, con una distancia media considerada de 25 km. Incluye la carga con la máquina, el amarre y cubrición de la carga, el traslado, la descarga, el repaso manual del acopio residual y la limpieza de la zona de carga. Medido en volumen de material esponjado realmente retirado.</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E143" t="n">
         <v>1</v>
       </c>
       <c r="F143" t="n">
-        <v>3.46</v>
+        <v>12.22</v>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Pintura interior</t>
+          <t>Transporte de tierras</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -5880,33 +5880,33 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Movimiento de tierras</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+          <t>Acopio provisional de tierra en obra para su reutilización.</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+          <t>Traslado interno y acopio provisional en obra del material de excavación apto para ser reutilizado en los rellenos posteriores, evitando el doble coste de botarlo y luego comprar material de préstamo. Incluye el traslado del material al punto de acopio, su amontonamiento con talud estable y alejado de los bordes de excavación, su cubrición con lámina plástica para evitar el lavado por lluvia y el aumento de humedad, y su posterior recuperación para el relleno. Medido en volumen de material realmente acopiado.</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E144" t="n">
         <v>1</v>
       </c>
       <c r="F144" t="n">
-        <v>5.23</v>
+        <v>3.44</v>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Esmaltes sobre madera y metal</t>
+          <t>Transporte de tierras</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -5918,36 +5918,872 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
+          <t>Movimiento de tierras</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Suministro y transporte de material de préstamo a obra.</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>Suministro de material granular de préstamo desde cantera o proveedor autorizado y su transporte y descarga en obra, en el punto de acopio indicado. Incluye la comprobación de la granulometría y la limpieza del material a la llegada, el rechazo de la carga si no cumple, la descarga en el punto acordado y el registro de los volúmenes recibidos por vale de entrega. Medido en volumen de material realmente recibido en obra.</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>1</v>
+      </c>
+      <c r="F145" t="n">
+        <v>28.35</v>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Transporte de tierras</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Paredes y tabiquería</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Tabique de bloque de concreto de 10 cm, recibido con mortero de pega.</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Tabique interior no estructural de 10 cm de espesor, ejecutado con bloque hueco de concreto de 10x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Incluye replanteo y trazado sobre el piso, colocación de hiladas a nivel y plomo con la ayuda de reglas y cuerda, formación de huecos de paso, anclaje del tabique a los paramentos existentes, humedecido previo de las piezas y limpieza de restos. No incluye el friso ni los dinteles de los huecos, que se valoran aparte. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>1</v>
+      </c>
+      <c r="F146" t="n">
+        <v>18.29</v>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Bloque de concreto</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Paredes y tabiquería</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>1</v>
+      </c>
+      <c r="F147" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Tabiquería de yeso laminado</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Frisos y revestimientos de pared</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>1</v>
+      </c>
+      <c r="F148" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Frisos y enlucidos de mortero</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Frisos y revestimientos de pared</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>1</v>
+      </c>
+      <c r="F149" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Enchapado cerámico y porcelanato</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>1</v>
+      </c>
+      <c r="F150" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Bases, contrapisos y nivelación</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>1</v>
+      </c>
+      <c r="F151" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Pisos cerámicos y porcelanato</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>1</v>
+      </c>
+      <c r="F152" t="n">
+        <v>12.51</v>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Pisos cerámicos y porcelanato</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>1</v>
+      </c>
+      <c r="F153" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Rodapiés y remates de piso</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Cielos rasos</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>1</v>
+      </c>
+      <c r="F154" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Yeso laminado continuo</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>1</v>
+      </c>
+      <c r="F155" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Tuberías y montantes de agua</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>1</v>
+      </c>
+      <c r="F156" t="n">
+        <v>37.22</v>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Puntos de agua</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>1</v>
+      </c>
+      <c r="F157" t="n">
+        <v>13.52</v>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Llaves y valvulería</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>1</v>
+      </c>
+      <c r="F158" t="n">
+        <v>23.45</v>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Instalación de lavamanos con su grifería y desagüe.</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>1</v>
+      </c>
+      <c r="F159" t="n">
+        <v>36.45</v>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>1</v>
+      </c>
+      <c r="F160" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Tuberías y bajantes de desagüe</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Punto de desagüe para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>1</v>
+      </c>
+      <c r="F161" t="n">
+        <v>33.84</v>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Puntos de desagüe</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>1</v>
+      </c>
+      <c r="F162" t="n">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Canalizaciones y cableado</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>1</v>
+      </c>
+      <c r="F163" t="n">
+        <v>8.720000000000001</v>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Puntos, mecanismos y tomas</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E164" t="n">
+        <v>1</v>
+      </c>
+      <c r="F164" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>Preparación de soportes</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>1</v>
+      </c>
+      <c r="F165" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Pintura interior</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E166" t="n">
+        <v>1</v>
+      </c>
+      <c r="F166" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Esmaltes sobre madera y metal</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
           <t>Gestión de residuos y limpieza</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr">
+      <c r="B167" t="inlineStr">
         <is>
           <t>Retirada y transporte de escombro a vertedero autorizado.</t>
         </is>
       </c>
-      <c r="C145" s="2" t="inlineStr">
+      <c r="C167" s="2" t="inlineStr">
         <is>
           <t>Retirada de escombro procedente de demoliciones desde el punto de acopio de la obra y transporte en camión volqueta hasta vertedero o botadero autorizado, incluido el canon de vertido. Incluye la carga manual del escombro sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado con una distancia media considerada de 25 km, la descarga y la limpieza de la zona de carga. Medido por metro cúbico de escombro esponjado realmente retirado.</t>
         </is>
       </c>
-      <c r="D145" t="inlineStr">
+      <c r="D167" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="E145" t="n">
-        <v>1</v>
-      </c>
-      <c r="F145" t="n">
+      <c r="E167" t="n">
+        <v>1</v>
+      </c>
+      <c r="F167" t="n">
         <v>16.07</v>
       </c>
-      <c r="G145" t="inlineStr">
+      <c r="G167" t="inlineStr">
         <is>
           <t>Retiro y transporte de escombro</t>
         </is>
       </c>
-      <c r="H145" t="inlineStr">
+      <c r="H167" t="inlineStr">
         <is>
           <t>incluida</t>
         </is>

</xml_diff>

<commit_message>
Cerrar el capitulo 04 Fundaciones con 25 partidas en 5 subcapitulos
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/catalogo_partidas.xlsx
+++ b/basedatos_partidas/salida/catalogo_partidas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H167"/>
+  <dimension ref="A1:H192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5956,17 +5956,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Paredes y tabiquería</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Tabique de bloque de concreto de 10 cm, recibido con mortero de pega.</t>
+          <t>Concreto pobre de limpieza bajo fundaciones, 5 cm de espesor.</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>Tabique interior no estructural de 10 cm de espesor, ejecutado con bloque hueco de concreto de 10x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Incluye replanteo y trazado sobre el piso, colocación de hiladas a nivel y plomo con la ayuda de reglas y cuerda, formación de huecos de paso, anclaje del tabique a los paramentos existentes, humedecido previo de las piezas y limpieza de restos. No incluye el friso ni los dinteles de los huecos, que se valoran aparte. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Capa de concreto pobre de limpieza de 5 cm de espesor medio, vaciada sobre el fondo de excavación antes de armar la fundación. Cumple una función que no es estructural sino de ejecución: aísla el acero del terreno, evita que la tierra contamine el concreto estructural y proporciona una superficie limpia y a nivel donde replantear y apoyar los separadores. Incluye el repaso y compactación del fondo, el vaciado y extendido del concreto, su reglado a nivel y el marcado de los ejes de la fundación sobre la capa endurecida. Medido en superficie realmente ejecutada.</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -5978,11 +5978,11 @@
         <v>1</v>
       </c>
       <c r="F146" t="n">
-        <v>18.29</v>
+        <v>8.41</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Bloque de concreto</t>
+          <t>Bases y zapatas</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
@@ -5994,33 +5994,33 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Paredes y tabiquería</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
+          <t>Acero de refuerzo en zapatas y bases.</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Suministro, corte, doblado, armado y colocación de acero de refuerzo en cabillas corrugadas de límite elástico 4.200 kg/cm2 en zapatas y bases de fundación, según los planos de despiece. Incluye el corte y doblado en obra o el recibo del acero ya elaborado, el armado de las parrillas con amarre de alambre en todos los cruces del perímetro y alternos en el interior, la colocación de separadores para garantizar el recubrimiento especificado por todas las caras, el arriostramiento del armado para que no se desplace durante el vaciado y la revisión del despiece antes de autorizar el concreto. Medido en peso de acero realmente colocado, sin incluir despuntes ni solapes no previstos en el despiece.</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E147" t="n">
         <v>1</v>
       </c>
       <c r="F147" t="n">
-        <v>52.4</v>
+        <v>2.3</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Tabiquería de yeso laminado</t>
+          <t>Bases y zapatas</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
@@ -6032,17 +6032,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Frisos y revestimientos de pared</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+          <t>Encofrado y desencofrado de zapata.</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Encofrado de las caras laterales de zapata mediante paneles de madera con sus puntales y arriostramientos, y su posterior desencofrado. Incluye el replanteo y montaje de los paneles, la comprobación de escuadras, plomos y dimensiones antes del vaciado, el apuntalamiento y arriostramiento que impide la apertura del encofrado por el empuje del concreto fresco, la aplicación de desmoldeante, el desencofrado cuidadoso una vez alcanzada la resistencia necesaria, y la limpieza y acopio de los paneles para su reutilización. Medido en superficie de encofrado en contacto con el concreto.</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -6054,11 +6054,11 @@
         <v>1</v>
       </c>
       <c r="F148" t="n">
-        <v>10.75</v>
+        <v>13.77</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Frisos y enlucidos de mortero</t>
+          <t>Bases y zapatas</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
@@ -6070,33 +6070,33 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Frisos y revestimientos de pared</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+          <t>Concreto para zapata aislada.</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Concreto premezclado de resistencia 210 kg/cm2 vaciado en zapata aislada, incluida su compactación por vibrado y su curado. Incluye la revisión previa del armado, del encofrado y del recubrimiento, la recepción y comprobación del concreto a la llegada con rechazo de la carga si no cumple el asentamiento, el vaciado por capas evitando la segregación, la compactación con vibrador de aguja sin tocar el armado ni el encofrado, el reglado de la cara superior, el curado durante los primeros días y la toma de probetas cuando el control de calidad lo exija. Medido en volumen teórico según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E149" t="n">
         <v>1</v>
       </c>
       <c r="F149" t="n">
-        <v>10.87</v>
+        <v>167.7</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Enchapado cerámico y porcelanato</t>
+          <t>Bases y zapatas</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
@@ -6108,33 +6108,33 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+          <t>Concreto para zapata corrida.</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+          <t>Concreto premezclado de resistencia 210 kg/cm2 vaciado en zapata corrida bajo muro o hilera de columnas, incluida su compactación por vibrado y su curado. El vaciado en zanja continua rinde algo mejor que el de zapatas aisladas por la continuidad del frente de trabajo. Incluye la revisión previa del armado y del recubrimiento, la recepción y comprobación del concreto, el vaciado por capas, la compactación con vibrador de aguja, el reglado de la cara superior a la cota prevista y el curado durante los primeros días. Medido en volumen teórico según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E150" t="n">
         <v>1</v>
       </c>
       <c r="F150" t="n">
-        <v>8.02</v>
+        <v>166.6</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Bases, contrapisos y nivelación</t>
+          <t>Bases y zapatas</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -6146,33 +6146,33 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+          <t>Pedestal de concreto armado sobre fundación.</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Pedestal de concreto armado de resistencia 210 kg/cm2 que arranca de la zapata y eleva el apoyo de la columna hasta la cota de arranque, incluidos su encofrado, su vaciado y su curado. Incluye el replanteo sobre la zapata, el montaje y aplomado del encofrado con arriostramiento en las cuatro caras, la comprobación de que las cabillas de espera quedan en su posición y con la longitud de solape prevista, el vaciado y vibrado por capas, el desencofrado y el curado. No incluye el acero de refuerzo, que se valora por su peso. Medido en volumen teórico según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E151" t="n">
         <v>1</v>
       </c>
       <c r="F151" t="n">
-        <v>9.17</v>
+        <v>243.11</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Pisos cerámicos y porcelanato</t>
+          <t>Bases y zapatas</t>
         </is>
       </c>
       <c r="H151" t="inlineStr">
@@ -6184,33 +6184,33 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+          <t>Acero de refuerzo en vigas de riostra.</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Suministro, corte, doblado, armado y colocación de acero de refuerzo en cabillas corrugadas en vigas de riostra, según los planos de despiece. El armado de viga exige más tiempo por kilogramo que el de zapata por el montaje de los estribos y por el trabajo en zanja estrecha. Incluye el corte y doblado de barras y estribos, el armado de la canasta con la separación de estribos indicada y su reducción en las zonas de confinamiento junto a los apoyos, el amarre con alambre, la colocación de separadores por las cuatro caras, el anclaje o solape con las esperas de las zapatas y la revisión del despiece antes del vaciado. Medido en peso de acero realmente colocado.</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E152" t="n">
         <v>1</v>
       </c>
       <c r="F152" t="n">
-        <v>12.51</v>
+        <v>2.39</v>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>Pisos cerámicos y porcelanato</t>
+          <t>Vigas de riostra</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
@@ -6222,33 +6222,33 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+          <t>Encofrado y desencofrado de viga de riostra.</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+          <t>Encofrado de las caras laterales de viga de riostra mediante paneles de madera con puntales y arriostramientos, y su posterior desencofrado. Incluye el replanteo y montaje de los paneles, la comprobación de alineación, plomo y sección antes del vaciado, el arriostramiento que impide la apertura por el empuje del concreto, la aplicación de desmoldeante, el desencofrado una vez alcanzada la resistencia necesaria y la limpieza y acopio de los paneles para su reutilización. Medido en superficie de encofrado en contacto con el concreto.</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E153" t="n">
         <v>1</v>
       </c>
       <c r="F153" t="n">
-        <v>1.69</v>
+        <v>14.29</v>
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>Rodapiés y remates de piso</t>
+          <t>Vigas de riostra</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
@@ -6260,33 +6260,33 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Cielos rasos</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+          <t>Concreto para viga de riostra.</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+          <t>Concreto premezclado de resistencia 210 kg/cm2 vaciado en viga de riostra, incluida su compactación por vibrado y su curado. La viga de riostra ata las fundaciones entre sí y es la que absorbe los asientos diferenciales, por lo que su continuidad y la correcta ejecución de los nudos con las zapatas son determinantes. Incluye la revisión previa del armado y del recubrimiento, la recepción del concreto, el vaciado continuo evitando juntas frías en los nudos, la compactación con vibrador de aguja, el reglado de la cara superior y el curado. Medido en volumen teórico según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E154" t="n">
         <v>1</v>
       </c>
       <c r="F154" t="n">
-        <v>18.47</v>
+        <v>171.91</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>Yeso laminado continuo</t>
+          <t>Vigas de riostra</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
@@ -6298,33 +6298,33 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+          <t>Barrera de vapor de polietileno bajo losa de fundación.</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+          <t>Colocación de lámina de polietileno de alta densidad sobre la base compactada, como barrera de vapor que impide el ascenso capilar de humedad desde el terreno hacia la losa y el piso terminado. Es una capa barata cuya omisión provoca humedades permanentes en el piso, imposibles de corregir después sin demoler. Incluye la comprobación de que la base no presenta aristas que puedan perforar la lámina, el extendido con solapes de 20 cm sellados con cinta, el remonte en el perímetro hasta la cota superior de la losa y la reparación de cualquier perforación producida durante el armado. Medido en superficie realmente cubierta.</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E155" t="n">
         <v>1</v>
       </c>
       <c r="F155" t="n">
-        <v>7.45</v>
+        <v>1.29</v>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>Tuberías y montantes de agua</t>
+          <t>Losas de fundación</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
@@ -6336,33 +6336,33 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+          <t>Acero de refuerzo en losa de fundación.</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+          <t>Suministro, corte, doblado, armado y colocación de acero de refuerzo en cabillas corrugadas en losa de fundación, en parrillas inferior y superior según los planos de despiece. Incluye el corte y doblado, el armado de las parrillas con amarre de alambre, la colocación de separadores inferiores y de caballetes o soportes que mantienen la parrilla superior en su cota durante el vaciado, los refuerzos de borde y de esquina, y la revisión del despiece y del recubrimiento antes de autorizar el concreto. Medido en peso de acero realmente colocado.</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E156" t="n">
         <v>1</v>
       </c>
       <c r="F156" t="n">
-        <v>37.22</v>
+        <v>2.27</v>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>Puntos de agua</t>
+          <t>Losas de fundación</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
@@ -6374,33 +6374,33 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+          <t>Malla electrosoldada de refuerzo en losa.</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+          <t>Suministro y colocación de malla electrosoldada de acero como refuerzo de losa, sobre separadores que garantizan su posición dentro del espesor. Incluye el replanteo, el corte de los paños, su colocación con los solapes mínimos de dos retículas amarrados con alambre, la colocación de separadores y caballetes, y el repaso de la posición de la malla inmediatamente antes del vaciado, ya que es habitual que quede pisada y apoyada en el fondo, con lo que pierde por completo su función. Medido en superficie realmente reforzada.</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E157" t="n">
         <v>1</v>
       </c>
       <c r="F157" t="n">
-        <v>13.52</v>
+        <v>7.37</v>
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Llaves y valvulería</t>
+          <t>Losas de fundación</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -6412,33 +6412,33 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+          <t>Encofrado perimetral de losa de fundación.</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+          <t>Encofrado del borde perimetral de losa de fundación mediante tablones de madera con estacas y arriostramiento, y su posterior desencofrado. Incluye el replanteo del perímetro, el montaje de los tablones a la cota exacta de la cara superior de la losa, su fijación y arriostramiento contra el empuje del concreto, la aplicación de desmoldeante, el desencofrado y la limpieza y acopio del material. Medido en superficie de encofrado en contacto con el concreto.</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E158" t="n">
         <v>1</v>
       </c>
       <c r="F158" t="n">
-        <v>23.45</v>
+        <v>14.11</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Losas de fundación</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
@@ -6450,33 +6450,33 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Instalación de lavamanos con su grifería y desagüe.</t>
+          <t>Concreto para losa de fundación.</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
+          <t>Concreto premezclado de resistencia 250 kg/cm2 vaciado en losa de fundación, incluida su compactación por vibrado. Incluye la revisión previa del armado, de los separadores y de la barrera de vapor, la recepción y comprobación del concreto, el vaciado continuo por franjas evitando las juntas frías, la compactación con vibrador de aguja, el reglado a la cota mediante maestras y el sangrado del agua de exudación antes del acabado. No incluye el acabado superficial ni el curado, que se valoran en la partida siguiente. Medido en volumen teórico según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E159" t="n">
         <v>1</v>
       </c>
       <c r="F159" t="n">
-        <v>36.45</v>
+        <v>182.77</v>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Losas de fundación</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
@@ -6488,33 +6488,33 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+          <t>Acabado y curado de losa de fundación.</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+          <t>Acabado superficial de la losa mediante alisado mecánico y su curado posterior. Incluye el reglado y flotado inicial, el alisado con alisadora mecánica en las pasadas necesarias hasta obtener la textura requerida según vaya a recibir un piso adherido o quedar visto, el aserrado de las juntas de retracción en el momento adecuado, y el curado mediante curador de membrana o riego continuo durante los primeros días, sin el cual la losa fisura por retracción plástica por muy bien vaciada que esté. Medido en superficie realmente acabada.</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E160" t="n">
         <v>1</v>
       </c>
       <c r="F160" t="n">
-        <v>11.04</v>
+        <v>2.48</v>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>Tuberías y bajantes de desagüe</t>
+          <t>Losas de fundación</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
@@ -6526,33 +6526,33 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Punto de desagüe para aparato sanitario.</t>
+          <t>Encofrado a dos caras de muro de contención.</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+          <t>Encofrado a dos caras de muro de contención mediante paneles de madera con sus tirantes pasantes, puntales y arriostramientos, y su posterior desencofrado. Incluye el replanteo, el montaje y aplomado de la primera cara, la colocación de los tirantes y separadores que fijan el espesor, el cierre de la segunda cara tras la revisión del armado, el arriostramiento frente al empuje del concreto fresco que en un muro alto es considerable, la aplicación de desmoldeante, el desencofrado y el sellado de los agujeros de los tirantes. Medido en superficie de encofrado en contacto con el concreto, contando ambas caras.</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E161" t="n">
         <v>1</v>
       </c>
       <c r="F161" t="n">
-        <v>33.84</v>
+        <v>16.43</v>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Puntos de desagüe</t>
+          <t>Muros de contención</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
@@ -6564,33 +6564,33 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Instalaciones eléctricas</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+          <t>Acero de refuerzo en muro de contención.</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+          <t>Suministro, corte, doblado, armado y colocación de acero de refuerzo en cabillas corrugadas en muro de contención, según los planos de despiece. Incluye el corte y doblado, el armado de las dos parrillas verticales con sus ganchos de arranque solapados a las esperas de la fundación, el amarre con alambre, la colocación de separadores en ambas caras para garantizar el recubrimiento, los refuerzos de borde y de esquina, y la comprobación de que la parrilla del lado del terreno queda en la cara traccionada correcta, error frecuente y de consecuencias graves. Medido en peso de acero realmente colocado.</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E162" t="n">
         <v>1</v>
       </c>
       <c r="F162" t="n">
-        <v>8.369999999999999</v>
+        <v>2.37</v>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>Canalizaciones y cableado</t>
+          <t>Muros de contención</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -6602,33 +6602,33 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Instalaciones eléctricas</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+          <t>Concreto para muro de contención.</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+          <t>Concreto premezclado de resistencia 250 kg/cm2 vaciado en muro de contención, incluida su compactación por vibrado y su curado. Incluye la revisión previa del armado, del encofrado y de los recubrimientos, la recepción del concreto, el vaciado por capas de altura limitada y por puntos alternos para no descuadrar el encofrado, el uso de tubo de descarga cuando la altura de caída pueda provocar segregación, la compactación con vibrador de aguja en cada capa, el curado prolongado y el desencofrado una vez alcanzada la resistencia. Medido en volumen teórico según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E163" t="n">
         <v>1</v>
       </c>
       <c r="F163" t="n">
-        <v>8.720000000000001</v>
+        <v>191.39</v>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>Puntos, mecanismos y tomas</t>
+          <t>Muros de contención</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
@@ -6640,17 +6640,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+          <t>Impermeabilización del trasdós de muro de contención.</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Impermeabilización de la cara del muro en contacto con el terreno mediante imprimación y dos manos de emulsión asfáltica, con protección posterior. Es la única oportunidad de ejecutarla: una vez rellenado el trasdós, corregir una filtración obliga a excavar de nuevo. Incluye la limpieza y el repaso de la superficie con eliminación de rebabas y coqueras, la reparación de los agujeros de los tirantes del encofrado, la aplicación de la imprimación, las dos manos de emulsión asfáltica con especial cuidado en el encuentro con la fundación, y la colocación de la lámina de protección antes del relleno. Medido en superficie realmente impermeabilizada.</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -6662,11 +6662,11 @@
         <v>1</v>
       </c>
       <c r="F164" t="n">
-        <v>2.82</v>
+        <v>11.62</v>
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>Preparación de soportes</t>
+          <t>Muros de contención</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
@@ -6678,33 +6678,33 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+          <t>Drenaje de trasdós de muro con tubería y grava.</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Drenaje longitudinal en la base del trasdós del muro, formado por tubería corrugada perforada envuelta en geotextil y capa de piedra picada de relleno drenante, con salida a punto de evacuación. Su función es eliminar el empuje hidrostático sobre el muro, que es la causa más común del fallo de los muros de contención, mucho más que el empuje de tierras. Incluye la formación del asiento con pendiente hacia la salida, la colocación del geotextil envolvente, el tendido de la tubería, el relleno con piedra picada, el cierre del geotextil y la conexión a la salida de evacuación. Medido en longitud realmente ejecutada.</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E165" t="n">
         <v>1</v>
       </c>
       <c r="F165" t="n">
-        <v>3.46</v>
+        <v>21.94</v>
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>Pintura interior</t>
+          <t>Muros de contención</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -6716,33 +6716,33 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Fundaciones</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+          <t>Perforación para pilote vaciado en sitio.</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+          <t>Perforación rotatoria para pilote vaciado en sitio, en terreno de consistencia media, con equipo de perforación y su operador. Incluye el traslado y emplazamiento del equipo, el replanteo y centrado sobre el eje del pilote, la perforación hasta la cota de proyecto con control de la verticalidad, la extracción y acopio del material perforado, la limpieza del fondo de la perforación antes de introducir el armado y la protección o entubado provisional de la boca para evitar desprendimientos. Medido en longitud realmente perforada.</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E166" t="n">
         <v>1</v>
       </c>
       <c r="F166" t="n">
-        <v>5.23</v>
+        <v>21.85</v>
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>Esmaltes sobre madera y metal</t>
+          <t>Pilotes y fundaciones profundas</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
@@ -6754,36 +6754,986 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
+          <t>Fundaciones</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Acero de refuerzo en pilote.</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>Suministro, corte, doblado, armado y colocación de la canasta de acero de refuerzo del pilote, con sus barras longitudinales y su zuncho helicoidal. Incluye el armado de la canasta en superficie, la colocación de separadores circulares que centran la canasta dentro de la perforación y garantizan el recubrimiento, el izado y descenso controlado de la canasta dentro del pilote sin que roce las paredes y arrastre tierra, su suspensión a la cota correcta durante el vaciado y la disposición de las esperas de conexión con el cabezal. Medido en peso de acero realmente colocado.</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E167" t="n">
+        <v>1</v>
+      </c>
+      <c r="F167" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Pilotes y fundaciones profundas</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Fundaciones</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Concreto para pilote vaciado en sitio.</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>Concreto premezclado de resistencia 250 kg/cm2 vaciado en pilote perforado, colocado mediante tubo tremie o embudo con tubo de descarga. Incluye la comprobación de la limpieza del fondo y de la posición de la canasta, la recepción del concreto con la fluidez adecuada para un vaciado sin vibrado en toda la profundidad, el vaciado continuo desde el fondo hacia arriba sin interrupciones que provoquen discontinuidades, el control del volumen realmente colocado frente al teórico como indicador de posibles sobreanchos o pérdidas, y el rebose de la cabeza para desalojar el concreto contaminado. Medido en volumen teórico según el diámetro y la longitud de proyecto.</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E168" t="n">
+        <v>1</v>
+      </c>
+      <c r="F168" t="n">
+        <v>217.58</v>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Pilotes y fundaciones profundas</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Fundaciones</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Descabezado de pilote.</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>Demolición de la cabeza del pilote hasta la cota de proyecto, eliminando el concreto contaminado del rebose, y preparación de las esperas de acero para su conexión con el cabezal o la viga de atado. Incluye el marcado de la cota de corte, la demolición con martillo eléctrico sin dañar las barras de espera ni fisurar el concreto que permanece, el enderezado y limpieza de las esperas, el repicado de la superficie de contacto para dar adherencia al elemento superior y el retiro del escombro. Medido por pilote realmente descabezado.</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E169" t="n">
+        <v>1</v>
+      </c>
+      <c r="F169" t="n">
+        <v>26.64</v>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Pilotes y fundaciones profundas</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Fundaciones</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Cabezal de pilotes de concreto armado.</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>Cabezal de concreto armado de resistencia 250 kg/cm2 que recibe y reparte la carga de la columna entre el grupo de pilotes, incluidos su encofrado, su vaciado, su vibrado y su curado. Incluye el replanteo sobre las cabezas descabezadas, el montaje y arriostramiento del encofrado, la comprobación de que las esperas de los pilotes quedan embebidas con la longitud de anclaje prevista, el vaciado por capas con vibrado, el desencofrado y el curado. No incluye el acero de refuerzo, que se valora por su peso. Medido en volumen teórico según las dimensiones de proyecto.</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E170" t="n">
+        <v>1</v>
+      </c>
+      <c r="F170" t="n">
+        <v>231.7</v>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Pilotes y fundaciones profundas</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Paredes y tabiquería</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Tabique de bloque de concreto de 10 cm, recibido con mortero de pega.</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>Tabique interior no estructural de 10 cm de espesor, ejecutado con bloque hueco de concreto de 10x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Incluye replanteo y trazado sobre el piso, colocación de hiladas a nivel y plomo con la ayuda de reglas y cuerda, formación de huecos de paso, anclaje del tabique a los paramentos existentes, humedecido previo de las piezas y limpieza de restos. No incluye el friso ni los dinteles de los huecos, que se valoran aparte. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>1</v>
+      </c>
+      <c r="F171" t="n">
+        <v>18.29</v>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Bloque de concreto</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Paredes y tabiquería</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>1</v>
+      </c>
+      <c r="F172" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Tabiquería de yeso laminado</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Frisos y revestimientos de pared</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>1</v>
+      </c>
+      <c r="F173" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Frisos y enlucidos de mortero</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Frisos y revestimientos de pared</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>1</v>
+      </c>
+      <c r="F174" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Enchapado cerámico y porcelanato</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>1</v>
+      </c>
+      <c r="F175" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Bases, contrapisos y nivelación</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>1</v>
+      </c>
+      <c r="F176" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Pisos cerámicos y porcelanato</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>1</v>
+      </c>
+      <c r="F177" t="n">
+        <v>12.51</v>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Pisos cerámicos y porcelanato</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>1</v>
+      </c>
+      <c r="F178" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Rodapiés y remates de piso</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Cielos rasos</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E179" t="n">
+        <v>1</v>
+      </c>
+      <c r="F179" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Yeso laminado continuo</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E180" t="n">
+        <v>1</v>
+      </c>
+      <c r="F180" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Tuberías y montantes de agua</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E181" t="n">
+        <v>1</v>
+      </c>
+      <c r="F181" t="n">
+        <v>37.22</v>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Puntos de agua</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E182" t="n">
+        <v>1</v>
+      </c>
+      <c r="F182" t="n">
+        <v>13.52</v>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Llaves y valvulería</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E183" t="n">
+        <v>1</v>
+      </c>
+      <c r="F183" t="n">
+        <v>23.45</v>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Instalación de lavamanos con su grifería y desagüe.</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E184" t="n">
+        <v>1</v>
+      </c>
+      <c r="F184" t="n">
+        <v>36.45</v>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E185" t="n">
+        <v>1</v>
+      </c>
+      <c r="F185" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Tuberías y bajantes de desagüe</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Punto de desagüe para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C186" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E186" t="n">
+        <v>1</v>
+      </c>
+      <c r="F186" t="n">
+        <v>33.84</v>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Puntos de desagüe</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E187" t="n">
+        <v>1</v>
+      </c>
+      <c r="F187" t="n">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Canalizaciones y cableado</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+        </is>
+      </c>
+      <c r="C188" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E188" t="n">
+        <v>1</v>
+      </c>
+      <c r="F188" t="n">
+        <v>8.720000000000001</v>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Puntos, mecanismos y tomas</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+        </is>
+      </c>
+      <c r="C189" s="2" t="inlineStr">
+        <is>
+          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E189" t="n">
+        <v>1</v>
+      </c>
+      <c r="F189" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Preparación de soportes</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+        </is>
+      </c>
+      <c r="C190" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E190" t="n">
+        <v>1</v>
+      </c>
+      <c r="F190" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Pintura interior</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+        </is>
+      </c>
+      <c r="C191" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E191" t="n">
+        <v>1</v>
+      </c>
+      <c r="F191" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Esmaltes sobre madera y metal</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
           <t>Gestión de residuos y limpieza</t>
         </is>
       </c>
-      <c r="B167" t="inlineStr">
+      <c r="B192" t="inlineStr">
         <is>
           <t>Retirada y transporte de escombro a vertedero autorizado.</t>
         </is>
       </c>
-      <c r="C167" s="2" t="inlineStr">
+      <c r="C192" s="2" t="inlineStr">
         <is>
           <t>Retirada de escombro procedente de demoliciones desde el punto de acopio de la obra y transporte en camión volqueta hasta vertedero o botadero autorizado, incluido el canon de vertido. Incluye la carga manual del escombro sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado con una distancia media considerada de 25 km, la descarga y la limpieza de la zona de carga. Medido por metro cúbico de escombro esponjado realmente retirado.</t>
         </is>
       </c>
-      <c r="D167" t="inlineStr">
+      <c r="D192" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="E167" t="n">
-        <v>1</v>
-      </c>
-      <c r="F167" t="n">
+      <c r="E192" t="n">
+        <v>1</v>
+      </c>
+      <c r="F192" t="n">
         <v>16.07</v>
       </c>
-      <c r="G167" t="inlineStr">
+      <c r="G192" t="inlineStr">
         <is>
           <t>Retiro y transporte de escombro</t>
         </is>
       </c>
-      <c r="H167" t="inlineStr">
+      <c r="H192" t="inlineStr">
         <is>
           <t>incluida</t>
         </is>

</xml_diff>

<commit_message>
Cerrar el capitulo 05 Estructuras con 35 partidas en 6 subcapitulos
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/catalogo_partidas.xlsx
+++ b/basedatos_partidas/salida/catalogo_partidas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H192"/>
+  <dimension ref="A1:H227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6906,33 +6906,33 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Paredes y tabiquería</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Tabique de bloque de concreto de 10 cm, recibido con mortero de pega.</t>
+          <t>Acero de refuerzo en columnas.</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>Tabique interior no estructural de 10 cm de espesor, ejecutado con bloque hueco de concreto de 10x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Incluye replanteo y trazado sobre el piso, colocación de hiladas a nivel y plomo con la ayuda de reglas y cuerda, formación de huecos de paso, anclaje del tabique a los paramentos existentes, humedecido previo de las piezas y limpieza de restos. No incluye el friso ni los dinteles de los huecos, que se valoran aparte. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Suministro, corte, doblado, armado y colocación de acero de refuerzo en cabillas corrugadas de límite elástico 4.200 kg/cm2 en columnas, según los planos de despiece. El rendimiento por kilogramo es de los más bajos del acero de obra por el trabajo en vertical y por la cantidad de estribos. Incluye el corte y doblado de barras y estribos, el armado de la canasta con la separación de estribos indicada y su reducción en las zonas de confinamiento de los extremos, el amarre con alambre en todos los cruces, el solape con las esperas de la fundación o del nivel inferior respetando la longitud prevista, la colocación de separadores en las cuatro caras y el aplomado y arriostramiento del armado antes del encofrado. Medido en peso de acero realmente colocado.</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E171" t="n">
         <v>1</v>
       </c>
       <c r="F171" t="n">
-        <v>18.29</v>
+        <v>2.48</v>
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>Bloque de concreto</t>
+          <t>Concreto armado vaciado en sitio</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
@@ -6944,17 +6944,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Paredes y tabiquería</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
+          <t>Encofrado y desencofrado de columna.</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Encofrado de columna mediante paneles de madera con abrazaderas, puntales y arriostramiento, y su posterior desencofrado. Incluye el replanteo sobre el nivel, el montaje de los paneles alrededor del armado, el aplomado en las dos direcciones y su arriostramiento, la comprobación de la escuadría y del recubrimiento, la aplicación de desmoldeante, la previsión de la ventana de limpieza en la base, el desencofrado una vez alcanzada la resistencia y la limpieza y acopio de los paneles para su reutilización. Medido en superficie de encofrado en contacto con el concreto.</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -6966,11 +6966,11 @@
         <v>1</v>
       </c>
       <c r="F172" t="n">
-        <v>52.4</v>
+        <v>17.25</v>
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Tabiquería de yeso laminado</t>
+          <t>Concreto armado vaciado en sitio</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
@@ -6982,33 +6982,33 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Frisos y revestimientos de pared</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+          <t>Concreto para columna.</t>
         </is>
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Concreto premezclado de resistencia 250 kg/cm2 vaciado en columna, incluida su compactación por vibrado y su curado. Incluye la limpieza del fondo del encofrado por la ventana prevista antes de cerrarla, la recepción y comprobación del concreto, el vaciado por capas de altura limitada empleando tubo de descarga para evitar la segregación por caída libre, la compactación con vibrador de aguja en cada capa sin tocar el armado, el enrase de la cabeza dejando la superficie rugosa para la junta con la viga superior, el desencofrado y el curado. Medido en volumen teórico según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E173" t="n">
         <v>1</v>
       </c>
       <c r="F173" t="n">
-        <v>10.75</v>
+        <v>193.28</v>
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Frisos y enlucidos de mortero</t>
+          <t>Concreto armado vaciado en sitio</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -7020,33 +7020,33 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Frisos y revestimientos de pared</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+          <t>Acero de refuerzo en vigas.</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Suministro, corte, doblado, armado y colocación de acero de refuerzo en cabillas corrugadas en vigas, según los planos de despiece. Incluye el corte y doblado de barras y estribos, el armado de la canasta con la separación de estribos indicada y su reducción en las zonas de confinamiento junto a los apoyos, la disposición del refuerzo superior sobre los apoyos y del inferior en el centro del vano conforme al diagrama de momentos, el amarre con alambre, la colocación de separadores, el anclaje en los nudos con las columnas y la revisión del despiece antes de autorizar el vaciado. Medido en peso de acero realmente colocado.</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E174" t="n">
         <v>1</v>
       </c>
       <c r="F174" t="n">
-        <v>10.87</v>
+        <v>2.43</v>
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>Enchapado cerámico y porcelanato</t>
+          <t>Concreto armado vaciado en sitio</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
@@ -7058,17 +7058,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+          <t>Encofrado y desencofrado de viga.</t>
         </is>
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+          <t>Encofrado de viga mediante fondo y laterales de madera sobre puntales, con sus arriostramientos, y su posterior desencofrado. Es el encofrado más laborioso de la estructura por el apuntalamiento y la nivelación del fondo. Incluye el replanteo de la cota inferior, el montaje y nivelación del fondo sobre puntales con la contraflecha prevista, el montaje y aplomado de los laterales, la comprobación de sección y alineación, la aplicación de desmoldeante, el desencofrado escalonado retirando primero los laterales y manteniendo el fondo y los puntales hasta alcanzar la resistencia de proyecto, y la limpieza y acopio del material. Medido en superficie de encofrado en contacto con el concreto.</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -7080,11 +7080,11 @@
         <v>1</v>
       </c>
       <c r="F175" t="n">
-        <v>8.02</v>
+        <v>20.02</v>
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>Bases, contrapisos y nivelación</t>
+          <t>Concreto armado vaciado en sitio</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
@@ -7096,33 +7096,33 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+          <t>Concreto para viga.</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Concreto premezclado de resistencia 250 kg/cm2 vaciado en viga, incluida su compactación por vibrado y su curado. Incluye la revisión previa del armado, del apuntalamiento y del recubrimiento, la recepción y comprobación del concreto, el vaciado continuo evitando juntas frías y respetando la posición de las juntas de construcción previstas en el tercio central del vano, la compactación con vibrador de aguja, el reglado de la cara superior, el curado y el desapuntalamiento escalonado una vez alcanzada la resistencia. Medido en volumen teórico según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E176" t="n">
         <v>1</v>
       </c>
       <c r="F176" t="n">
-        <v>9.17</v>
+        <v>189.76</v>
       </c>
       <c r="G176" t="inlineStr">
         <is>
-          <t>Pisos cerámicos y porcelanato</t>
+          <t>Concreto armado vaciado en sitio</t>
         </is>
       </c>
       <c r="H176" t="inlineStr">
@@ -7134,33 +7134,33 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+          <t>Acero de refuerzo en pantalla o muro estructural.</t>
         </is>
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Suministro, corte, doblado, armado y colocación de acero de refuerzo en cabillas corrugadas en pantalla o muro estructural de concreto armado, en dos parrillas verticales, según los planos de despiece. Incluye el corte y doblado, el armado de ambas parrillas con sus barras verticales y horizontales, la colocación de los ganchos o grapas de unión entre parrillas que impiden su separación durante el vaciado, el solape con las esperas del nivel inferior, la disposición de los refuerzos de borde y de los elementos de confinamiento en los extremos, la colocación de separadores en ambas caras y la revisión del despiece. Medido en peso de acero realmente colocado.</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E177" t="n">
         <v>1</v>
       </c>
       <c r="F177" t="n">
-        <v>12.51</v>
+        <v>2.34</v>
       </c>
       <c r="G177" t="inlineStr">
         <is>
-          <t>Pisos cerámicos y porcelanato</t>
+          <t>Concreto armado vaciado en sitio</t>
         </is>
       </c>
       <c r="H177" t="inlineStr">
@@ -7172,33 +7172,33 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+          <t>Encofrado a dos caras de pantalla estructural.</t>
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+          <t>Encofrado a dos caras de pantalla o muro estructural mediante paneles de madera con tirantes pasantes, puntales y arriostramientos, y su posterior desencofrado. Incluye el replanteo, el montaje y aplomado de la primera cara, la colocación de los tirantes y separadores de espesor, el cierre de la segunda cara tras la revisión del armado, el arriostramiento frente al empuje del concreto fresco, la aplicación de desmoldeante, el desencofrado y el sellado de los agujeros de los tirantes. Medido en superficie de encofrado en contacto con el concreto, contando ambas caras.</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E178" t="n">
         <v>1</v>
       </c>
       <c r="F178" t="n">
-        <v>1.69</v>
+        <v>17.21</v>
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>Rodapiés y remates de piso</t>
+          <t>Concreto armado vaciado en sitio</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
@@ -7210,33 +7210,33 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Cielos rasos</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+          <t>Concreto para pantalla estructural.</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+          <t>Concreto premezclado de resistencia 250 kg/cm2 vaciado en pantalla o muro estructural, incluida su compactación por vibrado y su curado. Incluye la revisión previa del armado, del encofrado y de los recubrimientos, la recepción del concreto, el vaciado por capas de altura limitada y por puntos alternos para no descuadrar el encofrado, el empleo de tubo de descarga para evitar la segregación, la compactación con vibrador de aguja en cada capa, el curado prolongado y el desencofrado una vez alcanzada la resistencia. Medido en volumen teórico según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E179" t="n">
         <v>1</v>
       </c>
       <c r="F179" t="n">
-        <v>18.47</v>
+        <v>190.5</v>
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>Yeso laminado continuo</t>
+          <t>Concreto armado vaciado en sitio</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
@@ -7248,33 +7248,33 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+          <t>Suministro y montaje de estructura metálica.</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+          <t>Suministro, izado y montaje de estructura metálica de acero formada por perfiles laminados, con sus cartelas, rigidizadores y elementos de conexión, montada mediante soldadura y tornillería estructural. Incluye la recepción y verificación del material contra los planos de taller, el replanteo y comprobación de la posición de las placas base, el izado con grúa y el presentado de las piezas, el aplomado y nivelación provisional mediante arriostramientos y tornillos de montaje, la ejecución de las uniones definitivas, la verificación geométrica del conjunto montado y la retirada de los elementos provisionales. No incluye la protección anticorrosiva ni la protección contra incendios. Medido en peso de estructura realmente montada.</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E180" t="n">
         <v>1</v>
       </c>
       <c r="F180" t="n">
-        <v>7.45</v>
+        <v>3.89</v>
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>Tuberías y montantes de agua</t>
+          <t>Estructura metálica</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
@@ -7286,17 +7286,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+          <t>Placa base con pernos de anclaje para columna metálica.</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+          <t>Placa base de acero con sus pernos de anclaje, cartelas y nivelación con grout de retracción compensada, para el apoyo de columna metálica sobre fundación de concreto. Incluye el replanteo preciso de la posición de los pernos, que es la operación crítica del conjunto porque un error aquí obliga a rehacer anclajes en concreto endurecido, la colocación de la plantilla de pernos antes del vaciado de la fundación o el anclaje químico posterior, el nivelado de la placa mediante cuñas o tuercas de nivelación, el relleno del espacio bajo la placa con grout fluido sin retracción, el apriete de tuercas al par especificado y la protección del conjunto. Medido por unidad realmente ejecutada.</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -7308,11 +7308,11 @@
         <v>1</v>
       </c>
       <c r="F181" t="n">
-        <v>37.22</v>
+        <v>107.48</v>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>Puntos de agua</t>
+          <t>Estructura metálica</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
@@ -7324,33 +7324,33 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+          <t>Soldadura de conexiones estructurales en obra.</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+          <t>Ejecución de cordón de soldadura de conexión estructural en obra, con preparación de bordes, precalentamiento cuando el espesor lo requiera y limpieza entre pasadas. Incluye la limpieza y preparación de las superficies a unir con esmerilado hasta metal sano, el punteado y verificación de la posición antes del cordón definitivo, la ejecución de la soldadura en las pasadas necesarias según el espesor, la eliminación de escoria entre pasadas, la inspección visual del cordón terminado y el retoque de la protección anticorrosiva en la zona afectada por el calor. Medido en longitud de cordón realmente ejecutado.</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E182" t="n">
         <v>1</v>
       </c>
       <c r="F182" t="n">
-        <v>13.52</v>
+        <v>8.35</v>
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>Llaves y valvulería</t>
+          <t>Estructura metálica</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
@@ -7362,33 +7362,33 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+          <t>Imprimación anticorrosiva de estructura metálica.</t>
         </is>
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+          <t>Preparación de la superficie y aplicación de dos manos de imprimación anticorrosiva sobre estructura metálica. La durabilidad del recubrimiento depende mucho más de la preparación previa que de la calidad de la pintura, de modo que el grado de limpieza alcanzado es lo determinante. Incluye la eliminación de óxido, calamina, grasa y restos de escoria mediante cepillo de púas y esmerilado, el desengrasado, la aplicación de la primera mano cubriendo aristas, cantos y zonas de difícil acceso que son las que primero fallan, el respeto del tiempo de repintado y la aplicación de la segunda mano. Medido en superficie realmente tratada, desarrollando todas las caras del perfil.</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E183" t="n">
         <v>1</v>
       </c>
       <c r="F183" t="n">
-        <v>23.45</v>
+        <v>6.2</v>
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Estructura metálica</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
@@ -7400,33 +7400,33 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Instalación de lavamanos con su grifería y desagüe.</t>
+          <t>Correas metálicas para estructura de techo.</t>
         </is>
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
+          <t>Suministro y montaje de correas metálicas de perfil conformado para el soporte de la cubierta, fijadas a la estructura principal mediante tornillería o soldadura, con sus tensores y separadores. Incluye la recepción y verificación del material, el replanteo de la separación entre correas según la luz admisible del material de cubrición, el izado y presentado, la fijación a la estructura principal, la colocación de los tensores que evitan el pandeo lateral y la comprobación de la alineación y del plano de apoyo de la cubierta. Medido en peso realmente montado.</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E184" t="n">
         <v>1</v>
       </c>
       <c r="F184" t="n">
-        <v>36.45</v>
+        <v>3.43</v>
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Estructura metálica</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
@@ -7438,33 +7438,33 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+          <t>Suministro y montaje de estructura de madera.</t>
         </is>
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+          <t>Suministro y montaje de estructura de madera aserrada formada por vigas, pares y tirantes, con uniones ejecutadas mediante herrajes metálicos o ensambles tradicionales. Incluye la recepción y verificación de la escuadría, la humedad y la ausencia de defectos que comprometan la capacidad, el corte y labra de las piezas, el presentado y ajuste de las uniones, el izado y montaje con apeo provisional, la fijación definitiva, la comprobación geométrica del conjunto y el ajuste de contraflechas. No incluye el tratamiento preservante ni los herrajes, que se valoran aparte. Medido en volumen de madera realmente colocada.</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E185" t="n">
         <v>1</v>
       </c>
       <c r="F185" t="n">
-        <v>11.04</v>
+        <v>563.24</v>
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>Tuberías y bajantes de desagüe</t>
+          <t>Estructura de madera</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
@@ -7476,33 +7476,33 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Punto de desagüe para aparato sanitario.</t>
+          <t>Correas y viguetas de madera para cubierta o entrepiso.</t>
         </is>
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+          <t>Suministro y montaje de correas o viguetas de madera para el soporte de cubierta o entrepiso, fijadas a la estructura principal con herrajes o clavado. Incluye la recepción y selección de las piezas, el replanteo de la separación entre ejes, el corte a medida, el presentado y nivelación, la fijación a los apoyos, la colocación de los arriostramientos o crucetas que impiden el vuelco lateral y la comprobación del plano de apoyo. Medido en longitud realmente colocada.</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E186" t="n">
         <v>1</v>
       </c>
       <c r="F186" t="n">
-        <v>33.84</v>
+        <v>12.68</v>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>Puntos de desagüe</t>
+          <t>Estructura de madera</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
@@ -7514,33 +7514,33 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Instalaciones eléctricas</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+          <t>Tratamiento preservante de madera estructural.</t>
         </is>
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+          <t>Aplicación de tratamiento preservante fungicida e insecticida sobre madera estructural, mediante dos manos a brocha o por inmersión. En clima tropical este tratamiento no es opcional: la madera sin proteger tiene una vida útil corta frente al comején y a los hongos de pudrición. Incluye el lijado y limpieza previa de la superficie, la aplicación de la primera mano con especial atención a testas, ensambles y zonas de apoyo que son las de mayor riesgo, el respeto del tiempo de absorción y la aplicación de la segunda mano. Medido en superficie realmente tratada, desarrollando todas las caras.</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E187" t="n">
         <v>1</v>
       </c>
       <c r="F187" t="n">
-        <v>8.369999999999999</v>
+        <v>3.81</v>
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>Canalizaciones y cableado</t>
+          <t>Estructura de madera</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
@@ -7552,17 +7552,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Instalaciones eléctricas</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+          <t>Herraje o conector metálico para unión de estructura de madera.</t>
         </is>
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+          <t>Suministro y colocación de herraje metálico galvanizado de unión en estructura de madera, tal como estribo, placa, ángulo o conector de pares, con su tornillería específica. Incluye el replanteo de la posición, el pretaladrado de la madera con el diámetro correcto para no fisurarla, la colocación del herraje, el atornillado o clavado con la totalidad de los agujeros ocupados, requisito del que depende la capacidad declarada del herraje, y la comprobación del apriete. Medido por unidad realmente colocada.</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -7574,11 +7574,11 @@
         <v>1</v>
       </c>
       <c r="F188" t="n">
-        <v>8.720000000000001</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Puntos, mecanismos y tomas</t>
+          <t>Estructura de madera</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -7590,17 +7590,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+          <t>Encofrado de losa maciza sobre puntales.</t>
         </is>
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Encofrado de losa maciza mediante tablero de madera sobre soleras y puntales metálicos, con su nivelación y contraflecha, y su posterior desencofrado. Incluye el replanteo de la cota inferior, el montaje de la retícula de puntales con la separación indicada, la colocación de soleras y del tablero, la nivelación del conjunto con la contraflecha prevista, el sellado de juntas del tablero para evitar la pérdida de lechada, la aplicación de desmoldeante, el desencofrado escalonado manteniendo los puntales de seguridad hasta alcanzar la resistencia de proyecto, y la limpieza y acopio del material. Medido en superficie de encofrado en contacto con el concreto.</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -7612,11 +7612,11 @@
         <v>1</v>
       </c>
       <c r="F189" t="n">
-        <v>2.82</v>
+        <v>22.28</v>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>Preparación de soportes</t>
+          <t>Losas y entrepisos</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
@@ -7628,33 +7628,33 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+          <t>Acero de refuerzo en losa maciza.</t>
         </is>
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Suministro, corte, doblado, armado y colocación de acero de refuerzo en cabillas corrugadas en losa maciza, en parrillas inferior y superior según los planos de despiece. Incluye el corte y doblado, el armado de las parrillas con amarre de alambre, la colocación de separadores inferiores y de caballetes que sostienen la parrilla superior en su cota, los refuerzos sobre los apoyos y en los bordes de huecos, y el repaso de la posición del armado inmediatamente antes del vaciado. Medido en peso de acero realmente colocado.</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E190" t="n">
         <v>1</v>
       </c>
       <c r="F190" t="n">
-        <v>3.46</v>
+        <v>2.27</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Pintura interior</t>
+          <t>Losas y entrepisos</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
@@ -7666,33 +7666,33 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Estructuras</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+          <t>Concreto para losa maciza.</t>
         </is>
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+          <t>Concreto premezclado de resistencia 250 kg/cm2 vaciado en losa maciza de entrepiso o techo, incluida su compactación por vibrado y su curado. Incluye la revisión previa del encofrado, del apuntalamiento, del armado y de los recubrimientos, la recepción y comprobación del concreto, el vaciado continuo por franjas evitando juntas frías, la compactación con vibrador de aguja, el reglado a la cota mediante maestras, el flotado de la superficie y el curado durante los primeros días. Medido en volumen teórico según las dimensiones de proyecto.</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="E191" t="n">
         <v>1</v>
       </c>
       <c r="F191" t="n">
-        <v>5.23</v>
+        <v>185.81</v>
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>Esmaltes sobre madera y metal</t>
+          <t>Losas y entrepisos</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
@@ -7704,36 +7704,1366 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
+          <t>Estructuras</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Losa nervada con bloques de arcilla de aliviano.</t>
+        </is>
+      </c>
+      <c r="C192" s="2" t="inlineStr">
+        <is>
+          <t>Losa nervada de entrepiso o techo formada por nervios de concreto armado y bloques de arcilla de aliviano, con su loseta de compresión y malla de retracción. Incluye el encofrado y apuntalamiento del fondo, la colocación de los bloques de aliviano dejando el ancho de nervio previsto, el armado de los nervios con su refuerzo inferior y superior, la colocación de la malla electrosoldada de la loseta de compresión, el vaciado y vibrado del concreto, el reglado, el curado y el desapuntalamiento escalonado. Medido en superficie de losa realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E192" t="n">
+        <v>1</v>
+      </c>
+      <c r="F192" t="n">
+        <v>70.77</v>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Losas y entrepisos</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Estructuras</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Losa nervada con bloques de poliestireno de aliviano.</t>
+        </is>
+      </c>
+      <c r="C193" s="2" t="inlineStr">
+        <is>
+          <t>Losa nervada de entrepiso o techo formada por nervios de concreto armado y bloques de poliestireno expandido de aliviano, con su loseta de compresión y malla de retracción. Frente al bloque de arcilla reduce notablemente el peso propio de la losa, lo que repercute en el dimensionado de vigas, columnas y fundaciones, y mejora el aislamiento térmico. Incluye el encofrado y apuntalamiento, la colocación de los bloques, el armado de los nervios, la malla de la loseta de compresión, el vaciado y vibrado, el reglado, el curado y el desapuntalamiento escalonado. Medido en superficie de losa realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E193" t="n">
+        <v>1</v>
+      </c>
+      <c r="F193" t="n">
+        <v>77.36</v>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Losas y entrepisos</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Estructuras</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Losa con viguetas prefabricadas pretensadas.</t>
+        </is>
+      </c>
+      <c r="C194" s="2" t="inlineStr">
+        <is>
+          <t>Losa de entrepiso o techo formada por viguetas prefabricadas pretensadas, bloques de aliviano, loseta de compresión y malla de retracción. Al trabajar la vigueta como elemento resistente durante el montaje, el apuntalamiento necesario es mucho menor que en una losa nervada tradicional, lo que acelera la ejecución. Incluye el replanteo y colocación de las viguetas sobre sus apoyos con la entrega mínima requerida, el apuntalamiento intermedio, la colocación de los bloques, el armado de negativos sobre apoyos, la malla de la loseta, el vaciado y vibrado, el curado y el desapuntalamiento escalonado. Medido en superficie de losa realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E194" t="n">
+        <v>1</v>
+      </c>
+      <c r="F194" t="n">
+        <v>61.39</v>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Losas y entrepisos</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Estructuras</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Apuntalamiento de losa durante el vaciado y el fraguado.</t>
+        </is>
+      </c>
+      <c r="C195" s="2" t="inlineStr">
+        <is>
+          <t>Apuntalamiento de losa mediante puntales metálicos telescópicos sobre durmientes de reparto, dimensionado para soportar el peso del concreto fresco, del encofrado y de las cargas de ejecución, y mantenido hasta que la losa alcanza la resistencia de proyecto. El desapuntalamiento prematuro es una de las causas más frecuentes de flechas excesivas y de fisuración permanente. Incluye el replanteo de la retícula, la colocación de durmientes en cabeza y base, el montaje y puesta en carga de los puntales, la comprobación de que la carga se transmite a un nivel inferior con capacidad suficiente, la revisión durante el vaciado y el desapuntalamiento escalonado. Medido en superficie de losa realmente apuntalada.</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E195" t="n">
+        <v>1</v>
+      </c>
+      <c r="F195" t="n">
+        <v>11.93</v>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Losas y entrepisos</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Estructuras</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Encofrado de escalera de concreto armado.</t>
+        </is>
+      </c>
+      <c r="C196" s="2" t="inlineStr">
+        <is>
+          <t>Encofrado de escalera de concreto armado, comprendiendo el fondo de la losa inclinada sobre puntales, los laterales de cierre y los tabicones de formación de peldaños, y su posterior desencofrado. Es de los encofrados más laboriosos por la geometría inclinada y por el replanteo de la huella y la contrahuella, que debe ser exacto y constante porque cualquier diferencia entre peldaños se percibe al caminar y compromete la seguridad. Incluye el replanteo, el montaje y nivelación del fondo, los laterales, los tabicones de peldaño, el arriostramiento, el desmoldeante, el desencofrado y la limpieza del material. Medido en superficie de encofrado en contacto con el concreto.</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E196" t="n">
+        <v>1</v>
+      </c>
+      <c r="F196" t="n">
+        <v>29.15</v>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Escaleras estructurales</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Estructuras</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Acero de refuerzo en escalera.</t>
+        </is>
+      </c>
+      <c r="C197" s="2" t="inlineStr">
+        <is>
+          <t>Suministro, corte, doblado, armado y colocación de acero de refuerzo en cabillas corrugadas en escalera de concreto armado, según los planos de despiece. Incluye el corte y doblado, el armado de la parrilla principal de la losa inclinada con su refuerzo de reparto, la disposición de los refuerzos en los quiebres de la geometría donde el trazado del acero debe respetar el sentido de las tracciones, el anclaje en los apoyos de arranque y llegada, el amarre con alambre y la colocación de separadores. Medido en peso de acero realmente colocado.</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E197" t="n">
+        <v>1</v>
+      </c>
+      <c r="F197" t="n">
+        <v>2.46</v>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Escaleras estructurales</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Estructuras</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Concreto para escalera de concreto armado.</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t>Concreto premezclado de resistencia 250 kg/cm2 vaciado en escalera, incluida su compactación por vibrado y su curado. El vaciado en pendiente exige un concreto de consistencia más seca de lo habitual para que no escurra por la rampa, y debe ejecutarse de forma ascendente desde el arranque. Incluye la revisión previa del encofrado, el apuntalamiento y el armado, la recepción del concreto con el asentamiento adecuado, el vaciado ascendente por peldaños, la compactación con vibrador, el fratasado de huellas y contrahuellas, el curado y el desapuntalamiento escalonado. Medido en volumen teórico según las dimensiones de proyecto.</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>1</v>
+      </c>
+      <c r="F198" t="n">
+        <v>199.24</v>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Escaleras estructurales</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Estructuras</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Escalera metálica estructural.</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y montaje de escalera metálica estructural formada por zancas de perfil laminado, peldaños y descansos, con sus anclajes a la estructura. Incluye la verificación en obra de las cotas reales de arranque y llegada antes de la fabricación, paso imprescindible porque una escalera metálica no admite ajustes en sitio, el izado y presentado de las zancas, su nivelación y aplomado, la ejecución de las uniones soldadas o atornilladas, el montaje de peldaños y descansos y la comprobación de que huella y contrahuella se mantienen constantes en todo el tramo. No incluye barandas ni el acabado del peldaño. Medido en peso realmente montado.</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E199" t="n">
+        <v>1</v>
+      </c>
+      <c r="F199" t="n">
+        <v>4.71</v>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Escaleras estructurales</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Estructuras</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Reparación superficial de concreto con mortero estructural.</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>Reparación de concreto deteriorado por coqueras, desprendimientos o carbonatación, mediante saneado del área y reposición con mortero tixotrópico de reparación estructural, de 3 cm de espesor medio. Incluye la delimitación del área con corte perimetral perpendicular para evitar bordes en bisel que se desprenden, el picado del concreto suelto hasta alcanzar concreto sano, la limpieza y saturación del soporte, la aplicación del puente de adherencia, la reposición del mortero por capas respetando el espesor máximo por capa y el curado del material aplicado. Medido en superficie realmente reparada.</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E200" t="n">
+        <v>1</v>
+      </c>
+      <c r="F200" t="n">
+        <v>173.12</v>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Refuerzos y reparaciones estructurales</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Estructuras</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Tratamiento pasivante de acero de refuerzo corroído.</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr">
+        <is>
+          <t>Limpieza y tratamiento del acero de refuerzo afectado por corrosión, descubierto tras el saneado del concreto, mediante cepillado hasta grado de limpieza adecuado y aplicación de recubrimiento pasivante con inhibidor. Es el paso que decide si la reparación dura: si se repone el mortero sobre acero oxidado, la corrosión continúa por debajo y vuelve a reventar el recubrimiento en pocos años. Incluye el descubrimiento del acero en todo su perímetro dejando espacio libre por detrás de la barra, la eliminación del óxido con cepillo de púas y esmeril, la valoración de la pérdida de sección y el aviso al proyectista si supera lo admisible, y la aplicación de dos manos de pasivante. Medido en superficie de elemento realmente tratada.</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E201" t="n">
+        <v>1</v>
+      </c>
+      <c r="F201" t="n">
+        <v>12.49</v>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Refuerzos y reparaciones estructurales</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Estructuras</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Inyección de fisuras en concreto con resina epóxica.</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>Sellado y restitución del monolitismo de fisuras en elementos de concreto mediante inyección de resina epóxica de baja viscosidad a través de boquillas. Incluye el mapeo previo y el registro del ancho y recorrido de las fisuras, la determinación de si la fisura está viva o estabilizada, ya que inyectar con resina rígida una fisura en movimiento provoca su reaparición junto al sello, la limpieza del recorrido, la colocación de boquillas y el sellado superficial del labio, la inyección progresiva de boquilla en boquilla hasta rebose en la siguiente, el fraguado y el retiro de boquillas y sello con repaso de la superficie. Medido en longitud de fisura realmente inyectada.</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E202" t="n">
+        <v>1</v>
+      </c>
+      <c r="F202" t="n">
+        <v>15.65</v>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Refuerzos y reparaciones estructurales</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Estructuras</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Refuerzo estructural con tejido de fibra de carbono.</t>
+        </is>
+      </c>
+      <c r="C203" s="2" t="inlineStr">
+        <is>
+          <t>Refuerzo de elemento estructural de concreto mediante encolado de tejido de fibra de carbono con resina epóxica de saturación. Aporta capacidad a flexión o a cortante sin apenas añadir peso ni modificar la geometría, lo que lo hace idóneo en rehabilitación donde no se puede aumentar la sección. Incluye la regularización y lijado del soporte hasta obtener una superficie plana y sin lechada, el redondeo de las aristas por las que ha de doblar el tejido, la imprimación, la aplicación de la resina de saturación, la colocación del tejido en la dirección de las tracciones eliminando burbujas con rodillo, la segunda capa de resina y el curado. Medido en superficie de tejido realmente colocada.</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E203" t="n">
+        <v>1</v>
+      </c>
+      <c r="F203" t="n">
+        <v>92.44</v>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Refuerzos y reparaciones estructurales</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Estructuras</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Encamisado de columna de concreto armado.</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t>Refuerzo de columna existente mediante encamisado de concreto armado, aumentando su sección con una capa perimetral de concreto con su propio armado, conectada al núcleo original. Incluye el apeo previo de la estructura que descarga la columna, el repicado de la superficie existente para dar adherencia, la perforación y anclaje químico de los conectores que cosen el encamisado al núcleo, el armado longitudinal y de estribos de confinamiento, el encofrado, el vaciado con concreto de retracción compensada o mortero fluido dado el reducido espesor, el curado y el desapeo escalonado. Medido en longitud de columna realmente encamisada.</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E204" t="n">
+        <v>1</v>
+      </c>
+      <c r="F204" t="n">
+        <v>180.34</v>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Refuerzos y reparaciones estructurales</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Estructuras</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Anclaje químico de barra de acero en concreto.</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t>Anclaje de barra de acero en elemento de concreto existente mediante resina epóxica bicomponente inyectada en perforación, para conexión de elementos nuevos a la estructura existente. Incluye el replanteo del punto evitando la armadura existente mediante detección previa, la perforación con el diámetro y la profundidad especificados por el fabricante de la resina, la limpieza del taladro mediante soplado y cepillado repetidos, operación de la que depende por completo la capacidad del anclaje y que es la que más se omite en obra, la inyección de la resina desde el fondo, la introducción de la barra con giro y el respeto del tiempo de curado antes de cargarla. Medido por unidad realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E205" t="n">
+        <v>1</v>
+      </c>
+      <c r="F205" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>Refuerzos y reparaciones estructurales</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Paredes y tabiquería</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Tabique de bloque de concreto de 10 cm, recibido con mortero de pega.</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t>Tabique interior no estructural de 10 cm de espesor, ejecutado con bloque hueco de concreto de 10x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Incluye replanteo y trazado sobre el piso, colocación de hiladas a nivel y plomo con la ayuda de reglas y cuerda, formación de huecos de paso, anclaje del tabique a los paramentos existentes, humedecido previo de las piezas y limpieza de restos. No incluye el friso ni los dinteles de los huecos, que se valoran aparte. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E206" t="n">
+        <v>1</v>
+      </c>
+      <c r="F206" t="n">
+        <v>18.29</v>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Bloque de concreto</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Paredes y tabiquería</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
+        </is>
+      </c>
+      <c r="C207" s="2" t="inlineStr">
+        <is>
+          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E207" t="n">
+        <v>1</v>
+      </c>
+      <c r="F207" t="n">
+        <v>52.4</v>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>Tabiquería de yeso laminado</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Frisos y revestimientos de pared</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E208" t="n">
+        <v>1</v>
+      </c>
+      <c r="F208" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>Frisos y enlucidos de mortero</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Frisos y revestimientos de pared</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E209" t="n">
+        <v>1</v>
+      </c>
+      <c r="F209" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Enchapado cerámico y porcelanato</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+        </is>
+      </c>
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>1</v>
+      </c>
+      <c r="F210" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>Bases, contrapisos y nivelación</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>1</v>
+      </c>
+      <c r="F211" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>Pisos cerámicos y porcelanato</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C212" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E212" t="n">
+        <v>1</v>
+      </c>
+      <c r="F212" t="n">
+        <v>12.51</v>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>Pisos cerámicos y porcelanato</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E213" t="n">
+        <v>1</v>
+      </c>
+      <c r="F213" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>Rodapiés y remates de piso</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Cielos rasos</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>1</v>
+      </c>
+      <c r="F214" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>Yeso laminado continuo</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E215" t="n">
+        <v>1</v>
+      </c>
+      <c r="F215" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>Tuberías y montantes de agua</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E216" t="n">
+        <v>1</v>
+      </c>
+      <c r="F216" t="n">
+        <v>37.22</v>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>Puntos de agua</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+        </is>
+      </c>
+      <c r="C217" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E217" t="n">
+        <v>1</v>
+      </c>
+      <c r="F217" t="n">
+        <v>13.52</v>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>Llaves y valvulería</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E218" t="n">
+        <v>1</v>
+      </c>
+      <c r="F218" t="n">
+        <v>23.45</v>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Instalación de lavamanos con su grifería y desagüe.</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E219" t="n">
+        <v>1</v>
+      </c>
+      <c r="F219" t="n">
+        <v>36.45</v>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E220" t="n">
+        <v>1</v>
+      </c>
+      <c r="F220" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>Tuberías y bajantes de desagüe</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Punto de desagüe para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E221" t="n">
+        <v>1</v>
+      </c>
+      <c r="F221" t="n">
+        <v>33.84</v>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>Puntos de desagüe</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E222" t="n">
+        <v>1</v>
+      </c>
+      <c r="F222" t="n">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>Canalizaciones y cableado</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E223" t="n">
+        <v>1</v>
+      </c>
+      <c r="F223" t="n">
+        <v>8.720000000000001</v>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>Puntos, mecanismos y tomas</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr">
+        <is>
+          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E224" t="n">
+        <v>1</v>
+      </c>
+      <c r="F224" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>Preparación de soportes</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E225" t="n">
+        <v>1</v>
+      </c>
+      <c r="F225" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>Pintura interior</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E226" t="n">
+        <v>1</v>
+      </c>
+      <c r="F226" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>Esmaltes sobre madera y metal</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
           <t>Gestión de residuos y limpieza</t>
         </is>
       </c>
-      <c r="B192" t="inlineStr">
+      <c r="B227" t="inlineStr">
         <is>
           <t>Retirada y transporte de escombro a vertedero autorizado.</t>
         </is>
       </c>
-      <c r="C192" s="2" t="inlineStr">
+      <c r="C227" s="2" t="inlineStr">
         <is>
           <t>Retirada de escombro procedente de demoliciones desde el punto de acopio de la obra y transporte en camión volqueta hasta vertedero o botadero autorizado, incluido el canon de vertido. Incluye la carga manual del escombro sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado con una distancia media considerada de 25 km, la descarga y la limpieza de la zona de carga. Medido por metro cúbico de escombro esponjado realmente retirado.</t>
         </is>
       </c>
-      <c r="D192" t="inlineStr">
+      <c r="D227" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="E192" t="n">
-        <v>1</v>
-      </c>
-      <c r="F192" t="n">
+      <c r="E227" t="n">
+        <v>1</v>
+      </c>
+      <c r="F227" t="n">
         <v>16.07</v>
       </c>
-      <c r="G192" t="inlineStr">
+      <c r="G227" t="inlineStr">
         <is>
           <t>Retiro y transporte de escombro</t>
         </is>
       </c>
-      <c r="H192" t="inlineStr">
+      <c r="H227" t="inlineStr">
         <is>
           <t>incluida</t>
         </is>

</xml_diff>

<commit_message>
Cerrar el capitulo 06 Paredes y tabiqueria con 25 partidas en 5 subcapitulos
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/catalogo_partidas.xlsx
+++ b/basedatos_partidas/salida/catalogo_partidas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H227"/>
+  <dimension ref="A1:H250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8279,12 +8279,12 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
+          <t>Pared de bloque de concreto de 15 cm.</t>
         </is>
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
+          <t>Pared de 15 cm de espesor ejecutada con bloque hueco de concreto de 15x20x40 cm recibido con mortero de pega, aparejado a soga con juntas de 1 cm enrasadas. Se emplea en paredes divisorias de mayor exigencia acústica y en cerramientos de fachada de una sola hoja. Incluye el replanteo y trazado sobre el piso, el humedecido previo de las piezas, la colocación de hiladas a nivel y plomo con ayuda de reglas y cuerda, la formación de huecos de paso, el amarre a los paramentos y a la estructura existente mediante conectores, y la limpieza de restos. No incluye el friso ni los dinteles. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -8296,11 +8296,11 @@
         <v>1</v>
       </c>
       <c r="F207" t="n">
-        <v>52.4</v>
+        <v>23.83</v>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>Tabiquería de yeso laminado</t>
+          <t>Bloque de concreto</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
@@ -8312,17 +8312,17 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Frisos y revestimientos de pared</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+          <t>Pared de bloque de concreto de 20 cm.</t>
         </is>
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Pared de 20 cm de espesor ejecutada con bloque hueco de concreto de 20x20x40 cm recibido con mortero de pega, aparejado a soga con juntas enrasadas. Se emplea en cerramientos de fachada, paredes de linderos y en cualquier paño que deba aportar masa por razones acústicas o de seguridad. Incluye el replanteo, el humedecido de las piezas, la colocación de hiladas a nivel y plomo, la formación de huecos, el amarre a la estructura mediante conectores y la limpieza. No incluye el friso ni los dinteles. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -8334,11 +8334,11 @@
         <v>1</v>
       </c>
       <c r="F208" t="n">
-        <v>10.75</v>
+        <v>28.63</v>
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>Frisos y enlucidos de mortero</t>
+          <t>Bloque de concreto</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
@@ -8350,17 +8350,17 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Frisos y revestimientos de pared</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+          <t>Pared de bloque de concreto a la vista.</t>
         </is>
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Pared de bloque de concreto ejecutada con acabado a la vista, sin friso posterior, con selección previa de las piezas y junta trabajada y rehundida. Al no haber friso que corrija los defectos, el trabajo exige un aparejo cuidado, plomos y niveles exactos y limpieza continua de la superficie, lo que reduce sensiblemente el rendimiento frente a una pared destinada a frisar. Incluye la selección y descarte de piezas defectuosas o descantilladas, el replanteo del despiece para evitar cortes en zonas vistas, la colocación con junta constante, el rehundido y perfilado de la junta con el mortero aún fresco y la limpieza inmediata de los rebabes. No incluye el tratamiento hidrofugante final. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -8372,11 +8372,11 @@
         <v>1</v>
       </c>
       <c r="F209" t="n">
-        <v>10.87</v>
+        <v>28.37</v>
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>Enchapado cerámico y porcelanato</t>
+          <t>Bloque de concreto</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
@@ -8388,33 +8388,33 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+          <t>Machón o columna de confinamiento en pared de bloque.</t>
         </is>
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+          <t>Machón o columna de confinamiento de concreto armado vaciado dentro del paño de mampostería, que junto con la viga de corona conforma el sistema de mampostería confinada. Su función es dotar a la pared de capacidad frente a acciones sísmicas, por lo que su ejecución no es opcional en los paños que el proyecto define como confinados. Incluye el armado con sus cabillas longitudinales y estribos, el amarre de las esperas a la fundación y a la viga superior, el dentado o la colocación de conectores en el borde de la mampostería para garantizar la trabazón, el encofrado, el vaciado con concreto de 210 kg/cm2, el vibrado y el desencofrado. Medido en longitud realmente ejecutada.</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E210" t="n">
         <v>1</v>
       </c>
       <c r="F210" t="n">
-        <v>8.02</v>
+        <v>33.5</v>
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>Bases, contrapisos y nivelación</t>
+          <t>Bloque de concreto</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
@@ -8426,33 +8426,33 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+          <t>Viga de corona o de amarre en pared de bloque.</t>
         </is>
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Viga de corona de concreto armado vaciada en la coronación del paño de mampostería, que cierra el marco de confinamiento junto con los machones y reparte las cargas hacia ellos. Incluye el armado con sus cabillas longitudinales y estribos, el anclaje en los machones extremos, el encofrado apoyado sobre la última hilada, el vaciado con concreto de 210 kg/cm2, el vibrado, el curado y el desencofrado. Medido en longitud realmente ejecutada.</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E211" t="n">
         <v>1</v>
       </c>
       <c r="F211" t="n">
-        <v>9.17</v>
+        <v>29.72</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>Pisos cerámicos y porcelanato</t>
+          <t>Bloque de concreto</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
@@ -8464,17 +8464,17 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+          <t>Pared de bloque de arcilla de 10 cm.</t>
         </is>
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Pared divisoria de 10 cm de espesor ejecutada con bloque hueco de arcilla de 10x20x30 cm recibido con mortero de pega, aparejado a soga con juntas enrasadas. El bloque de arcilla es más ligero que el de concreto y ofrece mejor comportamiento térmico, aunque menor resistencia mecánica, por lo que se reserva a paños divisorios sin función estructural. Incluye el replanteo, el humedecido previo de las piezas, la colocación de hiladas a nivel y plomo, la formación de huecos de paso, el amarre a los paramentos existentes y la limpieza. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -8486,11 +8486,11 @@
         <v>1</v>
       </c>
       <c r="F212" t="n">
-        <v>12.51</v>
+        <v>18.73</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>Pisos cerámicos y porcelanato</t>
+          <t>Bloque y ladrillo de arcilla</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
@@ -8502,33 +8502,33 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+          <t>Pared de bloque de arcilla de 15 cm.</t>
         </is>
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+          <t>Pared de 15 cm de espesor ejecutada con bloque hueco de arcilla de 15x20x30 cm recibido con mortero de pega, aparejado a soga con juntas enrasadas. Incluye el replanteo, el humedecido previo de las piezas, la colocación de hiladas a nivel y plomo, la formación de huecos de paso, el amarre a la estructura mediante conectores y la limpieza de restos. No incluye el friso ni los dinteles. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E213" t="n">
         <v>1</v>
       </c>
       <c r="F213" t="n">
-        <v>1.69</v>
+        <v>23.75</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>Rodapiés y remates de piso</t>
+          <t>Bloque y ladrillo de arcilla</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
@@ -8540,17 +8540,17 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Cielos rasos</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+          <t>Pared de ladrillo macizo de arcilla.</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+          <t>Pared ejecutada con ladrillo macizo de arcilla cocida recibido con mortero de pega, aparejado a soga con juntas enrasadas. El tamaño reducido de la pieza multiplica el número de unidades por metro cuadrado y hace de esta la mampostería de menor rendimiento, aunque aporta la mayor masa y resistencia. Incluye el replanteo, el humedecido previo de las piezas que en el ladrillo de arcilla es determinante porque absorbe el agua del mortero y compromete su fraguado, la colocación de hiladas a nivel y plomo con trabazón, la formación de huecos y la limpieza. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
@@ -8562,11 +8562,11 @@
         <v>1</v>
       </c>
       <c r="F214" t="n">
-        <v>18.47</v>
+        <v>40.79</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>Yeso laminado continuo</t>
+          <t>Bloque y ladrillo de arcilla</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
@@ -8578,33 +8578,33 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+          <t>Pared de ladrillo de arcilla a la vista.</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+          <t>Pared de ladrillo de arcilla ejecutada con acabado a la vista, con selección de piezas, aparejo replanteado y junta trabajada y rehundida. Es el trabajo de mampostería de menor rendimiento del catálogo: sin friso posterior que corrija nada, cada pieza y cada junta quedan expuestas. Incluye la selección y descarte de piezas descantilladas o de tono discordante, el replanteo del aparejo para resolver los encuentros y los huecos sin piezas partidas a la vista, el humedecido, la colocación con junta constante controlada con plantilla, el rehundido y perfilado de la junta y la limpieza inmediata de rebabes antes de que fragüen. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E215" t="n">
         <v>1</v>
       </c>
       <c r="F215" t="n">
-        <v>7.45</v>
+        <v>45.76</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>Tuberías y montantes de agua</t>
+          <t>Bloque y ladrillo de arcilla</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
@@ -8616,33 +8616,33 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+          <t>Tabique autoportante de placa de yeso laminado 15+70+15, doble placa por cara.</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+          <t>Tabique autoportante de 100 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm, montantes cada 600 mm y canales fijados a piso y techo, con doble placa de yeso laminado de 15 mm atornillada a cada cara y aislamiento interior de lana mineral de 60 mm. Incluye replanteo, banda estanca perimetral, tratamiento de juntas con cinta y pasta, lijado hasta dejar el paramento listo para pintar, y retirada de restos. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E216" t="n">
         <v>1</v>
       </c>
       <c r="F216" t="n">
-        <v>37.22</v>
+        <v>52.4</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>Puntos de agua</t>
+          <t>Tabiquería de yeso laminado</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
@@ -8654,33 +8654,33 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+          <t>Tabique autoportante de yeso laminado 12,5+70+12,5, placa simple.</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+          <t>Tabique autoportante de 95 mm de espesor total, ejecutado con estructura de perfiles de acero galvanizado de 70 mm con montantes cada 600 mm, placa de yeso laminado de 12,5 mm atornillada a cada cara y aislamiento de lana mineral en la cámara. Es la solución estándar para divisiones interiores sin exigencias especiales, y frente al tabique de doble placa reduce a la mitad el material de placa y buena parte de la mano de obra. Incluye el replanteo, la banda estanca perimetral, el montaje de canales y montantes, el atornillado de las placas, la colocación del aislamiento, el tratamiento de juntas con cinta y pasta y el lijado hasta dejar el paramento listo para pintar. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E217" t="n">
         <v>1</v>
       </c>
       <c r="F217" t="n">
-        <v>13.52</v>
+        <v>35.46</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>Llaves y valvulería</t>
+          <t>Tabiquería de yeso laminado</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
@@ -8692,33 +8692,33 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+          <t>Tabique de yeso laminado con placa resistente a la humedad.</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+          <t>Tabique autoportante ejecutado con placa de yeso laminado resistente a la humedad en las caras expuestas, para baños, cocinas y áreas de servicio. La placa resistente a la humedad no es impermeable: retrasa la absorción, pero en las zonas de contacto directo con el agua debe complementarse con una impermeabilización bajo el enchapado, que se valora aparte. Incluye el replanteo, la banda estanca perimetral, el montaje de canales y montantes con la separación reducida que exige recibir el enchapado, el atornillado de las placas, el aislamiento de la cámara, el tratamiento de juntas y el lijado. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E218" t="n">
         <v>1</v>
       </c>
       <c r="F218" t="n">
-        <v>23.45</v>
+        <v>45.15</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Tabiquería de yeso laminado</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
@@ -8730,33 +8730,33 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Instalación de lavamanos con su grifería y desagüe.</t>
+          <t>Trasdosado autoportante de yeso laminado.</t>
         </is>
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
+          <t>Trasdosado autoportante de placa de yeso laminado sobre estructura independiente separada del muro existente, con aislamiento en la cámara. Se emplea para regularizar paredes desplomadas o en mal estado, para alojar instalaciones sin picar el muro y para mejorar el aislamiento térmico y acústico. Al no apoyarse en el muro, admite soportes muy irregulares sin trasladar sus defectos al paramento final. Incluye el replanteo, la banda estanca, el montaje de canales y montantes, el aislamiento, el atornillado de la placa, el tratamiento de juntas y el lijado. Medido en superficie realmente ejecutada, descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E219" t="n">
         <v>1</v>
       </c>
       <c r="F219" t="n">
-        <v>36.45</v>
+        <v>24.19</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Tabiquería de yeso laminado</t>
         </is>
       </c>
       <c r="H219" t="inlineStr">
@@ -8768,33 +8768,33 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+          <t>Trasdosado directo de placa de yeso laminado pegada al muro.</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+          <t>Trasdosado directo mediante placa de yeso laminado adherida al muro existente con pelladas de pasta de agarre. Es la solución más rápida y económica para regularizar y renovar un paramento, pero exige que el muro esté razonablemente plomado y sano, y no permite alojar instalaciones ni aislamiento. Incluye la limpieza y comprobación del soporte, la aplicación de las pelladas con la separación indicada, la colocación y reglado de las placas comprobando plomo y planitud antes del fraguado, el tratamiento de juntas y el lijado. Medido en superficie realmente ejecutada, descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E220" t="n">
         <v>1</v>
       </c>
       <c r="F220" t="n">
-        <v>11.04</v>
+        <v>13.23</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>Tuberías y bajantes de desagüe</t>
+          <t>Tabiquería de yeso laminado</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
@@ -8806,17 +8806,17 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Punto de desagüe para aparato sanitario.</t>
+          <t>Refuerzo interior para anclaje de cargas en tabique de yeso laminado.</t>
         </is>
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+          <t>Colocación de refuerzo interior de madera o perfil metálico entre montantes del tabique de yeso laminado, en la posición prevista para colgar mobiliario, televisores, lavamanos suspendidos, barras de apoyo o cualquier carga puntual. Debe replantearse y montarse antes de cerrar el tabique: resolverlo después obliga a abrir la placa. Incluye el replanteo de la altura y posición exactas según el elemento a soportar, el corte y fijación del refuerzo a los montantes, y el registro de su posición en el plano para poder localizarlo una vez cerrado y acabado el tabique. Medido por refuerzo realmente colocado.</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
@@ -8828,11 +8828,11 @@
         <v>1</v>
       </c>
       <c r="F221" t="n">
-        <v>33.84</v>
+        <v>5.93</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>Puntos de desagüe</t>
+          <t>Tabiquería de yeso laminado</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
@@ -8844,33 +8844,33 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Instalaciones eléctricas</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+          <t>Pared de bloque de vidrio.</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+          <t>Paño de bloque de vidrio recibido con mortero, con separadores plásticos que garantizan la constancia de la junta y refuerzo de cabilla en las juntas horizontales y verticales. Aporta luz natural manteniendo la privacidad, y es habitual en baños y en divisiones interiores. Exige un paño con sus cuatro bordes confinados y con junta de dilatación perimetral, ya que el vidrio no admite deformaciones del entorno. Incluye el replanteo del despiece que debe resolverse con piezas enteras porque el bloque no se corta, la colocación con separadores, el armado de las juntas con cabilla, el rejuntado y la limpieza final de las caras. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E222" t="n">
         <v>1</v>
       </c>
       <c r="F222" t="n">
-        <v>8.369999999999999</v>
+        <v>186.85</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>Canalizaciones y cableado</t>
+          <t>Tabiquería de otros materiales</t>
         </is>
       </c>
       <c r="H222" t="inlineStr">
@@ -8882,33 +8882,33 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Instalaciones eléctricas</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+          <t>Tabique de placa de cemento sobre estructura metálica.</t>
         </is>
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+          <t>Tabique autoportante ejecutado con placa de cemento reforzada con fibra sobre estructura de perfiles de acero galvanizado, para áreas húmedas, exteriores protegidos y zonas donde la placa de yeso no es apta. La placa de cemento admite humedad permanente y constituye un soporte estable para recibir enchapado en duchas y fachadas de patio. Incluye el replanteo, el montaje de canales y montantes, el atornillado de las placas con tornillería específica, el tratamiento de juntas con cinta de malla y mortero, y el remate perimetral. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E223" t="n">
         <v>1</v>
       </c>
       <c r="F223" t="n">
-        <v>8.720000000000001</v>
+        <v>53.64</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>Puntos, mecanismos y tomas</t>
+          <t>Tabiquería de otros materiales</t>
         </is>
       </c>
       <c r="H223" t="inlineStr">
@@ -8920,17 +8920,17 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+          <t>Tabique de paneles livianos prefabricados.</t>
         </is>
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Tabique ejecutado con paneles livianos prefabricados de núcleo aligerado y caras de mortero, montados machihembrados entre sí y recibidos en piso y techo. Su ventaja es la rapidez de montaje y el bajo peso propio, lo que lo hace idóneo para dividir sobre losas existentes sin sobrecargarlas, situación frecuente en remodelación de plantas altas. Incluye el replanteo, la fijación de la guía inferior, el montaje de los paneles con adhesivo en las juntas machihembradas, el ajuste y acuñado contra el techo, el sellado del perímetro y el tratamiento de juntas dejando la superficie lista para pintar. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
@@ -8942,11 +8942,11 @@
         <v>1</v>
       </c>
       <c r="F224" t="n">
-        <v>2.82</v>
+        <v>30.12</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>Preparación de soportes</t>
+          <t>Tabiquería de otros materiales</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
@@ -8958,17 +8958,17 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+          <t>División liviana de machihembrado de madera.</t>
         </is>
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>División interior ejecutada con machihembrado de madera sobre rastreles, fijada a piso, techo y paramentos. Se emplea en divisiones ligeras, forros y cerramientos de carácter decorativo o en construcción tradicional. Incluye el replanteo, el montaje y nivelación del rastrelado, la aplicación de preservante en las piezas y muy especialmente en las testas y zonas de apoyo, el montaje del machihembrado con encaje a presión, el remate perimetral con molduras y el lijado final. Medido a cinta corrida descontando huecos mayores de 2 m².</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
@@ -8980,11 +8980,11 @@
         <v>1</v>
       </c>
       <c r="F225" t="n">
-        <v>3.46</v>
+        <v>31.59</v>
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>Pintura interior</t>
+          <t>Tabiquería de otros materiales</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
@@ -8996,33 +8996,33 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Paredes y tabiquería</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+          <t>Dintel prefabricado de concreto sobre vano.</t>
         </is>
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+          <t>Colocación de dintel prefabricado de concreto armado sobre vano de puerta o ventana en pared de mampostería, con la entrega mínima de apoyo a cada lado. Incluye la comprobación de que el apoyo disponible a cada lado alcanza la entrega mínima exigida, requisito del que depende que el dintel trabaje como tal y no se limite a rellenar el hueco, la nivelación del asiento con mortero, la colocación de la pieza a nivel y plomo, el macizado de los apoyos y el relleno de la junta superior. Medido en longitud realmente colocada, incluidas las entregas.</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E226" t="n">
         <v>1</v>
       </c>
       <c r="F226" t="n">
-        <v>5.23</v>
+        <v>13.48</v>
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>Esmaltes sobre madera y metal</t>
+          <t>Dinteles, brocales y remates de vano</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
@@ -9034,36 +9034,910 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
+          <t>Paredes y tabiquería</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Dintel de concreto armado vaciado en sitio.</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="inlineStr">
+        <is>
+          <t>Dintel de concreto armado vaciado en sitio sobre vano de puerta o ventana, con su armado, encofrado y entregas de apoyo. Se emplea cuando la luz del vano, la carga que recibe o la geometría no admiten un dintel prefabricado. Incluye el apeo provisional de la fábrica superior, el armado con sus cabillas y estribos, el encofrado del fondo y los laterales apoyado sobre puntales, el vaciado con concreto de 210 kg/cm2, el vibrado, el curado y el desencofrado y desapeo una vez alcanzada la resistencia. Medido en longitud realmente ejecutada, incluidas las entregas.</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E227" t="n">
+        <v>1</v>
+      </c>
+      <c r="F227" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>Dinteles, brocales y remates de vano</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Paredes y tabiquería</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Brocal o antepecho de ventana.</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr">
+        <is>
+          <t>Formación del brocal o antepecho de ventana en pared de mampostería, con su remate superior conformado con la pendiente hacia el exterior que evacúa el agua de lluvia. Esa pendiente y el goterón inferior son lo que impide que el agua escurra por la fachada y termine filtrando bajo la ventana, patología muy frecuente cuando el brocal se ejecuta plano. Incluye el replanteo de la cota, la ejecución de la fábrica del antepecho, la conformación de la pendiente y del goterón, y el macizado de los apoyos laterales. No incluye el alféizar de acabado. Medido en longitud realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E228" t="n">
+        <v>1</v>
+      </c>
+      <c r="F228" t="n">
+        <v>13.43</v>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>Dinteles, brocales y remates de vano</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Paredes y tabiquería</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Formación de jambas y mochetas de vano.</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr">
+        <is>
+          <t>Formación y repaso de las jambas y mochetas de un vano de puerta o ventana, dejándolas aplomadas, escuadradas y con las dimensiones exactas para recibir la carpintería. Es la operación que determina si la carpintería entra sin forzarla: un vano fuera de escuadra obliga a rehacerlo o a resolverlo con calzos y sellados que se ven. Incluye el repicado de los excesos, el macizado y regularización con mortero de las zonas deficientes, la comprobación de plomos, escuadras y diagonales, y el acabado de la superficie lista para frisar. Medido en longitud de jamba realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E229" t="n">
+        <v>1</v>
+      </c>
+      <c r="F229" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>Dinteles, brocales y remates de vano</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Paredes y tabiquería</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Remate y sellado del encuentro de pared con estructura.</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>Tratamiento del encuentro entre la pared de mampostería o tabiquería y los elementos estructurales de concreto, mediante malla de refuerzo de junta y sellado elástico donde el proyecto prevea movimiento diferencial. La junta entre dos materiales de distinto comportamiento es donde aparece la fisura casi con seguridad si se frisa por encima sin tratarla, y es uno de los defectos por los que más se reclama tras la entrega. Incluye la limpieza y apertura de la junta, la colocación de la malla o banda de refuerzo solapada a ambos lados, la aplicación del sellador elástico donde corresponda y el repaso previo al friso. Medido en longitud de encuentro realmente tratada.</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E230" t="n">
+        <v>1</v>
+      </c>
+      <c r="F230" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>Dinteles, brocales y remates de vano</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Frisos y revestimientos de pared</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Friso de mortero maestreado sobre paramento interior, 1,5 cm de espesor.</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="inlineStr">
+        <is>
+          <t>Friso de mortero de cemento y arena cernida sobre paramento interior de bloque o ladrillo, de 1,5 cm de espesor medio, maestreado y acabado a la llana. Incluye limpieza y humedecido previo del soporte, colocación de maestras y cantoneras en esquinas y encuentros, malla de refuerzo en los cambios de material, tendido y reglado del mortero, y acabado fratasado dejando la superficie plana y aplomada, lista para recibir pintura o revestimiento cerámico. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E231" t="n">
+        <v>1</v>
+      </c>
+      <c r="F231" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>Frisos y enlucidos de mortero</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Frisos y revestimientos de pared</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr">
+        <is>
+          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E232" t="n">
+        <v>1</v>
+      </c>
+      <c r="F232" t="n">
+        <v>10.87</v>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>Enchapado cerámico y porcelanato</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E233" t="n">
+        <v>1</v>
+      </c>
+      <c r="F233" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>Bases, contrapisos y nivelación</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E234" t="n">
+        <v>1</v>
+      </c>
+      <c r="F234" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>Pisos cerámicos y porcelanato</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E235" t="n">
+        <v>1</v>
+      </c>
+      <c r="F235" t="n">
+        <v>12.51</v>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>Pisos cerámicos y porcelanato</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E236" t="n">
+        <v>1</v>
+      </c>
+      <c r="F236" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>Rodapiés y remates de piso</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Cielos rasos</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E237" t="n">
+        <v>1</v>
+      </c>
+      <c r="F237" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>Yeso laminado continuo</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E238" t="n">
+        <v>1</v>
+      </c>
+      <c r="F238" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>Tuberías y montantes de agua</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E239" t="n">
+        <v>1</v>
+      </c>
+      <c r="F239" t="n">
+        <v>37.22</v>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>Puntos de agua</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E240" t="n">
+        <v>1</v>
+      </c>
+      <c r="F240" t="n">
+        <v>13.52</v>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>Llaves y valvulería</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E241" t="n">
+        <v>1</v>
+      </c>
+      <c r="F241" t="n">
+        <v>23.45</v>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Instalación de lavamanos con su grifería y desagüe.</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E242" t="n">
+        <v>1</v>
+      </c>
+      <c r="F242" t="n">
+        <v>36.45</v>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E243" t="n">
+        <v>1</v>
+      </c>
+      <c r="F243" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>Tuberías y bajantes de desagüe</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Punto de desagüe para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E244" t="n">
+        <v>1</v>
+      </c>
+      <c r="F244" t="n">
+        <v>33.84</v>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>Puntos de desagüe</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E245" t="n">
+        <v>1</v>
+      </c>
+      <c r="F245" t="n">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>Canalizaciones y cableado</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E246" t="n">
+        <v>1</v>
+      </c>
+      <c r="F246" t="n">
+        <v>8.720000000000001</v>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>Puntos, mecanismos y tomas</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E247" t="n">
+        <v>1</v>
+      </c>
+      <c r="F247" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>Preparación de soportes</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E248" t="n">
+        <v>1</v>
+      </c>
+      <c r="F248" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>Pintura interior</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E249" t="n">
+        <v>1</v>
+      </c>
+      <c r="F249" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>Esmaltes sobre madera y metal</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
           <t>Gestión de residuos y limpieza</t>
         </is>
       </c>
-      <c r="B227" t="inlineStr">
+      <c r="B250" t="inlineStr">
         <is>
           <t>Retirada y transporte de escombro a vertedero autorizado.</t>
         </is>
       </c>
-      <c r="C227" s="2" t="inlineStr">
+      <c r="C250" s="2" t="inlineStr">
         <is>
           <t>Retirada de escombro procedente de demoliciones desde el punto de acopio de la obra y transporte en camión volqueta hasta vertedero o botadero autorizado, incluido el canon de vertido. Incluye la carga manual del escombro sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado con una distancia media considerada de 25 km, la descarga y la limpieza de la zona de carga. Medido por metro cúbico de escombro esponjado realmente retirado.</t>
         </is>
       </c>
-      <c r="D227" t="inlineStr">
+      <c r="D250" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="E227" t="n">
-        <v>1</v>
-      </c>
-      <c r="F227" t="n">
+      <c r="E250" t="n">
+        <v>1</v>
+      </c>
+      <c r="F250" t="n">
         <v>16.07</v>
       </c>
-      <c r="G227" t="inlineStr">
+      <c r="G250" t="inlineStr">
         <is>
           <t>Retiro y transporte de escombro</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr">
+      <c r="H250" t="inlineStr">
         <is>
           <t>incluida</t>
         </is>

</xml_diff>

<commit_message>
Cerrar el capitulo 07 Frisos y revestimientos de pared con 25 partidas en 5 subcapitulos
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/catalogo_partidas.xlsx
+++ b/basedatos_partidas/salida/catalogo_partidas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H250"/>
+  <dimension ref="A1:H273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9229,12 +9229,12 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
+          <t>Friso de mortero con hidrófugo en paramento exterior.</t>
         </is>
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Friso de mortero de cemento y arena con aditivo hidrófugo de masa, de 2 cm de espesor medio, maestreado y fratasado sobre paramento exterior de bloque o ladrillo. El hidrófugo reduce la absorción capilar del mortero, que es la vía por la que la lluvia batiente termina apareciendo como humedad en la cara interior. Incluye el trabajo desde andamio, la limpieza y humedecido del soporte, la colocación de maestras y cantoneras, la malla de refuerzo en los encuentros de materiales distintos, el tendido y reglado del mortero en dos capas, el fratasado final y el curado durante los primeros días, sin el cual el friso exterior fisura por retracción. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
@@ -9246,11 +9246,11 @@
         <v>1</v>
       </c>
       <c r="F232" t="n">
-        <v>10.87</v>
+        <v>17.52</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
-          <t>Enchapado cerámico y porcelanato</t>
+          <t>Frisos y enlucidos de mortero</t>
         </is>
       </c>
       <c r="H232" t="inlineStr">
@@ -9262,17 +9262,17 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+          <t>Friso rústico texturado en fachada.</t>
         </is>
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+          <t>Revestimiento de fachada con friso rústico texturado, aplicado sobre friso base o directamente sobre la mampostería, con acabado obtenido por proyección o por peinado según la textura elegida. Incluye el trabajo desde andamio, la preparación y humedecido del soporte, la aplicación de la capa base, la ejecución de la textura de forma continua por paños completos entre juntas o quiebres para evitar que se marquen las paradas de trabajo, y el curado. La uniformidad del acabado depende de mantener la misma cuadrilla y la misma dosificación en todo el paño. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -9284,11 +9284,11 @@
         <v>1</v>
       </c>
       <c r="F233" t="n">
-        <v>8.02</v>
+        <v>16.45</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>Bases, contrapisos y nivelación</t>
+          <t>Frisos y enlucidos de mortero</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
@@ -9300,17 +9300,17 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+          <t>Mortero impermeabilizante en área húmeda, base para enchapado.</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Aplicación de mortero impermeabilizante cementoso flexible en dos manos sobre el paramento de zonas de ducha y áreas de contacto directo con agua, como base bajo el enchapado. Es la capa que realmente impide el paso del agua: la cerámica y su boquilla no son estancas, y sin esta base la humedad termina apareciendo en la habitación contigua. Incluye la regularización previa del soporte, el redondeo o refuerzo con banda elástica de los encuentros de pared con piso y de las esquinas, que son los puntos por donde falla el sistema, la aplicación de las dos manos cruzadas respetando el tiempo entre ellas y la prueba de estanqueidad antes de enchapar. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -9322,11 +9322,11 @@
         <v>1</v>
       </c>
       <c r="F234" t="n">
-        <v>9.17</v>
+        <v>12.4</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>Pisos cerámicos y porcelanato</t>
+          <t>Frisos y enlucidos de mortero</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
@@ -9338,17 +9338,17 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+          <t>Regularización y repello de paramento existente.</t>
         </is>
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Regularización de paramento existente mediante repello de mortero de espesor variable, para corregir desplomes, resanar zonas picadas y dejar la superficie apta para recibir el acabado. Se emplea en reforma cuando el friso existente está sano en su mayor parte y solo requiere reparación y nivelación, evitando el picado completo. Incluye el sondeo por golpeo para delimitar y retirar las zonas huecas, la limpieza y humedecido, la aplicación del puente de adherencia en las zonas de mayor espesor, el tendido y reglado del mortero enrasando con el friso existente, y el fratasado dejando una transición imperceptible entre lo nuevo y lo conservado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -9360,11 +9360,11 @@
         <v>1</v>
       </c>
       <c r="F235" t="n">
-        <v>12.51</v>
+        <v>12.23</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>Pisos cerámicos y porcelanato</t>
+          <t>Frisos y enlucidos de mortero</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
@@ -9376,33 +9376,33 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Pisos y pavimentos</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+          <t>Friso de pasta de yeso en paramento interior.</t>
         </is>
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+          <t>Friso de pasta de yeso de 1,2 cm de espesor medio aplicado sobre paramento interior de mampostería, maestreado y acabado a la llana. Frente al friso de mortero ofrece un acabado más liso y un rendimiento notablemente mayor, pero no admite humedad, por lo que queda descartado en baños, cocinas expuestas y paredes en contacto con el exterior. Incluye la limpieza del soporte, la colocación de maestras y cantoneras, el amasado de la pasta en cantidades ajustadas al tiempo de trabajabilidad, el tendido y reglado, y el acabado a la llana hasta dejar la superficie lista para pintar. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E236" t="n">
         <v>1</v>
       </c>
       <c r="F236" t="n">
-        <v>1.69</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>Rodapiés y remates de piso</t>
+          <t>Pastas y acabados de yeso</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
@@ -9414,17 +9414,17 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Cielos rasos</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+          <t>Estucado fino de pasta sobre friso.</t>
         </is>
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+          <t>Capa de acabado fino de pasta aplicada sobre friso de mortero o de yeso, de 2 a 3 mm de espesor, para obtener una superficie tersa apta para pinturas de alto brillo o para acabados donde cualquier irregularidad se marca con la luz rasante. Incluye la comprobación y el sellado previo del soporte, la aplicación de la pasta en dos manos cruzadas con llana, el lijado entre manos y el lijado final con aspiración, y la revisión con luz rasante para detectar y corregir los defectos que solo aparecen bajo esa iluminación. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -9436,11 +9436,11 @@
         <v>1</v>
       </c>
       <c r="F237" t="n">
-        <v>18.47</v>
+        <v>6.38</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>Yeso laminado continuo</t>
+          <t>Pastas y acabados de yeso</t>
         </is>
       </c>
       <c r="H237" t="inlineStr">
@@ -9452,33 +9452,33 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+          <t>Alisado de paramento con pasta de nivelación.</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+          <t>Alisado de paramento existente mediante aplicación de pasta de nivelación a llana, para corregir irregularidades menores, marcas de rodillo, gotelé fino o restos de acabados anteriores, dejando la superficie plana. Es la alternativa económica al picado y refriso cuando el paramento está sano pero con textura o defectos superficiales. Incluye el raspado de las partes sueltas, la aplicación del fondo fijador, el extendido de la pasta en una o dos manos según el defecto a corregir, el lijado con aspiración y el repaso final. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E238" t="n">
         <v>1</v>
       </c>
       <c r="F238" t="n">
-        <v>7.45</v>
+        <v>4.34</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>Tuberías y montantes de agua</t>
+          <t>Pastas y acabados de yeso</t>
         </is>
       </c>
       <c r="H238" t="inlineStr">
@@ -9490,33 +9490,33 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+          <t>Moldura decorativa corrida de yeso.</t>
         </is>
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+          <t>Suministro y colocación de moldura decorativa corrida de yeso o poliuretano en el encuentro de pared y cielo raso o como elemento decorativo en paramento, recibida con pasta de agarre. Incluye el replanteo de la línea de referencia con nivel, el corte a inglete de los encuentros en esquinas interiores y exteriores, la colocación con pasta, el relleno y alisado de las juntas entre piezas hasta hacerlas imperceptibles, y el repaso final dejando la moldura lista para pintar. Medido en longitud realmente colocada.</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E239" t="n">
         <v>1</v>
       </c>
       <c r="F239" t="n">
-        <v>37.22</v>
+        <v>7.77</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>Puntos de agua</t>
+          <t>Pastas y acabados de yeso</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
@@ -9528,33 +9528,33 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+          <t>Reparación puntual de friso de yeso.</t>
         </is>
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+          <t>Reparación de zonas puntuales de friso de yeso deteriorado por golpes, humedades ya resueltas o desprendimientos, con reposición del material y enrase con el friso existente. Incluye la delimitación y retirada del material suelto hasta encontrar friso sano y bien adherido, la limpieza y humedecido del borde, la aplicación del puente de adherencia, la reposición por capas de la pasta, el enrase con la superficie existente y el lijado de la transición. En reparaciones sobre humedades es imprescindible haber eliminado antes la causa, porque de lo contrario la zona vuelve a fallar. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E240" t="n">
         <v>1</v>
       </c>
       <c r="F240" t="n">
-        <v>13.52</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>Llaves y valvulería</t>
+          <t>Pastas y acabados de yeso</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
@@ -9566,33 +9566,33 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+          <t>Alicatado de paramento interior con pieza cerámica o porcelanato, en capa fina.</t>
         </is>
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+          <t>Alicatado de paramento interior en baños, cocinas y áreas húmedas con pieza cerámica o de porcelanato rectificado, sobre soporte previamente frisado y regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE de deslizamiento reducido aplicado con llana dentada, nivelación mediante crucetas y cuñas, y rejuntado con mortero CG2. Incluye replanteo de hiladas para evitar piezas cortadas en zonas vistas, cortes y taladros para el paso de instalaciones y mecanismos, resolución de encuentros y esquinas, y limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E241" t="n">
         <v>1</v>
       </c>
       <c r="F241" t="n">
-        <v>23.45</v>
+        <v>10.87</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Enchapado cerámico y porcelanato</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
@@ -9604,33 +9604,33 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Instalación de lavamanos con su grifería y desagüe.</t>
+          <t>Enchapado de porcelanato de gran formato en pared.</t>
         </is>
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
+          <t>Colocación en pared de pieza de porcelanato rectificado de gran formato, tipo 60x120 cm o superior, en capa fina con adhesivo cementoso mejorado y doble encolado. En vertical el gran formato exige un soporte perfectamente plano y el empleo de sistemas de nivelación y de apoyo provisional que sostengan la pieza mientras el adhesivo agarra, porque su peso tiende a hacerla descolgar. Incluye la comprobación y regularización previa de la planitud, el replanteo del despiece, el doble encolado, la nivelación con cuñas, los cortes con cortadora de disco refrigerada, el rejuntado y la limpieza final. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E242" t="n">
         <v>1</v>
       </c>
       <c r="F242" t="n">
-        <v>36.45</v>
+        <v>14.5</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Enchapado cerámico y porcelanato</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
@@ -9642,33 +9642,33 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+          <t>Enchapado cerámico en fachada o paramento exterior.</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+          <t>Colocación de enchapado cerámico o de porcelanato en fachada o paramento exterior, en capa fina con adhesivo cementoso de altas prestaciones tipo C2 con deslizamiento reducido, con juntas de dilatación en paños y encuentros. En exterior el revestimiento sufre dilataciones térmicas y humedad, de modo que el adhesivo, la junta ancha y las juntas de dilatación dejan de ser opcionales: son lo que impide el desprendimiento de piezas. Incluye el trabajo desde andamio, la comprobación del soporte, el replanteo, el doble encolado, la ejecución de las juntas de dilatación, el rejuntado con mortero para exterior y la limpieza. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E243" t="n">
         <v>1</v>
       </c>
       <c r="F243" t="n">
-        <v>11.04</v>
+        <v>16.33</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>Tuberías y bajantes de desagüe</t>
+          <t>Enchapado cerámico y porcelanato</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
@@ -9680,33 +9680,33 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Punto de desagüe para aparato sanitario.</t>
+          <t>Cenefa o listelo decorativo en enchapado.</t>
         </is>
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+          <t>Colocación de cenefa, listelo o pieza decorativa corrida dentro del enchapado cerámico, recibida con adhesivo y rejuntada a juego. Incluye el replanteo de la línea que debe coordinarse con el despiece general para que la cenefa coincida con la junta de las piezas y no obligue a cortes forzados, la colocación pieza a pieza con nivelación, los cortes de ajuste en esquinas y encuentros, el rejuntado y la limpieza. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente colocada.</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E244" t="n">
         <v>1</v>
       </c>
       <c r="F244" t="n">
-        <v>33.84</v>
+        <v>2.99</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>Puntos de desagüe</t>
+          <t>Enchapado cerámico y porcelanato</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
@@ -9718,17 +9718,17 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Instalaciones eléctricas</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+          <t>Perfil de remate, esquinero o transición en enchapado.</t>
         </is>
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+          <t>Suministro y colocación de perfil de aluminio o PVC de remate, esquinero o transición en el enchapado, recibido con el propio adhesivo bajo el borde de la pieza. Protege la arista del enchapado, que es donde se producen los desportillados, y resuelve el encuentro entre materiales distintos con una línea limpia. Incluye el replanteo, el corte a medida y a inglete en los encuentros, la colocación embebida en el adhesivo antes de asentar la pieza contigua y la limpieza. Medido en longitud realmente colocada.</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -9740,11 +9740,11 @@
         <v>1</v>
       </c>
       <c r="F245" t="n">
-        <v>8.369999999999999</v>
+        <v>5.25</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>Canalizaciones y cableado</t>
+          <t>Enchapado cerámico y porcelanato</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
@@ -9756,33 +9756,33 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Instalaciones eléctricas</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+          <t>Enchapado de mármol o granito en pared, colocación en capa fina.</t>
         </is>
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+          <t>Colocación en pared de pieza de mármol o granito en capa fina, con adhesivo cementoso blanco de altas prestaciones. El adhesivo blanco no es un capricho: los mármoles claros son translúcidos y un adhesivo gris se transparenta y mancha la pieza de forma irreversible. Incluye la comprobación y regularización del soporte, el replanteo del despiece atendiendo a la veta y al tono para que la composición sea continua, el doble encolado, la nivelación, los cortes con disco refrigerado, el rejuntado con junta mínima a juego y la limpieza con productos no ácidos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E246" t="n">
         <v>1</v>
       </c>
       <c r="F246" t="n">
-        <v>8.720000000000001</v>
+        <v>14.61</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
-          <t>Puntos, mecanismos y tomas</t>
+          <t>Enchapado de piedra natural</t>
         </is>
       </c>
       <c r="H246" t="inlineStr">
@@ -9794,17 +9794,17 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+          <t>Enchapado de laja o piedra natural irregular.</t>
         </is>
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Colocación de laja o piedra natural de formato irregular en paramento interior o exterior, recibida con mortero o adhesivo de alta deformabilidad según el espesor y el peso de la pieza. Al no existir un despiece regular, el trabajo consiste en componer el paño pieza a pieza buscando el encaje y la distribución de tonos, lo que reduce el rendimiento respecto a cualquier enchapado modular. Incluye la selección y clasificación previa del material, el replanteo del paño, la colocación con junta irregular controlada, el rejuntado o el acabado a hueso según el diseño, la limpieza y la aplicación del sellador hidrofugante. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -9816,11 +9816,11 @@
         <v>1</v>
       </c>
       <c r="F247" t="n">
-        <v>2.82</v>
+        <v>23.82</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>Preparación de soportes</t>
+          <t>Enchapado de piedra natural</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
@@ -9832,17 +9832,17 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+          <t>Enchapado de piedra natural con anclaje mecánico.</t>
         </is>
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Colocación de piezas de piedra natural en fachada mediante anclaje mecánico de acero inoxidable, sin depender del adhesivo como elemento portante. Es la solución obligada a partir de cierta altura, espesor o peso de pieza, donde un enchapado adherido no ofrece seguridad suficiente frente al desprendimiento. Incluye el trabajo desde andamio, el replanteo, el taladrado de los alojamientos en el canto de la pieza y en el soporte, la colocación de los anclajes con su resina, el aplomado y nivelación de cada pieza, el sellado de juntas y la limpieza. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -9854,11 +9854,11 @@
         <v>1</v>
       </c>
       <c r="F248" t="n">
-        <v>3.46</v>
+        <v>31.46</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>Pintura interior</t>
+          <t>Enchapado de piedra natural</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
@@ -9870,33 +9870,33 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Frisos y revestimientos de pared</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+          <t>Zócalo de piedra natural.</t>
         </is>
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+          <t>Colocación de zócalo de piedra natural a juego con el piso o el paramento, recibido con adhesivo cementoso blanco. Incluye el replanteo de la altura, los cortes a inglete en esquinas y encuentros, la colocación con nivelación, el rejuntado y el sellado de la junta inferior con el piso. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente colocada.</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E249" t="n">
         <v>1</v>
       </c>
       <c r="F249" t="n">
-        <v>5.23</v>
+        <v>2.95</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>Esmaltes sobre madera y metal</t>
+          <t>Enchapado de piedra natural</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
@@ -9908,36 +9908,910 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
+          <t>Frisos y revestimientos de pared</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Pulido y abrillantado de enchapado de piedra natural.</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>Pulido y abrillantado en obra de enchapado de piedra natural, para igualar el plano entre piezas y recuperar o dar el brillo final. Se ejecuta cuando la piedra se coloca en bruto o cuando los pequeños resaltos entre piezas hacen necesario rectificar el plano completo. Incluye la protección del entorno, el pulido con pasadas sucesivas de grano decreciente con aporte de agua, la recogida y evacuación del lodo generado, el abrillantado con cristalizador, la limpieza y la aplicación del sellador hidrofugante y antimanchas. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E250" t="n">
+        <v>1</v>
+      </c>
+      <c r="F250" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>Enchapado de piedra natural</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Frisos y revestimientos de pared</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Revestimiento de paramento con papel tapiz.</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de papel tapiz sobre paramento interior previamente preparado, con pegamento mural. Incluye la comprobación de que el soporte está liso, seco y con absorción uniforme, condición sin la cual las juntas se abren o se marcan las irregularidades, la aplicación del fondo sellador, el replanteo de la primera plomada, el corte de los paños respetando el ajuste del dibujo, el encolado y colocación con eliminación de burbujas y arrugas, el recorte de los excesos en rodapié y cielo, y la limpieza de restos de pegamento. El papel lo elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E251" t="n">
+        <v>1</v>
+      </c>
+      <c r="F251" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>Revestimientos decorativos y especiales</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Frisos y revestimientos de pared</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Estuco veneciano o acabado decorativo mineral.</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>Acabado decorativo tipo estuco veneciano a la cal, aplicado en varias capas a espátula sobre paramento interior preparado, con bruñido final que produce el brillo característico. Es un trabajo de acabado puro en el que el resultado depende casi por completo de la mano del aplicador, por lo que conviene ejecutar una muestra previa aprobada por el cliente antes de acometer el paño. Incluye la preparación y sellado del soporte, la aplicación de las capas sucesivas con la espátula, el bruñido y el encerado final de protección. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E252" t="n">
+        <v>1</v>
+      </c>
+      <c r="F252" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>Revestimientos decorativos y especiales</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Frisos y revestimientos de pared</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Revestimiento de paramento con paneles decorativos.</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de paneles decorativos de PVC, madera técnica, laminado o material similar sobre paramento interior, montados sobre rastrelado o adheridos según el sistema. Incluye el replanteo del despiece para centrar el paño y evitar piezas estrechas en los bordes, el montaje y nivelación del rastrelado cuando el sistema lo requiera, la colocación de los paneles con su sistema de encaje o adhesivo, el ajuste alrededor de mecanismos y huecos, y la colocación de los perfiles de remate perimetrales. El panel lo elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E253" t="n">
+        <v>1</v>
+      </c>
+      <c r="F253" t="n">
+        <v>13.64</v>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>Revestimientos decorativos y especiales</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Frisos y revestimientos de pared</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Forro de pared con machihembrado de madera.</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>Forro de paramento interior con machihembrado de madera montado sobre rastrelado fijado a la pared, con cámara de ventilación posterior. La cámara y el tratamiento preservante son lo que evita que la madera se pudra por la humedad que pueda transmitir el muro, problema habitual cuando el machihembrado se clava directamente contra el paramento. Incluye el replanteo, el montaje y nivelación del rastrelado, la aplicación del preservante en todas las caras y testas, el montaje del machihembrado con encaje a presión, el remate perimetral con molduras y el lijado final. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E254" t="n">
+        <v>1</v>
+      </c>
+      <c r="F254" t="n">
+        <v>30.64</v>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>Revestimientos decorativos y especiales</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Frisos y revestimientos de pared</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Revestimiento continuo de microcemento en paramento vertical.</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>Revestimiento continuo de microcemento en paramento vertical, aplicado en capas sucesivas con malla de refuerzo, con acabado sellado. Ofrece una superficie continua sin juntas, muy demandada en baños y espacios contemporáneos, pero es extremadamente sensible a la calidad del soporte: cualquier fisura o movimiento del paramento se refleja en el acabado. Incluye la comprobación y estabilización del soporte, la imprimación, la aplicación de la capa base con malla, las capas de acabado con la textura elegida, el lijado entre capas y la aplicación de las manos de sellador protector. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E255" t="n">
+        <v>1</v>
+      </c>
+      <c r="F255" t="n">
+        <v>42.94</v>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>Revestimientos decorativos y especiales</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Recrecido con mortero autonivelante de 5 mm de espesor medio.</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>Regularización de soporte mediante mortero autonivelante de base cemento, de 5 mm de espesor medio, para dejar la superficie en condiciones de planitud aptas para recibir pavimento cerámico, incluso de gran formato. Incluye limpieza y aspirado previo del soporte, aplicación de imprimación tapaporos para regular la absorción, colocación de banda perimetral de desolidarización, amasado mecánico, vertido, extendido y desaireado del producto, y espera hasta transitabilidad. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E256" t="n">
+        <v>1</v>
+      </c>
+      <c r="F256" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>Bases, contrapisos y nivelación</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E257" t="n">
+        <v>1</v>
+      </c>
+      <c r="F257" t="n">
+        <v>9.17</v>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>Pisos cerámicos y porcelanato</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E258" t="n">
+        <v>1</v>
+      </c>
+      <c r="F258" t="n">
+        <v>12.51</v>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>Pisos cerámicos y porcelanato</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E259" t="n">
+        <v>1</v>
+      </c>
+      <c r="F259" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>Rodapiés y remates de piso</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Cielos rasos</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E260" t="n">
+        <v>1</v>
+      </c>
+      <c r="F260" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>Yeso laminado continuo</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E261" t="n">
+        <v>1</v>
+      </c>
+      <c r="F261" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>Tuberías y montantes de agua</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E262" t="n">
+        <v>1</v>
+      </c>
+      <c r="F262" t="n">
+        <v>37.22</v>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>Puntos de agua</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E263" t="n">
+        <v>1</v>
+      </c>
+      <c r="F263" t="n">
+        <v>13.52</v>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>Llaves y valvulería</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E264" t="n">
+        <v>1</v>
+      </c>
+      <c r="F264" t="n">
+        <v>23.45</v>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Instalación de lavamanos con su grifería y desagüe.</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E265" t="n">
+        <v>1</v>
+      </c>
+      <c r="F265" t="n">
+        <v>36.45</v>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E266" t="n">
+        <v>1</v>
+      </c>
+      <c r="F266" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>Tuberías y bajantes de desagüe</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Punto de desagüe para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E267" t="n">
+        <v>1</v>
+      </c>
+      <c r="F267" t="n">
+        <v>33.84</v>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Puntos de desagüe</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E268" t="n">
+        <v>1</v>
+      </c>
+      <c r="F268" t="n">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>Canalizaciones y cableado</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E269" t="n">
+        <v>1</v>
+      </c>
+      <c r="F269" t="n">
+        <v>8.720000000000001</v>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>Puntos, mecanismos y tomas</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E270" t="n">
+        <v>1</v>
+      </c>
+      <c r="F270" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>Preparación de soportes</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E271" t="n">
+        <v>1</v>
+      </c>
+      <c r="F271" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>Pintura interior</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E272" t="n">
+        <v>1</v>
+      </c>
+      <c r="F272" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>Esmaltes sobre madera y metal</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
           <t>Gestión de residuos y limpieza</t>
         </is>
       </c>
-      <c r="B250" t="inlineStr">
+      <c r="B273" t="inlineStr">
         <is>
           <t>Retirada y transporte de escombro a vertedero autorizado.</t>
         </is>
       </c>
-      <c r="C250" s="2" t="inlineStr">
+      <c r="C273" s="2" t="inlineStr">
         <is>
           <t>Retirada de escombro procedente de demoliciones desde el punto de acopio de la obra y transporte en camión volqueta hasta vertedero o botadero autorizado, incluido el canon de vertido. Incluye la carga manual del escombro sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado con una distancia media considerada de 25 km, la descarga y la limpieza de la zona de carga. Medido por metro cúbico de escombro esponjado realmente retirado.</t>
         </is>
       </c>
-      <c r="D250" t="inlineStr">
+      <c r="D273" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="E250" t="n">
-        <v>1</v>
-      </c>
-      <c r="F250" t="n">
+      <c r="E273" t="n">
+        <v>1</v>
+      </c>
+      <c r="F273" t="n">
         <v>16.07</v>
       </c>
-      <c r="G250" t="inlineStr">
+      <c r="G273" t="inlineStr">
         <is>
           <t>Retiro y transporte de escombro</t>
         </is>
       </c>
-      <c r="H250" t="inlineStr">
+      <c r="H273" t="inlineStr">
         <is>
           <t>incluida</t>
         </is>

</xml_diff>

<commit_message>
Cerrar el capitulo 08 Pisos y pavimentos con 39 partidas en 8 subcapitulos
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/catalogo_partidas.xlsx
+++ b/basedatos_partidas/salida/catalogo_partidas.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H273"/>
+  <dimension ref="A1:H308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10179,12 +10179,12 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
+          <t>Contrapiso de mortero de nivelación, 4 cm de espesor.</t>
         </is>
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Contrapiso de mortero de cemento y arena de 4 cm de espesor medio, maestreado y reglado, ejecutado sobre losa o base compactada para recibir el piso de acabado. Es la capa que define el nivel y la planitud definitivos del piso, de modo que los defectos que se dejen aquí se arrastran a todo el acabado posterior. Incluye la limpieza y humedecido del soporte, la colocación de maestras a la cota de proyecto, el tendido y reglado del mortero, el fratasado de la superficie y el curado durante los primeros días. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -10196,11 +10196,11 @@
         <v>1</v>
       </c>
       <c r="F257" t="n">
-        <v>9.17</v>
+        <v>17.86</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>Pisos cerámicos y porcelanato</t>
+          <t>Bases, contrapisos y nivelación</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
@@ -10217,12 +10217,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
+          <t>Contrapiso de concreto sobre terreno, 8 cm de espesor.</t>
         </is>
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Contrapiso de concreto de 8 cm de espesor con malla electrosoldada de retracción, vaciado sobre base de piedra picada compactada y barrera de vapor, con juntas de control aserradas. Incluye la comprobación de la base, la colocación de la barrera de vapor y de la malla sobre separadores, el vaciado y vibrado, el reglado a nivel, el fratasado, el aserrado de las juntas de control en el momento adecuado, que es lo que evita la fisuración anárquica por retracción, y el curado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -10234,11 +10234,11 @@
         <v>1</v>
       </c>
       <c r="F258" t="n">
-        <v>12.51</v>
+        <v>24.83</v>
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>Pisos cerámicos y porcelanato</t>
+          <t>Bases, contrapisos y nivelación</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
@@ -10255,28 +10255,28 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+          <t>Nivelación con mortero seco compactado.</t>
         </is>
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+          <t>Capa de nivelación con mortero seco de consistencia de tierra húmeda, extendido y compactado, empleada cuando hay que salvar desniveles importantes o embeber instalaciones bajo el piso sin recurrir a un espesor de mortero convencional que resultaría costoso y pesado. Incluye la limpieza del soporte, el replanteo de niveles con maestras, el extendido y compactado del mortero por capas, el reglado final y la aplicación de la lechada de cierre superficial que sella la capa y permite recibir el adhesivo del piso. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E259" t="n">
         <v>1</v>
       </c>
       <c r="F259" t="n">
-        <v>1.69</v>
+        <v>21.62</v>
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>Rodapiés y remates de piso</t>
+          <t>Bases, contrapisos y nivelación</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
@@ -10288,17 +10288,17 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Cielos rasos</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+          <t>Preparación y puente de adherencia sobre losa existente.</t>
         </is>
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+          <t>Preparación de losa o piso existente que permanece como base, mediante limpieza, saneado y aplicación de puente de adherencia, para recibir una capa de recrecido o un piso adherido. Se emplea en reforma cuando no se demuele la base y hay que garantizar que la capa nueva no se despegue. Incluye el sondeo por golpeo y el saneado de las zonas huecas, el desengrasado y eliminación de restos de adhesivos o pinturas, el aspirado del polvo, la apertura del poro mediante lijado o repicado ligero y la aplicación del puente de adherencia respetando el tiempo abierto antes de recibir la capa siguiente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -10310,11 +10310,11 @@
         <v>1</v>
       </c>
       <c r="F260" t="n">
-        <v>18.47</v>
+        <v>7.19</v>
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>Yeso laminado continuo</t>
+          <t>Bases, contrapisos y nivelación</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
@@ -10326,33 +10326,33 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+          <t>Colocación de pavimento cerámico o porcelanato de formato estándar, en capa fina.</t>
         </is>
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+          <t>Colocación de pavimento con pieza cerámica o de porcelanato de formato estándar, hasta 60x60 cm, sobre soporte previamente regularizado y limpio. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE aplicado con llana dentada y doble encolado en la pieza, nivelación con sistema de crucetas y cuñas, y rejuntado con mortero cementoso CG2 en el color elegido. Incluye replanteo previo para centrar el despiece, cortes y ajustes en encuentros y pasos de instalaciones, limpieza final de la superficie y retirada de restos. La pieza cerámica la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E261" t="n">
         <v>1</v>
       </c>
       <c r="F261" t="n">
-        <v>7.45</v>
+        <v>9.17</v>
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>Tuberías y montantes de agua</t>
+          <t>Pisos cerámicos y porcelanato</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
@@ -10364,33 +10364,33 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+          <t>Colocación de pavimento de porcelanato de gran formato, en capa fina.</t>
         </is>
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+          <t>Colocación de pavimento con pieza de porcelanato rectificado de gran formato, tipo 120x60 cm o superior, sobre soporte previamente regularizado. Ejecución en capa fina con adhesivo cementoso mejorado C2 TE mediante doble encolado, manipulación de las piezas con juego de ventosas, nivelación con cuñas para garantizar la planitud que exige el formato y junta mínima rejuntada con mortero CG2. Incluye comprobación previa de la planitud del soporte, replanteo del despiece, cortes con cortadora de disco de diamante refrigerada por agua, limpieza final y retirada de restos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E262" t="n">
         <v>1</v>
       </c>
       <c r="F262" t="n">
-        <v>37.22</v>
+        <v>12.51</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t>Puntos de agua</t>
+          <t>Pisos cerámicos y porcelanato</t>
         </is>
       </c>
       <c r="H262" t="inlineStr">
@@ -10402,33 +10402,33 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+          <t>Piso cerámico en área húmeda con pendiente a desagüe.</t>
         </is>
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+          <t>Colocación de piso cerámico o de porcelanato en área húmeda, con formación de las pendientes hacia el desagüe y tratamiento del encuentro con el sumidero. La ejecución correcta de la pendiente es lo que determina que el agua evacúe y no quede empozada, defecto que en una ducha o en un lavadero se detecta el primer día de uso. Incluye el replanteo de las pendientes desde los bordes hacia el desagüe, el corte y ajuste de las piezas alrededor del sumidero, el doble encolado, la nivelación respetando la pendiente, el rejuntado con mortero apto para zonas húmedas y el sellado elástico del encuentro con paredes y con el sumidero. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E263" t="n">
         <v>1</v>
       </c>
       <c r="F263" t="n">
-        <v>13.52</v>
+        <v>13.18</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>Llaves y valvulería</t>
+          <t>Pisos cerámicos y porcelanato</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
@@ -10440,33 +10440,33 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+          <t>Piso cerámico en terraza o área exterior.</t>
         </is>
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+          <t>Colocación de piso cerámico o de porcelanato en terraza, patio o área exterior, con adhesivo cementoso de altas prestaciones, junta ancha y juntas de dilatación perimetrales y en paños. En exterior el piso sufre dilataciones térmicas y humedad bajo la pieza, de modo que la junta ancha y las juntas de dilatación son las que evitan el abombamiento y el desprendimiento por acumulación de tensiones. Incluye la comprobación de la pendiente de evacuación del soporte, el replanteo, el doble encolado, la ejecución de las juntas de dilatación, el rejuntado con mortero para exterior y el sellado perimetral. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E264" t="n">
         <v>1</v>
       </c>
       <c r="F264" t="n">
-        <v>23.45</v>
+        <v>13.86</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Pisos cerámicos y porcelanato</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
@@ -10478,33 +10478,33 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Instalación de lavamanos con su grifería y desagüe.</t>
+          <t>Piso cerámico colocado en capa gruesa sobre mortero.</t>
         </is>
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
+          <t>Colocación de piso cerámico por el método tradicional de capa gruesa, asentando la pieza sobre una capa de mortero fresco que a la vez recibe la pieza y forma el nivel. Se emplea cuando el soporte presenta desniveles que harían inviable la capa fina, ya que permite corregir cota y planitud en una sola operación, aunque exige más material y más pericia del solador. Incluye el replanteo de niveles con maestras, el extendido del mortero, la espolvoreada de cemento, el asentado y golpeteo de la pieza hasta el nivel, la comprobación continua con regla y nivel, el rejuntado y la limpieza. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E265" t="n">
         <v>1</v>
       </c>
       <c r="F265" t="n">
-        <v>36.45</v>
+        <v>19.41</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>Aparatos sanitarios y grifería</t>
+          <t>Pisos cerámicos y porcelanato</t>
         </is>
       </c>
       <c r="H265" t="inlineStr">
@@ -10516,33 +10516,33 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+          <t>Piso de mármol o granito en capa fina.</t>
         </is>
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+          <t>Colocación de piso de mármol o granito en capa fina con adhesivo cementoso blanco de altas prestaciones, con junta mínima. El adhesivo blanco es obligado en mármoles claros porque el gris se transparenta a través de la pieza y produce manchas irreversibles. Incluye la comprobación y regularización previa del soporte, el replanteo del despiece atendiendo a la veta y al tono para que la composición sea continua, el doble encolado, la nivelación con cuñas, los cortes con disco refrigerado, el rejuntado a juego y la limpieza con productos no ácidos, ya que el ácido ataca el mármol de forma permanente. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E266" t="n">
         <v>1</v>
       </c>
       <c r="F266" t="n">
-        <v>11.04</v>
+        <v>15.31</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
-          <t>Tuberías y bajantes de desagüe</t>
+          <t>Pisos de piedra natural y granito</t>
         </is>
       </c>
       <c r="H266" t="inlineStr">
@@ -10554,33 +10554,33 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Instalaciones sanitarias</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Punto de desagüe para aparato sanitario.</t>
+          <t>Piso de granito vaciado en sitio.</t>
         </is>
       </c>
       <c r="C267" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+          <t>Piso continuo de granito vaciado en sitio, formado por capa de mortero con grano de mármol, dividida en paños mediante platinas divisorias, con pulido y abrillantado final. Es un piso tradicional muy usado en Venezuela, de gran durabilidad y sin juntas de pieza, cuyo resultado depende de la homogeneidad de la mezcla y de la ejecución del pulido. Incluye la preparación del soporte, el replanteo y colocación de las platinas divisorias que absorben la retracción y definen los paños, el vaciado y reglado de la capa de grano, el curado, el pulido en pasadas de grano decreciente con aporte de agua, el resane de poros y el abrillantado final. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E267" t="n">
         <v>1</v>
       </c>
       <c r="F267" t="n">
-        <v>33.84</v>
+        <v>49.71</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>Puntos de desagüe</t>
+          <t>Pisos de piedra natural y granito</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
@@ -10592,33 +10592,33 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Instalaciones eléctricas</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+          <t>Piso de laja o piedra natural irregular.</t>
         </is>
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+          <t>Colocación de piso de laja o piedra natural de formato irregular, recibida con mortero o adhesivo de alta deformabilidad según el espesor de la pieza. Al no existir despiece regular, el paño se compone pieza a pieza buscando el encaje y la distribución de tonos, lo que reduce sensiblemente el rendimiento. Incluye la selección y clasificación previa del material, el replanteo del paño, la colocación con junta irregular controlada, el rejuntado, la limpieza y la aplicación del sellador hidrofugante que protege la piedra y facilita su mantenimiento. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E268" t="n">
         <v>1</v>
       </c>
       <c r="F268" t="n">
-        <v>8.369999999999999</v>
+        <v>23.21</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>Canalizaciones y cableado</t>
+          <t>Pisos de piedra natural y granito</t>
         </is>
       </c>
       <c r="H268" t="inlineStr">
@@ -10630,33 +10630,33 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Instalaciones eléctricas</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+          <t>Piso de baldosa de granito prefabricado.</t>
         </is>
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+          <t>Colocación de piso con baldosa de granito o terrazo prefabricado, recibida con mortero o adhesivo según el espesor, con pulido de igualación en obra. Incluye el replanteo del despiece, la colocación con nivelación y junta mínima, el rejuntado con lechada de cemento a juego, el pulido de igualación que elimina los resaltos entre piezas y unifica el plano, el resane de poros y el abrillantado. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>ud</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="E269" t="n">
         <v>1</v>
       </c>
       <c r="F269" t="n">
-        <v>8.720000000000001</v>
+        <v>24.78</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>Puntos, mecanismos y tomas</t>
+          <t>Pisos de piedra natural y granito</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
@@ -10668,17 +10668,17 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+          <t>Pulido y abrillantado de piso de piedra existente.</t>
         </is>
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Pulido y abrillantado de piso existente de mármol, granito o terrazo, para recuperar el brillo perdido y eliminar rayaduras y manchas superficiales. Es una alternativa muy rentable frente a la sustitución del piso, ya que devuelve el aspecto original a una fracción del costo. Incluye la protección del entorno y de los rodapiés, el pulido con pasadas sucesivas de grano decreciente con aporte de agua, la recogida y evacuación del lodo generado, el resane de poros y pequeños desconchados, el abrillantado con cristalizador y la aplicación del sellador antimanchas. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -10690,11 +10690,11 @@
         <v>1</v>
       </c>
       <c r="F270" t="n">
-        <v>2.82</v>
+        <v>12.88</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>Preparación de soportes</t>
+          <t>Pisos de piedra natural y granito</t>
         </is>
       </c>
       <c r="H270" t="inlineStr">
@@ -10706,17 +10706,17 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+          <t>Piso laminado flotante con manta acústica.</t>
         </is>
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+          <t>Colocación de piso laminado flotante sobre manta acústica, montado por encastre sin adhesivo, con junta perimetral de dilatación. El sistema flotante exige que la junta perimetral quede libre en todo el contorno y oculta bajo el rodapié: si el piso queda a tope contra la pared, al dilatar se abomba y levanta. Incluye la comprobación de la planitud y humedad del contrapiso, el extendido de la manta con solapes sellados, el replanteo del sentido de las tablas y del ancho de la última hilera, el montaje por encastre con cuñas perimetrales, los cortes de ajuste en marcos y tuberías y el retiro de las cuñas. El piso lo elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -10728,11 +10728,11 @@
         <v>1</v>
       </c>
       <c r="F271" t="n">
-        <v>3.46</v>
+        <v>4.89</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>Pintura interior</t>
+          <t>Pisos de madera y laminados</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
@@ -10744,17 +10744,17 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Pintura y acabados</t>
+          <t>Pisos y pavimentos</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+          <t>Piso de madera maciza clavada sobre rastreles.</t>
         </is>
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+          <t>Piso de tabla de madera maciza clavada sobre rastreles fijados al contrapiso, con cámara ventilada. Es la solución tradicional y la más duradera, ya que la madera maciza admite varios lijados a lo largo de su vida. Incluye la aplicación de preservante en los rastreles y en la cara inferior de la tabla, el replanteo y nivelación del rastrelado, la ventilación de la cámara mediante rejillas perimetrales, el clavado oculto de la tabla, la junta perimetral de dilatación y el remate. No incluye el lijado y barnizado final, que se valora aparte. La madera la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -10766,11 +10766,11 @@
         <v>1</v>
       </c>
       <c r="F272" t="n">
-        <v>5.23</v>
+        <v>15.04</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>Esmaltes sobre madera y metal</t>
+          <t>Pisos de madera y laminados</t>
         </is>
       </c>
       <c r="H272" t="inlineStr">
@@ -10782,36 +10782,1366 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Piso de parquet encolado sobre contrapiso.</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de parquet encolado directamente sobre el contrapiso con adhesivo de poliuretano, sin rastreles. Exige un contrapiso perfectamente plano, seco y sin humedad residual: el parquet encolado sobre una base húmeda se abomba y se despega sin remedio, por lo que la medición de humedad del soporte antes de colocar no es un trámite sino la condición del trabajo. Incluye la comprobación de planitud y humedad, la imprimación del soporte si el adhesivo la requiere, el replanteo del despiece, el encolado y colocación con presión, la junta perimetral y el retiro de restos de adhesivo. No incluye el lijado y barnizado. El parquet lo elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E273" t="n">
+        <v>1</v>
+      </c>
+      <c r="F273" t="n">
+        <v>12.93</v>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>Pisos de madera y laminados</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Lijado y barnizado de piso de madera.</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>Lijado y acabado con barniz de poliuretano de piso de madera nuevo o existente, en tres manos con lijado intermedio. En pisos existentes esta operación recupera por completo el aspecto de la madera y evita su sustitución. Incluye el hundido de las puntas que sobresalgan y el resane de juntas y grietas con masilla al tono, el lijado en pasadas de grano decreciente con lijadora de banda y orilladora en perímetros y rincones, el aspirado exhaustivo entre pasadas porque cualquier partícula queda atrapada bajo el barniz, la aplicación de las manos de barniz con lijado suave intermedio y el respeto de los tiempos de secado antes de pisar. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E274" t="n">
+        <v>1</v>
+      </c>
+      <c r="F274" t="n">
+        <v>12.91</v>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Pisos de madera y laminados</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Piso de deck de madera o madera técnica para exterior.</t>
+        </is>
+      </c>
+      <c r="C275" s="2" t="inlineStr">
+        <is>
+          <t>Piso de deck para exterior con tablas de madera tratada o madera técnica, montado sobre rastreles con separación entre tablas para el drenaje y la ventilación. La separación entre tablas y la ventilación inferior no son estéticas: son lo que permite que el agua evacúe y que la madera seque, evitando la pudrición. Incluye el replanteo y nivelación del rastrelado con pendiente de evacuación, la aplicación de preservante en los cortes y testas, el montaje de las tablas con clip oculto o tornillo de acero inoxidable, la separación constante mediante plantilla y el remate perimetral. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E275" t="n">
+        <v>1</v>
+      </c>
+      <c r="F275" t="n">
+        <v>29.69</v>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>Pisos de madera y laminados</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Piso vinílico en lámina.</t>
+        </is>
+      </c>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de piso vinílico en lámina continua, encolado al contrapiso, con soldadura o sellado de las juntas entre paños. Su ventaja frente a la baldosa es la ausencia casi total de juntas, lo que lo hace idóneo en áreas de higiene exigente. Requiere un soporte perfectamente liso, ya que el vinílico es un material fino que copia y hace visible cualquier grano o irregularidad del contrapiso. Incluye la nivelación fina previa si el soporte la requiere, el corte y presentado de los paños dejándolos relajar, el encolado, el paso de rodillo para eliminar aire, la soldadura o sellado de juntas y el remate perimetral. El material lo elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E276" t="n">
+        <v>1</v>
+      </c>
+      <c r="F276" t="n">
+        <v>5.02</v>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>Pisos vinílicos y flexibles</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Piso vinílico en baldosa o lama.</t>
+        </is>
+      </c>
+      <c r="C277" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de piso vinílico en baldosa o lama, tipo LVT, autoadhesivo, encolado o de encastre según el sistema. Combina la facilidad de reposición pieza a pieza con un aspecto muy próximo al de la madera o la piedra. Incluye la comprobación de planitud, limpieza y humedad del soporte, el replanteo del despiece para centrar el paño y evitar piezas estrechas en los bordes, la colocación con junta a matajunta, el paso de rodillo en los sistemas encolados, los cortes de ajuste en marcos y tuberías y el remate perimetral. El material lo elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E277" t="n">
+        <v>1</v>
+      </c>
+      <c r="F277" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>Pisos vinílicos y flexibles</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Piso de caucho o pavimento deportivo.</t>
+        </is>
+      </c>
+      <c r="C278" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de piso de caucho en rollo o en losetas, encolado al soporte, para gimnasios, áreas deportivas, cuartos de máquinas y zonas de tránsito intenso. Incluye la preparación y nivelación del soporte, el corte y presentado del material dejándolo relajar para que recupere su dimensión antes de fijarlo, el encolado, el paso de rodillo, el ajuste y sellado de juntas y el remate perimetral con media caña o perfil. El material lo elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E278" t="n">
+        <v>1</v>
+      </c>
+      <c r="F278" t="n">
+        <v>5.79</v>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Pisos vinílicos y flexibles</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Alfombra o moqueta.</t>
+        </is>
+      </c>
+      <c r="C279" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de alfombra o moqueta, mediante encolado directo o sistema de tiras tensoras según el tipo, con su remate perimetral. Incluye la comprobación de limpieza y sequedad del soporte, la colocación de la manta base cuando el sistema lo requiera, el corte y presentado de los paños respetando el sentido del pelo, que debe ser el mismo en todo el ambiente porque de lo contrario los paños se ven de distinto tono, el encolado o tensado, el sellado de las uniones y el remate en umbrales y perímetro. El material lo elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E279" t="n">
+        <v>1</v>
+      </c>
+      <c r="F279" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Pisos vinílicos y flexibles</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Piso de concreto alisado mecánicamente.</t>
+        </is>
+      </c>
+      <c r="C280" s="2" t="inlineStr">
+        <is>
+          <t>Piso continuo de concreto con acabado alisado mecánicamente mediante alisadora de aspas, con juntas de control aserradas y curado. Incluye el vaciado y reglado del concreto, el flotado inicial, el alisado mecánico en las pasadas necesarias hasta obtener la textura y el cerrado de poro requeridos, el aserrado de las juntas de control en el momento en que el concreto lo admite sin desgranarse ni fisurar, y el curado, que en un piso alisado es determinante porque toda la calidad superficial se pierde si el agua de fraguado se evapora demasiado rápido. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E280" t="n">
+        <v>1</v>
+      </c>
+      <c r="F280" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Pisos continuos de concreto y microcemento</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Piso de concreto estampado.</t>
+        </is>
+      </c>
+      <c r="C281" s="2" t="inlineStr">
+        <is>
+          <t>Piso de concreto con acabado estampado mediante moldes texturados y desmoldeante pigmentado, con sellado final. Se emplea en accesos, patios y áreas exteriores donde se busca el aspecto de piedra o adoquín con la continuidad de un piso de concreto. Incluye el vaciado y reglado, la aplicación del endurecedor color en polvo, la espolvoreada del desmoldeante pigmentado, el estampado con los moldes en el punto exacto de fraguado, ventana de tiempo estrecha de la que depende por completo el resultado, el aserrado de juntas, el lavado del exceso de desmoldeante y la aplicación de las manos de sellador. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E281" t="n">
+        <v>1</v>
+      </c>
+      <c r="F281" t="n">
+        <v>38.82</v>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Pisos continuos de concreto y microcemento</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Piso continuo de microcemento.</t>
+        </is>
+      </c>
+      <c r="C282" s="2" t="inlineStr">
+        <is>
+          <t>Revestimiento continuo de microcemento sobre piso existente o contrapiso, aplicado en capas con malla de refuerzo y sellado con varias manos de barniz de protección. Permite renovar un piso sin demolerlo y sin apenas ganar cota, lo que en reforma resuelve el problema de los umbrales y las puertas. Es muy sensible al soporte: cualquier fisura o movimiento se refleja en el acabado. Incluye la comprobación y estabilización del soporte, la imprimación, la capa base con malla, las capas de acabado con la textura elegida, el lijado entre capas y las manos de sellador de alto tránsito. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E282" t="n">
+        <v>1</v>
+      </c>
+      <c r="F282" t="n">
+        <v>47.79</v>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>Pisos continuos de concreto y microcemento</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Piso epóxico autonivelante.</t>
+        </is>
+      </c>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>Piso continuo de resina epóxica autonivelante, con imprimación y capa de acabado, para áreas industriales, cocinas, laboratorios y estacionamientos. Ofrece una superficie sin juntas, impermeable y resistente a productos químicos. Exige un soporte con humedad por debajo del límite del fabricante: aplicado sobre concreto húmedo, la presión de vapor despega la resina en escamas. Incluye el granallado o lijado del soporte para abrir el poro, la medición de humedad, la imprimación, el sellado de fisuras y juntas, la aplicación de la capa autonivelante con desaireado por rodillo de púas y el respeto de los tiempos de curado antes de la puesta en servicio. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E283" t="n">
+        <v>1</v>
+      </c>
+      <c r="F283" t="n">
+        <v>35.15</v>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Pisos continuos de concreto y microcemento</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Endurecedor superficial y sellado de piso de concreto.</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
+          <t>Tratamiento de piso de concreto mediante endurecedor superficial espolvoreado y sellado final, para aumentar su resistencia a la abrasión y reducir el desprendimiento de polvo. Es la solución económica para estacionamientos, depósitos y áreas de servicio donde no se justifica un piso epóxico. Incluye la espolvoreada del endurecedor sobre el concreto fresco en el momento adecuado, su incorporación mediante alisado mecánico, el curado y la aplicación de las manos de sellador acrílico una vez seco. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E284" t="n">
+        <v>1</v>
+      </c>
+      <c r="F284" t="n">
+        <v>10.47</v>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>Pisos continuos de concreto y microcemento</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié cerámico o de porcelanato.</t>
+        </is>
+      </c>
+      <c r="C285" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié de pieza cerámica o de porcelanato, a juego con el pavimento, recibido con adhesivo cementoso mejorado C2 TE sobre paramento previamente regularizado. Incluye replanteo, cortes a inglete en esquinas y encuentros, ajuste a los marcos de carpintería, rejuntado con mortero CG2 y sellado de la junta inferior con el pavimento. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud realmente ejecutada, descontando los huecos de paso.</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E285" t="n">
+        <v>1</v>
+      </c>
+      <c r="F285" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Rodapiés y remates de piso</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Rodapié de madera o MDF.</t>
+        </is>
+      </c>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de rodapié de madera o MDF lacado, fijado al paramento con adhesivo y clavado oculto, con cortes a inglete en esquinas. Incluye el replanteo, el corte a inglete en esquinas interiores y exteriores, el ajuste alrededor de los marcos de puerta, la fijación combinando adhesivo y puntas, el relleno y disimulo de los puntos de clavado y el sellado de la junta superior con la pared cuando el acabado lo requiera. El rodapié lo elige el cliente y se presupuesta aparte. Medido en longitud realmente colocada.</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E286" t="n">
+        <v>1</v>
+      </c>
+      <c r="F286" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>Rodapiés y remates de piso</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Rodapié de mortero con media caña sanitaria.</t>
+        </is>
+      </c>
+      <c r="C287" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de rodapié corrido de mortero con media caña en el encuentro con el piso, acabado a la llana. La media caña elimina la arista interior, que es donde se acumula la suciedad y por donde penetra el agua de la limpieza, por lo que es la solución habitual en cocinas industriales, áreas de servicio y locales de higiene exigente. Incluye el replanteo de la altura, la limpieza y humedecido, el tendido del mortero, la conformación de la media caña con plantilla y el fratasado dejando la superficie lista para pintar o sellar. Medido en longitud realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E287" t="n">
+        <v>1</v>
+      </c>
+      <c r="F287" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Rodapiés y remates de piso</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Perfil de transición entre pisos.</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y colocación de perfil de transición de aluminio entre pisos de distinto material o de distinto nivel, generalmente en umbrales de puerta. Resuelve el encuentro protegiendo los cantos de ambos pisos y absorbiendo la diferencia de cota, que es donde se producen los tropiezos y los desportillados. Incluye el replanteo, el corte a medida, el taladrado y fijación con tacos o el encolado según el sistema, y el sellado de los bordes. Medido en longitud realmente colocada.</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E288" t="n">
+        <v>1</v>
+      </c>
+      <c r="F288" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>Rodapiés y remates de piso</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Junta de dilatación en piso.</t>
+        </is>
+      </c>
+      <c r="C289" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de junta de dilatación en piso mediante perfil con elemento elástico, que absorbe los movimientos del soporte e impide que la tensión se descargue rompiendo el piso. Es obligada en paños extensos, en los cambios de ambiente y coincidiendo con las juntas estructurales del edificio: una junta estructural que se cubre con piso continuo se refleja como fisura en pocos meses. Incluye el replanteo coordinado con las juntas del soporte, la formación del alojamiento, la colocación y nivelación del perfil y el sellado de los bordes. Medido en longitud realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E289" t="n">
+        <v>1</v>
+      </c>
+      <c r="F289" t="n">
+        <v>10.17</v>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Rodapiés y remates de piso</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Revestimiento de escalera con cerámica o porcelanato.</t>
+        </is>
+      </c>
+      <c r="C290" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de piezas cerámicas o de porcelanato en huellas y contrahuellas de escalera, con pieza de nariz o canto redondeado. El rendimiento es sensiblemente menor que en un piso corrido por la posición de trabajo, por la fragmentación en peldaños y porque cada huella exige un corte a medida. Incluye el replanteo comprobando que huella y contrahuella se mantengan constantes en todo el tramo, requisito de seguridad porque una diferencia entre peldaños provoca tropiezos, los cortes, el doble encolado, la colocación de la pieza de nariz, el rejuntado y la limpieza. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, desarrollando huella y contrahuella.</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E290" t="n">
+        <v>1</v>
+      </c>
+      <c r="F290" t="n">
+        <v>18.02</v>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>Revestimiento de escaleras</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Revestimiento de escalera con piedra natural.</t>
+        </is>
+      </c>
+      <c r="C291" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de piezas de mármol, granito o piedra natural en huellas y contrahuellas de escalera, recibidas con adhesivo cementoso blanco de altas prestaciones. Es el revestimiento de escalera de menor rendimiento, por el peso de las piezas, la exigencia de nivelación y el corte a medida de cada peldaño. Incluye el replanteo verificando la constancia de huella y contrahuella, el corte y pulido del canto de la huella, el doble encolado, la nivelación, el rejuntado a juego y la limpieza con productos no ácidos. La pieza la elige el cliente y se presupuesta aparte. Medido en superficie realmente ejecutada, desarrollando huella y contrahuella.</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E291" t="n">
+        <v>1</v>
+      </c>
+      <c r="F291" t="n">
+        <v>24.57</v>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Revestimiento de escaleras</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Peldaño de madera sobre escalera de concreto.</t>
+        </is>
+      </c>
+      <c r="C292" s="2" t="inlineStr">
+        <is>
+          <t>Colocación de huella y contrahuella de madera sobre escalera de concreto existente, fijadas con adhesivo y tornillería oculta. Es una solución muy habitual en reforma para renovar una escalera sin demolerla. Incluye la comprobación y regularización de la superficie del peldaño de concreto, la toma de medidas peldaño a peldaño porque en una escalera existente rara vez son todos iguales, el corte y ajuste de cada pieza, el encolado y atornillado oculto, la colocación de la pieza de nariz y el remate lateral. La madera la elige el cliente y se presupuesta aparte. Medido en longitud de peldaño realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E292" t="n">
+        <v>1</v>
+      </c>
+      <c r="F292" t="n">
+        <v>9.49</v>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Revestimiento de escaleras</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Cinta o perfil antideslizante en nariz de peldaño.</t>
+        </is>
+      </c>
+      <c r="C293" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y colocación de cinta o perfil antideslizante en la nariz del peldaño, encolado o atornillado según el sistema. Es un elemento de seguridad exigible en escaleras de uso público y muy recomendable en cualquier escalera con revestimiento pulido, donde el riesgo de resbalón es real. Incluye el replanteo de la línea, la limpieza y desengrasado de la zona de apoyo, el corte a medida, la colocación con presión o el atornillado y el sellado de los extremos. Medido en longitud realmente colocada.</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E293" t="n">
+        <v>1</v>
+      </c>
+      <c r="F293" t="n">
+        <v>7.67</v>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>Revestimiento de escaleras</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Pisos y pavimentos</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Zócalo escalonado de escalera.</t>
+        </is>
+      </c>
+      <c r="C294" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución del zócalo o rodapié escalonado que acompaña a la escalera en su encuentro con el paramento, con la pieza cortada siguiendo el perfil de peldaños. Es el remate que da el acabado a la escalera y el trabajo de rodapié de menor rendimiento, ya que cada pieza exige un corte doble en ángulo ajustado al peldaño. Incluye el replanteo de la línea inclinada, el corte de las piezas siguiendo el perfil, la colocación con adhesivo y nivelación, el rejuntado y el sellado de la junta con el peldaño. La pieza la elige el cliente y se presupuesta aparte. Medido en longitud real de la línea inclinada del zócalo.</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E294" t="n">
+        <v>1</v>
+      </c>
+      <c r="F294" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>Revestimiento de escaleras</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Cielos rasos</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo de placa de yeso laminado, estructura oculta suspendida.</t>
+        </is>
+      </c>
+      <c r="C295" s="2" t="inlineStr">
+        <is>
+          <t>Cielo raso continuo formado por una placa de yeso laminado de 12,5 mm atornillada a estructura oculta de perfilería de acero galvanizado, suspendida de la losa mediante varilla y horquilla, con ángulo perimetral en todo el contorno. Incluye replanteo y nivelación con manguera o láser, colocación del perímetro, montaje y nivelación de las maestras, atornillado de las placas, tratamiento de juntas con cinta y pasta, lijado hasta dejar la superficie lista para pintar, y previsión de los huecos de luminarias y rejillas. Medido en superficie realmente ejecutada.</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>1</v>
+      </c>
+      <c r="F295" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Yeso laminado continuo</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Tubería de agua de PPR de 20 mm, empotrada, incluso roza y resane.</t>
+        </is>
+      </c>
+      <c r="C296" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de polipropileno PPR de 20 mm para distribución de agua fría o caliente, empotrada en paramento. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación de la tubería con uniones por termofusión, accesorios y piezas especiales, fijación con abrazaderas, prueba de estanqueidad a presión y tapado de roza con mortero de reparación, dejando el paramento listo para su revestimiento. No incluye el acabado final del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E296" t="n">
+        <v>1</v>
+      </c>
+      <c r="F296" t="n">
+        <v>7.45</v>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>Tuberías y montantes de agua</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Punto de agua fría y caliente para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C297" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de agua para aparato sanitario, formado por las derivaciones de agua fría y caliente en tubería de PPR de 20 mm desde el montante más próximo hasta la salida del aparato, con una longitud media de 2,5 m por punto. Incluye replanteo de la altura y separación normalizadas de las tomas, apertura de roza, montaje de la tubería con uniones por termofusión, codos de salida con refuerzo metálico anclados al paramento, prueba de estanqueidad a presión de la derivación, taponado provisional hasta la instalación del aparato y tapado de roza con mortero de reparación. No incluye la grifería ni el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E297" t="n">
+        <v>1</v>
+      </c>
+      <c r="F297" t="n">
+        <v>37.22</v>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>Puntos de agua</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Llave de paso de PPR de 20 mm, empotrada.</t>
+        </is>
+      </c>
+      <c r="C298" s="2" t="inlineStr">
+        <is>
+          <t>Suministro y montaje de llave de paso de esfera de PPR de 20 mm, empotrada en paramento, para el corte sectorizado del suministro de agua. Incluye apertura del hueco, montaje intercalado en la tubería mediante termofusión, comprobación de la maniobrabilidad del volante, prueba de estanqueidad y resane del paramento, dejando el embellecedor enrasado. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E298" t="n">
+        <v>1</v>
+      </c>
+      <c r="F298" t="n">
+        <v>13.52</v>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>Llaves y valvulería</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro con su conexión de agua y desagüe.</t>
+        </is>
+      </c>
+      <c r="C299" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de inodoro sobre punto de agua y desagüe previamente ejecutados. Incluye replanteo y presentación de la pieza, montaje del anillo de cera o junta de estanqueidad, anclaje al piso con tornillería inoxidable y tacos, conexión al desagüe, montaje del tanque y sus herrajes internos, conexión de la alimentación mediante tubo de abasto flexible con llave de escuadra, sellado perimetral con silicona sanitaria antihongos, regulación del mecanismo de descarga y prueba de funcionamiento y estanqueidad. El aparato lo elige el cliente y se presupuesta aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E299" t="n">
+        <v>1</v>
+      </c>
+      <c r="F299" t="n">
+        <v>23.45</v>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Instalación de lavamanos con su grifería y desagüe.</t>
+        </is>
+      </c>
+      <c r="C300" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de lavamanos, ya sea de pedestal, sobre encimera o suspendido, sobre puntos de agua y desagüe previamente ejecutados. Incluye replanteo de la altura de uso, taladrado y anclaje al paramento o fijación sobre el mueble, montaje de la grifería con sus juntas, conexión de las tomas de agua fría y caliente mediante tubos de abasto flexibles con llaves de escuadra, montaje del desagüe con su válvula y sifón, sellado perimetral con silicona sanitaria, y prueba de funcionamiento, evacuación y estanqueidad. El aparato y la grifería los elige el cliente y se presupuestan aparte. Medido por unidad instalada y probada.</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E300" t="n">
+        <v>1</v>
+      </c>
+      <c r="F300" t="n">
+        <v>36.45</v>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>Aparatos sanitarios y grifería</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Tubería de desagüe de PVC sanitario de 4 pulgadas.</t>
+        </is>
+      </c>
+      <c r="C301" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de tubería de PVC sanitario de 4 pulgadas para red de desagüe, colocada con la pendiente de proyecto. Incluye replanteo, cortes, limpieza y cementado de las uniones, accesorios como codos, yees y sifones, fijación mediante abrazaderas o apoyo sobre cama según el trazado, y prueba de estanqueidad de la red. No incluye la apertura de rozas ni la obra civil de canalización, que se valoran aparte. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E301" t="n">
+        <v>1</v>
+      </c>
+      <c r="F301" t="n">
+        <v>11.04</v>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>Tuberías y bajantes de desagüe</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Instalaciones sanitarias</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Punto de desagüe para aparato sanitario.</t>
+        </is>
+      </c>
+      <c r="C302" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto de desagüe para aparato sanitario, formado por la derivación en tubería de PVC sanitario desde el aparato hasta la bajante o colector más próximo, con una longitud media de 2 m y la pendiente reglamentaria. Incluye replanteo, apertura del paso en piso o paramento, montaje de la tubería con uniones cementadas, sifón y accesorios, fijación mediante abrazaderas, prueba de estanqueidad con agua, taponado provisional hasta la instalación del aparato y resane del paso. No incluye el aparato. Medido por punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E302" t="n">
+        <v>1</v>
+      </c>
+      <c r="F302" t="n">
+        <v>33.84</v>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>Puntos de desagüe</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Canalización eléctrica empotrada con conduit de 20 mm y conductor 12 AWG.</t>
+        </is>
+      </c>
+      <c r="C303" s="2" t="inlineStr">
+        <is>
+          <t>Instalación de canalización eléctrica empotrada formada por tubería conduit corrugada de PVC de 20 mm y tres conductores de cobre THW calibre 12 AWG, incluyendo fase, neutro y tierra. Incluye replanteo del trazado, apertura de roza con rozadora eléctrica con captación de polvo, colocación y fijación del conduit, guiado y tendido de los conductores, identificación de circuitos y tapado de roza con mortero de reparación. No incluye cajas, mecanismos ni el acabado del paramento. Medido en longitud realmente instalada.</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E303" t="n">
+        <v>1</v>
+      </c>
+      <c r="F303" t="n">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>Canalizaciones y cableado</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Instalaciones eléctricas</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Punto de interruptor o tomacorriente, incluso caja y mecanismo.</t>
+        </is>
+      </c>
+      <c r="C304" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución de punto eléctrico de interruptor o tomacorriente, formado por caja de mecanismo empotrada, conexionado de los conductores del circuito correspondiente, mecanismo de gama estándar y placa embellecedora. Incluye apertura del hueco de la caja, fijación y enrase con el paramento, conexionado con apriete y verificación de continuidad y polaridad, colocación del mecanismo y comprobación de funcionamiento. Medido por unidad de punto terminado y probado.</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="E304" t="n">
+        <v>1</v>
+      </c>
+      <c r="F304" t="n">
+        <v>8.720000000000001</v>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>Puntos, mecanismos y tomas</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Preparación de paramento interior para pintura: resane, alisado y fondo.</t>
+        </is>
+      </c>
+      <c r="C305" s="2" t="inlineStr">
+        <is>
+          <t>Preparación completa de paramento interior antes de pintar. Incluye protección de pisos, carpintería y mobiliario con plástico y cinta de enmascarar, retirada de partes sueltas, resane de grietas y huecos con masilla de reparación, alisado y lijado hasta obtener superficie uniforme, eliminación del polvo residual y aplicación de una mano de fondo fijador para consolidar el soporte y regular su absorción. Deja el paramento listo para recibir el acabado. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E305" t="n">
+        <v>1</v>
+      </c>
+      <c r="F305" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>Preparación de soportes</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Pintura de caucho mate lavable en paramento interior, dos manos.</t>
+        </is>
+      </c>
+      <c r="C306" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de pintura de caucho acrílico mate lavable sobre paramento interior previamente preparado e imprimado, aplicada con rodillo y brocha en encuentros y remates, con el lijado intermedio necesario entre manos y respetando los tiempos de secado del fabricante. Incluye protección del entorno, recorte de cantos y esquinas, repasos finales y limpieza del área de trabajo. El color lo elige el cliente. Medido en superficie realmente ejecutada, descontando huecos mayores de 1 m².</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E306" t="n">
+        <v>1</v>
+      </c>
+      <c r="F306" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>Pintura interior</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Pintura y acabados</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Esmalte sintético sobre carpintería metálica o de madera, dos manos.</t>
+        </is>
+      </c>
+      <c r="C307" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación de dos manos de esmalte sintético brillante sobre carpintería metálica o de madera, previa preparación del soporte mediante lijado, desengrasado y eliminación de óxido o restos de acabados anteriores. Incluye enmascarado de vidrios, herrajes y paramentos contiguos, aplicación a brocha en perfiles y molduras, lijado suave entre manos y retirada de protecciones. Medido en superficie realmente tratada, midiendo ambas caras por separado.</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="E307" t="n">
+        <v>1</v>
+      </c>
+      <c r="F307" t="n">
+        <v>5.23</v>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>Esmaltes sobre madera y metal</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>incluida</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
           <t>Gestión de residuos y limpieza</t>
         </is>
       </c>
-      <c r="B273" t="inlineStr">
+      <c r="B308" t="inlineStr">
         <is>
           <t>Retirada y transporte de escombro a vertedero autorizado.</t>
         </is>
       </c>
-      <c r="C273" s="2" t="inlineStr">
+      <c r="C308" s="2" t="inlineStr">
         <is>
           <t>Retirada de escombro procedente de demoliciones desde el punto de acopio de la obra y transporte en camión volqueta hasta vertedero o botadero autorizado, incluido el canon de vertido. Incluye la carga manual del escombro sobre el vehículo, el amarre y cubrición de la carga para evitar derrames durante el trayecto, el traslado con una distancia media considerada de 25 km, la descarga y la limpieza de la zona de carga. Medido por metro cúbico de escombro esponjado realmente retirado.</t>
         </is>
       </c>
-      <c r="D273" t="inlineStr">
+      <c r="D308" t="inlineStr">
         <is>
           <t>m3</t>
         </is>
       </c>
-      <c r="E273" t="n">
-        <v>1</v>
-      </c>
-      <c r="F273" t="n">
+      <c r="E308" t="n">
+        <v>1</v>
+      </c>
+      <c r="F308" t="n">
         <v>16.07</v>
       </c>
-      <c r="G273" t="inlineStr">
+      <c r="G308" t="inlineStr">
         <is>
           <t>Retiro y transporte de escombro</t>
         </is>
       </c>
-      <c r="H273" t="inlineStr">
+      <c r="H308" t="inlineStr">
         <is>
           <t>incluida</t>
         </is>

</xml_diff>

<commit_message>
Contrastar 66 precios de material con el mercado venezolano y documentar fuentes
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/basedatos_partidas/salida/catalogo_partidas.xlsx
+++ b/basedatos_partidas/salida/catalogo_partidas.xlsx
@@ -620,7 +620,7 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>19.59</v>
+        <v>22.35</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -810,7 +810,7 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>83.14</v>
+        <v>88.92</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>9.609999999999999</v>
+        <v>8.67</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1532,7 +1532,7 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>146.84</v>
+        <v>166.53</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -3584,7 +3584,7 @@
         <v>1</v>
       </c>
       <c r="F83" t="n">
-        <v>18.8</v>
+        <v>17.86</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -6054,7 +6054,7 @@
         <v>1</v>
       </c>
       <c r="F148" t="n">
-        <v>34.71</v>
+        <v>31.43</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
@@ -6130,7 +6130,7 @@
         <v>1</v>
       </c>
       <c r="F150" t="n">
-        <v>45.36</v>
+        <v>48.5</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
@@ -6320,7 +6320,7 @@
         <v>1</v>
       </c>
       <c r="F155" t="n">
-        <v>28.35</v>
+        <v>25.73</v>
       </c>
       <c r="G155" t="inlineStr">
         <is>
@@ -6396,7 +6396,7 @@
         <v>1</v>
       </c>
       <c r="F157" t="n">
-        <v>8.41</v>
+        <v>7.68</v>
       </c>
       <c r="G157" t="inlineStr">
         <is>
@@ -6434,7 +6434,7 @@
         <v>1</v>
       </c>
       <c r="F158" t="n">
-        <v>2.3</v>
+        <v>2.09</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
@@ -6510,7 +6510,7 @@
         <v>1</v>
       </c>
       <c r="F160" t="n">
-        <v>167.7</v>
+        <v>158.13</v>
       </c>
       <c r="G160" t="inlineStr">
         <is>
@@ -6548,7 +6548,7 @@
         <v>1</v>
       </c>
       <c r="F161" t="n">
-        <v>166.6</v>
+        <v>157.04</v>
       </c>
       <c r="G161" t="inlineStr">
         <is>
@@ -6586,7 +6586,7 @@
         <v>1</v>
       </c>
       <c r="F162" t="n">
-        <v>243.11</v>
+        <v>233.47</v>
       </c>
       <c r="G162" t="inlineStr">
         <is>
@@ -6624,7 +6624,7 @@
         <v>1</v>
       </c>
       <c r="F163" t="n">
-        <v>95</v>
+        <v>85.34999999999999</v>
       </c>
       <c r="G163" t="inlineStr">
         <is>
@@ -6662,7 +6662,7 @@
         <v>1</v>
       </c>
       <c r="F164" t="n">
-        <v>137.83</v>
+        <v>133.39</v>
       </c>
       <c r="G164" t="inlineStr">
         <is>
@@ -6700,7 +6700,7 @@
         <v>1</v>
       </c>
       <c r="F165" t="n">
-        <v>134.64</v>
+        <v>128.28</v>
       </c>
       <c r="G165" t="inlineStr">
         <is>
@@ -6738,7 +6738,7 @@
         <v>1</v>
       </c>
       <c r="F166" t="n">
-        <v>2.39</v>
+        <v>2.18</v>
       </c>
       <c r="G166" t="inlineStr">
         <is>
@@ -6814,7 +6814,7 @@
         <v>1</v>
       </c>
       <c r="F168" t="n">
-        <v>171.91</v>
+        <v>162.27</v>
       </c>
       <c r="G168" t="inlineStr">
         <is>
@@ -6890,7 +6890,7 @@
         <v>1</v>
       </c>
       <c r="F170" t="n">
-        <v>2.27</v>
+        <v>2.07</v>
       </c>
       <c r="G170" t="inlineStr">
         <is>
@@ -6928,7 +6928,7 @@
         <v>1</v>
       </c>
       <c r="F171" t="n">
-        <v>7.37</v>
+        <v>7.96</v>
       </c>
       <c r="G171" t="inlineStr">
         <is>
@@ -7004,7 +7004,7 @@
         <v>1</v>
       </c>
       <c r="F173" t="n">
-        <v>182.77</v>
+        <v>173.21</v>
       </c>
       <c r="G173" t="inlineStr">
         <is>
@@ -7080,7 +7080,7 @@
         <v>1</v>
       </c>
       <c r="F175" t="n">
-        <v>16.43</v>
+        <v>16.33</v>
       </c>
       <c r="G175" t="inlineStr">
         <is>
@@ -7118,7 +7118,7 @@
         <v>1</v>
       </c>
       <c r="F176" t="n">
-        <v>2.37</v>
+        <v>2.16</v>
       </c>
       <c r="G176" t="inlineStr">
         <is>
@@ -7156,7 +7156,7 @@
         <v>1</v>
       </c>
       <c r="F177" t="n">
-        <v>191.39</v>
+        <v>181.73</v>
       </c>
       <c r="G177" t="inlineStr">
         <is>
@@ -7232,7 +7232,7 @@
         <v>1</v>
       </c>
       <c r="F179" t="n">
-        <v>21.94</v>
+        <v>22.78</v>
       </c>
       <c r="G179" t="inlineStr">
         <is>
@@ -7308,7 +7308,7 @@
         <v>1</v>
       </c>
       <c r="F181" t="n">
-        <v>2.61</v>
+        <v>2.41</v>
       </c>
       <c r="G181" t="inlineStr">
         <is>
@@ -7346,7 +7346,7 @@
         <v>1</v>
       </c>
       <c r="F182" t="n">
-        <v>217.58</v>
+        <v>207.01</v>
       </c>
       <c r="G182" t="inlineStr">
         <is>
@@ -7422,7 +7422,7 @@
         <v>1</v>
       </c>
       <c r="F184" t="n">
-        <v>231.7</v>
+        <v>222.05</v>
       </c>
       <c r="G184" t="inlineStr">
         <is>
@@ -7460,7 +7460,7 @@
         <v>1</v>
       </c>
       <c r="F185" t="n">
-        <v>2.48</v>
+        <v>2.27</v>
       </c>
       <c r="G185" t="inlineStr">
         <is>
@@ -7536,7 +7536,7 @@
         <v>1</v>
       </c>
       <c r="F187" t="n">
-        <v>193.28</v>
+        <v>183.55</v>
       </c>
       <c r="G187" t="inlineStr">
         <is>
@@ -7574,7 +7574,7 @@
         <v>1</v>
       </c>
       <c r="F188" t="n">
-        <v>2.43</v>
+        <v>2.22</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -7650,7 +7650,7 @@
         <v>1</v>
       </c>
       <c r="F190" t="n">
-        <v>189.76</v>
+        <v>180.1</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -7688,7 +7688,7 @@
         <v>1</v>
       </c>
       <c r="F191" t="n">
-        <v>2.34</v>
+        <v>2.13</v>
       </c>
       <c r="G191" t="inlineStr">
         <is>
@@ -7726,7 +7726,7 @@
         <v>1</v>
       </c>
       <c r="F192" t="n">
-        <v>17.21</v>
+        <v>17.12</v>
       </c>
       <c r="G192" t="inlineStr">
         <is>
@@ -7764,7 +7764,7 @@
         <v>1</v>
       </c>
       <c r="F193" t="n">
-        <v>190.5</v>
+        <v>180.86</v>
       </c>
       <c r="G193" t="inlineStr">
         <is>
@@ -7802,7 +7802,7 @@
         <v>1</v>
       </c>
       <c r="F194" t="n">
-        <v>3.89</v>
+        <v>4.02</v>
       </c>
       <c r="G194" t="inlineStr">
         <is>
@@ -7840,7 +7840,7 @@
         <v>1</v>
       </c>
       <c r="F195" t="n">
-        <v>107.48</v>
+        <v>103.01</v>
       </c>
       <c r="G195" t="inlineStr">
         <is>
@@ -7954,7 +7954,7 @@
         <v>1</v>
       </c>
       <c r="F198" t="n">
-        <v>3.43</v>
+        <v>3.58</v>
       </c>
       <c r="G198" t="inlineStr">
         <is>
@@ -7992,7 +7992,7 @@
         <v>1</v>
       </c>
       <c r="F199" t="n">
-        <v>563.24</v>
+        <v>514.53</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -8030,7 +8030,7 @@
         <v>1</v>
       </c>
       <c r="F200" t="n">
-        <v>12.68</v>
+        <v>12.03</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -8182,7 +8182,7 @@
         <v>1</v>
       </c>
       <c r="F204" t="n">
-        <v>2.27</v>
+        <v>2.07</v>
       </c>
       <c r="G204" t="inlineStr">
         <is>
@@ -8220,7 +8220,7 @@
         <v>1</v>
       </c>
       <c r="F205" t="n">
-        <v>185.81</v>
+        <v>176.24</v>
       </c>
       <c r="G205" t="inlineStr">
         <is>
@@ -8258,7 +8258,7 @@
         <v>1</v>
       </c>
       <c r="F206" t="n">
-        <v>70.77</v>
+        <v>69.23</v>
       </c>
       <c r="G206" t="inlineStr">
         <is>
@@ -8296,7 +8296,7 @@
         <v>1</v>
       </c>
       <c r="F207" t="n">
-        <v>77.36</v>
+        <v>75.81999999999999</v>
       </c>
       <c r="G207" t="inlineStr">
         <is>
@@ -8334,7 +8334,7 @@
         <v>1</v>
       </c>
       <c r="F208" t="n">
-        <v>61.39</v>
+        <v>60.67</v>
       </c>
       <c r="G208" t="inlineStr">
         <is>
@@ -8410,7 +8410,7 @@
         <v>1</v>
       </c>
       <c r="F210" t="n">
-        <v>68.54000000000001</v>
+        <v>68.33</v>
       </c>
       <c r="G210" t="inlineStr">
         <is>
@@ -8448,7 +8448,7 @@
         <v>1</v>
       </c>
       <c r="F211" t="n">
-        <v>123.59</v>
+        <v>119.2</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -8524,7 +8524,7 @@
         <v>1</v>
       </c>
       <c r="F213" t="n">
-        <v>2.46</v>
+        <v>2.25</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -8562,7 +8562,7 @@
         <v>1</v>
       </c>
       <c r="F214" t="n">
-        <v>199.24</v>
+        <v>189.49</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -8600,7 +8600,7 @@
         <v>1</v>
       </c>
       <c r="F215" t="n">
-        <v>4.71</v>
+        <v>4.89</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -8790,7 +8790,7 @@
         <v>1</v>
       </c>
       <c r="F220" t="n">
-        <v>180.34</v>
+        <v>174.2</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -8828,7 +8828,7 @@
         <v>1</v>
       </c>
       <c r="F221" t="n">
-        <v>6.1</v>
+        <v>5.97</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -8866,7 +8866,7 @@
         <v>1</v>
       </c>
       <c r="F222" t="n">
-        <v>192.82</v>
+        <v>187.82</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -8904,7 +8904,7 @@
         <v>1</v>
       </c>
       <c r="F223" t="n">
-        <v>18.29</v>
+        <v>16.17</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -8942,7 +8942,7 @@
         <v>1</v>
       </c>
       <c r="F224" t="n">
-        <v>23.83</v>
+        <v>20.45</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -8980,7 +8980,7 @@
         <v>1</v>
       </c>
       <c r="F225" t="n">
-        <v>28.63</v>
+        <v>24.23</v>
       </c>
       <c r="G225" t="inlineStr">
         <is>
@@ -9018,7 +9018,7 @@
         <v>1</v>
       </c>
       <c r="F226" t="n">
-        <v>28.37</v>
+        <v>24.78</v>
       </c>
       <c r="G226" t="inlineStr">
         <is>
@@ -9056,7 +9056,7 @@
         <v>1</v>
       </c>
       <c r="F227" t="n">
-        <v>33.5</v>
+        <v>32.01</v>
       </c>
       <c r="G227" t="inlineStr">
         <is>
@@ -9094,7 +9094,7 @@
         <v>1</v>
       </c>
       <c r="F228" t="n">
-        <v>29.72</v>
+        <v>28.38</v>
       </c>
       <c r="G228" t="inlineStr">
         <is>
@@ -9132,7 +9132,7 @@
         <v>1</v>
       </c>
       <c r="F229" t="n">
-        <v>20.81</v>
+        <v>18.1</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -9170,7 +9170,7 @@
         <v>1</v>
       </c>
       <c r="F230" t="n">
-        <v>18.73</v>
+        <v>16.98</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -9208,7 +9208,7 @@
         <v>1</v>
       </c>
       <c r="F231" t="n">
-        <v>23.75</v>
+        <v>21.92</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -9246,7 +9246,7 @@
         <v>1</v>
       </c>
       <c r="F232" t="n">
-        <v>40.79</v>
+        <v>34.55</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -9284,7 +9284,7 @@
         <v>1</v>
       </c>
       <c r="F233" t="n">
-        <v>45.76</v>
+        <v>39.17</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -9322,7 +9322,7 @@
         <v>1</v>
       </c>
       <c r="F234" t="n">
-        <v>52.4</v>
+        <v>64.05</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -9360,7 +9360,7 @@
         <v>1</v>
       </c>
       <c r="F235" t="n">
-        <v>35.46</v>
+        <v>39.99</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -9398,7 +9398,7 @@
         <v>1</v>
       </c>
       <c r="F236" t="n">
-        <v>45.15</v>
+        <v>57.76</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -9436,7 +9436,7 @@
         <v>1</v>
       </c>
       <c r="F237" t="n">
-        <v>24.19</v>
+        <v>26.21</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -9474,7 +9474,7 @@
         <v>1</v>
       </c>
       <c r="F238" t="n">
-        <v>13.23</v>
+        <v>15.59</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -9550,7 +9550,7 @@
         <v>1</v>
       </c>
       <c r="F240" t="n">
-        <v>186.85</v>
+        <v>185.85</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -9588,7 +9588,7 @@
         <v>1</v>
       </c>
       <c r="F241" t="n">
-        <v>53.64</v>
+        <v>52.62</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -9626,7 +9626,7 @@
         <v>1</v>
       </c>
       <c r="F242" t="n">
-        <v>30.12</v>
+        <v>29.65</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -9664,7 +9664,7 @@
         <v>1</v>
       </c>
       <c r="F243" t="n">
-        <v>31.59</v>
+        <v>29.46</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -9702,7 +9702,7 @@
         <v>1</v>
       </c>
       <c r="F244" t="n">
-        <v>13.48</v>
+        <v>13.04</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -9740,7 +9740,7 @@
         <v>1</v>
       </c>
       <c r="F245" t="n">
-        <v>33.2</v>
+        <v>31.95</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -9778,7 +9778,7 @@
         <v>1</v>
       </c>
       <c r="F246" t="n">
-        <v>13.43</v>
+        <v>11.01</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -9816,7 +9816,7 @@
         <v>1</v>
       </c>
       <c r="F247" t="n">
-        <v>7.25</v>
+        <v>6.38</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -9854,7 +9854,7 @@
         <v>1</v>
       </c>
       <c r="F248" t="n">
-        <v>5.75</v>
+        <v>5.55</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -9892,7 +9892,7 @@
         <v>1</v>
       </c>
       <c r="F249" t="n">
-        <v>47.92</v>
+        <v>42.46</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -9930,7 +9930,7 @@
         <v>1</v>
       </c>
       <c r="F250" t="n">
-        <v>59.77</v>
+        <v>52.18</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -9968,7 +9968,7 @@
         <v>1</v>
       </c>
       <c r="F251" t="n">
-        <v>32.29</v>
+        <v>29.98</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -10006,7 +10006,7 @@
         <v>1</v>
       </c>
       <c r="F252" t="n">
-        <v>11.13</v>
+        <v>10.5</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -10044,7 +10044,7 @@
         <v>1</v>
       </c>
       <c r="F253" t="n">
-        <v>12.55</v>
+        <v>11.28</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -10082,7 +10082,7 @@
         <v>1</v>
       </c>
       <c r="F254" t="n">
-        <v>34.63</v>
+        <v>33.85</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -10120,7 +10120,7 @@
         <v>1</v>
       </c>
       <c r="F255" t="n">
-        <v>83.48999999999999</v>
+        <v>80.95999999999999</v>
       </c>
       <c r="G255" t="inlineStr">
         <is>
@@ -10158,7 +10158,7 @@
         <v>1</v>
       </c>
       <c r="F256" t="n">
-        <v>217.43</v>
+        <v>214.5</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -10348,7 +10348,7 @@
         <v>1</v>
       </c>
       <c r="F261" t="n">
-        <v>10.75</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -10386,7 +10386,7 @@
         <v>1</v>
       </c>
       <c r="F262" t="n">
-        <v>17.52</v>
+        <v>14.85</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -10424,7 +10424,7 @@
         <v>1</v>
       </c>
       <c r="F263" t="n">
-        <v>16.45</v>
+        <v>14.26</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -10462,7 +10462,7 @@
         <v>1</v>
       </c>
       <c r="F264" t="n">
-        <v>12.4</v>
+        <v>11.47</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -10500,7 +10500,7 @@
         <v>1</v>
       </c>
       <c r="F265" t="n">
-        <v>12.23</v>
+        <v>10.5</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -10538,7 +10538,7 @@
         <v>1</v>
       </c>
       <c r="F266" t="n">
-        <v>10.92</v>
+        <v>8.720000000000001</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -10576,7 +10576,7 @@
         <v>1</v>
       </c>
       <c r="F267" t="n">
-        <v>3.59</v>
+        <v>3.15</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -10614,7 +10614,7 @@
         <v>1</v>
       </c>
       <c r="F268" t="n">
-        <v>4.89</v>
+        <v>4.33</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -10690,7 +10690,7 @@
         <v>1</v>
       </c>
       <c r="F270" t="n">
-        <v>6.38</v>
+        <v>6.59</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -10728,7 +10728,7 @@
         <v>1</v>
       </c>
       <c r="F271" t="n">
-        <v>4.34</v>
+        <v>4.52</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -10766,7 +10766,7 @@
         <v>1</v>
       </c>
       <c r="F272" t="n">
-        <v>7.77</v>
+        <v>7.66</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -10842,7 +10842,7 @@
         <v>1</v>
       </c>
       <c r="F274" t="n">
-        <v>10.87</v>
+        <v>9.74</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -10880,7 +10880,7 @@
         <v>1</v>
       </c>
       <c r="F275" t="n">
-        <v>14.5</v>
+        <v>12.8</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -10918,7 +10918,7 @@
         <v>1</v>
       </c>
       <c r="F276" t="n">
-        <v>16.33</v>
+        <v>14.94</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -10956,7 +10956,7 @@
         <v>1</v>
       </c>
       <c r="F277" t="n">
-        <v>2.99</v>
+        <v>2.85</v>
       </c>
       <c r="G277" t="inlineStr">
         <is>
@@ -10994,7 +10994,7 @@
         <v>1</v>
       </c>
       <c r="F278" t="n">
-        <v>5.25</v>
+        <v>5.17</v>
       </c>
       <c r="G278" t="inlineStr">
         <is>
@@ -11032,7 +11032,7 @@
         <v>1</v>
       </c>
       <c r="F279" t="n">
-        <v>14.13</v>
+        <v>12.92</v>
       </c>
       <c r="G279" t="inlineStr">
         <is>
@@ -11070,7 +11070,7 @@
         <v>1</v>
       </c>
       <c r="F280" t="n">
-        <v>3.06</v>
+        <v>2.91</v>
       </c>
       <c r="G280" t="inlineStr">
         <is>
@@ -11108,7 +11108,7 @@
         <v>1</v>
       </c>
       <c r="F281" t="n">
-        <v>14.61</v>
+        <v>12.53</v>
       </c>
       <c r="G281" t="inlineStr">
         <is>
@@ -11146,7 +11146,7 @@
         <v>1</v>
       </c>
       <c r="F282" t="n">
-        <v>23.82</v>
+        <v>21.03</v>
       </c>
       <c r="G282" t="inlineStr">
         <is>
@@ -11184,7 +11184,7 @@
         <v>1</v>
       </c>
       <c r="F283" t="n">
-        <v>31.46</v>
+        <v>30.59</v>
       </c>
       <c r="G283" t="inlineStr">
         <is>
@@ -11222,7 +11222,7 @@
         <v>1</v>
       </c>
       <c r="F284" t="n">
-        <v>2.95</v>
+        <v>2.67</v>
       </c>
       <c r="G284" t="inlineStr">
         <is>
@@ -11298,7 +11298,7 @@
         <v>1</v>
       </c>
       <c r="F286" t="n">
-        <v>4.24</v>
+        <v>4.41</v>
       </c>
       <c r="G286" t="inlineStr">
         <is>
@@ -11336,7 +11336,7 @@
         <v>1</v>
       </c>
       <c r="F287" t="n">
-        <v>16.2</v>
+        <v>16.38</v>
       </c>
       <c r="G287" t="inlineStr">
         <is>
@@ -11374,7 +11374,7 @@
         <v>1</v>
       </c>
       <c r="F288" t="n">
-        <v>13.64</v>
+        <v>13.33</v>
       </c>
       <c r="G288" t="inlineStr">
         <is>
@@ -11412,7 +11412,7 @@
         <v>1</v>
       </c>
       <c r="F289" t="n">
-        <v>30.64</v>
+        <v>28.52</v>
       </c>
       <c r="G289" t="inlineStr">
         <is>
@@ -11488,7 +11488,7 @@
         <v>1</v>
       </c>
       <c r="F291" t="n">
-        <v>29.84</v>
+        <v>29.57</v>
       </c>
       <c r="G291" t="inlineStr">
         <is>
@@ -11564,7 +11564,7 @@
         <v>1</v>
       </c>
       <c r="F293" t="n">
-        <v>17.86</v>
+        <v>13.75</v>
       </c>
       <c r="G293" t="inlineStr">
         <is>
@@ -11602,7 +11602,7 @@
         <v>1</v>
       </c>
       <c r="F294" t="n">
-        <v>24.83</v>
+        <v>24.61</v>
       </c>
       <c r="G294" t="inlineStr">
         <is>
@@ -11640,7 +11640,7 @@
         <v>1</v>
       </c>
       <c r="F295" t="n">
-        <v>21.62</v>
+        <v>16.82</v>
       </c>
       <c r="G295" t="inlineStr">
         <is>
@@ -11716,7 +11716,7 @@
         <v>1</v>
       </c>
       <c r="F297" t="n">
-        <v>13.64</v>
+        <v>12.64</v>
       </c>
       <c r="G297" t="inlineStr">
         <is>
@@ -11754,7 +11754,7 @@
         <v>1</v>
       </c>
       <c r="F298" t="n">
-        <v>9.17</v>
+        <v>8.15</v>
       </c>
       <c r="G298" t="inlineStr">
         <is>
@@ -11792,7 +11792,7 @@
         <v>1</v>
       </c>
       <c r="F299" t="n">
-        <v>12.51</v>
+        <v>11.01</v>
       </c>
       <c r="G299" t="inlineStr">
         <is>
@@ -11830,7 +11830,7 @@
         <v>1</v>
       </c>
       <c r="F300" t="n">
-        <v>13.18</v>
+        <v>12.08</v>
       </c>
       <c r="G300" t="inlineStr">
         <is>
@@ -11868,7 +11868,7 @@
         <v>1</v>
       </c>
       <c r="F301" t="n">
-        <v>13.86</v>
+        <v>12.58</v>
       </c>
       <c r="G301" t="inlineStr">
         <is>
@@ -11906,7 +11906,7 @@
         <v>1</v>
       </c>
       <c r="F302" t="n">
-        <v>19.41</v>
+        <v>16.54</v>
       </c>
       <c r="G302" t="inlineStr">
         <is>
@@ -11944,7 +11944,7 @@
         <v>1</v>
       </c>
       <c r="F303" t="n">
-        <v>21.18</v>
+        <v>18.97</v>
       </c>
       <c r="G303" t="inlineStr">
         <is>
@@ -11982,7 +11982,7 @@
         <v>1</v>
       </c>
       <c r="F304" t="n">
-        <v>15.31</v>
+        <v>13.38</v>
       </c>
       <c r="G304" t="inlineStr">
         <is>
@@ -12020,7 +12020,7 @@
         <v>1</v>
       </c>
       <c r="F305" t="n">
-        <v>49.71</v>
+        <v>49.8</v>
       </c>
       <c r="G305" t="inlineStr">
         <is>
@@ -12058,7 +12058,7 @@
         <v>1</v>
       </c>
       <c r="F306" t="n">
-        <v>23.21</v>
+        <v>20.59</v>
       </c>
       <c r="G306" t="inlineStr">
         <is>
@@ -12096,7 +12096,7 @@
         <v>1</v>
       </c>
       <c r="F307" t="n">
-        <v>24.78</v>
+        <v>22.48</v>
       </c>
       <c r="G307" t="inlineStr">
         <is>
@@ -12286,7 +12286,7 @@
         <v>1</v>
       </c>
       <c r="F312" t="n">
-        <v>12.91</v>
+        <v>12.27</v>
       </c>
       <c r="G312" t="inlineStr">
         <is>
@@ -12552,7 +12552,7 @@
         <v>1</v>
       </c>
       <c r="F319" t="n">
-        <v>26.2</v>
+        <v>25.93</v>
       </c>
       <c r="G319" t="inlineStr">
         <is>
@@ -12590,7 +12590,7 @@
         <v>1</v>
       </c>
       <c r="F320" t="n">
-        <v>38.82</v>
+        <v>38.49</v>
       </c>
       <c r="G320" t="inlineStr">
         <is>
@@ -12742,7 +12742,7 @@
         <v>1</v>
       </c>
       <c r="F324" t="n">
-        <v>20.01</v>
+        <v>16.8</v>
       </c>
       <c r="G324" t="inlineStr">
         <is>
@@ -12780,7 +12780,7 @@
         <v>1</v>
       </c>
       <c r="F325" t="n">
-        <v>21.45</v>
+        <v>18.43</v>
       </c>
       <c r="G325" t="inlineStr">
         <is>
@@ -12818,7 +12818,7 @@
         <v>1</v>
       </c>
       <c r="F326" t="n">
-        <v>1.69</v>
+        <v>1.59</v>
       </c>
       <c r="G326" t="inlineStr">
         <is>
@@ -12856,7 +12856,7 @@
         <v>1</v>
       </c>
       <c r="F327" t="n">
-        <v>2.13</v>
+        <v>2.08</v>
       </c>
       <c r="G327" t="inlineStr">
         <is>
@@ -12894,7 +12894,7 @@
         <v>1</v>
       </c>
       <c r="F328" t="n">
-        <v>4.06</v>
+        <v>3.55</v>
       </c>
       <c r="G328" t="inlineStr">
         <is>
@@ -12970,7 +12970,7 @@
         <v>1</v>
       </c>
       <c r="F330" t="n">
-        <v>10.17</v>
+        <v>10.04</v>
       </c>
       <c r="G330" t="inlineStr">
         <is>
@@ -13008,7 +13008,7 @@
         <v>1</v>
       </c>
       <c r="F331" t="n">
-        <v>10.69</v>
+        <v>10.01</v>
       </c>
       <c r="G331" t="inlineStr">
         <is>
@@ -13046,7 +13046,7 @@
         <v>1</v>
       </c>
       <c r="F332" t="n">
-        <v>18.02</v>
+        <v>16.63</v>
       </c>
       <c r="G332" t="inlineStr">
         <is>
@@ -13084,7 +13084,7 @@
         <v>1</v>
       </c>
       <c r="F333" t="n">
-        <v>24.57</v>
+        <v>22.24</v>
       </c>
       <c r="G333" t="inlineStr">
         <is>
@@ -13198,7 +13198,7 @@
         <v>1</v>
       </c>
       <c r="F336" t="n">
-        <v>3.68</v>
+        <v>3.55</v>
       </c>
       <c r="G336" t="inlineStr">
         <is>
@@ -13236,7 +13236,7 @@
         <v>1</v>
       </c>
       <c r="F337" t="n">
-        <v>18.47</v>
+        <v>22.07</v>
       </c>
       <c r="G337" t="inlineStr">
         <is>
@@ -13274,7 +13274,7 @@
         <v>1</v>
       </c>
       <c r="F338" t="n">
-        <v>22.02</v>
+        <v>29.8</v>
       </c>
       <c r="G338" t="inlineStr">
         <is>
@@ -13312,7 +13312,7 @@
         <v>1</v>
       </c>
       <c r="F339" t="n">
-        <v>34.68</v>
+        <v>41.27</v>
       </c>
       <c r="G339" t="inlineStr">
         <is>
@@ -13350,7 +13350,7 @@
         <v>1</v>
       </c>
       <c r="F340" t="n">
-        <v>20.11</v>
+        <v>23.24</v>
       </c>
       <c r="G340" t="inlineStr">
         <is>
@@ -13388,7 +13388,7 @@
         <v>1</v>
       </c>
       <c r="F341" t="n">
-        <v>22.8</v>
+        <v>23.14</v>
       </c>
       <c r="G341" t="inlineStr">
         <is>
@@ -13426,7 +13426,7 @@
         <v>1</v>
       </c>
       <c r="F342" t="n">
-        <v>30.17</v>
+        <v>35.06</v>
       </c>
       <c r="G342" t="inlineStr">
         <is>
@@ -13578,7 +13578,7 @@
         <v>1</v>
       </c>
       <c r="F346" t="n">
-        <v>27.04</v>
+        <v>27.72</v>
       </c>
       <c r="G346" t="inlineStr">
         <is>
@@ -13616,7 +13616,7 @@
         <v>1</v>
       </c>
       <c r="F347" t="n">
-        <v>32.51</v>
+        <v>30.38</v>
       </c>
       <c r="G347" t="inlineStr">
         <is>
@@ -13654,7 +13654,7 @@
         <v>1</v>
       </c>
       <c r="F348" t="n">
-        <v>7.55</v>
+        <v>7.45</v>
       </c>
       <c r="G348" t="inlineStr">
         <is>
@@ -13692,7 +13692,7 @@
         <v>1</v>
       </c>
       <c r="F349" t="n">
-        <v>13.33</v>
+        <v>13.52</v>
       </c>
       <c r="G349" t="inlineStr">
         <is>
@@ -13730,7 +13730,7 @@
         <v>1</v>
       </c>
       <c r="F350" t="n">
-        <v>26.04</v>
+        <v>28.12</v>
       </c>
       <c r="G350" t="inlineStr">
         <is>
@@ -13768,7 +13768,7 @@
         <v>1</v>
       </c>
       <c r="F351" t="n">
-        <v>18.55</v>
+        <v>16.25</v>
       </c>
       <c r="G351" t="inlineStr">
         <is>
@@ -13806,7 +13806,7 @@
         <v>1</v>
       </c>
       <c r="F352" t="n">
-        <v>20.4</v>
+        <v>18.94</v>
       </c>
       <c r="G352" t="inlineStr">
         <is>
@@ -13882,7 +13882,7 @@
         <v>1</v>
       </c>
       <c r="F354" t="n">
-        <v>17.73</v>
+        <v>15.82</v>
       </c>
       <c r="G354" t="inlineStr">
         <is>
@@ -13920,7 +13920,7 @@
         <v>1</v>
       </c>
       <c r="F355" t="n">
-        <v>34.33</v>
+        <v>30.13</v>
       </c>
       <c r="G355" t="inlineStr">
         <is>
@@ -13958,7 +13958,7 @@
         <v>1</v>
       </c>
       <c r="F356" t="n">
-        <v>12.29</v>
+        <v>11.4</v>
       </c>
       <c r="G356" t="inlineStr">
         <is>
@@ -13996,7 +13996,7 @@
         <v>1</v>
       </c>
       <c r="F357" t="n">
-        <v>23.53</v>
+        <v>22.18</v>
       </c>
       <c r="G357" t="inlineStr">
         <is>
@@ -14072,7 +14072,7 @@
         <v>1</v>
       </c>
       <c r="F359" t="n">
-        <v>19.6</v>
+        <v>18.6</v>
       </c>
       <c r="G359" t="inlineStr">
         <is>
@@ -14110,7 +14110,7 @@
         <v>1</v>
       </c>
       <c r="F360" t="n">
-        <v>24.99</v>
+        <v>23.88</v>
       </c>
       <c r="G360" t="inlineStr">
         <is>
@@ -14186,7 +14186,7 @@
         <v>1</v>
       </c>
       <c r="F362" t="n">
-        <v>21.12</v>
+        <v>20.02</v>
       </c>
       <c r="G362" t="inlineStr">
         <is>
@@ -14224,7 +14224,7 @@
         <v>1</v>
       </c>
       <c r="F363" t="n">
-        <v>18.99</v>
+        <v>17.99</v>
       </c>
       <c r="G363" t="inlineStr">
         <is>
@@ -14376,7 +14376,7 @@
         <v>1</v>
       </c>
       <c r="F367" t="n">
-        <v>4.15</v>
+        <v>4.29</v>
       </c>
       <c r="G367" t="inlineStr">
         <is>
@@ -14414,7 +14414,7 @@
         <v>1</v>
       </c>
       <c r="F368" t="n">
-        <v>55.38</v>
+        <v>53.46</v>
       </c>
       <c r="G368" t="inlineStr">
         <is>
@@ -14452,7 +14452,7 @@
         <v>1</v>
       </c>
       <c r="F369" t="n">
-        <v>46.46</v>
+        <v>42.96</v>
       </c>
       <c r="G369" t="inlineStr">
         <is>
@@ -14490,7 +14490,7 @@
         <v>1</v>
       </c>
       <c r="F370" t="n">
-        <v>36.02</v>
+        <v>40.26</v>
       </c>
       <c r="G370" t="inlineStr">
         <is>
@@ -14528,7 +14528,7 @@
         <v>1</v>
       </c>
       <c r="F371" t="n">
-        <v>15.2</v>
+        <v>14.55</v>
       </c>
       <c r="G371" t="inlineStr">
         <is>
@@ -14566,7 +14566,7 @@
         <v>1</v>
       </c>
       <c r="F372" t="n">
-        <v>22.52</v>
+        <v>24.4</v>
       </c>
       <c r="G372" t="inlineStr">
         <is>
@@ -14680,7 +14680,7 @@
         <v>1</v>
       </c>
       <c r="F375" t="n">
-        <v>178</v>
+        <v>175.47</v>
       </c>
       <c r="G375" t="inlineStr">
         <is>
@@ -14718,7 +14718,7 @@
         <v>1</v>
       </c>
       <c r="F376" t="n">
-        <v>18.62</v>
+        <v>15.07</v>
       </c>
       <c r="G376" t="inlineStr">
         <is>
@@ -14756,7 +14756,7 @@
         <v>1</v>
       </c>
       <c r="F377" t="n">
-        <v>26.6</v>
+        <v>23.39</v>
       </c>
       <c r="G377" t="inlineStr">
         <is>
@@ -14908,7 +14908,7 @@
         <v>1</v>
       </c>
       <c r="F381" t="n">
-        <v>31.72</v>
+        <v>31.33</v>
       </c>
       <c r="G381" t="inlineStr">
         <is>
@@ -14946,7 +14946,7 @@
         <v>1</v>
       </c>
       <c r="F382" t="n">
-        <v>17.12</v>
+        <v>16.5</v>
       </c>
       <c r="G382" t="inlineStr">
         <is>
@@ -15022,7 +15022,7 @@
         <v>1</v>
       </c>
       <c r="F384" t="n">
-        <v>23.91</v>
+        <v>22.2</v>
       </c>
       <c r="G384" t="inlineStr">
         <is>
@@ -15060,7 +15060,7 @@
         <v>1</v>
       </c>
       <c r="F385" t="n">
-        <v>7.45</v>
+        <v>7.44</v>
       </c>
       <c r="G385" t="inlineStr">
         <is>
@@ -15098,7 +15098,7 @@
         <v>1</v>
       </c>
       <c r="F386" t="n">
-        <v>8.15</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="G386" t="inlineStr">
         <is>
@@ -15136,7 +15136,7 @@
         <v>1</v>
       </c>
       <c r="F387" t="n">
-        <v>10.43</v>
+        <v>10.35</v>
       </c>
       <c r="G387" t="inlineStr">
         <is>
@@ -15174,7 +15174,7 @@
         <v>1</v>
       </c>
       <c r="F388" t="n">
-        <v>37.22</v>
+        <v>36.71</v>
       </c>
       <c r="G388" t="inlineStr">
         <is>
@@ -15212,7 +15212,7 @@
         <v>1</v>
       </c>
       <c r="F389" t="n">
-        <v>13.52</v>
+        <v>13.26</v>
       </c>
       <c r="G389" t="inlineStr">
         <is>
@@ -15326,7 +15326,7 @@
         <v>1</v>
       </c>
       <c r="F392" t="n">
-        <v>17.78</v>
+        <v>17.58</v>
       </c>
       <c r="G392" t="inlineStr">
         <is>
@@ -15402,7 +15402,7 @@
         <v>1</v>
       </c>
       <c r="F394" t="n">
-        <v>52.2</v>
+        <v>51.66</v>
       </c>
       <c r="G394" t="inlineStr">
         <is>
@@ -15554,7 +15554,7 @@
         <v>1</v>
       </c>
       <c r="F398" t="n">
-        <v>11.04</v>
+        <v>8.33</v>
       </c>
       <c r="G398" t="inlineStr">
         <is>
@@ -15592,7 +15592,7 @@
         <v>1</v>
       </c>
       <c r="F399" t="n">
-        <v>146.58</v>
+        <v>137.97</v>
       </c>
       <c r="G399" t="inlineStr">
         <is>
@@ -15630,7 +15630,7 @@
         <v>1</v>
       </c>
       <c r="F400" t="n">
-        <v>99.52</v>
+        <v>86.79000000000001</v>
       </c>
       <c r="G400" t="inlineStr">
         <is>
@@ -15668,7 +15668,7 @@
         <v>1</v>
       </c>
       <c r="F401" t="n">
-        <v>33.84</v>
+        <v>28.87</v>
       </c>
       <c r="G401" t="inlineStr">
         <is>
@@ -15706,7 +15706,7 @@
         <v>1</v>
       </c>
       <c r="F402" t="n">
-        <v>91.56</v>
+        <v>96.02</v>
       </c>
       <c r="G402" t="inlineStr">
         <is>
@@ -15744,7 +15744,7 @@
         <v>1</v>
       </c>
       <c r="F403" t="n">
-        <v>131.04</v>
+        <v>132.48</v>
       </c>
       <c r="G403" t="inlineStr">
         <is>
@@ -15782,7 +15782,7 @@
         <v>1</v>
       </c>
       <c r="F404" t="n">
-        <v>208.94</v>
+        <v>212.22</v>
       </c>
       <c r="G404" t="inlineStr">
         <is>
@@ -15820,7 +15820,7 @@
         <v>1</v>
       </c>
       <c r="F405" t="n">
-        <v>129.55</v>
+        <v>116.29</v>
       </c>
       <c r="G405" t="inlineStr">
         <is>
@@ -15858,7 +15858,7 @@
         <v>1</v>
       </c>
       <c r="F406" t="n">
-        <v>8.369999999999999</v>
+        <v>6.72</v>
       </c>
       <c r="G406" t="inlineStr">
         <is>
@@ -15896,7 +15896,7 @@
         <v>1</v>
       </c>
       <c r="F407" t="n">
-        <v>8.199999999999999</v>
+        <v>6.55</v>
       </c>
       <c r="G407" t="inlineStr">
         <is>
@@ -15934,7 +15934,7 @@
         <v>1</v>
       </c>
       <c r="F408" t="n">
-        <v>13.34</v>
+        <v>10.43</v>
       </c>
       <c r="G408" t="inlineStr">
         <is>
@@ -15972,7 +15972,7 @@
         <v>1</v>
       </c>
       <c r="F409" t="n">
-        <v>8.720000000000001</v>
+        <v>7.93</v>
       </c>
       <c r="G409" t="inlineStr">
         <is>
@@ -16010,7 +16010,7 @@
         <v>1</v>
       </c>
       <c r="F410" t="n">
-        <v>77.81999999999999</v>
+        <v>60.65</v>
       </c>
       <c r="G410" t="inlineStr">
         <is>
@@ -16048,7 +16048,7 @@
         <v>1</v>
       </c>
       <c r="F411" t="n">
-        <v>35.4</v>
+        <v>29.99</v>
       </c>
       <c r="G411" t="inlineStr">
         <is>
@@ -16086,7 +16086,7 @@
         <v>1</v>
       </c>
       <c r="F412" t="n">
-        <v>145.44</v>
+        <v>131.13</v>
       </c>
       <c r="G412" t="inlineStr">
         <is>
@@ -16124,7 +16124,7 @@
         <v>1</v>
       </c>
       <c r="F413" t="n">
-        <v>14.92</v>
+        <v>13.25</v>
       </c>
       <c r="G413" t="inlineStr">
         <is>
@@ -16162,7 +16162,7 @@
         <v>1</v>
       </c>
       <c r="F414" t="n">
-        <v>47.67</v>
+        <v>47.12</v>
       </c>
       <c r="G414" t="inlineStr">
         <is>
@@ -16238,7 +16238,7 @@
         <v>1</v>
       </c>
       <c r="F416" t="n">
-        <v>5.2</v>
+        <v>4.56</v>
       </c>
       <c r="G416" t="inlineStr">
         <is>
@@ -16276,7 +16276,7 @@
         <v>1</v>
       </c>
       <c r="F417" t="n">
-        <v>5.94</v>
+        <v>5.37</v>
       </c>
       <c r="G417" t="inlineStr">
         <is>
@@ -16314,7 +16314,7 @@
         <v>1</v>
       </c>
       <c r="F418" t="n">
-        <v>12.44</v>
+        <v>11.9</v>
       </c>
       <c r="G418" t="inlineStr">
         <is>
@@ -16352,7 +16352,7 @@
         <v>1</v>
       </c>
       <c r="F419" t="n">
-        <v>10.57</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="G419" t="inlineStr">
         <is>
@@ -16390,7 +16390,7 @@
         <v>1</v>
       </c>
       <c r="F420" t="n">
-        <v>55.41</v>
+        <v>43.32</v>
       </c>
       <c r="G420" t="inlineStr">
         <is>
@@ -16428,7 +16428,7 @@
         <v>1</v>
       </c>
       <c r="F421" t="n">
-        <v>159.8</v>
+        <v>132.07</v>
       </c>
       <c r="G421" t="inlineStr">
         <is>
@@ -16466,7 +16466,7 @@
         <v>1</v>
       </c>
       <c r="F422" t="n">
-        <v>65.88</v>
+        <v>58.2</v>
       </c>
       <c r="G422" t="inlineStr">
         <is>
@@ -16504,7 +16504,7 @@
         <v>1</v>
       </c>
       <c r="F423" t="n">
-        <v>61.8</v>
+        <v>52.74</v>
       </c>
       <c r="G423" t="inlineStr">
         <is>
@@ -16542,7 +16542,7 @@
         <v>1</v>
       </c>
       <c r="F424" t="n">
-        <v>50.08</v>
+        <v>48.62</v>
       </c>
       <c r="G424" t="inlineStr">
         <is>
@@ -16580,7 +16580,7 @@
         <v>1</v>
       </c>
       <c r="F425" t="n">
-        <v>72.27</v>
+        <v>68.67</v>
       </c>
       <c r="G425" t="inlineStr">
         <is>
@@ -16618,7 +16618,7 @@
         <v>1</v>
       </c>
       <c r="F426" t="n">
-        <v>46.8</v>
+        <v>44.15</v>
       </c>
       <c r="G426" t="inlineStr">
         <is>
@@ -16656,7 +16656,7 @@
         <v>1</v>
       </c>
       <c r="F427" t="n">
-        <v>50.83</v>
+        <v>48.93</v>
       </c>
       <c r="G427" t="inlineStr">
         <is>
@@ -16694,7 +16694,7 @@
         <v>1</v>
       </c>
       <c r="F428" t="n">
-        <v>153.26</v>
+        <v>151.94</v>
       </c>
       <c r="G428" t="inlineStr">
         <is>
@@ -16770,7 +16770,7 @@
         <v>1</v>
       </c>
       <c r="F430" t="n">
-        <v>58.73</v>
+        <v>57.08</v>
       </c>
       <c r="G430" t="inlineStr">
         <is>
@@ -16998,7 +16998,7 @@
         <v>1</v>
       </c>
       <c r="F436" t="n">
-        <v>119.8</v>
+        <v>119.02</v>
       </c>
       <c r="G436" t="inlineStr">
         <is>
@@ -17074,7 +17074,7 @@
         <v>1</v>
       </c>
       <c r="F438" t="n">
-        <v>44.1</v>
+        <v>43.82</v>
       </c>
       <c r="G438" t="inlineStr">
         <is>
@@ -17112,7 +17112,7 @@
         <v>1</v>
       </c>
       <c r="F439" t="n">
-        <v>293.57</v>
+        <v>295.33</v>
       </c>
       <c r="G439" t="inlineStr">
         <is>
@@ -17150,7 +17150,7 @@
         <v>1</v>
       </c>
       <c r="F440" t="n">
-        <v>253.28</v>
+        <v>228.18</v>
       </c>
       <c r="G440" t="inlineStr">
         <is>
@@ -17188,7 +17188,7 @@
         <v>1</v>
       </c>
       <c r="F441" t="n">
-        <v>137.74</v>
+        <v>121.32</v>
       </c>
       <c r="G441" t="inlineStr">
         <is>
@@ -17226,7 +17226,7 @@
         <v>1</v>
       </c>
       <c r="F442" t="n">
-        <v>168.39</v>
+        <v>145.02</v>
       </c>
       <c r="G442" t="inlineStr">
         <is>
@@ -17378,7 +17378,7 @@
         <v>1</v>
       </c>
       <c r="F446" t="n">
-        <v>60.42</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="G446" t="inlineStr">
         <is>
@@ -17416,7 +17416,7 @@
         <v>1</v>
       </c>
       <c r="F447" t="n">
-        <v>114.78</v>
+        <v>108.49</v>
       </c>
       <c r="G447" t="inlineStr">
         <is>
@@ -17454,7 +17454,7 @@
         <v>1</v>
       </c>
       <c r="F448" t="n">
-        <v>19.03</v>
+        <v>19.19</v>
       </c>
       <c r="G448" t="inlineStr">
         <is>
@@ -17530,7 +17530,7 @@
         <v>1</v>
       </c>
       <c r="F450" t="n">
-        <v>98.72</v>
+        <v>84.75</v>
       </c>
       <c r="G450" t="inlineStr">
         <is>
@@ -17568,7 +17568,7 @@
         <v>1</v>
       </c>
       <c r="F451" t="n">
-        <v>171.91</v>
+        <v>161.28</v>
       </c>
       <c r="G451" t="inlineStr">
         <is>
@@ -17606,7 +17606,7 @@
         <v>1</v>
       </c>
       <c r="F452" t="n">
-        <v>104.45</v>
+        <v>100.52</v>
       </c>
       <c r="G452" t="inlineStr">
         <is>
@@ -17644,7 +17644,7 @@
         <v>1</v>
       </c>
       <c r="F453" t="n">
-        <v>109.98</v>
+        <v>103.09</v>
       </c>
       <c r="G453" t="inlineStr">
         <is>
@@ -17682,7 +17682,7 @@
         <v>1</v>
       </c>
       <c r="F454" t="n">
-        <v>117.65</v>
+        <v>110.75</v>
       </c>
       <c r="G454" t="inlineStr">
         <is>
@@ -17720,7 +17720,7 @@
         <v>1</v>
       </c>
       <c r="F455" t="n">
-        <v>97.25</v>
+        <v>92.04000000000001</v>
       </c>
       <c r="G455" t="inlineStr">
         <is>
@@ -17796,7 +17796,7 @@
         <v>1</v>
       </c>
       <c r="F457" t="n">
-        <v>122.04</v>
+        <v>115.15</v>
       </c>
       <c r="G457" t="inlineStr">
         <is>
@@ -17834,7 +17834,7 @@
         <v>1</v>
       </c>
       <c r="F458" t="n">
-        <v>75.54000000000001</v>
+        <v>68.84</v>
       </c>
       <c r="G458" t="inlineStr">
         <is>
@@ -17872,7 +17872,7 @@
         <v>1</v>
       </c>
       <c r="F459" t="n">
-        <v>87.18000000000001</v>
+        <v>77.73</v>
       </c>
       <c r="G459" t="inlineStr">
         <is>
@@ -17910,7 +17910,7 @@
         <v>1</v>
       </c>
       <c r="F460" t="n">
-        <v>99.37</v>
+        <v>93.06999999999999</v>
       </c>
       <c r="G460" t="inlineStr">
         <is>
@@ -17948,7 +17948,7 @@
         <v>1</v>
       </c>
       <c r="F461" t="n">
-        <v>70.47</v>
+        <v>64.17</v>
       </c>
       <c r="G461" t="inlineStr">
         <is>
@@ -17986,7 +17986,7 @@
         <v>1</v>
       </c>
       <c r="F462" t="n">
-        <v>4.25</v>
+        <v>4.24</v>
       </c>
       <c r="G462" t="inlineStr">
         <is>
@@ -18024,7 +18024,7 @@
         <v>1</v>
       </c>
       <c r="F463" t="n">
-        <v>121.32</v>
+        <v>131.56</v>
       </c>
       <c r="G463" t="inlineStr">
         <is>
@@ -18062,7 +18062,7 @@
         <v>1</v>
       </c>
       <c r="F464" t="n">
-        <v>79.38</v>
+        <v>83.56</v>
       </c>
       <c r="G464" t="inlineStr">
         <is>
@@ -18100,7 +18100,7 @@
         <v>1</v>
       </c>
       <c r="F465" t="n">
-        <v>31.12</v>
+        <v>32.89</v>
       </c>
       <c r="G465" t="inlineStr">
         <is>
@@ -18214,7 +18214,7 @@
         <v>1</v>
       </c>
       <c r="F468" t="n">
-        <v>129.18</v>
+        <v>122.89</v>
       </c>
       <c r="G468" t="inlineStr">
         <is>
@@ -18252,7 +18252,7 @@
         <v>1</v>
       </c>
       <c r="F469" t="n">
-        <v>163.81</v>
+        <v>155.94</v>
       </c>
       <c r="G469" t="inlineStr">
         <is>
@@ -18290,7 +18290,7 @@
         <v>1</v>
       </c>
       <c r="F470" t="n">
-        <v>21.1</v>
+        <v>20.64</v>
       </c>
       <c r="G470" t="inlineStr">
         <is>
@@ -18328,7 +18328,7 @@
         <v>1</v>
       </c>
       <c r="F471" t="n">
-        <v>85.59</v>
+        <v>80.87</v>
       </c>
       <c r="G471" t="inlineStr">
         <is>
@@ -18366,7 +18366,7 @@
         <v>1</v>
       </c>
       <c r="F472" t="n">
-        <v>2.82</v>
+        <v>3.12</v>
       </c>
       <c r="G472" t="inlineStr">
         <is>
@@ -18404,7 +18404,7 @@
         <v>1</v>
       </c>
       <c r="F473" t="n">
-        <v>4.45</v>
+        <v>4.86</v>
       </c>
       <c r="G473" t="inlineStr">
         <is>
@@ -18480,7 +18480,7 @@
         <v>1</v>
       </c>
       <c r="F475" t="n">
-        <v>3.46</v>
+        <v>3.41</v>
       </c>
       <c r="G475" t="inlineStr">
         <is>
@@ -18518,7 +18518,7 @@
         <v>1</v>
       </c>
       <c r="F476" t="n">
-        <v>3.76</v>
+        <v>3.71</v>
       </c>
       <c r="G476" t="inlineStr">
         <is>
@@ -18556,7 +18556,7 @@
         <v>1</v>
       </c>
       <c r="F477" t="n">
-        <v>4.46</v>
+        <v>4.41</v>
       </c>
       <c r="G477" t="inlineStr">
         <is>
@@ -18594,7 +18594,7 @@
         <v>1</v>
       </c>
       <c r="F478" t="n">
-        <v>5.11</v>
+        <v>5.04</v>
       </c>
       <c r="G478" t="inlineStr">
         <is>
@@ -18632,7 +18632,7 @@
         <v>1</v>
       </c>
       <c r="F479" t="n">
-        <v>13.17</v>
+        <v>11.93</v>
       </c>
       <c r="G479" t="inlineStr">
         <is>
@@ -18670,7 +18670,7 @@
         <v>1</v>
       </c>
       <c r="F480" t="n">
-        <v>6.83</v>
+        <v>7.23</v>
       </c>
       <c r="G480" t="inlineStr">
         <is>
@@ -18708,7 +18708,7 @@
         <v>1</v>
       </c>
       <c r="F481" t="n">
-        <v>5.23</v>
+        <v>5.4</v>
       </c>
       <c r="G481" t="inlineStr">
         <is>
@@ -18746,7 +18746,7 @@
         <v>1</v>
       </c>
       <c r="F482" t="n">
-        <v>5.68</v>
+        <v>6.15</v>
       </c>
       <c r="G482" t="inlineStr">
         <is>
@@ -18822,7 +18822,7 @@
         <v>1</v>
       </c>
       <c r="F484" t="n">
-        <v>8.18</v>
+        <v>8.35</v>
       </c>
       <c r="G484" t="inlineStr">
         <is>
@@ -18860,7 +18860,7 @@
         <v>1</v>
       </c>
       <c r="F485" t="n">
-        <v>7.53</v>
+        <v>7.23</v>
       </c>
       <c r="G485" t="inlineStr">
         <is>
@@ -18936,7 +18936,7 @@
         <v>1</v>
       </c>
       <c r="F487" t="n">
-        <v>124.88</v>
+        <v>134.33</v>
       </c>
       <c r="G487" t="inlineStr">
         <is>
@@ -18974,7 +18974,7 @@
         <v>1</v>
       </c>
       <c r="F488" t="n">
-        <v>122.4</v>
+        <v>124.37</v>
       </c>
       <c r="G488" t="inlineStr">
         <is>
@@ -19012,7 +19012,7 @@
         <v>1</v>
       </c>
       <c r="F489" t="n">
-        <v>169.75</v>
+        <v>176.06</v>
       </c>
       <c r="G489" t="inlineStr">
         <is>
@@ -19050,7 +19050,7 @@
         <v>1</v>
       </c>
       <c r="F490" t="n">
-        <v>54.73</v>
+        <v>53.08</v>
       </c>
       <c r="G490" t="inlineStr">
         <is>
@@ -19126,7 +19126,7 @@
         <v>1</v>
       </c>
       <c r="F492" t="n">
-        <v>178.66</v>
+        <v>187.33</v>
       </c>
       <c r="G492" t="inlineStr">
         <is>
@@ -19164,7 +19164,7 @@
         <v>1</v>
       </c>
       <c r="F493" t="n">
-        <v>22.59</v>
+        <v>22.14</v>
       </c>
       <c r="G493" t="inlineStr">
         <is>
@@ -19202,7 +19202,7 @@
         <v>1</v>
       </c>
       <c r="F494" t="n">
-        <v>76.04000000000001</v>
+        <v>74.14</v>
       </c>
       <c r="G494" t="inlineStr">
         <is>
@@ -19240,7 +19240,7 @@
         <v>1</v>
       </c>
       <c r="F495" t="n">
-        <v>6.06</v>
+        <v>5.88</v>
       </c>
       <c r="G495" t="inlineStr">
         <is>
@@ -19278,7 +19278,7 @@
         <v>1</v>
       </c>
       <c r="F496" t="n">
-        <v>20.7</v>
+        <v>20.32</v>
       </c>
       <c r="G496" t="inlineStr">
         <is>
@@ -19316,7 +19316,7 @@
         <v>1</v>
       </c>
       <c r="F497" t="n">
-        <v>32.77</v>
+        <v>26.47</v>
       </c>
       <c r="G497" t="inlineStr">
         <is>
@@ -19392,7 +19392,7 @@
         <v>1</v>
       </c>
       <c r="F499" t="n">
-        <v>13.69</v>
+        <v>13.34</v>
       </c>
       <c r="G499" t="inlineStr">
         <is>
@@ -19430,7 +19430,7 @@
         <v>1</v>
       </c>
       <c r="F500" t="n">
-        <v>67</v>
+        <v>62.27</v>
       </c>
       <c r="G500" t="inlineStr">
         <is>
@@ -19506,7 +19506,7 @@
         <v>1</v>
       </c>
       <c r="F502" t="n">
-        <v>27.48</v>
+        <v>29.13</v>
       </c>
       <c r="G502" t="inlineStr">
         <is>
@@ -19544,7 +19544,7 @@
         <v>1</v>
       </c>
       <c r="F503" t="n">
-        <v>120.08</v>
+        <v>129.94</v>
       </c>
       <c r="G503" t="inlineStr">
         <is>
@@ -19582,7 +19582,7 @@
         <v>1</v>
       </c>
       <c r="F504" t="n">
-        <v>28.26</v>
+        <v>27.82</v>
       </c>
       <c r="G504" t="inlineStr">
         <is>
@@ -19696,7 +19696,7 @@
         <v>1</v>
       </c>
       <c r="F507" t="n">
-        <v>38.14</v>
+        <v>37.57</v>
       </c>
       <c r="G507" t="inlineStr">
         <is>
@@ -19734,7 +19734,7 @@
         <v>1</v>
       </c>
       <c r="F508" t="n">
-        <v>90.3</v>
+        <v>86.48</v>
       </c>
       <c r="G508" t="inlineStr">
         <is>
@@ -19772,7 +19772,7 @@
         <v>1</v>
       </c>
       <c r="F509" t="n">
-        <v>16.74</v>
+        <v>15.55</v>
       </c>
       <c r="G509" t="inlineStr">
         <is>
@@ -19810,7 +19810,7 @@
         <v>1</v>
       </c>
       <c r="F510" t="n">
-        <v>26.6</v>
+        <v>26.38</v>
       </c>
       <c r="G510" t="inlineStr">
         <is>
@@ -19848,7 +19848,7 @@
         <v>1</v>
       </c>
       <c r="F511" t="n">
-        <v>45.05</v>
+        <v>44.01</v>
       </c>
       <c r="G511" t="inlineStr">
         <is>
@@ -19886,7 +19886,7 @@
         <v>1</v>
       </c>
       <c r="F512" t="n">
-        <v>113.89</v>
+        <v>99.27</v>
       </c>
       <c r="G512" t="inlineStr">
         <is>
@@ -19924,7 +19924,7 @@
         <v>1</v>
       </c>
       <c r="F513" t="n">
-        <v>54.99</v>
+        <v>47.05</v>
       </c>
       <c r="G513" t="inlineStr">
         <is>
@@ -19962,7 +19962,7 @@
         <v>1</v>
       </c>
       <c r="F514" t="n">
-        <v>34.1</v>
+        <v>33.83</v>
       </c>
       <c r="G514" t="inlineStr">
         <is>
@@ -20000,7 +20000,7 @@
         <v>1</v>
       </c>
       <c r="F515" t="n">
-        <v>121.24</v>
+        <v>116.73</v>
       </c>
       <c r="G515" t="inlineStr">
         <is>
@@ -20114,7 +20114,7 @@
         <v>1</v>
       </c>
       <c r="F518" t="n">
-        <v>8.83</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="G518" t="inlineStr">
         <is>
@@ -20152,7 +20152,7 @@
         <v>1</v>
       </c>
       <c r="F519" t="n">
-        <v>48.45</v>
+        <v>38.36</v>
       </c>
       <c r="G519" t="inlineStr">
         <is>
@@ -20190,7 +20190,7 @@
         <v>1</v>
       </c>
       <c r="F520" t="n">
-        <v>35.78</v>
+        <v>35.06</v>
       </c>
       <c r="G520" t="inlineStr">
         <is>
@@ -20228,7 +20228,7 @@
         <v>1</v>
       </c>
       <c r="F521" t="n">
-        <v>94.47</v>
+        <v>91.77</v>
       </c>
       <c r="G521" t="inlineStr">
         <is>
@@ -20266,7 +20266,7 @@
         <v>1</v>
       </c>
       <c r="F522" t="n">
-        <v>63.92</v>
+        <v>56.52</v>
       </c>
       <c r="G522" t="inlineStr">
         <is>
@@ -20646,7 +20646,7 @@
         <v>1</v>
       </c>
       <c r="F532" t="n">
-        <v>9.15</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G532" t="inlineStr">
         <is>
@@ -20684,7 +20684,7 @@
         <v>1</v>
       </c>
       <c r="F533" t="n">
-        <v>23.78</v>
+        <v>20.63</v>
       </c>
       <c r="G533" t="inlineStr">
         <is>

</xml_diff>